<commit_message>
Calibrage sur comptes consolidés EDUSERVICES 4.0 (EBITDA 14,6%, D&A 6%, ~8,2k/étudiant)
CA/étudiant 8276 EUR (réel 8232) ; marge EBITDA N-1 14,6% (réel 14,6%) via
ajout des autres charges d'exploitation ; D&A porté à 6% du CA.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="C3" s="56">
-        <f>'02_Leviers'!$D$23</f>
+        <f>'02_Leviers'!$D$24</f>
         <v/>
       </c>
       <c r="E3" s="19" t="inlineStr">
@@ -2021,7 +2021,7 @@
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Coûts directs (ens.+pédago+mktg)</t>
+          <t xml:space="preserve">  Coûts directs (ens.+pédago+mktg+autres)</t>
         </is>
       </c>
       <c r="C8" s="16">
@@ -2029,7 +2029,7 @@
         <v/>
       </c>
       <c r="D8" s="17">
-        <f>-(SUM('08_Moteur'!$AJ$3:$AJ$60)+SUM('08_Moteur'!$AK$3:$AK$60)+SUM('08_Moteur'!$AL$3:$AL$60))</f>
+        <f>-(SUM('08_Moteur'!$AJ$3:$AJ$60)+SUM('08_Moteur'!$AK$3:$AK$60)+SUM('08_Moteur'!$AL$3:$AL$60)+'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)*SUM('08_Moteur'!$AD$3:$AD$60))</f>
         <v/>
       </c>
       <c r="E8" s="66">
@@ -6472,7 +6472,7 @@
         </is>
       </c>
       <c r="C8" s="17">
-        <f>0.01*'02_Leviers'!$D$20*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$AM$3:$AM$60)-0.01*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$H$3:$H$60*'08_Moteur'!$S$3:$S$60*(1+'08_Moteur'!$Y$3:$Y$60))</f>
+        <f>0.01*'02_Leviers'!$D$21*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$AM$3:$AM$60)-0.01*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$H$3:$H$60*'08_Moteur'!$S$3:$S$60*(1+'08_Moteur'!$Y$3:$Y$60))</f>
         <v/>
       </c>
       <c r="D8" s="73" t="inlineStr">
@@ -6737,7 +6737,7 @@
         <v/>
       </c>
       <c r="D14" s="53">
-        <f>'02_Leviers'!$D$19</f>
+        <f>'02_Leviers'!$D$20</f>
         <v/>
       </c>
       <c r="E14" s="53">
@@ -6756,7 +6756,7 @@
         <v/>
       </c>
       <c r="D15" s="76">
-        <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$G$3:$G$60*'08_Moteur'!$L$3:$L$60)*(1-'02_Leviers'!$D$19)</f>
+        <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$G$3:$G$60*'08_Moteur'!$L$3:$L$60)*(1-'02_Leviers'!$D$20)</f>
         <v/>
       </c>
       <c r="E15" s="77">
@@ -7126,7 +7126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G23"/>
+  <dimension ref="B2:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7504,24 +7504,24 @@
     <row r="19">
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Sécurisation N-1 — REPLI</t>
+          <t>Autres charges d'exploitation / étudiant</t>
         </is>
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D19" s="32" t="n">
-        <v>0.86</v>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="n">
+        <v>380</v>
       </c>
       <c r="E19" s="29" t="inlineStr">
         <is>
-          <t>repli (sinon mesuré par programme)</t>
+          <t>réel (achats, sous-traitance, IT)</t>
         </is>
       </c>
       <c r="F19" s="30" t="n"/>
-      <c r="G19" s="26">
+      <c r="G19" s="31">
         <f>D19</f>
         <v/>
       </c>
@@ -7529,24 +7529,24 @@
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Élasticité marketing — REPLI</t>
+          <t>Sécurisation N-1 — REPLI</t>
         </is>
       </c>
       <c r="C20" s="24" t="inlineStr">
         <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D20" s="33" t="n">
-        <v>0.5</v>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="n">
+        <v>0.86</v>
       </c>
       <c r="E20" s="29" t="inlineStr">
         <is>
-          <t>repli (sinon mesurée N-2/N-1)</t>
+          <t>repli (sinon mesuré par programme)</t>
         </is>
       </c>
       <c r="F20" s="30" t="n"/>
-      <c r="G20" s="34">
+      <c r="G20" s="26">
         <f>D20</f>
         <v/>
       </c>
@@ -7554,48 +7554,74 @@
     <row r="21">
       <c r="B21" s="8" t="inlineStr">
         <is>
+          <t>Élasticité marketing — REPLI</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>repli (sinon mesurée N-2/N-1)</t>
+        </is>
+      </c>
+      <c r="F21" s="30" t="n"/>
+      <c r="G21" s="34">
+        <f>D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="8" t="inlineStr">
+        <is>
           <t>Conversion candidature→inscrit — REPLI</t>
         </is>
       </c>
-      <c r="C21" s="24" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D21" s="32" t="n">
+      <c r="D22" s="32" t="n">
         <v>0.372</v>
       </c>
-      <c r="E21" s="29" t="inlineStr">
+      <c r="E22" s="29" t="inlineStr">
         <is>
           <t>repli (sinon mesurée par cellule)</t>
         </is>
       </c>
-      <c r="F21" s="30" t="n"/>
-      <c r="G21" s="26">
-        <f>D21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="19" t="inlineStr">
+      <c r="F22" s="30" t="n"/>
+      <c r="G22" s="26">
+        <f>D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>Driver d'allocation :</t>
         </is>
       </c>
-      <c r="D23" s="21" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>Effectifs</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B24:C24"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="E22:F22"/>
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="E18:F18"/>
@@ -7605,7 +7631,7 @@
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Cadrage,Optimiste,Prudent"</formula1>
     </dataValidation>
-    <dataValidation sqref="D23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Effectifs,Chiffre d'affaires,Surface m2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12812,7 +12838,7 @@
         <v>81600</v>
       </c>
       <c r="F66" s="43">
-        <f>IFERROR((C66/B66-1)/(E66/D66-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C66/B66-1)/(E66/D66-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G66" s="25" t="n">
@@ -12838,7 +12864,7 @@
         <v>92400</v>
       </c>
       <c r="F67" s="43">
-        <f>IFERROR((C67/B67-1)/(E67/D67-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C67/B67-1)/(E67/D67-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G67" s="25" t="n">
@@ -12864,7 +12890,7 @@
         <v>54080</v>
       </c>
       <c r="F68" s="43">
-        <f>IFERROR((C68/B68-1)/(E68/D68-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C68/B68-1)/(E68/D68-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G68" s="25" t="n">
@@ -12890,7 +12916,7 @@
         <v>60600</v>
       </c>
       <c r="F69" s="43">
-        <f>IFERROR((C69/B69-1)/(E69/D69-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C69/B69-1)/(E69/D69-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G69" s="25" t="n">
@@ -12916,7 +12942,7 @@
         <v>41600</v>
       </c>
       <c r="F70" s="43">
-        <f>IFERROR((C70/B70-1)/(E70/D70-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C70/B70-1)/(E70/D70-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G70" s="25" t="n">
@@ -12942,7 +12968,7 @@
         <v>16500</v>
       </c>
       <c r="F71" s="43">
-        <f>IFERROR((C71/B71-1)/(E71/D71-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C71/B71-1)/(E71/D71-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G71" s="25" t="n">
@@ -12968,7 +12994,7 @@
         <v>26240</v>
       </c>
       <c r="F72" s="43">
-        <f>IFERROR((C72/B72-1)/(E72/D72-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C72/B72-1)/(E72/D72-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G72" s="25" t="n">
@@ -12994,7 +13020,7 @@
         <v>27840</v>
       </c>
       <c r="F73" s="43">
-        <f>IFERROR((C73/B73-1)/(E73/D73-1),'02_Leviers'!$D$20)</f>
+        <f>IFERROR((C73/B73-1)/(E73/D73-1),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="G73" s="25" t="n">
@@ -13114,7 +13140,7 @@
         <v>2467250</v>
       </c>
       <c r="E4" s="42" t="n">
-        <v>1896050</v>
+        <v>1785470</v>
       </c>
       <c r="F4" s="42" t="n">
         <v>271000</v>
@@ -13127,7 +13153,7 @@
         <v/>
       </c>
       <c r="I4" s="42" t="n">
-        <v>74000</v>
+        <v>148000</v>
       </c>
       <c r="J4" s="40" t="n">
         <v>2328</v>
@@ -13155,7 +13181,7 @@
         <v>2102540</v>
       </c>
       <c r="E5" s="42" t="n">
-        <v>1625420</v>
+        <v>1531180</v>
       </c>
       <c r="F5" s="42" t="n">
         <v>231000</v>
@@ -13168,7 +13194,7 @@
         <v/>
       </c>
       <c r="I5" s="42" t="n">
-        <v>63000</v>
+        <v>126000</v>
       </c>
       <c r="J5" s="40" t="n">
         <v>1984</v>
@@ -13196,7 +13222,7 @@
         <v>1898640</v>
       </c>
       <c r="E6" s="42" t="n">
-        <v>1436400</v>
+        <v>1351280</v>
       </c>
       <c r="F6" s="42" t="n">
         <v>209000</v>
@@ -13209,7 +13235,7 @@
         <v/>
       </c>
       <c r="I6" s="42" t="n">
-        <v>57000</v>
+        <v>114000</v>
       </c>
       <c r="J6" s="40" t="n">
         <v>1792</v>
@@ -13237,7 +13263,7 @@
         <v>1619880</v>
       </c>
       <c r="E7" s="42" t="n">
-        <v>1177800</v>
+        <v>1105220</v>
       </c>
       <c r="F7" s="42" t="n">
         <v>178000</v>
@@ -13250,7 +13276,7 @@
         <v/>
       </c>
       <c r="I7" s="42" t="n">
-        <v>49000</v>
+        <v>97000</v>
       </c>
       <c r="J7" s="40" t="n">
         <v>1528</v>
@@ -13278,7 +13304,7 @@
         <v>2280350</v>
       </c>
       <c r="E8" s="42" t="n">
-        <v>1692040</v>
+        <v>1589820</v>
       </c>
       <c r="F8" s="42" t="n">
         <v>251000</v>
@@ -13291,7 +13317,7 @@
         <v/>
       </c>
       <c r="I8" s="42" t="n">
-        <v>68000</v>
+        <v>137000</v>
       </c>
       <c r="J8" s="40" t="n">
         <v>2152</v>
@@ -13319,7 +13345,7 @@
         <v>1585200</v>
       </c>
       <c r="E9" s="42" t="n">
-        <v>1097030</v>
+        <v>1025970</v>
       </c>
       <c r="F9" s="42" t="n">
         <v>174000</v>
@@ -13332,7 +13358,7 @@
         <v/>
       </c>
       <c r="I9" s="42" t="n">
-        <v>48000</v>
+        <v>95000</v>
       </c>
       <c r="J9" s="40" t="n">
         <v>1496</v>
@@ -13360,7 +13386,7 @@
         <v>1483250</v>
       </c>
       <c r="E10" s="42" t="n">
-        <v>1004320</v>
+        <v>937820</v>
       </c>
       <c r="F10" s="42" t="n">
         <v>163000</v>
@@ -13373,7 +13399,7 @@
         <v/>
       </c>
       <c r="I10" s="42" t="n">
-        <v>44000</v>
+        <v>89000</v>
       </c>
       <c r="J10" s="40" t="n">
         <v>1400</v>
@@ -13401,7 +13427,7 @@
         <v>1044500</v>
       </c>
       <c r="E11" s="42" t="n">
-        <v>784220</v>
+        <v>734820</v>
       </c>
       <c r="F11" s="42" t="n">
         <v>115000</v>
@@ -13414,7 +13440,7 @@
         <v/>
       </c>
       <c r="I11" s="42" t="n">
-        <v>31000</v>
+        <v>63000</v>
       </c>
       <c r="J11" s="40" t="n">
         <v>1040</v>
@@ -13442,7 +13468,7 @@
         <v>835600</v>
       </c>
       <c r="E12" s="42" t="n">
-        <v>618560</v>
+        <v>579040</v>
       </c>
       <c r="F12" s="42" t="n">
         <v>92000</v>
@@ -13455,7 +13481,7 @@
         <v/>
       </c>
       <c r="I12" s="42" t="n">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="J12" s="40" t="n">
         <v>832</v>
@@ -13483,7 +13509,7 @@
         <v>835600</v>
       </c>
       <c r="E13" s="42" t="n">
-        <v>618560</v>
+        <v>579040</v>
       </c>
       <c r="F13" s="42" t="n">
         <v>92000</v>
@@ -13496,7 +13522,7 @@
         <v/>
       </c>
       <c r="I13" s="42" t="n">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="J13" s="40" t="n">
         <v>832</v>
@@ -13524,7 +13550,7 @@
         <v>1130470</v>
       </c>
       <c r="E14" s="42" t="n">
-        <v>768030</v>
+        <v>711410</v>
       </c>
       <c r="F14" s="42" t="n">
         <v>124000</v>
@@ -13537,7 +13563,7 @@
         <v/>
       </c>
       <c r="I14" s="42" t="n">
-        <v>34000</v>
+        <v>68000</v>
       </c>
       <c r="J14" s="40" t="n">
         <v>1192</v>
@@ -13565,7 +13591,7 @@
         <v>887850</v>
       </c>
       <c r="E15" s="42" t="n">
-        <v>649480</v>
+        <v>605020</v>
       </c>
       <c r="F15" s="42" t="n">
         <v>98000</v>
@@ -13578,7 +13604,7 @@
         <v/>
       </c>
       <c r="I15" s="42" t="n">
-        <v>27000</v>
+        <v>53000</v>
       </c>
       <c r="J15" s="40" t="n">
         <v>936</v>
@@ -13606,7 +13632,7 @@
         <v>980230</v>
       </c>
       <c r="E16" s="42" t="n">
-        <v>722130</v>
+        <v>675770</v>
       </c>
       <c r="F16" s="42" t="n">
         <v>108000</v>
@@ -13619,7 +13645,7 @@
         <v/>
       </c>
       <c r="I16" s="42" t="n">
-        <v>29000</v>
+        <v>59000</v>
       </c>
       <c r="J16" s="40" t="n">
         <v>976</v>
@@ -13647,7 +13673,7 @@
         <v>835600</v>
       </c>
       <c r="E17" s="42" t="n">
-        <v>616960</v>
+        <v>577440</v>
       </c>
       <c r="F17" s="42" t="n">
         <v>92000</v>
@@ -13660,7 +13686,7 @@
         <v/>
       </c>
       <c r="I17" s="42" t="n">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="J17" s="40" t="n">
         <v>832</v>
@@ -14092,7 +14118,7 @@
         <v/>
       </c>
       <c r="X3" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C3,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C3,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y3" s="53">
@@ -14104,7 +14130,7 @@
         <v/>
       </c>
       <c r="AA3" s="53">
-        <f>IF(F3=1,IFERROR(H3/J3,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F3=1,IFERROR(H3/J3,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB3" s="51">
@@ -14128,7 +14154,7 @@
         <v/>
       </c>
       <c r="AG3" s="43">
-        <f>IF(E3="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C3,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C3,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E3="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C3,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C3,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH3" s="17">
@@ -14152,7 +14178,7 @@
         <v/>
       </c>
       <c r="AM3" s="55">
-        <f>AH3-AJ3-AK3-AL3</f>
+        <f>AH3-AJ3-AK3-AL3-AD3*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN3" s="53">
@@ -14262,7 +14288,7 @@
         <v/>
       </c>
       <c r="X4" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C4,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C4,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y4" s="53">
@@ -14274,7 +14300,7 @@
         <v/>
       </c>
       <c r="AA4" s="53">
-        <f>IF(F4=1,IFERROR(H4/J4,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F4=1,IFERROR(H4/J4,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB4" s="51">
@@ -14298,7 +14324,7 @@
         <v/>
       </c>
       <c r="AG4" s="43">
-        <f>IF(E4="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C4,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C4,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E4="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C4,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C4,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH4" s="17">
@@ -14322,7 +14348,7 @@
         <v/>
       </c>
       <c r="AM4" s="55">
-        <f>AH4-AJ4-AK4-AL4</f>
+        <f>AH4-AJ4-AK4-AL4-AD4*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN4" s="53">
@@ -14432,7 +14458,7 @@
         <v/>
       </c>
       <c r="X5" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C5,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C5,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y5" s="53">
@@ -14444,7 +14470,7 @@
         <v/>
       </c>
       <c r="AA5" s="53">
-        <f>IF(F5=1,IFERROR(H5/J5,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F5=1,IFERROR(H5/J5,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB5" s="51">
@@ -14468,7 +14494,7 @@
         <v/>
       </c>
       <c r="AG5" s="43">
-        <f>IF(E5="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C5,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C5,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E5="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C5,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C5,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH5" s="17">
@@ -14492,7 +14518,7 @@
         <v/>
       </c>
       <c r="AM5" s="55">
-        <f>AH5-AJ5-AK5-AL5</f>
+        <f>AH5-AJ5-AK5-AL5-AD5*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN5" s="53">
@@ -14602,7 +14628,7 @@
         <v/>
       </c>
       <c r="X6" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C6,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C6,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y6" s="53">
@@ -14614,7 +14640,7 @@
         <v/>
       </c>
       <c r="AA6" s="53">
-        <f>IF(F6=1,IFERROR(H6/J6,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F6=1,IFERROR(H6/J6,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB6" s="51">
@@ -14638,7 +14664,7 @@
         <v/>
       </c>
       <c r="AG6" s="43">
-        <f>IF(E6="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C6,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C6,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E6="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C6,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C6,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH6" s="17">
@@ -14662,7 +14688,7 @@
         <v/>
       </c>
       <c r="AM6" s="55">
-        <f>AH6-AJ6-AK6-AL6</f>
+        <f>AH6-AJ6-AK6-AL6-AD6*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN6" s="53">
@@ -14772,7 +14798,7 @@
         <v/>
       </c>
       <c r="X7" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C7,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C7,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y7" s="53">
@@ -14784,7 +14810,7 @@
         <v/>
       </c>
       <c r="AA7" s="53">
-        <f>IF(F7=1,IFERROR(H7/J7,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F7=1,IFERROR(H7/J7,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB7" s="51">
@@ -14808,7 +14834,7 @@
         <v/>
       </c>
       <c r="AG7" s="43">
-        <f>IF(E7="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C7,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C7,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E7="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C7,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C7,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH7" s="17">
@@ -14832,7 +14858,7 @@
         <v/>
       </c>
       <c r="AM7" s="55">
-        <f>AH7-AJ7-AK7-AL7</f>
+        <f>AH7-AJ7-AK7-AL7-AD7*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN7" s="53">
@@ -14942,7 +14968,7 @@
         <v/>
       </c>
       <c r="X8" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C8,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C8,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y8" s="53">
@@ -14954,7 +14980,7 @@
         <v/>
       </c>
       <c r="AA8" s="53">
-        <f>IF(F8=1,IFERROR(H8/J8,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F8=1,IFERROR(H8/J8,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB8" s="51">
@@ -14978,7 +15004,7 @@
         <v/>
       </c>
       <c r="AG8" s="43">
-        <f>IF(E8="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C8,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C8,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E8="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C8,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C8,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH8" s="17">
@@ -15002,7 +15028,7 @@
         <v/>
       </c>
       <c r="AM8" s="55">
-        <f>AH8-AJ8-AK8-AL8</f>
+        <f>AH8-AJ8-AK8-AL8-AD8*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN8" s="53">
@@ -15112,7 +15138,7 @@
         <v/>
       </c>
       <c r="X9" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C9,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C9,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y9" s="53">
@@ -15124,7 +15150,7 @@
         <v/>
       </c>
       <c r="AA9" s="53">
-        <f>IF(F9=1,IFERROR(H9/J9,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F9=1,IFERROR(H9/J9,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB9" s="51">
@@ -15148,7 +15174,7 @@
         <v/>
       </c>
       <c r="AG9" s="43">
-        <f>IF(E9="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C9,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C9,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E9="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C9,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C9,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH9" s="17">
@@ -15172,7 +15198,7 @@
         <v/>
       </c>
       <c r="AM9" s="55">
-        <f>AH9-AJ9-AK9-AL9</f>
+        <f>AH9-AJ9-AK9-AL9-AD9*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN9" s="53">
@@ -15282,7 +15308,7 @@
         <v/>
       </c>
       <c r="X10" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C10,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C10,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y10" s="53">
@@ -15294,7 +15320,7 @@
         <v/>
       </c>
       <c r="AA10" s="53">
-        <f>IF(F10=1,IFERROR(H10/J10,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F10=1,IFERROR(H10/J10,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB10" s="51">
@@ -15318,7 +15344,7 @@
         <v/>
       </c>
       <c r="AG10" s="43">
-        <f>IF(E10="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C10,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C10,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E10="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C10,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C10,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH10" s="17">
@@ -15342,7 +15368,7 @@
         <v/>
       </c>
       <c r="AM10" s="55">
-        <f>AH10-AJ10-AK10-AL10</f>
+        <f>AH10-AJ10-AK10-AL10-AD10*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN10" s="53">
@@ -15452,7 +15478,7 @@
         <v/>
       </c>
       <c r="X11" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C11,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C11,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y11" s="53">
@@ -15464,7 +15490,7 @@
         <v/>
       </c>
       <c r="AA11" s="53">
-        <f>IF(F11=1,IFERROR(H11/J11,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F11=1,IFERROR(H11/J11,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB11" s="51">
@@ -15488,7 +15514,7 @@
         <v/>
       </c>
       <c r="AG11" s="43">
-        <f>IF(E11="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C11,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C11,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E11="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C11,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C11,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH11" s="17">
@@ -15512,7 +15538,7 @@
         <v/>
       </c>
       <c r="AM11" s="55">
-        <f>AH11-AJ11-AK11-AL11</f>
+        <f>AH11-AJ11-AK11-AL11-AD11*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN11" s="53">
@@ -15622,7 +15648,7 @@
         <v/>
       </c>
       <c r="X12" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C12,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C12,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y12" s="53">
@@ -15634,7 +15660,7 @@
         <v/>
       </c>
       <c r="AA12" s="53">
-        <f>IF(F12=1,IFERROR(H12/J12,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F12=1,IFERROR(H12/J12,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB12" s="51">
@@ -15658,7 +15684,7 @@
         <v/>
       </c>
       <c r="AG12" s="43">
-        <f>IF(E12="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C12,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C12,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E12="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C12,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C12,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH12" s="17">
@@ -15682,7 +15708,7 @@
         <v/>
       </c>
       <c r="AM12" s="55">
-        <f>AH12-AJ12-AK12-AL12</f>
+        <f>AH12-AJ12-AK12-AL12-AD12*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN12" s="53">
@@ -15792,7 +15818,7 @@
         <v/>
       </c>
       <c r="X13" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C13,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C13,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y13" s="53">
@@ -15804,7 +15830,7 @@
         <v/>
       </c>
       <c r="AA13" s="53">
-        <f>IF(F13=1,IFERROR(H13/J13,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F13=1,IFERROR(H13/J13,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB13" s="51">
@@ -15828,7 +15854,7 @@
         <v/>
       </c>
       <c r="AG13" s="43">
-        <f>IF(E13="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C13,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C13,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E13="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C13,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C13,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH13" s="17">
@@ -15852,7 +15878,7 @@
         <v/>
       </c>
       <c r="AM13" s="55">
-        <f>AH13-AJ13-AK13-AL13</f>
+        <f>AH13-AJ13-AK13-AL13-AD13*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN13" s="53">
@@ -15962,7 +15988,7 @@
         <v/>
       </c>
       <c r="X14" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C14,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C14,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y14" s="53">
@@ -15974,7 +16000,7 @@
         <v/>
       </c>
       <c r="AA14" s="53">
-        <f>IF(F14=1,IFERROR(H14/J14,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F14=1,IFERROR(H14/J14,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB14" s="51">
@@ -15998,7 +16024,7 @@
         <v/>
       </c>
       <c r="AG14" s="43">
-        <f>IF(E14="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C14,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C14,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E14="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C14,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C14,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH14" s="17">
@@ -16022,7 +16048,7 @@
         <v/>
       </c>
       <c r="AM14" s="55">
-        <f>AH14-AJ14-AK14-AL14</f>
+        <f>AH14-AJ14-AK14-AL14-AD14*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN14" s="53">
@@ -16132,7 +16158,7 @@
         <v/>
       </c>
       <c r="X15" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C15,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C15,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y15" s="53">
@@ -16144,7 +16170,7 @@
         <v/>
       </c>
       <c r="AA15" s="53">
-        <f>IF(F15=1,IFERROR(H15/J15,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F15=1,IFERROR(H15/J15,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB15" s="51">
@@ -16168,7 +16194,7 @@
         <v/>
       </c>
       <c r="AG15" s="43">
-        <f>IF(E15="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C15,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C15,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E15="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C15,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C15,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH15" s="17">
@@ -16192,7 +16218,7 @@
         <v/>
       </c>
       <c r="AM15" s="55">
-        <f>AH15-AJ15-AK15-AL15</f>
+        <f>AH15-AJ15-AK15-AL15-AD15*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN15" s="53">
@@ -16302,7 +16328,7 @@
         <v/>
       </c>
       <c r="X16" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C16,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C16,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y16" s="53">
@@ -16314,7 +16340,7 @@
         <v/>
       </c>
       <c r="AA16" s="53">
-        <f>IF(F16=1,IFERROR(H16/J16,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F16=1,IFERROR(H16/J16,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB16" s="51">
@@ -16338,7 +16364,7 @@
         <v/>
       </c>
       <c r="AG16" s="43">
-        <f>IF(E16="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C16,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C16,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E16="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C16,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C16,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH16" s="17">
@@ -16362,7 +16388,7 @@
         <v/>
       </c>
       <c r="AM16" s="55">
-        <f>AH16-AJ16-AK16-AL16</f>
+        <f>AH16-AJ16-AK16-AL16-AD16*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN16" s="53">
@@ -16472,7 +16498,7 @@
         <v/>
       </c>
       <c r="X17" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C17,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C17,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y17" s="53">
@@ -16484,7 +16510,7 @@
         <v/>
       </c>
       <c r="AA17" s="53">
-        <f>IF(F17=1,IFERROR(H17/J17,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F17=1,IFERROR(H17/J17,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB17" s="51">
@@ -16508,7 +16534,7 @@
         <v/>
       </c>
       <c r="AG17" s="43">
-        <f>IF(E17="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C17,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C17,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E17="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C17,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C17,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH17" s="17">
@@ -16532,7 +16558,7 @@
         <v/>
       </c>
       <c r="AM17" s="55">
-        <f>AH17-AJ17-AK17-AL17</f>
+        <f>AH17-AJ17-AK17-AL17-AD17*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN17" s="53">
@@ -16642,7 +16668,7 @@
         <v/>
       </c>
       <c r="X18" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C18,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C18,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y18" s="53">
@@ -16654,7 +16680,7 @@
         <v/>
       </c>
       <c r="AA18" s="53">
-        <f>IF(F18=1,IFERROR(H18/J18,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F18=1,IFERROR(H18/J18,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB18" s="51">
@@ -16678,7 +16704,7 @@
         <v/>
       </c>
       <c r="AG18" s="43">
-        <f>IF(E18="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C18,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C18,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E18="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C18,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C18,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH18" s="17">
@@ -16702,7 +16728,7 @@
         <v/>
       </c>
       <c r="AM18" s="55">
-        <f>AH18-AJ18-AK18-AL18</f>
+        <f>AH18-AJ18-AK18-AL18-AD18*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN18" s="53">
@@ -16812,7 +16838,7 @@
         <v/>
       </c>
       <c r="X19" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C19,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C19,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y19" s="53">
@@ -16824,7 +16850,7 @@
         <v/>
       </c>
       <c r="AA19" s="53">
-        <f>IF(F19=1,IFERROR(H19/J19,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F19=1,IFERROR(H19/J19,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB19" s="51">
@@ -16848,7 +16874,7 @@
         <v/>
       </c>
       <c r="AG19" s="43">
-        <f>IF(E19="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C19,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C19,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E19="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C19,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C19,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH19" s="17">
@@ -16872,7 +16898,7 @@
         <v/>
       </c>
       <c r="AM19" s="55">
-        <f>AH19-AJ19-AK19-AL19</f>
+        <f>AH19-AJ19-AK19-AL19-AD19*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN19" s="53">
@@ -16982,7 +17008,7 @@
         <v/>
       </c>
       <c r="X20" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C20,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C20,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y20" s="53">
@@ -16994,7 +17020,7 @@
         <v/>
       </c>
       <c r="AA20" s="53">
-        <f>IF(F20=1,IFERROR(H20/J20,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F20=1,IFERROR(H20/J20,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB20" s="51">
@@ -17018,7 +17044,7 @@
         <v/>
       </c>
       <c r="AG20" s="43">
-        <f>IF(E20="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C20,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C20,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E20="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C20,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C20,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH20" s="17">
@@ -17042,7 +17068,7 @@
         <v/>
       </c>
       <c r="AM20" s="55">
-        <f>AH20-AJ20-AK20-AL20</f>
+        <f>AH20-AJ20-AK20-AL20-AD20*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN20" s="53">
@@ -17152,7 +17178,7 @@
         <v/>
       </c>
       <c r="X21" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C21,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C21,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y21" s="53">
@@ -17164,7 +17190,7 @@
         <v/>
       </c>
       <c r="AA21" s="53">
-        <f>IF(F21=1,IFERROR(H21/J21,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F21=1,IFERROR(H21/J21,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB21" s="51">
@@ -17188,7 +17214,7 @@
         <v/>
       </c>
       <c r="AG21" s="43">
-        <f>IF(E21="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C21,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C21,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E21="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C21,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C21,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH21" s="17">
@@ -17212,7 +17238,7 @@
         <v/>
       </c>
       <c r="AM21" s="55">
-        <f>AH21-AJ21-AK21-AL21</f>
+        <f>AH21-AJ21-AK21-AL21-AD21*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN21" s="53">
@@ -17322,7 +17348,7 @@
         <v/>
       </c>
       <c r="X22" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C22,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C22,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y22" s="53">
@@ -17334,7 +17360,7 @@
         <v/>
       </c>
       <c r="AA22" s="53">
-        <f>IF(F22=1,IFERROR(H22/J22,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F22=1,IFERROR(H22/J22,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB22" s="51">
@@ -17358,7 +17384,7 @@
         <v/>
       </c>
       <c r="AG22" s="43">
-        <f>IF(E22="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C22,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C22,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E22="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C22,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C22,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH22" s="17">
@@ -17382,7 +17408,7 @@
         <v/>
       </c>
       <c r="AM22" s="55">
-        <f>AH22-AJ22-AK22-AL22</f>
+        <f>AH22-AJ22-AK22-AL22-AD22*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN22" s="53">
@@ -17492,7 +17518,7 @@
         <v/>
       </c>
       <c r="X23" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C23,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C23,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y23" s="53">
@@ -17504,7 +17530,7 @@
         <v/>
       </c>
       <c r="AA23" s="53">
-        <f>IF(F23=1,IFERROR(H23/J23,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F23=1,IFERROR(H23/J23,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB23" s="51">
@@ -17528,7 +17554,7 @@
         <v/>
       </c>
       <c r="AG23" s="43">
-        <f>IF(E23="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C23,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C23,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E23="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C23,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C23,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH23" s="17">
@@ -17552,7 +17578,7 @@
         <v/>
       </c>
       <c r="AM23" s="55">
-        <f>AH23-AJ23-AK23-AL23</f>
+        <f>AH23-AJ23-AK23-AL23-AD23*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN23" s="53">
@@ -17662,7 +17688,7 @@
         <v/>
       </c>
       <c r="X24" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C24,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C24,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y24" s="53">
@@ -17674,7 +17700,7 @@
         <v/>
       </c>
       <c r="AA24" s="53">
-        <f>IF(F24=1,IFERROR(H24/J24,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F24=1,IFERROR(H24/J24,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB24" s="51">
@@ -17698,7 +17724,7 @@
         <v/>
       </c>
       <c r="AG24" s="43">
-        <f>IF(E24="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C24,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C24,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E24="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C24,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C24,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH24" s="17">
@@ -17722,7 +17748,7 @@
         <v/>
       </c>
       <c r="AM24" s="55">
-        <f>AH24-AJ24-AK24-AL24</f>
+        <f>AH24-AJ24-AK24-AL24-AD24*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN24" s="53">
@@ -17832,7 +17858,7 @@
         <v/>
       </c>
       <c r="X25" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C25,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C25,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y25" s="53">
@@ -17844,7 +17870,7 @@
         <v/>
       </c>
       <c r="AA25" s="53">
-        <f>IF(F25=1,IFERROR(H25/J25,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F25=1,IFERROR(H25/J25,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB25" s="51">
@@ -17868,7 +17894,7 @@
         <v/>
       </c>
       <c r="AG25" s="43">
-        <f>IF(E25="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C25,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C25,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E25="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C25,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C25,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH25" s="17">
@@ -17892,7 +17918,7 @@
         <v/>
       </c>
       <c r="AM25" s="55">
-        <f>AH25-AJ25-AK25-AL25</f>
+        <f>AH25-AJ25-AK25-AL25-AD25*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN25" s="53">
@@ -18002,7 +18028,7 @@
         <v/>
       </c>
       <c r="X26" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C26,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C26,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y26" s="53">
@@ -18014,7 +18040,7 @@
         <v/>
       </c>
       <c r="AA26" s="53">
-        <f>IF(F26=1,IFERROR(H26/J26,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F26=1,IFERROR(H26/J26,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB26" s="51">
@@ -18038,7 +18064,7 @@
         <v/>
       </c>
       <c r="AG26" s="43">
-        <f>IF(E26="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C26,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C26,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E26="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C26,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C26,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH26" s="17">
@@ -18062,7 +18088,7 @@
         <v/>
       </c>
       <c r="AM26" s="55">
-        <f>AH26-AJ26-AK26-AL26</f>
+        <f>AH26-AJ26-AK26-AL26-AD26*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN26" s="53">
@@ -18172,7 +18198,7 @@
         <v/>
       </c>
       <c r="X27" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C27,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C27,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y27" s="53">
@@ -18184,7 +18210,7 @@
         <v/>
       </c>
       <c r="AA27" s="53">
-        <f>IF(F27=1,IFERROR(H27/J27,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F27=1,IFERROR(H27/J27,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB27" s="51">
@@ -18208,7 +18234,7 @@
         <v/>
       </c>
       <c r="AG27" s="43">
-        <f>IF(E27="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C27,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C27,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E27="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C27,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C27,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH27" s="17">
@@ -18232,7 +18258,7 @@
         <v/>
       </c>
       <c r="AM27" s="55">
-        <f>AH27-AJ27-AK27-AL27</f>
+        <f>AH27-AJ27-AK27-AL27-AD27*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN27" s="53">
@@ -18342,7 +18368,7 @@
         <v/>
       </c>
       <c r="X28" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C28,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C28,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y28" s="53">
@@ -18354,7 +18380,7 @@
         <v/>
       </c>
       <c r="AA28" s="53">
-        <f>IF(F28=1,IFERROR(H28/J28,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F28=1,IFERROR(H28/J28,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB28" s="51">
@@ -18378,7 +18404,7 @@
         <v/>
       </c>
       <c r="AG28" s="43">
-        <f>IF(E28="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C28,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C28,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E28="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C28,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C28,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH28" s="17">
@@ -18402,7 +18428,7 @@
         <v/>
       </c>
       <c r="AM28" s="55">
-        <f>AH28-AJ28-AK28-AL28</f>
+        <f>AH28-AJ28-AK28-AL28-AD28*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN28" s="53">
@@ -18512,7 +18538,7 @@
         <v/>
       </c>
       <c r="X29" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C29,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C29,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y29" s="53">
@@ -18524,7 +18550,7 @@
         <v/>
       </c>
       <c r="AA29" s="53">
-        <f>IF(F29=1,IFERROR(H29/J29,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F29=1,IFERROR(H29/J29,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB29" s="51">
@@ -18548,7 +18574,7 @@
         <v/>
       </c>
       <c r="AG29" s="43">
-        <f>IF(E29="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C29,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C29,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E29="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C29,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C29,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH29" s="17">
@@ -18572,7 +18598,7 @@
         <v/>
       </c>
       <c r="AM29" s="55">
-        <f>AH29-AJ29-AK29-AL29</f>
+        <f>AH29-AJ29-AK29-AL29-AD29*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN29" s="53">
@@ -18682,7 +18708,7 @@
         <v/>
       </c>
       <c r="X30" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C30,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C30,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y30" s="53">
@@ -18694,7 +18720,7 @@
         <v/>
       </c>
       <c r="AA30" s="53">
-        <f>IF(F30=1,IFERROR(H30/J30,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F30=1,IFERROR(H30/J30,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB30" s="51">
@@ -18718,7 +18744,7 @@
         <v/>
       </c>
       <c r="AG30" s="43">
-        <f>IF(E30="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C30,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C30,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E30="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C30,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C30,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH30" s="17">
@@ -18742,7 +18768,7 @@
         <v/>
       </c>
       <c r="AM30" s="55">
-        <f>AH30-AJ30-AK30-AL30</f>
+        <f>AH30-AJ30-AK30-AL30-AD30*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN30" s="53">
@@ -18852,7 +18878,7 @@
         <v/>
       </c>
       <c r="X31" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C31,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C31,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y31" s="53">
@@ -18864,7 +18890,7 @@
         <v/>
       </c>
       <c r="AA31" s="53">
-        <f>IF(F31=1,IFERROR(H31/J31,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F31=1,IFERROR(H31/J31,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB31" s="51">
@@ -18888,7 +18914,7 @@
         <v/>
       </c>
       <c r="AG31" s="43">
-        <f>IF(E31="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C31,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C31,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E31="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C31,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C31,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH31" s="17">
@@ -18912,7 +18938,7 @@
         <v/>
       </c>
       <c r="AM31" s="55">
-        <f>AH31-AJ31-AK31-AL31</f>
+        <f>AH31-AJ31-AK31-AL31-AD31*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN31" s="53">
@@ -19022,7 +19048,7 @@
         <v/>
       </c>
       <c r="X32" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C32,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C32,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y32" s="53">
@@ -19034,7 +19060,7 @@
         <v/>
       </c>
       <c r="AA32" s="53">
-        <f>IF(F32=1,IFERROR(H32/J32,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F32=1,IFERROR(H32/J32,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB32" s="51">
@@ -19058,7 +19084,7 @@
         <v/>
       </c>
       <c r="AG32" s="43">
-        <f>IF(E32="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C32,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C32,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E32="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C32,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C32,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH32" s="17">
@@ -19082,7 +19108,7 @@
         <v/>
       </c>
       <c r="AM32" s="55">
-        <f>AH32-AJ32-AK32-AL32</f>
+        <f>AH32-AJ32-AK32-AL32-AD32*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN32" s="53">
@@ -19192,7 +19218,7 @@
         <v/>
       </c>
       <c r="X33" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C33,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C33,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y33" s="53">
@@ -19204,7 +19230,7 @@
         <v/>
       </c>
       <c r="AA33" s="53">
-        <f>IF(F33=1,IFERROR(H33/J33,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F33=1,IFERROR(H33/J33,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB33" s="51">
@@ -19228,7 +19254,7 @@
         <v/>
       </c>
       <c r="AG33" s="43">
-        <f>IF(E33="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C33,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C33,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E33="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C33,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C33,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH33" s="17">
@@ -19252,7 +19278,7 @@
         <v/>
       </c>
       <c r="AM33" s="55">
-        <f>AH33-AJ33-AK33-AL33</f>
+        <f>AH33-AJ33-AK33-AL33-AD33*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN33" s="53">
@@ -19362,7 +19388,7 @@
         <v/>
       </c>
       <c r="X34" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C34,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C34,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y34" s="53">
@@ -19374,7 +19400,7 @@
         <v/>
       </c>
       <c r="AA34" s="53">
-        <f>IF(F34=1,IFERROR(H34/J34,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F34=1,IFERROR(H34/J34,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB34" s="51">
@@ -19398,7 +19424,7 @@
         <v/>
       </c>
       <c r="AG34" s="43">
-        <f>IF(E34="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C34,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C34,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E34="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C34,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C34,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH34" s="17">
@@ -19422,7 +19448,7 @@
         <v/>
       </c>
       <c r="AM34" s="55">
-        <f>AH34-AJ34-AK34-AL34</f>
+        <f>AH34-AJ34-AK34-AL34-AD34*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN34" s="53">
@@ -19532,7 +19558,7 @@
         <v/>
       </c>
       <c r="X35" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C35,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C35,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y35" s="53">
@@ -19544,7 +19570,7 @@
         <v/>
       </c>
       <c r="AA35" s="53">
-        <f>IF(F35=1,IFERROR(H35/J35,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F35=1,IFERROR(H35/J35,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB35" s="51">
@@ -19568,7 +19594,7 @@
         <v/>
       </c>
       <c r="AG35" s="43">
-        <f>IF(E35="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C35,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C35,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E35="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C35,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C35,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH35" s="17">
@@ -19592,7 +19618,7 @@
         <v/>
       </c>
       <c r="AM35" s="55">
-        <f>AH35-AJ35-AK35-AL35</f>
+        <f>AH35-AJ35-AK35-AL35-AD35*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN35" s="53">
@@ -19702,7 +19728,7 @@
         <v/>
       </c>
       <c r="X36" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C36,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C36,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y36" s="53">
@@ -19714,7 +19740,7 @@
         <v/>
       </c>
       <c r="AA36" s="53">
-        <f>IF(F36=1,IFERROR(H36/J36,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F36=1,IFERROR(H36/J36,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB36" s="51">
@@ -19738,7 +19764,7 @@
         <v/>
       </c>
       <c r="AG36" s="43">
-        <f>IF(E36="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C36,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C36,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E36="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C36,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C36,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH36" s="17">
@@ -19762,7 +19788,7 @@
         <v/>
       </c>
       <c r="AM36" s="55">
-        <f>AH36-AJ36-AK36-AL36</f>
+        <f>AH36-AJ36-AK36-AL36-AD36*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN36" s="53">
@@ -19872,7 +19898,7 @@
         <v/>
       </c>
       <c r="X37" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C37,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C37,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y37" s="53">
@@ -19884,7 +19910,7 @@
         <v/>
       </c>
       <c r="AA37" s="53">
-        <f>IF(F37=1,IFERROR(H37/J37,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F37=1,IFERROR(H37/J37,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB37" s="51">
@@ -19908,7 +19934,7 @@
         <v/>
       </c>
       <c r="AG37" s="43">
-        <f>IF(E37="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C37,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C37,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E37="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C37,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C37,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH37" s="17">
@@ -19932,7 +19958,7 @@
         <v/>
       </c>
       <c r="AM37" s="55">
-        <f>AH37-AJ37-AK37-AL37</f>
+        <f>AH37-AJ37-AK37-AL37-AD37*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN37" s="53">
@@ -20042,7 +20068,7 @@
         <v/>
       </c>
       <c r="X38" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C38,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C38,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y38" s="53">
@@ -20054,7 +20080,7 @@
         <v/>
       </c>
       <c r="AA38" s="53">
-        <f>IF(F38=1,IFERROR(H38/J38,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F38=1,IFERROR(H38/J38,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB38" s="51">
@@ -20078,7 +20104,7 @@
         <v/>
       </c>
       <c r="AG38" s="43">
-        <f>IF(E38="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C38,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C38,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E38="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C38,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C38,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH38" s="17">
@@ -20102,7 +20128,7 @@
         <v/>
       </c>
       <c r="AM38" s="55">
-        <f>AH38-AJ38-AK38-AL38</f>
+        <f>AH38-AJ38-AK38-AL38-AD38*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN38" s="53">
@@ -20212,7 +20238,7 @@
         <v/>
       </c>
       <c r="X39" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C39,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C39,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y39" s="53">
@@ -20224,7 +20250,7 @@
         <v/>
       </c>
       <c r="AA39" s="53">
-        <f>IF(F39=1,IFERROR(H39/J39,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F39=1,IFERROR(H39/J39,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB39" s="51">
@@ -20248,7 +20274,7 @@
         <v/>
       </c>
       <c r="AG39" s="43">
-        <f>IF(E39="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C39,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C39,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E39="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C39,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C39,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH39" s="17">
@@ -20272,7 +20298,7 @@
         <v/>
       </c>
       <c r="AM39" s="55">
-        <f>AH39-AJ39-AK39-AL39</f>
+        <f>AH39-AJ39-AK39-AL39-AD39*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN39" s="53">
@@ -20382,7 +20408,7 @@
         <v/>
       </c>
       <c r="X40" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C40,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C40,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y40" s="53">
@@ -20394,7 +20420,7 @@
         <v/>
       </c>
       <c r="AA40" s="53">
-        <f>IF(F40=1,IFERROR(H40/J40,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F40=1,IFERROR(H40/J40,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB40" s="51">
@@ -20418,7 +20444,7 @@
         <v/>
       </c>
       <c r="AG40" s="43">
-        <f>IF(E40="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C40,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C40,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E40="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C40,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C40,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH40" s="17">
@@ -20442,7 +20468,7 @@
         <v/>
       </c>
       <c r="AM40" s="55">
-        <f>AH40-AJ40-AK40-AL40</f>
+        <f>AH40-AJ40-AK40-AL40-AD40*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN40" s="53">
@@ -20552,7 +20578,7 @@
         <v/>
       </c>
       <c r="X41" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C41,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C41,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y41" s="53">
@@ -20564,7 +20590,7 @@
         <v/>
       </c>
       <c r="AA41" s="53">
-        <f>IF(F41=1,IFERROR(H41/J41,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F41=1,IFERROR(H41/J41,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB41" s="51">
@@ -20588,7 +20614,7 @@
         <v/>
       </c>
       <c r="AG41" s="43">
-        <f>IF(E41="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C41,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C41,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E41="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C41,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C41,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH41" s="17">
@@ -20612,7 +20638,7 @@
         <v/>
       </c>
       <c r="AM41" s="55">
-        <f>AH41-AJ41-AK41-AL41</f>
+        <f>AH41-AJ41-AK41-AL41-AD41*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN41" s="53">
@@ -20722,7 +20748,7 @@
         <v/>
       </c>
       <c r="X42" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C42,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C42,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y42" s="53">
@@ -20734,7 +20760,7 @@
         <v/>
       </c>
       <c r="AA42" s="53">
-        <f>IF(F42=1,IFERROR(H42/J42,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F42=1,IFERROR(H42/J42,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB42" s="51">
@@ -20758,7 +20784,7 @@
         <v/>
       </c>
       <c r="AG42" s="43">
-        <f>IF(E42="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C42,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C42,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E42="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C42,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C42,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH42" s="17">
@@ -20782,7 +20808,7 @@
         <v/>
       </c>
       <c r="AM42" s="55">
-        <f>AH42-AJ42-AK42-AL42</f>
+        <f>AH42-AJ42-AK42-AL42-AD42*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN42" s="53">
@@ -20892,7 +20918,7 @@
         <v/>
       </c>
       <c r="X43" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C43,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C43,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y43" s="53">
@@ -20904,7 +20930,7 @@
         <v/>
       </c>
       <c r="AA43" s="53">
-        <f>IF(F43=1,IFERROR(H43/J43,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F43=1,IFERROR(H43/J43,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB43" s="51">
@@ -20928,7 +20954,7 @@
         <v/>
       </c>
       <c r="AG43" s="43">
-        <f>IF(E43="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C43,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C43,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E43="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C43,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C43,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH43" s="17">
@@ -20952,7 +20978,7 @@
         <v/>
       </c>
       <c r="AM43" s="55">
-        <f>AH43-AJ43-AK43-AL43</f>
+        <f>AH43-AJ43-AK43-AL43-AD43*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN43" s="53">
@@ -21062,7 +21088,7 @@
         <v/>
       </c>
       <c r="X44" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C44,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C44,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y44" s="53">
@@ -21074,7 +21100,7 @@
         <v/>
       </c>
       <c r="AA44" s="53">
-        <f>IF(F44=1,IFERROR(H44/J44,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F44=1,IFERROR(H44/J44,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB44" s="51">
@@ -21098,7 +21124,7 @@
         <v/>
       </c>
       <c r="AG44" s="43">
-        <f>IF(E44="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C44,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C44,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E44="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C44,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C44,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH44" s="17">
@@ -21122,7 +21148,7 @@
         <v/>
       </c>
       <c r="AM44" s="55">
-        <f>AH44-AJ44-AK44-AL44</f>
+        <f>AH44-AJ44-AK44-AL44-AD44*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN44" s="53">
@@ -21232,7 +21258,7 @@
         <v/>
       </c>
       <c r="X45" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C45,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C45,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y45" s="53">
@@ -21244,7 +21270,7 @@
         <v/>
       </c>
       <c r="AA45" s="53">
-        <f>IF(F45=1,IFERROR(H45/J45,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F45=1,IFERROR(H45/J45,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB45" s="51">
@@ -21268,7 +21294,7 @@
         <v/>
       </c>
       <c r="AG45" s="43">
-        <f>IF(E45="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C45,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C45,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E45="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C45,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C45,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH45" s="17">
@@ -21292,7 +21318,7 @@
         <v/>
       </c>
       <c r="AM45" s="55">
-        <f>AH45-AJ45-AK45-AL45</f>
+        <f>AH45-AJ45-AK45-AL45-AD45*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN45" s="53">
@@ -21402,7 +21428,7 @@
         <v/>
       </c>
       <c r="X46" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C46,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C46,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y46" s="53">
@@ -21414,7 +21440,7 @@
         <v/>
       </c>
       <c r="AA46" s="53">
-        <f>IF(F46=1,IFERROR(H46/J46,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F46=1,IFERROR(H46/J46,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB46" s="51">
@@ -21438,7 +21464,7 @@
         <v/>
       </c>
       <c r="AG46" s="43">
-        <f>IF(E46="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C46,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C46,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E46="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C46,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C46,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH46" s="17">
@@ -21462,7 +21488,7 @@
         <v/>
       </c>
       <c r="AM46" s="55">
-        <f>AH46-AJ46-AK46-AL46</f>
+        <f>AH46-AJ46-AK46-AL46-AD46*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN46" s="53">
@@ -21572,7 +21598,7 @@
         <v/>
       </c>
       <c r="X47" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C47,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C47,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y47" s="53">
@@ -21584,7 +21610,7 @@
         <v/>
       </c>
       <c r="AA47" s="53">
-        <f>IF(F47=1,IFERROR(H47/J47,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F47=1,IFERROR(H47/J47,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB47" s="51">
@@ -21608,7 +21634,7 @@
         <v/>
       </c>
       <c r="AG47" s="43">
-        <f>IF(E47="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C47,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C47,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E47="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C47,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C47,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH47" s="17">
@@ -21632,7 +21658,7 @@
         <v/>
       </c>
       <c r="AM47" s="55">
-        <f>AH47-AJ47-AK47-AL47</f>
+        <f>AH47-AJ47-AK47-AL47-AD47*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN47" s="53">
@@ -21742,7 +21768,7 @@
         <v/>
       </c>
       <c r="X48" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C48,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C48,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y48" s="53">
@@ -21754,7 +21780,7 @@
         <v/>
       </c>
       <c r="AA48" s="53">
-        <f>IF(F48=1,IFERROR(H48/J48,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F48=1,IFERROR(H48/J48,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB48" s="51">
@@ -21778,7 +21804,7 @@
         <v/>
       </c>
       <c r="AG48" s="43">
-        <f>IF(E48="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C48,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C48,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E48="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C48,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C48,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH48" s="17">
@@ -21802,7 +21828,7 @@
         <v/>
       </c>
       <c r="AM48" s="55">
-        <f>AH48-AJ48-AK48-AL48</f>
+        <f>AH48-AJ48-AK48-AL48-AD48*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN48" s="53">
@@ -21912,7 +21938,7 @@
         <v/>
       </c>
       <c r="X49" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C49,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C49,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y49" s="53">
@@ -21924,7 +21950,7 @@
         <v/>
       </c>
       <c r="AA49" s="53">
-        <f>IF(F49=1,IFERROR(H49/J49,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F49=1,IFERROR(H49/J49,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB49" s="51">
@@ -21948,7 +21974,7 @@
         <v/>
       </c>
       <c r="AG49" s="43">
-        <f>IF(E49="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C49,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C49,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E49="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C49,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C49,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH49" s="17">
@@ -21972,7 +21998,7 @@
         <v/>
       </c>
       <c r="AM49" s="55">
-        <f>AH49-AJ49-AK49-AL49</f>
+        <f>AH49-AJ49-AK49-AL49-AD49*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN49" s="53">
@@ -22082,7 +22108,7 @@
         <v/>
       </c>
       <c r="X50" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C50,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C50,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y50" s="53">
@@ -22094,7 +22120,7 @@
         <v/>
       </c>
       <c r="AA50" s="53">
-        <f>IF(F50=1,IFERROR(H50/J50,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F50=1,IFERROR(H50/J50,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB50" s="51">
@@ -22118,7 +22144,7 @@
         <v/>
       </c>
       <c r="AG50" s="43">
-        <f>IF(E50="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C50,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C50,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E50="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C50,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C50,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH50" s="17">
@@ -22142,7 +22168,7 @@
         <v/>
       </c>
       <c r="AM50" s="55">
-        <f>AH50-AJ50-AK50-AL50</f>
+        <f>AH50-AJ50-AK50-AL50-AD50*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN50" s="53">
@@ -22252,7 +22278,7 @@
         <v/>
       </c>
       <c r="X51" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C51,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C51,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y51" s="53">
@@ -22264,7 +22290,7 @@
         <v/>
       </c>
       <c r="AA51" s="53">
-        <f>IF(F51=1,IFERROR(H51/J51,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F51=1,IFERROR(H51/J51,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB51" s="51">
@@ -22288,7 +22314,7 @@
         <v/>
       </c>
       <c r="AG51" s="43">
-        <f>IF(E51="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C51,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C51,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E51="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C51,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C51,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH51" s="17">
@@ -22312,7 +22338,7 @@
         <v/>
       </c>
       <c r="AM51" s="55">
-        <f>AH51-AJ51-AK51-AL51</f>
+        <f>AH51-AJ51-AK51-AL51-AD51*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN51" s="53">
@@ -22422,7 +22448,7 @@
         <v/>
       </c>
       <c r="X52" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C52,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C52,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y52" s="53">
@@ -22434,7 +22460,7 @@
         <v/>
       </c>
       <c r="AA52" s="53">
-        <f>IF(F52=1,IFERROR(H52/J52,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F52=1,IFERROR(H52/J52,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB52" s="51">
@@ -22458,7 +22484,7 @@
         <v/>
       </c>
       <c r="AG52" s="43">
-        <f>IF(E52="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C52,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C52,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E52="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C52,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C52,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH52" s="17">
@@ -22482,7 +22508,7 @@
         <v/>
       </c>
       <c r="AM52" s="55">
-        <f>AH52-AJ52-AK52-AL52</f>
+        <f>AH52-AJ52-AK52-AL52-AD52*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN52" s="53">
@@ -22592,7 +22618,7 @@
         <v/>
       </c>
       <c r="X53" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C53,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C53,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y53" s="53">
@@ -22604,7 +22630,7 @@
         <v/>
       </c>
       <c r="AA53" s="53">
-        <f>IF(F53=1,IFERROR(H53/J53,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F53=1,IFERROR(H53/J53,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB53" s="51">
@@ -22628,7 +22654,7 @@
         <v/>
       </c>
       <c r="AG53" s="43">
-        <f>IF(E53="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C53,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C53,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E53="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C53,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C53,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH53" s="17">
@@ -22652,7 +22678,7 @@
         <v/>
       </c>
       <c r="AM53" s="55">
-        <f>AH53-AJ53-AK53-AL53</f>
+        <f>AH53-AJ53-AK53-AL53-AD53*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN53" s="53">
@@ -22762,7 +22788,7 @@
         <v/>
       </c>
       <c r="X54" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C54,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C54,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y54" s="53">
@@ -22774,7 +22800,7 @@
         <v/>
       </c>
       <c r="AA54" s="53">
-        <f>IF(F54=1,IFERROR(H54/J54,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F54=1,IFERROR(H54/J54,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB54" s="51">
@@ -22798,7 +22824,7 @@
         <v/>
       </c>
       <c r="AG54" s="43">
-        <f>IF(E54="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C54,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C54,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E54="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C54,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C54,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH54" s="17">
@@ -22822,7 +22848,7 @@
         <v/>
       </c>
       <c r="AM54" s="55">
-        <f>AH54-AJ54-AK54-AL54</f>
+        <f>AH54-AJ54-AK54-AL54-AD54*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN54" s="53">
@@ -22932,7 +22958,7 @@
         <v/>
       </c>
       <c r="X55" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C55,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C55,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y55" s="53">
@@ -22944,7 +22970,7 @@
         <v/>
       </c>
       <c r="AA55" s="53">
-        <f>IF(F55=1,IFERROR(H55/J55,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F55=1,IFERROR(H55/J55,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB55" s="51">
@@ -22968,7 +22994,7 @@
         <v/>
       </c>
       <c r="AG55" s="43">
-        <f>IF(E55="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C55,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C55,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E55="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C55,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C55,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH55" s="17">
@@ -22992,7 +23018,7 @@
         <v/>
       </c>
       <c r="AM55" s="55">
-        <f>AH55-AJ55-AK55-AL55</f>
+        <f>AH55-AJ55-AK55-AL55-AD55*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN55" s="53">
@@ -23102,7 +23128,7 @@
         <v/>
       </c>
       <c r="X56" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C56,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C56,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y56" s="53">
@@ -23114,7 +23140,7 @@
         <v/>
       </c>
       <c r="AA56" s="53">
-        <f>IF(F56=1,IFERROR(H56/J56,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F56=1,IFERROR(H56/J56,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB56" s="51">
@@ -23138,7 +23164,7 @@
         <v/>
       </c>
       <c r="AG56" s="43">
-        <f>IF(E56="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C56,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C56,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E56="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C56,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C56,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH56" s="17">
@@ -23162,7 +23188,7 @@
         <v/>
       </c>
       <c r="AM56" s="55">
-        <f>AH56-AJ56-AK56-AL56</f>
+        <f>AH56-AJ56-AK56-AL56-AD56*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN56" s="53">
@@ -23272,7 +23298,7 @@
         <v/>
       </c>
       <c r="X57" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C57,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C57,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y57" s="53">
@@ -23284,7 +23310,7 @@
         <v/>
       </c>
       <c r="AA57" s="53">
-        <f>IF(F57=1,IFERROR(H57/J57,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F57=1,IFERROR(H57/J57,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB57" s="51">
@@ -23308,7 +23334,7 @@
         <v/>
       </c>
       <c r="AG57" s="43">
-        <f>IF(E57="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C57,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C57,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E57="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C57,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C57,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH57" s="17">
@@ -23332,7 +23358,7 @@
         <v/>
       </c>
       <c r="AM57" s="55">
-        <f>AH57-AJ57-AK57-AL57</f>
+        <f>AH57-AJ57-AK57-AL57-AD57*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN57" s="53">
@@ -23442,7 +23468,7 @@
         <v/>
       </c>
       <c r="X58" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C58,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C58,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y58" s="53">
@@ -23454,7 +23480,7 @@
         <v/>
       </c>
       <c r="AA58" s="53">
-        <f>IF(F58=1,IFERROR(H58/J58,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F58=1,IFERROR(H58/J58,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB58" s="51">
@@ -23478,7 +23504,7 @@
         <v/>
       </c>
       <c r="AG58" s="43">
-        <f>IF(E58="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C58,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C58,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E58="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C58,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C58,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH58" s="17">
@@ -23502,7 +23528,7 @@
         <v/>
       </c>
       <c r="AM58" s="55">
-        <f>AH58-AJ58-AK58-AL58</f>
+        <f>AH58-AJ58-AK58-AL58-AD58*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN58" s="53">
@@ -23612,7 +23638,7 @@
         <v/>
       </c>
       <c r="X59" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C59,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C59,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y59" s="53">
@@ -23624,7 +23650,7 @@
         <v/>
       </c>
       <c r="AA59" s="53">
-        <f>IF(F59=1,IFERROR(H59/J59,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F59=1,IFERROR(H59/J59,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB59" s="51">
@@ -23648,7 +23674,7 @@
         <v/>
       </c>
       <c r="AG59" s="43">
-        <f>IF(E59="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C59,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C59,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E59="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C59,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C59,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH59" s="17">
@@ -23672,7 +23698,7 @@
         <v/>
       </c>
       <c r="AM59" s="55">
-        <f>AH59-AJ59-AK59-AL59</f>
+        <f>AH59-AJ59-AK59-AL59-AD59*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN59" s="53">
@@ -23782,7 +23808,7 @@
         <v/>
       </c>
       <c r="X60" s="43">
-        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C60,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)</f>
+        <f>IFERROR(INDEX('06_Historique'!$F$66:$F$73,MATCH(C60,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$21)</f>
         <v/>
       </c>
       <c r="Y60" s="53">
@@ -23794,7 +23820,7 @@
         <v/>
       </c>
       <c r="AA60" s="53">
-        <f>IF(F60=1,IFERROR(H60/J60,'02_Leviers'!$D$21)+'02_Leviers'!$G$8,0)</f>
+        <f>IF(F60=1,IFERROR(H60/J60,'02_Leviers'!$D$22)+'02_Leviers'!$G$8,0)</f>
         <v/>
       </c>
       <c r="AB60" s="51">
@@ -23818,7 +23844,7 @@
         <v/>
       </c>
       <c r="AG60" s="43">
-        <f>IF(E60="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C60,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C60,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$19))*'02_Leviers'!$D$18,1)</f>
+        <f>IF(E60="ALT",IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C60,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20)+(1-IFERROR(INDEX('06_Historique'!$G$66:$G$73,MATCH(C60,'06_Historique'!$A$66:$A$73,0)),'02_Leviers'!$D$20))*'02_Leviers'!$D$18,1)</f>
         <v/>
       </c>
       <c r="AH60" s="17">
@@ -23842,7 +23868,7 @@
         <v/>
       </c>
       <c r="AM60" s="55">
-        <f>AH60-AJ60-AK60-AL60</f>
+        <f>AH60-AJ60-AK60-AL60-AD60*'02_Leviers'!$D$19*(1+'02_Leviers'!$G$11)</f>
         <v/>
       </c>
       <c r="AN60" s="53">

</xml_diff>

<commit_message>
Simulateur : dilution 360° symétrique (ouvrir enrichit tous, fermer appauvrit tous)
- 'Ouvrir +1 classe' capte désormais des étudiants (+1 classe remplie) : effectif
  total ↑ -> structure/étudiant ↓ -> TOUTES les promos voient leur structure
  allouée baisser et leur résultat tout compris monter (enrichissement), + la
  contribution marginale de la classe captée en EBITDA.
- 'Ne pas ouvrir' : effectif ↓ -> structure/étudiant ↑ -> tous absorbent plus.
- La base de dilution = effectif total APRÈS décisions, dans les deux sens.

Vérifié : 0 erreur ; ouvrir L6 -> L7/L8 s'enrichissent (struct↓, résultat↑),
EBITDA groupe +224k ; fermer L6 -> inverse. Marge 14,6% (réel).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -187,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -378,9 +378,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2324,7 +2321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:Q63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2335,20 +2332,21 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="42" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Simulateur &amp; conseil de décisions — logique CFO : on décide sur la MARGE DE CONTRIBUTION (col. H)</t>
+          <t>Simulateur &amp; conseil de décisions — logique CFO 360° : décider sur la CONTRIBUTION ; ouvrir/fermer redilue la structure sur TOUS</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2366,7 @@
         </is>
       </c>
       <c r="G2" s="54">
-        <f>SUM(P6:P63)</f>
+        <f>SUM(Q6:Q63)</f>
         <v/>
       </c>
       <c r="H2" s="30" t="n"/>
@@ -2383,7 +2381,7 @@
       </c>
       <c r="L2" s="30" t="n"/>
     </row>
-    <row r="3" ht="28" customHeight="1">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="19" t="inlineStr">
         <is>
           <t>Structure / étudiant — AVANT :</t>
@@ -2395,26 +2393,26 @@
       </c>
       <c r="E3" s="19" t="inlineStr">
         <is>
-          <t>APRÈS (dilution) :</t>
+          <t>APRÈS :</t>
         </is>
       </c>
       <c r="G3" s="20">
-        <f>IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
+        <f>IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
         <v/>
       </c>
       <c r="H3" s="30" t="n"/>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>🔴 promos contribution &lt; 0 :</t>
-        </is>
-      </c>
-      <c r="K3" s="68">
-        <f>SUMPRODUCT(--('08_Moteur'!$AM$3:$AM$60&lt;0))</f>
+          <t>Effectif total APRÈS :</t>
+        </is>
+      </c>
+      <c r="K3" s="53">
+        <f>SUM(M6:M63)</f>
         <v/>
       </c>
       <c r="M3" s="12" t="inlineStr">
         <is>
-          <t>⚠ Fermer une promo n'économise PAS la structure (loyer, permanents, siège) : elle RESTE et se redilue sur les autres → on ferme UNIQUEMENT si la contribution (H) est négative.</t>
+          <t>⚠ Fermer retire des étudiants → structure/étudiant ↑ (tous absorbent +). Ouvrir en capte → structure/étudiant ↓ (tous s'enrichissent). La structure totale ne bouge pas ; l'EBITDA groupe ne varie que des contributions.</t>
         </is>
       </c>
     </row>
@@ -2463,43 +2461,49 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
+          <t>Rempl.</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>🤖 Reco</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>Motif</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>Décision</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>Effectif
+après</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr">
+        <is>
+          <t>Contribution
+après</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
           <t>Structure allouée
 (après, dilution)</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="P5" s="13" t="inlineStr">
         <is>
           <t>Résultat tout
 compris (après)</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
-        <is>
-          <t>Rempl.</t>
-        </is>
-      </c>
-      <c r="L5" s="13" t="inlineStr">
-        <is>
-          <t>🤖 Reco</t>
-        </is>
-      </c>
-      <c r="M5" s="13" t="inlineStr">
-        <is>
-          <t>Motif</t>
-        </is>
-      </c>
-      <c r="N5" s="13" t="inlineStr">
-        <is>
-          <t>Décision</t>
-        </is>
-      </c>
-      <c r="O5" s="13" t="inlineStr">
-        <is>
-          <t>Contribution
-après</t>
-        </is>
-      </c>
-      <c r="P5" s="13" t="inlineStr">
+      <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>Δ EBITDA</t>
         </is>
@@ -2538,37 +2542,41 @@
         <f>'08_Moteur'!AM3</f>
         <v/>
       </c>
-      <c r="I6" s="17">
-        <f>IF(N6="Ne pas ouvrir",0,E6)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J6" s="17">
-        <f>O6-I6</f>
-        <v/>
-      </c>
-      <c r="K6" s="69">
+      <c r="I6" s="68">
         <f>'08_Moteur'!AN3</f>
         <v/>
       </c>
-      <c r="L6" s="70">
-        <f>IF(H6&lt;0,"🔴 Ne pas ouvrir",IF(K6&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K6&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M6" s="71">
-        <f>IF(H6&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K6&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K6&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N6" s="21" t="inlineStr">
+      <c r="J6" s="69">
+        <f>IF(H6&lt;0,"🔴 Ne pas ouvrir",IF(I6&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I6&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K6" s="70">
+        <f>IF(H6&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I6&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I6&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L6" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M6" s="50">
+        <f>IF(L6="Ne pas ouvrir",0,IF(L6="Ouvrir +1 classe",E6+'08_Moteur'!O3,E6))</f>
+        <v/>
+      </c>
+      <c r="N6" s="17">
+        <f>IF(L6="Ne pas ouvrir",0,IF(L6="Ouvrir +1 classe",H6+'08_Moteur'!O3*('08_Moteur'!AE3*'08_Moteur'!AF3-('08_Moteur'!R3+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S3)-'08_Moteur'!U3,IF(L6="Économiser 1 classe",H6+('08_Moteur'!AI3-MAX(1,'08_Moteur'!AI3-1))*'08_Moteur'!U3,H6)))</f>
+        <v/>
+      </c>
       <c r="O6" s="17">
-        <f>IF(N6="Ne pas ouvrir",0,IF(N6="Ouvrir +1 classe",H6-'08_Moteur'!U3,IF(N6="Économiser 1 classe",H6+('08_Moteur'!AI3-MAX(1,'08_Moteur'!AI3-1))*'08_Moteur'!U3,H6)))</f>
-        <v/>
-      </c>
-      <c r="P6" s="54">
-        <f>O6-H6</f>
+        <f>M6*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P6" s="17">
+        <f>N6-O6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="54">
+        <f>N6-H6</f>
         <v/>
       </c>
     </row>
@@ -2605,37 +2613,41 @@
         <f>'08_Moteur'!AM4</f>
         <v/>
       </c>
-      <c r="I7" s="17">
-        <f>IF(N7="Ne pas ouvrir",0,E7)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J7" s="17">
-        <f>O7-I7</f>
-        <v/>
-      </c>
-      <c r="K7" s="69">
+      <c r="I7" s="68">
         <f>'08_Moteur'!AN4</f>
         <v/>
       </c>
-      <c r="L7" s="70">
-        <f>IF(H7&lt;0,"🔴 Ne pas ouvrir",IF(K7&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K7&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M7" s="71">
-        <f>IF(H7&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K7&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K7&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N7" s="21" t="inlineStr">
+      <c r="J7" s="69">
+        <f>IF(H7&lt;0,"🔴 Ne pas ouvrir",IF(I7&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I7&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K7" s="70">
+        <f>IF(H7&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I7&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I7&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L7" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M7" s="50">
+        <f>IF(L7="Ne pas ouvrir",0,IF(L7="Ouvrir +1 classe",E7+'08_Moteur'!O4,E7))</f>
+        <v/>
+      </c>
+      <c r="N7" s="17">
+        <f>IF(L7="Ne pas ouvrir",0,IF(L7="Ouvrir +1 classe",H7+'08_Moteur'!O4*('08_Moteur'!AE4*'08_Moteur'!AF4-('08_Moteur'!R4+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S4)-'08_Moteur'!U4,IF(L7="Économiser 1 classe",H7+('08_Moteur'!AI4-MAX(1,'08_Moteur'!AI4-1))*'08_Moteur'!U4,H7)))</f>
+        <v/>
+      </c>
       <c r="O7" s="17">
-        <f>IF(N7="Ne pas ouvrir",0,IF(N7="Ouvrir +1 classe",H7-'08_Moteur'!U4,IF(N7="Économiser 1 classe",H7+('08_Moteur'!AI4-MAX(1,'08_Moteur'!AI4-1))*'08_Moteur'!U4,H7)))</f>
-        <v/>
-      </c>
-      <c r="P7" s="54">
-        <f>O7-H7</f>
+        <f>M7*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P7" s="17">
+        <f>N7-O7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="54">
+        <f>N7-H7</f>
         <v/>
       </c>
     </row>
@@ -2672,37 +2684,41 @@
         <f>'08_Moteur'!AM5</f>
         <v/>
       </c>
-      <c r="I8" s="17">
-        <f>IF(N8="Ne pas ouvrir",0,E8)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J8" s="17">
-        <f>O8-I8</f>
-        <v/>
-      </c>
-      <c r="K8" s="69">
+      <c r="I8" s="68">
         <f>'08_Moteur'!AN5</f>
         <v/>
       </c>
-      <c r="L8" s="70">
-        <f>IF(H8&lt;0,"🔴 Ne pas ouvrir",IF(K8&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K8&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M8" s="71">
-        <f>IF(H8&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K8&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K8&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N8" s="21" t="inlineStr">
+      <c r="J8" s="69">
+        <f>IF(H8&lt;0,"🔴 Ne pas ouvrir",IF(I8&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I8&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K8" s="70">
+        <f>IF(H8&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I8&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I8&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L8" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M8" s="50">
+        <f>IF(L8="Ne pas ouvrir",0,IF(L8="Ouvrir +1 classe",E8+'08_Moteur'!O5,E8))</f>
+        <v/>
+      </c>
+      <c r="N8" s="17">
+        <f>IF(L8="Ne pas ouvrir",0,IF(L8="Ouvrir +1 classe",H8+'08_Moteur'!O5*('08_Moteur'!AE5*'08_Moteur'!AF5-('08_Moteur'!R5+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S5)-'08_Moteur'!U5,IF(L8="Économiser 1 classe",H8+('08_Moteur'!AI5-MAX(1,'08_Moteur'!AI5-1))*'08_Moteur'!U5,H8)))</f>
+        <v/>
+      </c>
       <c r="O8" s="17">
-        <f>IF(N8="Ne pas ouvrir",0,IF(N8="Ouvrir +1 classe",H8-'08_Moteur'!U5,IF(N8="Économiser 1 classe",H8+('08_Moteur'!AI5-MAX(1,'08_Moteur'!AI5-1))*'08_Moteur'!U5,H8)))</f>
-        <v/>
-      </c>
-      <c r="P8" s="54">
-        <f>O8-H8</f>
+        <f>M8*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P8" s="17">
+        <f>N8-O8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="54">
+        <f>N8-H8</f>
         <v/>
       </c>
     </row>
@@ -2739,37 +2755,41 @@
         <f>'08_Moteur'!AM6</f>
         <v/>
       </c>
-      <c r="I9" s="17">
-        <f>IF(N9="Ne pas ouvrir",0,E9)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J9" s="17">
-        <f>O9-I9</f>
-        <v/>
-      </c>
-      <c r="K9" s="69">
+      <c r="I9" s="68">
         <f>'08_Moteur'!AN6</f>
         <v/>
       </c>
-      <c r="L9" s="70">
-        <f>IF(H9&lt;0,"🔴 Ne pas ouvrir",IF(K9&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K9&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M9" s="71">
-        <f>IF(H9&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K9&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K9&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N9" s="21" t="inlineStr">
+      <c r="J9" s="69">
+        <f>IF(H9&lt;0,"🔴 Ne pas ouvrir",IF(I9&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I9&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K9" s="70">
+        <f>IF(H9&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I9&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I9&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L9" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M9" s="50">
+        <f>IF(L9="Ne pas ouvrir",0,IF(L9="Ouvrir +1 classe",E9+'08_Moteur'!O6,E9))</f>
+        <v/>
+      </c>
+      <c r="N9" s="17">
+        <f>IF(L9="Ne pas ouvrir",0,IF(L9="Ouvrir +1 classe",H9+'08_Moteur'!O6*('08_Moteur'!AE6*'08_Moteur'!AF6-('08_Moteur'!R6+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S6)-'08_Moteur'!U6,IF(L9="Économiser 1 classe",H9+('08_Moteur'!AI6-MAX(1,'08_Moteur'!AI6-1))*'08_Moteur'!U6,H9)))</f>
+        <v/>
+      </c>
       <c r="O9" s="17">
-        <f>IF(N9="Ne pas ouvrir",0,IF(N9="Ouvrir +1 classe",H9-'08_Moteur'!U6,IF(N9="Économiser 1 classe",H9+('08_Moteur'!AI6-MAX(1,'08_Moteur'!AI6-1))*'08_Moteur'!U6,H9)))</f>
-        <v/>
-      </c>
-      <c r="P9" s="54">
-        <f>O9-H9</f>
+        <f>M9*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="17">
+        <f>N9-O9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="54">
+        <f>N9-H9</f>
         <v/>
       </c>
     </row>
@@ -2806,37 +2826,41 @@
         <f>'08_Moteur'!AM7</f>
         <v/>
       </c>
-      <c r="I10" s="17">
-        <f>IF(N10="Ne pas ouvrir",0,E10)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J10" s="17">
-        <f>O10-I10</f>
-        <v/>
-      </c>
-      <c r="K10" s="69">
+      <c r="I10" s="68">
         <f>'08_Moteur'!AN7</f>
         <v/>
       </c>
-      <c r="L10" s="70">
-        <f>IF(H10&lt;0,"🔴 Ne pas ouvrir",IF(K10&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K10&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M10" s="71">
-        <f>IF(H10&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K10&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K10&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N10" s="21" t="inlineStr">
+      <c r="J10" s="69">
+        <f>IF(H10&lt;0,"🔴 Ne pas ouvrir",IF(I10&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I10&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K10" s="70">
+        <f>IF(H10&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I10&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I10&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L10" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M10" s="50">
+        <f>IF(L10="Ne pas ouvrir",0,IF(L10="Ouvrir +1 classe",E10+'08_Moteur'!O7,E10))</f>
+        <v/>
+      </c>
+      <c r="N10" s="17">
+        <f>IF(L10="Ne pas ouvrir",0,IF(L10="Ouvrir +1 classe",H10+'08_Moteur'!O7*('08_Moteur'!AE7*'08_Moteur'!AF7-('08_Moteur'!R7+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S7)-'08_Moteur'!U7,IF(L10="Économiser 1 classe",H10+('08_Moteur'!AI7-MAX(1,'08_Moteur'!AI7-1))*'08_Moteur'!U7,H10)))</f>
+        <v/>
+      </c>
       <c r="O10" s="17">
-        <f>IF(N10="Ne pas ouvrir",0,IF(N10="Ouvrir +1 classe",H10-'08_Moteur'!U7,IF(N10="Économiser 1 classe",H10+('08_Moteur'!AI7-MAX(1,'08_Moteur'!AI7-1))*'08_Moteur'!U7,H10)))</f>
-        <v/>
-      </c>
-      <c r="P10" s="54">
-        <f>O10-H10</f>
+        <f>M10*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P10" s="17">
+        <f>N10-O10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="54">
+        <f>N10-H10</f>
         <v/>
       </c>
     </row>
@@ -2873,37 +2897,41 @@
         <f>'08_Moteur'!AM8</f>
         <v/>
       </c>
-      <c r="I11" s="17">
-        <f>IF(N11="Ne pas ouvrir",0,E11)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J11" s="17">
-        <f>O11-I11</f>
-        <v/>
-      </c>
-      <c r="K11" s="69">
+      <c r="I11" s="68">
         <f>'08_Moteur'!AN8</f>
         <v/>
       </c>
-      <c r="L11" s="70">
-        <f>IF(H11&lt;0,"🔴 Ne pas ouvrir",IF(K11&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K11&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M11" s="71">
-        <f>IF(H11&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K11&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K11&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N11" s="21" t="inlineStr">
+      <c r="J11" s="69">
+        <f>IF(H11&lt;0,"🔴 Ne pas ouvrir",IF(I11&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I11&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K11" s="70">
+        <f>IF(H11&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I11&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I11&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L11" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M11" s="50">
+        <f>IF(L11="Ne pas ouvrir",0,IF(L11="Ouvrir +1 classe",E11+'08_Moteur'!O8,E11))</f>
+        <v/>
+      </c>
+      <c r="N11" s="17">
+        <f>IF(L11="Ne pas ouvrir",0,IF(L11="Ouvrir +1 classe",H11+'08_Moteur'!O8*('08_Moteur'!AE8*'08_Moteur'!AF8-('08_Moteur'!R8+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S8)-'08_Moteur'!U8,IF(L11="Économiser 1 classe",H11+('08_Moteur'!AI8-MAX(1,'08_Moteur'!AI8-1))*'08_Moteur'!U8,H11)))</f>
+        <v/>
+      </c>
       <c r="O11" s="17">
-        <f>IF(N11="Ne pas ouvrir",0,IF(N11="Ouvrir +1 classe",H11-'08_Moteur'!U8,IF(N11="Économiser 1 classe",H11+('08_Moteur'!AI8-MAX(1,'08_Moteur'!AI8-1))*'08_Moteur'!U8,H11)))</f>
-        <v/>
-      </c>
-      <c r="P11" s="54">
-        <f>O11-H11</f>
+        <f>M11*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P11" s="17">
+        <f>N11-O11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="54">
+        <f>N11-H11</f>
         <v/>
       </c>
     </row>
@@ -2940,37 +2968,41 @@
         <f>'08_Moteur'!AM9</f>
         <v/>
       </c>
-      <c r="I12" s="17">
-        <f>IF(N12="Ne pas ouvrir",0,E12)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J12" s="17">
-        <f>O12-I12</f>
-        <v/>
-      </c>
-      <c r="K12" s="69">
+      <c r="I12" s="68">
         <f>'08_Moteur'!AN9</f>
         <v/>
       </c>
-      <c r="L12" s="70">
-        <f>IF(H12&lt;0,"🔴 Ne pas ouvrir",IF(K12&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K12&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M12" s="71">
-        <f>IF(H12&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K12&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K12&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N12" s="21" t="inlineStr">
+      <c r="J12" s="69">
+        <f>IF(H12&lt;0,"🔴 Ne pas ouvrir",IF(I12&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I12&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K12" s="70">
+        <f>IF(H12&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I12&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I12&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L12" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M12" s="50">
+        <f>IF(L12="Ne pas ouvrir",0,IF(L12="Ouvrir +1 classe",E12+'08_Moteur'!O9,E12))</f>
+        <v/>
+      </c>
+      <c r="N12" s="17">
+        <f>IF(L12="Ne pas ouvrir",0,IF(L12="Ouvrir +1 classe",H12+'08_Moteur'!O9*('08_Moteur'!AE9*'08_Moteur'!AF9-('08_Moteur'!R9+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S9)-'08_Moteur'!U9,IF(L12="Économiser 1 classe",H12+('08_Moteur'!AI9-MAX(1,'08_Moteur'!AI9-1))*'08_Moteur'!U9,H12)))</f>
+        <v/>
+      </c>
       <c r="O12" s="17">
-        <f>IF(N12="Ne pas ouvrir",0,IF(N12="Ouvrir +1 classe",H12-'08_Moteur'!U9,IF(N12="Économiser 1 classe",H12+('08_Moteur'!AI9-MAX(1,'08_Moteur'!AI9-1))*'08_Moteur'!U9,H12)))</f>
-        <v/>
-      </c>
-      <c r="P12" s="54">
-        <f>O12-H12</f>
+        <f>M12*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P12" s="17">
+        <f>N12-O12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="54">
+        <f>N12-H12</f>
         <v/>
       </c>
     </row>
@@ -3007,37 +3039,41 @@
         <f>'08_Moteur'!AM10</f>
         <v/>
       </c>
-      <c r="I13" s="17">
-        <f>IF(N13="Ne pas ouvrir",0,E13)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J13" s="17">
-        <f>O13-I13</f>
-        <v/>
-      </c>
-      <c r="K13" s="69">
+      <c r="I13" s="68">
         <f>'08_Moteur'!AN10</f>
         <v/>
       </c>
-      <c r="L13" s="70">
-        <f>IF(H13&lt;0,"🔴 Ne pas ouvrir",IF(K13&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K13&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M13" s="71">
-        <f>IF(H13&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K13&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K13&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N13" s="21" t="inlineStr">
+      <c r="J13" s="69">
+        <f>IF(H13&lt;0,"🔴 Ne pas ouvrir",IF(I13&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I13&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K13" s="70">
+        <f>IF(H13&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I13&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I13&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L13" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M13" s="50">
+        <f>IF(L13="Ne pas ouvrir",0,IF(L13="Ouvrir +1 classe",E13+'08_Moteur'!O10,E13))</f>
+        <v/>
+      </c>
+      <c r="N13" s="17">
+        <f>IF(L13="Ne pas ouvrir",0,IF(L13="Ouvrir +1 classe",H13+'08_Moteur'!O10*('08_Moteur'!AE10*'08_Moteur'!AF10-('08_Moteur'!R10+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S10)-'08_Moteur'!U10,IF(L13="Économiser 1 classe",H13+('08_Moteur'!AI10-MAX(1,'08_Moteur'!AI10-1))*'08_Moteur'!U10,H13)))</f>
+        <v/>
+      </c>
       <c r="O13" s="17">
-        <f>IF(N13="Ne pas ouvrir",0,IF(N13="Ouvrir +1 classe",H13-'08_Moteur'!U10,IF(N13="Économiser 1 classe",H13+('08_Moteur'!AI10-MAX(1,'08_Moteur'!AI10-1))*'08_Moteur'!U10,H13)))</f>
-        <v/>
-      </c>
-      <c r="P13" s="54">
-        <f>O13-H13</f>
+        <f>M13*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P13" s="17">
+        <f>N13-O13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="54">
+        <f>N13-H13</f>
         <v/>
       </c>
     </row>
@@ -3074,37 +3110,41 @@
         <f>'08_Moteur'!AM11</f>
         <v/>
       </c>
-      <c r="I14" s="17">
-        <f>IF(N14="Ne pas ouvrir",0,E14)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J14" s="17">
-        <f>O14-I14</f>
-        <v/>
-      </c>
-      <c r="K14" s="69">
+      <c r="I14" s="68">
         <f>'08_Moteur'!AN11</f>
         <v/>
       </c>
-      <c r="L14" s="70">
-        <f>IF(H14&lt;0,"🔴 Ne pas ouvrir",IF(K14&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K14&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M14" s="71">
-        <f>IF(H14&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K14&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K14&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N14" s="21" t="inlineStr">
+      <c r="J14" s="69">
+        <f>IF(H14&lt;0,"🔴 Ne pas ouvrir",IF(I14&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I14&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K14" s="70">
+        <f>IF(H14&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I14&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I14&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L14" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M14" s="50">
+        <f>IF(L14="Ne pas ouvrir",0,IF(L14="Ouvrir +1 classe",E14+'08_Moteur'!O11,E14))</f>
+        <v/>
+      </c>
+      <c r="N14" s="17">
+        <f>IF(L14="Ne pas ouvrir",0,IF(L14="Ouvrir +1 classe",H14+'08_Moteur'!O11*('08_Moteur'!AE11*'08_Moteur'!AF11-('08_Moteur'!R11+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S11)-'08_Moteur'!U11,IF(L14="Économiser 1 classe",H14+('08_Moteur'!AI11-MAX(1,'08_Moteur'!AI11-1))*'08_Moteur'!U11,H14)))</f>
+        <v/>
+      </c>
       <c r="O14" s="17">
-        <f>IF(N14="Ne pas ouvrir",0,IF(N14="Ouvrir +1 classe",H14-'08_Moteur'!U11,IF(N14="Économiser 1 classe",H14+('08_Moteur'!AI11-MAX(1,'08_Moteur'!AI11-1))*'08_Moteur'!U11,H14)))</f>
-        <v/>
-      </c>
-      <c r="P14" s="54">
-        <f>O14-H14</f>
+        <f>M14*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P14" s="17">
+        <f>N14-O14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="54">
+        <f>N14-H14</f>
         <v/>
       </c>
     </row>
@@ -3141,37 +3181,41 @@
         <f>'08_Moteur'!AM12</f>
         <v/>
       </c>
-      <c r="I15" s="17">
-        <f>IF(N15="Ne pas ouvrir",0,E15)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J15" s="17">
-        <f>O15-I15</f>
-        <v/>
-      </c>
-      <c r="K15" s="69">
+      <c r="I15" s="68">
         <f>'08_Moteur'!AN12</f>
         <v/>
       </c>
-      <c r="L15" s="70">
-        <f>IF(H15&lt;0,"🔴 Ne pas ouvrir",IF(K15&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K15&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M15" s="71">
-        <f>IF(H15&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K15&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K15&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N15" s="21" t="inlineStr">
+      <c r="J15" s="69">
+        <f>IF(H15&lt;0,"🔴 Ne pas ouvrir",IF(I15&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I15&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K15" s="70">
+        <f>IF(H15&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I15&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I15&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L15" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M15" s="50">
+        <f>IF(L15="Ne pas ouvrir",0,IF(L15="Ouvrir +1 classe",E15+'08_Moteur'!O12,E15))</f>
+        <v/>
+      </c>
+      <c r="N15" s="17">
+        <f>IF(L15="Ne pas ouvrir",0,IF(L15="Ouvrir +1 classe",H15+'08_Moteur'!O12*('08_Moteur'!AE12*'08_Moteur'!AF12-('08_Moteur'!R12+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S12)-'08_Moteur'!U12,IF(L15="Économiser 1 classe",H15+('08_Moteur'!AI12-MAX(1,'08_Moteur'!AI12-1))*'08_Moteur'!U12,H15)))</f>
+        <v/>
+      </c>
       <c r="O15" s="17">
-        <f>IF(N15="Ne pas ouvrir",0,IF(N15="Ouvrir +1 classe",H15-'08_Moteur'!U12,IF(N15="Économiser 1 classe",H15+('08_Moteur'!AI12-MAX(1,'08_Moteur'!AI12-1))*'08_Moteur'!U12,H15)))</f>
-        <v/>
-      </c>
-      <c r="P15" s="54">
-        <f>O15-H15</f>
+        <f>M15*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P15" s="17">
+        <f>N15-O15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="54">
+        <f>N15-H15</f>
         <v/>
       </c>
     </row>
@@ -3208,37 +3252,41 @@
         <f>'08_Moteur'!AM13</f>
         <v/>
       </c>
-      <c r="I16" s="17">
-        <f>IF(N16="Ne pas ouvrir",0,E16)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J16" s="17">
-        <f>O16-I16</f>
-        <v/>
-      </c>
-      <c r="K16" s="69">
+      <c r="I16" s="68">
         <f>'08_Moteur'!AN13</f>
         <v/>
       </c>
-      <c r="L16" s="70">
-        <f>IF(H16&lt;0,"🔴 Ne pas ouvrir",IF(K16&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K16&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M16" s="71">
-        <f>IF(H16&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K16&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K16&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N16" s="21" t="inlineStr">
+      <c r="J16" s="69">
+        <f>IF(H16&lt;0,"🔴 Ne pas ouvrir",IF(I16&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I16&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K16" s="70">
+        <f>IF(H16&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I16&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I16&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L16" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M16" s="50">
+        <f>IF(L16="Ne pas ouvrir",0,IF(L16="Ouvrir +1 classe",E16+'08_Moteur'!O13,E16))</f>
+        <v/>
+      </c>
+      <c r="N16" s="17">
+        <f>IF(L16="Ne pas ouvrir",0,IF(L16="Ouvrir +1 classe",H16+'08_Moteur'!O13*('08_Moteur'!AE13*'08_Moteur'!AF13-('08_Moteur'!R13+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S13)-'08_Moteur'!U13,IF(L16="Économiser 1 classe",H16+('08_Moteur'!AI13-MAX(1,'08_Moteur'!AI13-1))*'08_Moteur'!U13,H16)))</f>
+        <v/>
+      </c>
       <c r="O16" s="17">
-        <f>IF(N16="Ne pas ouvrir",0,IF(N16="Ouvrir +1 classe",H16-'08_Moteur'!U13,IF(N16="Économiser 1 classe",H16+('08_Moteur'!AI13-MAX(1,'08_Moteur'!AI13-1))*'08_Moteur'!U13,H16)))</f>
-        <v/>
-      </c>
-      <c r="P16" s="54">
-        <f>O16-H16</f>
+        <f>M16*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P16" s="17">
+        <f>N16-O16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="54">
+        <f>N16-H16</f>
         <v/>
       </c>
     </row>
@@ -3275,37 +3323,41 @@
         <f>'08_Moteur'!AM14</f>
         <v/>
       </c>
-      <c r="I17" s="17">
-        <f>IF(N17="Ne pas ouvrir",0,E17)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J17" s="17">
-        <f>O17-I17</f>
-        <v/>
-      </c>
-      <c r="K17" s="69">
+      <c r="I17" s="68">
         <f>'08_Moteur'!AN14</f>
         <v/>
       </c>
-      <c r="L17" s="70">
-        <f>IF(H17&lt;0,"🔴 Ne pas ouvrir",IF(K17&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K17&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M17" s="71">
-        <f>IF(H17&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K17&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K17&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N17" s="21" t="inlineStr">
+      <c r="J17" s="69">
+        <f>IF(H17&lt;0,"🔴 Ne pas ouvrir",IF(I17&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I17&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K17" s="70">
+        <f>IF(H17&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I17&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I17&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L17" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M17" s="50">
+        <f>IF(L17="Ne pas ouvrir",0,IF(L17="Ouvrir +1 classe",E17+'08_Moteur'!O14,E17))</f>
+        <v/>
+      </c>
+      <c r="N17" s="17">
+        <f>IF(L17="Ne pas ouvrir",0,IF(L17="Ouvrir +1 classe",H17+'08_Moteur'!O14*('08_Moteur'!AE14*'08_Moteur'!AF14-('08_Moteur'!R14+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S14)-'08_Moteur'!U14,IF(L17="Économiser 1 classe",H17+('08_Moteur'!AI14-MAX(1,'08_Moteur'!AI14-1))*'08_Moteur'!U14,H17)))</f>
+        <v/>
+      </c>
       <c r="O17" s="17">
-        <f>IF(N17="Ne pas ouvrir",0,IF(N17="Ouvrir +1 classe",H17-'08_Moteur'!U14,IF(N17="Économiser 1 classe",H17+('08_Moteur'!AI14-MAX(1,'08_Moteur'!AI14-1))*'08_Moteur'!U14,H17)))</f>
-        <v/>
-      </c>
-      <c r="P17" s="54">
-        <f>O17-H17</f>
+        <f>M17*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P17" s="17">
+        <f>N17-O17</f>
+        <v/>
+      </c>
+      <c r="Q17" s="54">
+        <f>N17-H17</f>
         <v/>
       </c>
     </row>
@@ -3342,37 +3394,41 @@
         <f>'08_Moteur'!AM15</f>
         <v/>
       </c>
-      <c r="I18" s="17">
-        <f>IF(N18="Ne pas ouvrir",0,E18)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J18" s="17">
-        <f>O18-I18</f>
-        <v/>
-      </c>
-      <c r="K18" s="69">
+      <c r="I18" s="68">
         <f>'08_Moteur'!AN15</f>
         <v/>
       </c>
-      <c r="L18" s="70">
-        <f>IF(H18&lt;0,"🔴 Ne pas ouvrir",IF(K18&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K18&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M18" s="71">
-        <f>IF(H18&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K18&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K18&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N18" s="21" t="inlineStr">
+      <c r="J18" s="69">
+        <f>IF(H18&lt;0,"🔴 Ne pas ouvrir",IF(I18&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I18&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K18" s="70">
+        <f>IF(H18&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I18&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I18&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L18" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M18" s="50">
+        <f>IF(L18="Ne pas ouvrir",0,IF(L18="Ouvrir +1 classe",E18+'08_Moteur'!O15,E18))</f>
+        <v/>
+      </c>
+      <c r="N18" s="17">
+        <f>IF(L18="Ne pas ouvrir",0,IF(L18="Ouvrir +1 classe",H18+'08_Moteur'!O15*('08_Moteur'!AE15*'08_Moteur'!AF15-('08_Moteur'!R15+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S15)-'08_Moteur'!U15,IF(L18="Économiser 1 classe",H18+('08_Moteur'!AI15-MAX(1,'08_Moteur'!AI15-1))*'08_Moteur'!U15,H18)))</f>
+        <v/>
+      </c>
       <c r="O18" s="17">
-        <f>IF(N18="Ne pas ouvrir",0,IF(N18="Ouvrir +1 classe",H18-'08_Moteur'!U15,IF(N18="Économiser 1 classe",H18+('08_Moteur'!AI15-MAX(1,'08_Moteur'!AI15-1))*'08_Moteur'!U15,H18)))</f>
-        <v/>
-      </c>
-      <c r="P18" s="54">
-        <f>O18-H18</f>
+        <f>M18*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P18" s="17">
+        <f>N18-O18</f>
+        <v/>
+      </c>
+      <c r="Q18" s="54">
+        <f>N18-H18</f>
         <v/>
       </c>
     </row>
@@ -3409,37 +3465,41 @@
         <f>'08_Moteur'!AM16</f>
         <v/>
       </c>
-      <c r="I19" s="17">
-        <f>IF(N19="Ne pas ouvrir",0,E19)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J19" s="17">
-        <f>O19-I19</f>
-        <v/>
-      </c>
-      <c r="K19" s="69">
+      <c r="I19" s="68">
         <f>'08_Moteur'!AN16</f>
         <v/>
       </c>
-      <c r="L19" s="70">
-        <f>IF(H19&lt;0,"🔴 Ne pas ouvrir",IF(K19&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K19&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M19" s="71">
-        <f>IF(H19&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K19&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K19&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N19" s="21" t="inlineStr">
+      <c r="J19" s="69">
+        <f>IF(H19&lt;0,"🔴 Ne pas ouvrir",IF(I19&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I19&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K19" s="70">
+        <f>IF(H19&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I19&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I19&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L19" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M19" s="50">
+        <f>IF(L19="Ne pas ouvrir",0,IF(L19="Ouvrir +1 classe",E19+'08_Moteur'!O16,E19))</f>
+        <v/>
+      </c>
+      <c r="N19" s="17">
+        <f>IF(L19="Ne pas ouvrir",0,IF(L19="Ouvrir +1 classe",H19+'08_Moteur'!O16*('08_Moteur'!AE16*'08_Moteur'!AF16-('08_Moteur'!R16+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S16)-'08_Moteur'!U16,IF(L19="Économiser 1 classe",H19+('08_Moteur'!AI16-MAX(1,'08_Moteur'!AI16-1))*'08_Moteur'!U16,H19)))</f>
+        <v/>
+      </c>
       <c r="O19" s="17">
-        <f>IF(N19="Ne pas ouvrir",0,IF(N19="Ouvrir +1 classe",H19-'08_Moteur'!U16,IF(N19="Économiser 1 classe",H19+('08_Moteur'!AI16-MAX(1,'08_Moteur'!AI16-1))*'08_Moteur'!U16,H19)))</f>
-        <v/>
-      </c>
-      <c r="P19" s="54">
-        <f>O19-H19</f>
+        <f>M19*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P19" s="17">
+        <f>N19-O19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="54">
+        <f>N19-H19</f>
         <v/>
       </c>
     </row>
@@ -3476,37 +3536,41 @@
         <f>'08_Moteur'!AM17</f>
         <v/>
       </c>
-      <c r="I20" s="17">
-        <f>IF(N20="Ne pas ouvrir",0,E20)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J20" s="17">
-        <f>O20-I20</f>
-        <v/>
-      </c>
-      <c r="K20" s="69">
+      <c r="I20" s="68">
         <f>'08_Moteur'!AN17</f>
         <v/>
       </c>
-      <c r="L20" s="70">
-        <f>IF(H20&lt;0,"🔴 Ne pas ouvrir",IF(K20&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K20&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M20" s="71">
-        <f>IF(H20&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K20&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K20&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N20" s="21" t="inlineStr">
+      <c r="J20" s="69">
+        <f>IF(H20&lt;0,"🔴 Ne pas ouvrir",IF(I20&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I20&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K20" s="70">
+        <f>IF(H20&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I20&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I20&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L20" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M20" s="50">
+        <f>IF(L20="Ne pas ouvrir",0,IF(L20="Ouvrir +1 classe",E20+'08_Moteur'!O17,E20))</f>
+        <v/>
+      </c>
+      <c r="N20" s="17">
+        <f>IF(L20="Ne pas ouvrir",0,IF(L20="Ouvrir +1 classe",H20+'08_Moteur'!O17*('08_Moteur'!AE17*'08_Moteur'!AF17-('08_Moteur'!R17+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S17)-'08_Moteur'!U17,IF(L20="Économiser 1 classe",H20+('08_Moteur'!AI17-MAX(1,'08_Moteur'!AI17-1))*'08_Moteur'!U17,H20)))</f>
+        <v/>
+      </c>
       <c r="O20" s="17">
-        <f>IF(N20="Ne pas ouvrir",0,IF(N20="Ouvrir +1 classe",H20-'08_Moteur'!U17,IF(N20="Économiser 1 classe",H20+('08_Moteur'!AI17-MAX(1,'08_Moteur'!AI17-1))*'08_Moteur'!U17,H20)))</f>
-        <v/>
-      </c>
-      <c r="P20" s="54">
-        <f>O20-H20</f>
+        <f>M20*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P20" s="17">
+        <f>N20-O20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="54">
+        <f>N20-H20</f>
         <v/>
       </c>
     </row>
@@ -3543,37 +3607,41 @@
         <f>'08_Moteur'!AM18</f>
         <v/>
       </c>
-      <c r="I21" s="17">
-        <f>IF(N21="Ne pas ouvrir",0,E21)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J21" s="17">
-        <f>O21-I21</f>
-        <v/>
-      </c>
-      <c r="K21" s="69">
+      <c r="I21" s="68">
         <f>'08_Moteur'!AN18</f>
         <v/>
       </c>
-      <c r="L21" s="70">
-        <f>IF(H21&lt;0,"🔴 Ne pas ouvrir",IF(K21&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K21&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M21" s="71">
-        <f>IF(H21&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K21&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K21&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N21" s="21" t="inlineStr">
+      <c r="J21" s="69">
+        <f>IF(H21&lt;0,"🔴 Ne pas ouvrir",IF(I21&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I21&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K21" s="70">
+        <f>IF(H21&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I21&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I21&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L21" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M21" s="50">
+        <f>IF(L21="Ne pas ouvrir",0,IF(L21="Ouvrir +1 classe",E21+'08_Moteur'!O18,E21))</f>
+        <v/>
+      </c>
+      <c r="N21" s="17">
+        <f>IF(L21="Ne pas ouvrir",0,IF(L21="Ouvrir +1 classe",H21+'08_Moteur'!O18*('08_Moteur'!AE18*'08_Moteur'!AF18-('08_Moteur'!R18+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S18)-'08_Moteur'!U18,IF(L21="Économiser 1 classe",H21+('08_Moteur'!AI18-MAX(1,'08_Moteur'!AI18-1))*'08_Moteur'!U18,H21)))</f>
+        <v/>
+      </c>
       <c r="O21" s="17">
-        <f>IF(N21="Ne pas ouvrir",0,IF(N21="Ouvrir +1 classe",H21-'08_Moteur'!U18,IF(N21="Économiser 1 classe",H21+('08_Moteur'!AI18-MAX(1,'08_Moteur'!AI18-1))*'08_Moteur'!U18,H21)))</f>
-        <v/>
-      </c>
-      <c r="P21" s="54">
-        <f>O21-H21</f>
+        <f>M21*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P21" s="17">
+        <f>N21-O21</f>
+        <v/>
+      </c>
+      <c r="Q21" s="54">
+        <f>N21-H21</f>
         <v/>
       </c>
     </row>
@@ -3610,37 +3678,41 @@
         <f>'08_Moteur'!AM19</f>
         <v/>
       </c>
-      <c r="I22" s="17">
-        <f>IF(N22="Ne pas ouvrir",0,E22)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J22" s="17">
-        <f>O22-I22</f>
-        <v/>
-      </c>
-      <c r="K22" s="69">
+      <c r="I22" s="68">
         <f>'08_Moteur'!AN19</f>
         <v/>
       </c>
-      <c r="L22" s="70">
-        <f>IF(H22&lt;0,"🔴 Ne pas ouvrir",IF(K22&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K22&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M22" s="71">
-        <f>IF(H22&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K22&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K22&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N22" s="21" t="inlineStr">
+      <c r="J22" s="69">
+        <f>IF(H22&lt;0,"🔴 Ne pas ouvrir",IF(I22&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I22&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K22" s="70">
+        <f>IF(H22&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I22&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I22&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L22" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M22" s="50">
+        <f>IF(L22="Ne pas ouvrir",0,IF(L22="Ouvrir +1 classe",E22+'08_Moteur'!O19,E22))</f>
+        <v/>
+      </c>
+      <c r="N22" s="17">
+        <f>IF(L22="Ne pas ouvrir",0,IF(L22="Ouvrir +1 classe",H22+'08_Moteur'!O19*('08_Moteur'!AE19*'08_Moteur'!AF19-('08_Moteur'!R19+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S19)-'08_Moteur'!U19,IF(L22="Économiser 1 classe",H22+('08_Moteur'!AI19-MAX(1,'08_Moteur'!AI19-1))*'08_Moteur'!U19,H22)))</f>
+        <v/>
+      </c>
       <c r="O22" s="17">
-        <f>IF(N22="Ne pas ouvrir",0,IF(N22="Ouvrir +1 classe",H22-'08_Moteur'!U19,IF(N22="Économiser 1 classe",H22+('08_Moteur'!AI19-MAX(1,'08_Moteur'!AI19-1))*'08_Moteur'!U19,H22)))</f>
-        <v/>
-      </c>
-      <c r="P22" s="54">
-        <f>O22-H22</f>
+        <f>M22*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P22" s="17">
+        <f>N22-O22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="54">
+        <f>N22-H22</f>
         <v/>
       </c>
     </row>
@@ -3677,37 +3749,41 @@
         <f>'08_Moteur'!AM20</f>
         <v/>
       </c>
-      <c r="I23" s="17">
-        <f>IF(N23="Ne pas ouvrir",0,E23)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J23" s="17">
-        <f>O23-I23</f>
-        <v/>
-      </c>
-      <c r="K23" s="69">
+      <c r="I23" s="68">
         <f>'08_Moteur'!AN20</f>
         <v/>
       </c>
-      <c r="L23" s="70">
-        <f>IF(H23&lt;0,"🔴 Ne pas ouvrir",IF(K23&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K23&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M23" s="71">
-        <f>IF(H23&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K23&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K23&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N23" s="21" t="inlineStr">
+      <c r="J23" s="69">
+        <f>IF(H23&lt;0,"🔴 Ne pas ouvrir",IF(I23&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I23&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K23" s="70">
+        <f>IF(H23&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I23&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I23&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L23" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M23" s="50">
+        <f>IF(L23="Ne pas ouvrir",0,IF(L23="Ouvrir +1 classe",E23+'08_Moteur'!O20,E23))</f>
+        <v/>
+      </c>
+      <c r="N23" s="17">
+        <f>IF(L23="Ne pas ouvrir",0,IF(L23="Ouvrir +1 classe",H23+'08_Moteur'!O20*('08_Moteur'!AE20*'08_Moteur'!AF20-('08_Moteur'!R20+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S20)-'08_Moteur'!U20,IF(L23="Économiser 1 classe",H23+('08_Moteur'!AI20-MAX(1,'08_Moteur'!AI20-1))*'08_Moteur'!U20,H23)))</f>
+        <v/>
+      </c>
       <c r="O23" s="17">
-        <f>IF(N23="Ne pas ouvrir",0,IF(N23="Ouvrir +1 classe",H23-'08_Moteur'!U20,IF(N23="Économiser 1 classe",H23+('08_Moteur'!AI20-MAX(1,'08_Moteur'!AI20-1))*'08_Moteur'!U20,H23)))</f>
-        <v/>
-      </c>
-      <c r="P23" s="54">
-        <f>O23-H23</f>
+        <f>M23*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P23" s="17">
+        <f>N23-O23</f>
+        <v/>
+      </c>
+      <c r="Q23" s="54">
+        <f>N23-H23</f>
         <v/>
       </c>
     </row>
@@ -3744,37 +3820,41 @@
         <f>'08_Moteur'!AM21</f>
         <v/>
       </c>
-      <c r="I24" s="17">
-        <f>IF(N24="Ne pas ouvrir",0,E24)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J24" s="17">
-        <f>O24-I24</f>
-        <v/>
-      </c>
-      <c r="K24" s="69">
+      <c r="I24" s="68">
         <f>'08_Moteur'!AN21</f>
         <v/>
       </c>
-      <c r="L24" s="70">
-        <f>IF(H24&lt;0,"🔴 Ne pas ouvrir",IF(K24&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K24&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M24" s="71">
-        <f>IF(H24&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K24&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K24&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N24" s="21" t="inlineStr">
+      <c r="J24" s="69">
+        <f>IF(H24&lt;0,"🔴 Ne pas ouvrir",IF(I24&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I24&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K24" s="70">
+        <f>IF(H24&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I24&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I24&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L24" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M24" s="50">
+        <f>IF(L24="Ne pas ouvrir",0,IF(L24="Ouvrir +1 classe",E24+'08_Moteur'!O21,E24))</f>
+        <v/>
+      </c>
+      <c r="N24" s="17">
+        <f>IF(L24="Ne pas ouvrir",0,IF(L24="Ouvrir +1 classe",H24+'08_Moteur'!O21*('08_Moteur'!AE21*'08_Moteur'!AF21-('08_Moteur'!R21+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S21)-'08_Moteur'!U21,IF(L24="Économiser 1 classe",H24+('08_Moteur'!AI21-MAX(1,'08_Moteur'!AI21-1))*'08_Moteur'!U21,H24)))</f>
+        <v/>
+      </c>
       <c r="O24" s="17">
-        <f>IF(N24="Ne pas ouvrir",0,IF(N24="Ouvrir +1 classe",H24-'08_Moteur'!U21,IF(N24="Économiser 1 classe",H24+('08_Moteur'!AI21-MAX(1,'08_Moteur'!AI21-1))*'08_Moteur'!U21,H24)))</f>
-        <v/>
-      </c>
-      <c r="P24" s="54">
-        <f>O24-H24</f>
+        <f>M24*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P24" s="17">
+        <f>N24-O24</f>
+        <v/>
+      </c>
+      <c r="Q24" s="54">
+        <f>N24-H24</f>
         <v/>
       </c>
     </row>
@@ -3811,37 +3891,41 @@
         <f>'08_Moteur'!AM22</f>
         <v/>
       </c>
-      <c r="I25" s="17">
-        <f>IF(N25="Ne pas ouvrir",0,E25)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J25" s="17">
-        <f>O25-I25</f>
-        <v/>
-      </c>
-      <c r="K25" s="69">
+      <c r="I25" s="68">
         <f>'08_Moteur'!AN22</f>
         <v/>
       </c>
-      <c r="L25" s="70">
-        <f>IF(H25&lt;0,"🔴 Ne pas ouvrir",IF(K25&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K25&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M25" s="71">
-        <f>IF(H25&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K25&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K25&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N25" s="21" t="inlineStr">
+      <c r="J25" s="69">
+        <f>IF(H25&lt;0,"🔴 Ne pas ouvrir",IF(I25&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I25&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K25" s="70">
+        <f>IF(H25&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I25&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I25&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L25" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M25" s="50">
+        <f>IF(L25="Ne pas ouvrir",0,IF(L25="Ouvrir +1 classe",E25+'08_Moteur'!O22,E25))</f>
+        <v/>
+      </c>
+      <c r="N25" s="17">
+        <f>IF(L25="Ne pas ouvrir",0,IF(L25="Ouvrir +1 classe",H25+'08_Moteur'!O22*('08_Moteur'!AE22*'08_Moteur'!AF22-('08_Moteur'!R22+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S22)-'08_Moteur'!U22,IF(L25="Économiser 1 classe",H25+('08_Moteur'!AI22-MAX(1,'08_Moteur'!AI22-1))*'08_Moteur'!U22,H25)))</f>
+        <v/>
+      </c>
       <c r="O25" s="17">
-        <f>IF(N25="Ne pas ouvrir",0,IF(N25="Ouvrir +1 classe",H25-'08_Moteur'!U22,IF(N25="Économiser 1 classe",H25+('08_Moteur'!AI22-MAX(1,'08_Moteur'!AI22-1))*'08_Moteur'!U22,H25)))</f>
-        <v/>
-      </c>
-      <c r="P25" s="54">
-        <f>O25-H25</f>
+        <f>M25*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P25" s="17">
+        <f>N25-O25</f>
+        <v/>
+      </c>
+      <c r="Q25" s="54">
+        <f>N25-H25</f>
         <v/>
       </c>
     </row>
@@ -3878,37 +3962,41 @@
         <f>'08_Moteur'!AM23</f>
         <v/>
       </c>
-      <c r="I26" s="17">
-        <f>IF(N26="Ne pas ouvrir",0,E26)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J26" s="17">
-        <f>O26-I26</f>
-        <v/>
-      </c>
-      <c r="K26" s="69">
+      <c r="I26" s="68">
         <f>'08_Moteur'!AN23</f>
         <v/>
       </c>
-      <c r="L26" s="70">
-        <f>IF(H26&lt;0,"🔴 Ne pas ouvrir",IF(K26&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K26&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M26" s="71">
-        <f>IF(H26&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K26&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K26&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N26" s="21" t="inlineStr">
+      <c r="J26" s="69">
+        <f>IF(H26&lt;0,"🔴 Ne pas ouvrir",IF(I26&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I26&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K26" s="70">
+        <f>IF(H26&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I26&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I26&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L26" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M26" s="50">
+        <f>IF(L26="Ne pas ouvrir",0,IF(L26="Ouvrir +1 classe",E26+'08_Moteur'!O23,E26))</f>
+        <v/>
+      </c>
+      <c r="N26" s="17">
+        <f>IF(L26="Ne pas ouvrir",0,IF(L26="Ouvrir +1 classe",H26+'08_Moteur'!O23*('08_Moteur'!AE23*'08_Moteur'!AF23-('08_Moteur'!R23+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S23)-'08_Moteur'!U23,IF(L26="Économiser 1 classe",H26+('08_Moteur'!AI23-MAX(1,'08_Moteur'!AI23-1))*'08_Moteur'!U23,H26)))</f>
+        <v/>
+      </c>
       <c r="O26" s="17">
-        <f>IF(N26="Ne pas ouvrir",0,IF(N26="Ouvrir +1 classe",H26-'08_Moteur'!U23,IF(N26="Économiser 1 classe",H26+('08_Moteur'!AI23-MAX(1,'08_Moteur'!AI23-1))*'08_Moteur'!U23,H26)))</f>
-        <v/>
-      </c>
-      <c r="P26" s="54">
-        <f>O26-H26</f>
+        <f>M26*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P26" s="17">
+        <f>N26-O26</f>
+        <v/>
+      </c>
+      <c r="Q26" s="54">
+        <f>N26-H26</f>
         <v/>
       </c>
     </row>
@@ -3945,37 +4033,41 @@
         <f>'08_Moteur'!AM24</f>
         <v/>
       </c>
-      <c r="I27" s="17">
-        <f>IF(N27="Ne pas ouvrir",0,E27)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J27" s="17">
-        <f>O27-I27</f>
-        <v/>
-      </c>
-      <c r="K27" s="69">
+      <c r="I27" s="68">
         <f>'08_Moteur'!AN24</f>
         <v/>
       </c>
-      <c r="L27" s="70">
-        <f>IF(H27&lt;0,"🔴 Ne pas ouvrir",IF(K27&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K27&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M27" s="71">
-        <f>IF(H27&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K27&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K27&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N27" s="21" t="inlineStr">
+      <c r="J27" s="69">
+        <f>IF(H27&lt;0,"🔴 Ne pas ouvrir",IF(I27&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I27&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K27" s="70">
+        <f>IF(H27&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I27&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I27&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L27" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M27" s="50">
+        <f>IF(L27="Ne pas ouvrir",0,IF(L27="Ouvrir +1 classe",E27+'08_Moteur'!O24,E27))</f>
+        <v/>
+      </c>
+      <c r="N27" s="17">
+        <f>IF(L27="Ne pas ouvrir",0,IF(L27="Ouvrir +1 classe",H27+'08_Moteur'!O24*('08_Moteur'!AE24*'08_Moteur'!AF24-('08_Moteur'!R24+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S24)-'08_Moteur'!U24,IF(L27="Économiser 1 classe",H27+('08_Moteur'!AI24-MAX(1,'08_Moteur'!AI24-1))*'08_Moteur'!U24,H27)))</f>
+        <v/>
+      </c>
       <c r="O27" s="17">
-        <f>IF(N27="Ne pas ouvrir",0,IF(N27="Ouvrir +1 classe",H27-'08_Moteur'!U24,IF(N27="Économiser 1 classe",H27+('08_Moteur'!AI24-MAX(1,'08_Moteur'!AI24-1))*'08_Moteur'!U24,H27)))</f>
-        <v/>
-      </c>
-      <c r="P27" s="54">
-        <f>O27-H27</f>
+        <f>M27*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P27" s="17">
+        <f>N27-O27</f>
+        <v/>
+      </c>
+      <c r="Q27" s="54">
+        <f>N27-H27</f>
         <v/>
       </c>
     </row>
@@ -4012,37 +4104,41 @@
         <f>'08_Moteur'!AM25</f>
         <v/>
       </c>
-      <c r="I28" s="17">
-        <f>IF(N28="Ne pas ouvrir",0,E28)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J28" s="17">
-        <f>O28-I28</f>
-        <v/>
-      </c>
-      <c r="K28" s="69">
+      <c r="I28" s="68">
         <f>'08_Moteur'!AN25</f>
         <v/>
       </c>
-      <c r="L28" s="70">
-        <f>IF(H28&lt;0,"🔴 Ne pas ouvrir",IF(K28&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K28&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M28" s="71">
-        <f>IF(H28&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K28&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K28&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N28" s="21" t="inlineStr">
+      <c r="J28" s="69">
+        <f>IF(H28&lt;0,"🔴 Ne pas ouvrir",IF(I28&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I28&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K28" s="70">
+        <f>IF(H28&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I28&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I28&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L28" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M28" s="50">
+        <f>IF(L28="Ne pas ouvrir",0,IF(L28="Ouvrir +1 classe",E28+'08_Moteur'!O25,E28))</f>
+        <v/>
+      </c>
+      <c r="N28" s="17">
+        <f>IF(L28="Ne pas ouvrir",0,IF(L28="Ouvrir +1 classe",H28+'08_Moteur'!O25*('08_Moteur'!AE25*'08_Moteur'!AF25-('08_Moteur'!R25+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S25)-'08_Moteur'!U25,IF(L28="Économiser 1 classe",H28+('08_Moteur'!AI25-MAX(1,'08_Moteur'!AI25-1))*'08_Moteur'!U25,H28)))</f>
+        <v/>
+      </c>
       <c r="O28" s="17">
-        <f>IF(N28="Ne pas ouvrir",0,IF(N28="Ouvrir +1 classe",H28-'08_Moteur'!U25,IF(N28="Économiser 1 classe",H28+('08_Moteur'!AI25-MAX(1,'08_Moteur'!AI25-1))*'08_Moteur'!U25,H28)))</f>
-        <v/>
-      </c>
-      <c r="P28" s="54">
-        <f>O28-H28</f>
+        <f>M28*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P28" s="17">
+        <f>N28-O28</f>
+        <v/>
+      </c>
+      <c r="Q28" s="54">
+        <f>N28-H28</f>
         <v/>
       </c>
     </row>
@@ -4079,37 +4175,41 @@
         <f>'08_Moteur'!AM26</f>
         <v/>
       </c>
-      <c r="I29" s="17">
-        <f>IF(N29="Ne pas ouvrir",0,E29)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J29" s="17">
-        <f>O29-I29</f>
-        <v/>
-      </c>
-      <c r="K29" s="69">
+      <c r="I29" s="68">
         <f>'08_Moteur'!AN26</f>
         <v/>
       </c>
-      <c r="L29" s="70">
-        <f>IF(H29&lt;0,"🔴 Ne pas ouvrir",IF(K29&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K29&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M29" s="71">
-        <f>IF(H29&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K29&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K29&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N29" s="21" t="inlineStr">
+      <c r="J29" s="69">
+        <f>IF(H29&lt;0,"🔴 Ne pas ouvrir",IF(I29&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I29&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K29" s="70">
+        <f>IF(H29&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I29&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I29&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L29" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M29" s="50">
+        <f>IF(L29="Ne pas ouvrir",0,IF(L29="Ouvrir +1 classe",E29+'08_Moteur'!O26,E29))</f>
+        <v/>
+      </c>
+      <c r="N29" s="17">
+        <f>IF(L29="Ne pas ouvrir",0,IF(L29="Ouvrir +1 classe",H29+'08_Moteur'!O26*('08_Moteur'!AE26*'08_Moteur'!AF26-('08_Moteur'!R26+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S26)-'08_Moteur'!U26,IF(L29="Économiser 1 classe",H29+('08_Moteur'!AI26-MAX(1,'08_Moteur'!AI26-1))*'08_Moteur'!U26,H29)))</f>
+        <v/>
+      </c>
       <c r="O29" s="17">
-        <f>IF(N29="Ne pas ouvrir",0,IF(N29="Ouvrir +1 classe",H29-'08_Moteur'!U26,IF(N29="Économiser 1 classe",H29+('08_Moteur'!AI26-MAX(1,'08_Moteur'!AI26-1))*'08_Moteur'!U26,H29)))</f>
-        <v/>
-      </c>
-      <c r="P29" s="54">
-        <f>O29-H29</f>
+        <f>M29*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P29" s="17">
+        <f>N29-O29</f>
+        <v/>
+      </c>
+      <c r="Q29" s="54">
+        <f>N29-H29</f>
         <v/>
       </c>
     </row>
@@ -4146,37 +4246,41 @@
         <f>'08_Moteur'!AM27</f>
         <v/>
       </c>
-      <c r="I30" s="17">
-        <f>IF(N30="Ne pas ouvrir",0,E30)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J30" s="17">
-        <f>O30-I30</f>
-        <v/>
-      </c>
-      <c r="K30" s="69">
+      <c r="I30" s="68">
         <f>'08_Moteur'!AN27</f>
         <v/>
       </c>
-      <c r="L30" s="70">
-        <f>IF(H30&lt;0,"🔴 Ne pas ouvrir",IF(K30&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K30&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M30" s="71">
-        <f>IF(H30&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K30&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K30&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N30" s="21" t="inlineStr">
+      <c r="J30" s="69">
+        <f>IF(H30&lt;0,"🔴 Ne pas ouvrir",IF(I30&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I30&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K30" s="70">
+        <f>IF(H30&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I30&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I30&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L30" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M30" s="50">
+        <f>IF(L30="Ne pas ouvrir",0,IF(L30="Ouvrir +1 classe",E30+'08_Moteur'!O27,E30))</f>
+        <v/>
+      </c>
+      <c r="N30" s="17">
+        <f>IF(L30="Ne pas ouvrir",0,IF(L30="Ouvrir +1 classe",H30+'08_Moteur'!O27*('08_Moteur'!AE27*'08_Moteur'!AF27-('08_Moteur'!R27+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S27)-'08_Moteur'!U27,IF(L30="Économiser 1 classe",H30+('08_Moteur'!AI27-MAX(1,'08_Moteur'!AI27-1))*'08_Moteur'!U27,H30)))</f>
+        <v/>
+      </c>
       <c r="O30" s="17">
-        <f>IF(N30="Ne pas ouvrir",0,IF(N30="Ouvrir +1 classe",H30-'08_Moteur'!U27,IF(N30="Économiser 1 classe",H30+('08_Moteur'!AI27-MAX(1,'08_Moteur'!AI27-1))*'08_Moteur'!U27,H30)))</f>
-        <v/>
-      </c>
-      <c r="P30" s="54">
-        <f>O30-H30</f>
+        <f>M30*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P30" s="17">
+        <f>N30-O30</f>
+        <v/>
+      </c>
+      <c r="Q30" s="54">
+        <f>N30-H30</f>
         <v/>
       </c>
     </row>
@@ -4213,37 +4317,41 @@
         <f>'08_Moteur'!AM28</f>
         <v/>
       </c>
-      <c r="I31" s="17">
-        <f>IF(N31="Ne pas ouvrir",0,E31)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J31" s="17">
-        <f>O31-I31</f>
-        <v/>
-      </c>
-      <c r="K31" s="69">
+      <c r="I31" s="68">
         <f>'08_Moteur'!AN28</f>
         <v/>
       </c>
-      <c r="L31" s="70">
-        <f>IF(H31&lt;0,"🔴 Ne pas ouvrir",IF(K31&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K31&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M31" s="71">
-        <f>IF(H31&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K31&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K31&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N31" s="21" t="inlineStr">
+      <c r="J31" s="69">
+        <f>IF(H31&lt;0,"🔴 Ne pas ouvrir",IF(I31&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I31&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K31" s="70">
+        <f>IF(H31&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I31&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I31&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L31" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M31" s="50">
+        <f>IF(L31="Ne pas ouvrir",0,IF(L31="Ouvrir +1 classe",E31+'08_Moteur'!O28,E31))</f>
+        <v/>
+      </c>
+      <c r="N31" s="17">
+        <f>IF(L31="Ne pas ouvrir",0,IF(L31="Ouvrir +1 classe",H31+'08_Moteur'!O28*('08_Moteur'!AE28*'08_Moteur'!AF28-('08_Moteur'!R28+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S28)-'08_Moteur'!U28,IF(L31="Économiser 1 classe",H31+('08_Moteur'!AI28-MAX(1,'08_Moteur'!AI28-1))*'08_Moteur'!U28,H31)))</f>
+        <v/>
+      </c>
       <c r="O31" s="17">
-        <f>IF(N31="Ne pas ouvrir",0,IF(N31="Ouvrir +1 classe",H31-'08_Moteur'!U28,IF(N31="Économiser 1 classe",H31+('08_Moteur'!AI28-MAX(1,'08_Moteur'!AI28-1))*'08_Moteur'!U28,H31)))</f>
-        <v/>
-      </c>
-      <c r="P31" s="54">
-        <f>O31-H31</f>
+        <f>M31*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P31" s="17">
+        <f>N31-O31</f>
+        <v/>
+      </c>
+      <c r="Q31" s="54">
+        <f>N31-H31</f>
         <v/>
       </c>
     </row>
@@ -4280,37 +4388,41 @@
         <f>'08_Moteur'!AM29</f>
         <v/>
       </c>
-      <c r="I32" s="17">
-        <f>IF(N32="Ne pas ouvrir",0,E32)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J32" s="17">
-        <f>O32-I32</f>
-        <v/>
-      </c>
-      <c r="K32" s="69">
+      <c r="I32" s="68">
         <f>'08_Moteur'!AN29</f>
         <v/>
       </c>
-      <c r="L32" s="70">
-        <f>IF(H32&lt;0,"🔴 Ne pas ouvrir",IF(K32&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K32&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M32" s="71">
-        <f>IF(H32&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K32&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K32&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N32" s="21" t="inlineStr">
+      <c r="J32" s="69">
+        <f>IF(H32&lt;0,"🔴 Ne pas ouvrir",IF(I32&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I32&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K32" s="70">
+        <f>IF(H32&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I32&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I32&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L32" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M32" s="50">
+        <f>IF(L32="Ne pas ouvrir",0,IF(L32="Ouvrir +1 classe",E32+'08_Moteur'!O29,E32))</f>
+        <v/>
+      </c>
+      <c r="N32" s="17">
+        <f>IF(L32="Ne pas ouvrir",0,IF(L32="Ouvrir +1 classe",H32+'08_Moteur'!O29*('08_Moteur'!AE29*'08_Moteur'!AF29-('08_Moteur'!R29+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S29)-'08_Moteur'!U29,IF(L32="Économiser 1 classe",H32+('08_Moteur'!AI29-MAX(1,'08_Moteur'!AI29-1))*'08_Moteur'!U29,H32)))</f>
+        <v/>
+      </c>
       <c r="O32" s="17">
-        <f>IF(N32="Ne pas ouvrir",0,IF(N32="Ouvrir +1 classe",H32-'08_Moteur'!U29,IF(N32="Économiser 1 classe",H32+('08_Moteur'!AI29-MAX(1,'08_Moteur'!AI29-1))*'08_Moteur'!U29,H32)))</f>
-        <v/>
-      </c>
-      <c r="P32" s="54">
-        <f>O32-H32</f>
+        <f>M32*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P32" s="17">
+        <f>N32-O32</f>
+        <v/>
+      </c>
+      <c r="Q32" s="54">
+        <f>N32-H32</f>
         <v/>
       </c>
     </row>
@@ -4347,37 +4459,41 @@
         <f>'08_Moteur'!AM30</f>
         <v/>
       </c>
-      <c r="I33" s="17">
-        <f>IF(N33="Ne pas ouvrir",0,E33)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J33" s="17">
-        <f>O33-I33</f>
-        <v/>
-      </c>
-      <c r="K33" s="69">
+      <c r="I33" s="68">
         <f>'08_Moteur'!AN30</f>
         <v/>
       </c>
-      <c r="L33" s="70">
-        <f>IF(H33&lt;0,"🔴 Ne pas ouvrir",IF(K33&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K33&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M33" s="71">
-        <f>IF(H33&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K33&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K33&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N33" s="21" t="inlineStr">
+      <c r="J33" s="69">
+        <f>IF(H33&lt;0,"🔴 Ne pas ouvrir",IF(I33&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I33&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K33" s="70">
+        <f>IF(H33&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I33&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I33&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L33" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M33" s="50">
+        <f>IF(L33="Ne pas ouvrir",0,IF(L33="Ouvrir +1 classe",E33+'08_Moteur'!O30,E33))</f>
+        <v/>
+      </c>
+      <c r="N33" s="17">
+        <f>IF(L33="Ne pas ouvrir",0,IF(L33="Ouvrir +1 classe",H33+'08_Moteur'!O30*('08_Moteur'!AE30*'08_Moteur'!AF30-('08_Moteur'!R30+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S30)-'08_Moteur'!U30,IF(L33="Économiser 1 classe",H33+('08_Moteur'!AI30-MAX(1,'08_Moteur'!AI30-1))*'08_Moteur'!U30,H33)))</f>
+        <v/>
+      </c>
       <c r="O33" s="17">
-        <f>IF(N33="Ne pas ouvrir",0,IF(N33="Ouvrir +1 classe",H33-'08_Moteur'!U30,IF(N33="Économiser 1 classe",H33+('08_Moteur'!AI30-MAX(1,'08_Moteur'!AI30-1))*'08_Moteur'!U30,H33)))</f>
-        <v/>
-      </c>
-      <c r="P33" s="54">
-        <f>O33-H33</f>
+        <f>M33*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P33" s="17">
+        <f>N33-O33</f>
+        <v/>
+      </c>
+      <c r="Q33" s="54">
+        <f>N33-H33</f>
         <v/>
       </c>
     </row>
@@ -4414,37 +4530,41 @@
         <f>'08_Moteur'!AM31</f>
         <v/>
       </c>
-      <c r="I34" s="17">
-        <f>IF(N34="Ne pas ouvrir",0,E34)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J34" s="17">
-        <f>O34-I34</f>
-        <v/>
-      </c>
-      <c r="K34" s="69">
+      <c r="I34" s="68">
         <f>'08_Moteur'!AN31</f>
         <v/>
       </c>
-      <c r="L34" s="70">
-        <f>IF(H34&lt;0,"🔴 Ne pas ouvrir",IF(K34&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K34&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M34" s="71">
-        <f>IF(H34&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K34&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K34&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N34" s="21" t="inlineStr">
+      <c r="J34" s="69">
+        <f>IF(H34&lt;0,"🔴 Ne pas ouvrir",IF(I34&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I34&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K34" s="70">
+        <f>IF(H34&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I34&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I34&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L34" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M34" s="50">
+        <f>IF(L34="Ne pas ouvrir",0,IF(L34="Ouvrir +1 classe",E34+'08_Moteur'!O31,E34))</f>
+        <v/>
+      </c>
+      <c r="N34" s="17">
+        <f>IF(L34="Ne pas ouvrir",0,IF(L34="Ouvrir +1 classe",H34+'08_Moteur'!O31*('08_Moteur'!AE31*'08_Moteur'!AF31-('08_Moteur'!R31+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S31)-'08_Moteur'!U31,IF(L34="Économiser 1 classe",H34+('08_Moteur'!AI31-MAX(1,'08_Moteur'!AI31-1))*'08_Moteur'!U31,H34)))</f>
+        <v/>
+      </c>
       <c r="O34" s="17">
-        <f>IF(N34="Ne pas ouvrir",0,IF(N34="Ouvrir +1 classe",H34-'08_Moteur'!U31,IF(N34="Économiser 1 classe",H34+('08_Moteur'!AI31-MAX(1,'08_Moteur'!AI31-1))*'08_Moteur'!U31,H34)))</f>
-        <v/>
-      </c>
-      <c r="P34" s="54">
-        <f>O34-H34</f>
+        <f>M34*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P34" s="17">
+        <f>N34-O34</f>
+        <v/>
+      </c>
+      <c r="Q34" s="54">
+        <f>N34-H34</f>
         <v/>
       </c>
     </row>
@@ -4481,37 +4601,41 @@
         <f>'08_Moteur'!AM32</f>
         <v/>
       </c>
-      <c r="I35" s="17">
-        <f>IF(N35="Ne pas ouvrir",0,E35)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J35" s="17">
-        <f>O35-I35</f>
-        <v/>
-      </c>
-      <c r="K35" s="69">
+      <c r="I35" s="68">
         <f>'08_Moteur'!AN32</f>
         <v/>
       </c>
-      <c r="L35" s="70">
-        <f>IF(H35&lt;0,"🔴 Ne pas ouvrir",IF(K35&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K35&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M35" s="71">
-        <f>IF(H35&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K35&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K35&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N35" s="21" t="inlineStr">
+      <c r="J35" s="69">
+        <f>IF(H35&lt;0,"🔴 Ne pas ouvrir",IF(I35&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I35&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K35" s="70">
+        <f>IF(H35&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I35&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I35&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L35" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M35" s="50">
+        <f>IF(L35="Ne pas ouvrir",0,IF(L35="Ouvrir +1 classe",E35+'08_Moteur'!O32,E35))</f>
+        <v/>
+      </c>
+      <c r="N35" s="17">
+        <f>IF(L35="Ne pas ouvrir",0,IF(L35="Ouvrir +1 classe",H35+'08_Moteur'!O32*('08_Moteur'!AE32*'08_Moteur'!AF32-('08_Moteur'!R32+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S32)-'08_Moteur'!U32,IF(L35="Économiser 1 classe",H35+('08_Moteur'!AI32-MAX(1,'08_Moteur'!AI32-1))*'08_Moteur'!U32,H35)))</f>
+        <v/>
+      </c>
       <c r="O35" s="17">
-        <f>IF(N35="Ne pas ouvrir",0,IF(N35="Ouvrir +1 classe",H35-'08_Moteur'!U32,IF(N35="Économiser 1 classe",H35+('08_Moteur'!AI32-MAX(1,'08_Moteur'!AI32-1))*'08_Moteur'!U32,H35)))</f>
-        <v/>
-      </c>
-      <c r="P35" s="54">
-        <f>O35-H35</f>
+        <f>M35*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P35" s="17">
+        <f>N35-O35</f>
+        <v/>
+      </c>
+      <c r="Q35" s="54">
+        <f>N35-H35</f>
         <v/>
       </c>
     </row>
@@ -4548,37 +4672,41 @@
         <f>'08_Moteur'!AM33</f>
         <v/>
       </c>
-      <c r="I36" s="17">
-        <f>IF(N36="Ne pas ouvrir",0,E36)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J36" s="17">
-        <f>O36-I36</f>
-        <v/>
-      </c>
-      <c r="K36" s="69">
+      <c r="I36" s="68">
         <f>'08_Moteur'!AN33</f>
         <v/>
       </c>
-      <c r="L36" s="70">
-        <f>IF(H36&lt;0,"🔴 Ne pas ouvrir",IF(K36&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K36&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M36" s="71">
-        <f>IF(H36&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K36&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K36&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N36" s="21" t="inlineStr">
+      <c r="J36" s="69">
+        <f>IF(H36&lt;0,"🔴 Ne pas ouvrir",IF(I36&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I36&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K36" s="70">
+        <f>IF(H36&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I36&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I36&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L36" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M36" s="50">
+        <f>IF(L36="Ne pas ouvrir",0,IF(L36="Ouvrir +1 classe",E36+'08_Moteur'!O33,E36))</f>
+        <v/>
+      </c>
+      <c r="N36" s="17">
+        <f>IF(L36="Ne pas ouvrir",0,IF(L36="Ouvrir +1 classe",H36+'08_Moteur'!O33*('08_Moteur'!AE33*'08_Moteur'!AF33-('08_Moteur'!R33+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S33)-'08_Moteur'!U33,IF(L36="Économiser 1 classe",H36+('08_Moteur'!AI33-MAX(1,'08_Moteur'!AI33-1))*'08_Moteur'!U33,H36)))</f>
+        <v/>
+      </c>
       <c r="O36" s="17">
-        <f>IF(N36="Ne pas ouvrir",0,IF(N36="Ouvrir +1 classe",H36-'08_Moteur'!U33,IF(N36="Économiser 1 classe",H36+('08_Moteur'!AI33-MAX(1,'08_Moteur'!AI33-1))*'08_Moteur'!U33,H36)))</f>
-        <v/>
-      </c>
-      <c r="P36" s="54">
-        <f>O36-H36</f>
+        <f>M36*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P36" s="17">
+        <f>N36-O36</f>
+        <v/>
+      </c>
+      <c r="Q36" s="54">
+        <f>N36-H36</f>
         <v/>
       </c>
     </row>
@@ -4615,37 +4743,41 @@
         <f>'08_Moteur'!AM34</f>
         <v/>
       </c>
-      <c r="I37" s="17">
-        <f>IF(N37="Ne pas ouvrir",0,E37)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J37" s="17">
-        <f>O37-I37</f>
-        <v/>
-      </c>
-      <c r="K37" s="69">
+      <c r="I37" s="68">
         <f>'08_Moteur'!AN34</f>
         <v/>
       </c>
-      <c r="L37" s="70">
-        <f>IF(H37&lt;0,"🔴 Ne pas ouvrir",IF(K37&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K37&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M37" s="71">
-        <f>IF(H37&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K37&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K37&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N37" s="21" t="inlineStr">
+      <c r="J37" s="69">
+        <f>IF(H37&lt;0,"🔴 Ne pas ouvrir",IF(I37&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I37&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K37" s="70">
+        <f>IF(H37&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I37&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I37&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L37" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M37" s="50">
+        <f>IF(L37="Ne pas ouvrir",0,IF(L37="Ouvrir +1 classe",E37+'08_Moteur'!O34,E37))</f>
+        <v/>
+      </c>
+      <c r="N37" s="17">
+        <f>IF(L37="Ne pas ouvrir",0,IF(L37="Ouvrir +1 classe",H37+'08_Moteur'!O34*('08_Moteur'!AE34*'08_Moteur'!AF34-('08_Moteur'!R34+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S34)-'08_Moteur'!U34,IF(L37="Économiser 1 classe",H37+('08_Moteur'!AI34-MAX(1,'08_Moteur'!AI34-1))*'08_Moteur'!U34,H37)))</f>
+        <v/>
+      </c>
       <c r="O37" s="17">
-        <f>IF(N37="Ne pas ouvrir",0,IF(N37="Ouvrir +1 classe",H37-'08_Moteur'!U34,IF(N37="Économiser 1 classe",H37+('08_Moteur'!AI34-MAX(1,'08_Moteur'!AI34-1))*'08_Moteur'!U34,H37)))</f>
-        <v/>
-      </c>
-      <c r="P37" s="54">
-        <f>O37-H37</f>
+        <f>M37*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P37" s="17">
+        <f>N37-O37</f>
+        <v/>
+      </c>
+      <c r="Q37" s="54">
+        <f>N37-H37</f>
         <v/>
       </c>
     </row>
@@ -4682,37 +4814,41 @@
         <f>'08_Moteur'!AM35</f>
         <v/>
       </c>
-      <c r="I38" s="17">
-        <f>IF(N38="Ne pas ouvrir",0,E38)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J38" s="17">
-        <f>O38-I38</f>
-        <v/>
-      </c>
-      <c r="K38" s="69">
+      <c r="I38" s="68">
         <f>'08_Moteur'!AN35</f>
         <v/>
       </c>
-      <c r="L38" s="70">
-        <f>IF(H38&lt;0,"🔴 Ne pas ouvrir",IF(K38&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K38&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M38" s="71">
-        <f>IF(H38&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K38&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K38&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N38" s="21" t="inlineStr">
+      <c r="J38" s="69">
+        <f>IF(H38&lt;0,"🔴 Ne pas ouvrir",IF(I38&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I38&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K38" s="70">
+        <f>IF(H38&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I38&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I38&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L38" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M38" s="50">
+        <f>IF(L38="Ne pas ouvrir",0,IF(L38="Ouvrir +1 classe",E38+'08_Moteur'!O35,E38))</f>
+        <v/>
+      </c>
+      <c r="N38" s="17">
+        <f>IF(L38="Ne pas ouvrir",0,IF(L38="Ouvrir +1 classe",H38+'08_Moteur'!O35*('08_Moteur'!AE35*'08_Moteur'!AF35-('08_Moteur'!R35+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S35)-'08_Moteur'!U35,IF(L38="Économiser 1 classe",H38+('08_Moteur'!AI35-MAX(1,'08_Moteur'!AI35-1))*'08_Moteur'!U35,H38)))</f>
+        <v/>
+      </c>
       <c r="O38" s="17">
-        <f>IF(N38="Ne pas ouvrir",0,IF(N38="Ouvrir +1 classe",H38-'08_Moteur'!U35,IF(N38="Économiser 1 classe",H38+('08_Moteur'!AI35-MAX(1,'08_Moteur'!AI35-1))*'08_Moteur'!U35,H38)))</f>
-        <v/>
-      </c>
-      <c r="P38" s="54">
-        <f>O38-H38</f>
+        <f>M38*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P38" s="17">
+        <f>N38-O38</f>
+        <v/>
+      </c>
+      <c r="Q38" s="54">
+        <f>N38-H38</f>
         <v/>
       </c>
     </row>
@@ -4749,37 +4885,41 @@
         <f>'08_Moteur'!AM36</f>
         <v/>
       </c>
-      <c r="I39" s="17">
-        <f>IF(N39="Ne pas ouvrir",0,E39)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J39" s="17">
-        <f>O39-I39</f>
-        <v/>
-      </c>
-      <c r="K39" s="69">
+      <c r="I39" s="68">
         <f>'08_Moteur'!AN36</f>
         <v/>
       </c>
-      <c r="L39" s="70">
-        <f>IF(H39&lt;0,"🔴 Ne pas ouvrir",IF(K39&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K39&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M39" s="71">
-        <f>IF(H39&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K39&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K39&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N39" s="21" t="inlineStr">
+      <c r="J39" s="69">
+        <f>IF(H39&lt;0,"🔴 Ne pas ouvrir",IF(I39&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I39&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K39" s="70">
+        <f>IF(H39&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I39&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I39&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L39" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M39" s="50">
+        <f>IF(L39="Ne pas ouvrir",0,IF(L39="Ouvrir +1 classe",E39+'08_Moteur'!O36,E39))</f>
+        <v/>
+      </c>
+      <c r="N39" s="17">
+        <f>IF(L39="Ne pas ouvrir",0,IF(L39="Ouvrir +1 classe",H39+'08_Moteur'!O36*('08_Moteur'!AE36*'08_Moteur'!AF36-('08_Moteur'!R36+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S36)-'08_Moteur'!U36,IF(L39="Économiser 1 classe",H39+('08_Moteur'!AI36-MAX(1,'08_Moteur'!AI36-1))*'08_Moteur'!U36,H39)))</f>
+        <v/>
+      </c>
       <c r="O39" s="17">
-        <f>IF(N39="Ne pas ouvrir",0,IF(N39="Ouvrir +1 classe",H39-'08_Moteur'!U36,IF(N39="Économiser 1 classe",H39+('08_Moteur'!AI36-MAX(1,'08_Moteur'!AI36-1))*'08_Moteur'!U36,H39)))</f>
-        <v/>
-      </c>
-      <c r="P39" s="54">
-        <f>O39-H39</f>
+        <f>M39*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P39" s="17">
+        <f>N39-O39</f>
+        <v/>
+      </c>
+      <c r="Q39" s="54">
+        <f>N39-H39</f>
         <v/>
       </c>
     </row>
@@ -4816,37 +4956,41 @@
         <f>'08_Moteur'!AM37</f>
         <v/>
       </c>
-      <c r="I40" s="17">
-        <f>IF(N40="Ne pas ouvrir",0,E40)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J40" s="17">
-        <f>O40-I40</f>
-        <v/>
-      </c>
-      <c r="K40" s="69">
+      <c r="I40" s="68">
         <f>'08_Moteur'!AN37</f>
         <v/>
       </c>
-      <c r="L40" s="70">
-        <f>IF(H40&lt;0,"🔴 Ne pas ouvrir",IF(K40&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K40&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M40" s="71">
-        <f>IF(H40&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K40&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K40&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N40" s="21" t="inlineStr">
+      <c r="J40" s="69">
+        <f>IF(H40&lt;0,"🔴 Ne pas ouvrir",IF(I40&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I40&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K40" s="70">
+        <f>IF(H40&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I40&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I40&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L40" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M40" s="50">
+        <f>IF(L40="Ne pas ouvrir",0,IF(L40="Ouvrir +1 classe",E40+'08_Moteur'!O37,E40))</f>
+        <v/>
+      </c>
+      <c r="N40" s="17">
+        <f>IF(L40="Ne pas ouvrir",0,IF(L40="Ouvrir +1 classe",H40+'08_Moteur'!O37*('08_Moteur'!AE37*'08_Moteur'!AF37-('08_Moteur'!R37+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S37)-'08_Moteur'!U37,IF(L40="Économiser 1 classe",H40+('08_Moteur'!AI37-MAX(1,'08_Moteur'!AI37-1))*'08_Moteur'!U37,H40)))</f>
+        <v/>
+      </c>
       <c r="O40" s="17">
-        <f>IF(N40="Ne pas ouvrir",0,IF(N40="Ouvrir +1 classe",H40-'08_Moteur'!U37,IF(N40="Économiser 1 classe",H40+('08_Moteur'!AI37-MAX(1,'08_Moteur'!AI37-1))*'08_Moteur'!U37,H40)))</f>
-        <v/>
-      </c>
-      <c r="P40" s="54">
-        <f>O40-H40</f>
+        <f>M40*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P40" s="17">
+        <f>N40-O40</f>
+        <v/>
+      </c>
+      <c r="Q40" s="54">
+        <f>N40-H40</f>
         <v/>
       </c>
     </row>
@@ -4883,37 +5027,41 @@
         <f>'08_Moteur'!AM38</f>
         <v/>
       </c>
-      <c r="I41" s="17">
-        <f>IF(N41="Ne pas ouvrir",0,E41)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J41" s="17">
-        <f>O41-I41</f>
-        <v/>
-      </c>
-      <c r="K41" s="69">
+      <c r="I41" s="68">
         <f>'08_Moteur'!AN38</f>
         <v/>
       </c>
-      <c r="L41" s="70">
-        <f>IF(H41&lt;0,"🔴 Ne pas ouvrir",IF(K41&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K41&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M41" s="71">
-        <f>IF(H41&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K41&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K41&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N41" s="21" t="inlineStr">
+      <c r="J41" s="69">
+        <f>IF(H41&lt;0,"🔴 Ne pas ouvrir",IF(I41&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I41&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K41" s="70">
+        <f>IF(H41&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I41&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I41&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L41" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M41" s="50">
+        <f>IF(L41="Ne pas ouvrir",0,IF(L41="Ouvrir +1 classe",E41+'08_Moteur'!O38,E41))</f>
+        <v/>
+      </c>
+      <c r="N41" s="17">
+        <f>IF(L41="Ne pas ouvrir",0,IF(L41="Ouvrir +1 classe",H41+'08_Moteur'!O38*('08_Moteur'!AE38*'08_Moteur'!AF38-('08_Moteur'!R38+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S38)-'08_Moteur'!U38,IF(L41="Économiser 1 classe",H41+('08_Moteur'!AI38-MAX(1,'08_Moteur'!AI38-1))*'08_Moteur'!U38,H41)))</f>
+        <v/>
+      </c>
       <c r="O41" s="17">
-        <f>IF(N41="Ne pas ouvrir",0,IF(N41="Ouvrir +1 classe",H41-'08_Moteur'!U38,IF(N41="Économiser 1 classe",H41+('08_Moteur'!AI38-MAX(1,'08_Moteur'!AI38-1))*'08_Moteur'!U38,H41)))</f>
-        <v/>
-      </c>
-      <c r="P41" s="54">
-        <f>O41-H41</f>
+        <f>M41*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P41" s="17">
+        <f>N41-O41</f>
+        <v/>
+      </c>
+      <c r="Q41" s="54">
+        <f>N41-H41</f>
         <v/>
       </c>
     </row>
@@ -4950,37 +5098,41 @@
         <f>'08_Moteur'!AM39</f>
         <v/>
       </c>
-      <c r="I42" s="17">
-        <f>IF(N42="Ne pas ouvrir",0,E42)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J42" s="17">
-        <f>O42-I42</f>
-        <v/>
-      </c>
-      <c r="K42" s="69">
+      <c r="I42" s="68">
         <f>'08_Moteur'!AN39</f>
         <v/>
       </c>
-      <c r="L42" s="70">
-        <f>IF(H42&lt;0,"🔴 Ne pas ouvrir",IF(K42&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K42&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M42" s="71">
-        <f>IF(H42&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K42&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K42&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N42" s="21" t="inlineStr">
+      <c r="J42" s="69">
+        <f>IF(H42&lt;0,"🔴 Ne pas ouvrir",IF(I42&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I42&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K42" s="70">
+        <f>IF(H42&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I42&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I42&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L42" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M42" s="50">
+        <f>IF(L42="Ne pas ouvrir",0,IF(L42="Ouvrir +1 classe",E42+'08_Moteur'!O39,E42))</f>
+        <v/>
+      </c>
+      <c r="N42" s="17">
+        <f>IF(L42="Ne pas ouvrir",0,IF(L42="Ouvrir +1 classe",H42+'08_Moteur'!O39*('08_Moteur'!AE39*'08_Moteur'!AF39-('08_Moteur'!R39+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S39)-'08_Moteur'!U39,IF(L42="Économiser 1 classe",H42+('08_Moteur'!AI39-MAX(1,'08_Moteur'!AI39-1))*'08_Moteur'!U39,H42)))</f>
+        <v/>
+      </c>
       <c r="O42" s="17">
-        <f>IF(N42="Ne pas ouvrir",0,IF(N42="Ouvrir +1 classe",H42-'08_Moteur'!U39,IF(N42="Économiser 1 classe",H42+('08_Moteur'!AI39-MAX(1,'08_Moteur'!AI39-1))*'08_Moteur'!U39,H42)))</f>
-        <v/>
-      </c>
-      <c r="P42" s="54">
-        <f>O42-H42</f>
+        <f>M42*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P42" s="17">
+        <f>N42-O42</f>
+        <v/>
+      </c>
+      <c r="Q42" s="54">
+        <f>N42-H42</f>
         <v/>
       </c>
     </row>
@@ -5017,37 +5169,41 @@
         <f>'08_Moteur'!AM40</f>
         <v/>
       </c>
-      <c r="I43" s="17">
-        <f>IF(N43="Ne pas ouvrir",0,E43)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J43" s="17">
-        <f>O43-I43</f>
-        <v/>
-      </c>
-      <c r="K43" s="69">
+      <c r="I43" s="68">
         <f>'08_Moteur'!AN40</f>
         <v/>
       </c>
-      <c r="L43" s="70">
-        <f>IF(H43&lt;0,"🔴 Ne pas ouvrir",IF(K43&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K43&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M43" s="71">
-        <f>IF(H43&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K43&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K43&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N43" s="21" t="inlineStr">
+      <c r="J43" s="69">
+        <f>IF(H43&lt;0,"🔴 Ne pas ouvrir",IF(I43&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I43&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K43" s="70">
+        <f>IF(H43&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I43&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I43&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L43" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M43" s="50">
+        <f>IF(L43="Ne pas ouvrir",0,IF(L43="Ouvrir +1 classe",E43+'08_Moteur'!O40,E43))</f>
+        <v/>
+      </c>
+      <c r="N43" s="17">
+        <f>IF(L43="Ne pas ouvrir",0,IF(L43="Ouvrir +1 classe",H43+'08_Moteur'!O40*('08_Moteur'!AE40*'08_Moteur'!AF40-('08_Moteur'!R40+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S40)-'08_Moteur'!U40,IF(L43="Économiser 1 classe",H43+('08_Moteur'!AI40-MAX(1,'08_Moteur'!AI40-1))*'08_Moteur'!U40,H43)))</f>
+        <v/>
+      </c>
       <c r="O43" s="17">
-        <f>IF(N43="Ne pas ouvrir",0,IF(N43="Ouvrir +1 classe",H43-'08_Moteur'!U40,IF(N43="Économiser 1 classe",H43+('08_Moteur'!AI40-MAX(1,'08_Moteur'!AI40-1))*'08_Moteur'!U40,H43)))</f>
-        <v/>
-      </c>
-      <c r="P43" s="54">
-        <f>O43-H43</f>
+        <f>M43*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P43" s="17">
+        <f>N43-O43</f>
+        <v/>
+      </c>
+      <c r="Q43" s="54">
+        <f>N43-H43</f>
         <v/>
       </c>
     </row>
@@ -5084,37 +5240,41 @@
         <f>'08_Moteur'!AM41</f>
         <v/>
       </c>
-      <c r="I44" s="17">
-        <f>IF(N44="Ne pas ouvrir",0,E44)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J44" s="17">
-        <f>O44-I44</f>
-        <v/>
-      </c>
-      <c r="K44" s="69">
+      <c r="I44" s="68">
         <f>'08_Moteur'!AN41</f>
         <v/>
       </c>
-      <c r="L44" s="70">
-        <f>IF(H44&lt;0,"🔴 Ne pas ouvrir",IF(K44&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K44&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M44" s="71">
-        <f>IF(H44&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K44&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K44&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N44" s="21" t="inlineStr">
+      <c r="J44" s="69">
+        <f>IF(H44&lt;0,"🔴 Ne pas ouvrir",IF(I44&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I44&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K44" s="70">
+        <f>IF(H44&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I44&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I44&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L44" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M44" s="50">
+        <f>IF(L44="Ne pas ouvrir",0,IF(L44="Ouvrir +1 classe",E44+'08_Moteur'!O41,E44))</f>
+        <v/>
+      </c>
+      <c r="N44" s="17">
+        <f>IF(L44="Ne pas ouvrir",0,IF(L44="Ouvrir +1 classe",H44+'08_Moteur'!O41*('08_Moteur'!AE41*'08_Moteur'!AF41-('08_Moteur'!R41+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S41)-'08_Moteur'!U41,IF(L44="Économiser 1 classe",H44+('08_Moteur'!AI41-MAX(1,'08_Moteur'!AI41-1))*'08_Moteur'!U41,H44)))</f>
+        <v/>
+      </c>
       <c r="O44" s="17">
-        <f>IF(N44="Ne pas ouvrir",0,IF(N44="Ouvrir +1 classe",H44-'08_Moteur'!U41,IF(N44="Économiser 1 classe",H44+('08_Moteur'!AI41-MAX(1,'08_Moteur'!AI41-1))*'08_Moteur'!U41,H44)))</f>
-        <v/>
-      </c>
-      <c r="P44" s="54">
-        <f>O44-H44</f>
+        <f>M44*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P44" s="17">
+        <f>N44-O44</f>
+        <v/>
+      </c>
+      <c r="Q44" s="54">
+        <f>N44-H44</f>
         <v/>
       </c>
     </row>
@@ -5151,37 +5311,41 @@
         <f>'08_Moteur'!AM42</f>
         <v/>
       </c>
-      <c r="I45" s="17">
-        <f>IF(N45="Ne pas ouvrir",0,E45)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J45" s="17">
-        <f>O45-I45</f>
-        <v/>
-      </c>
-      <c r="K45" s="69">
+      <c r="I45" s="68">
         <f>'08_Moteur'!AN42</f>
         <v/>
       </c>
-      <c r="L45" s="70">
-        <f>IF(H45&lt;0,"🔴 Ne pas ouvrir",IF(K45&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K45&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M45" s="71">
-        <f>IF(H45&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K45&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K45&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N45" s="21" t="inlineStr">
+      <c r="J45" s="69">
+        <f>IF(H45&lt;0,"🔴 Ne pas ouvrir",IF(I45&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I45&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K45" s="70">
+        <f>IF(H45&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I45&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I45&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L45" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M45" s="50">
+        <f>IF(L45="Ne pas ouvrir",0,IF(L45="Ouvrir +1 classe",E45+'08_Moteur'!O42,E45))</f>
+        <v/>
+      </c>
+      <c r="N45" s="17">
+        <f>IF(L45="Ne pas ouvrir",0,IF(L45="Ouvrir +1 classe",H45+'08_Moteur'!O42*('08_Moteur'!AE42*'08_Moteur'!AF42-('08_Moteur'!R42+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S42)-'08_Moteur'!U42,IF(L45="Économiser 1 classe",H45+('08_Moteur'!AI42-MAX(1,'08_Moteur'!AI42-1))*'08_Moteur'!U42,H45)))</f>
+        <v/>
+      </c>
       <c r="O45" s="17">
-        <f>IF(N45="Ne pas ouvrir",0,IF(N45="Ouvrir +1 classe",H45-'08_Moteur'!U42,IF(N45="Économiser 1 classe",H45+('08_Moteur'!AI42-MAX(1,'08_Moteur'!AI42-1))*'08_Moteur'!U42,H45)))</f>
-        <v/>
-      </c>
-      <c r="P45" s="54">
-        <f>O45-H45</f>
+        <f>M45*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P45" s="17">
+        <f>N45-O45</f>
+        <v/>
+      </c>
+      <c r="Q45" s="54">
+        <f>N45-H45</f>
         <v/>
       </c>
     </row>
@@ -5218,37 +5382,41 @@
         <f>'08_Moteur'!AM43</f>
         <v/>
       </c>
-      <c r="I46" s="17">
-        <f>IF(N46="Ne pas ouvrir",0,E46)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J46" s="17">
-        <f>O46-I46</f>
-        <v/>
-      </c>
-      <c r="K46" s="69">
+      <c r="I46" s="68">
         <f>'08_Moteur'!AN43</f>
         <v/>
       </c>
-      <c r="L46" s="70">
-        <f>IF(H46&lt;0,"🔴 Ne pas ouvrir",IF(K46&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K46&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M46" s="71">
-        <f>IF(H46&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K46&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K46&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N46" s="21" t="inlineStr">
+      <c r="J46" s="69">
+        <f>IF(H46&lt;0,"🔴 Ne pas ouvrir",IF(I46&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I46&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K46" s="70">
+        <f>IF(H46&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I46&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I46&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L46" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M46" s="50">
+        <f>IF(L46="Ne pas ouvrir",0,IF(L46="Ouvrir +1 classe",E46+'08_Moteur'!O43,E46))</f>
+        <v/>
+      </c>
+      <c r="N46" s="17">
+        <f>IF(L46="Ne pas ouvrir",0,IF(L46="Ouvrir +1 classe",H46+'08_Moteur'!O43*('08_Moteur'!AE43*'08_Moteur'!AF43-('08_Moteur'!R43+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S43)-'08_Moteur'!U43,IF(L46="Économiser 1 classe",H46+('08_Moteur'!AI43-MAX(1,'08_Moteur'!AI43-1))*'08_Moteur'!U43,H46)))</f>
+        <v/>
+      </c>
       <c r="O46" s="17">
-        <f>IF(N46="Ne pas ouvrir",0,IF(N46="Ouvrir +1 classe",H46-'08_Moteur'!U43,IF(N46="Économiser 1 classe",H46+('08_Moteur'!AI43-MAX(1,'08_Moteur'!AI43-1))*'08_Moteur'!U43,H46)))</f>
-        <v/>
-      </c>
-      <c r="P46" s="54">
-        <f>O46-H46</f>
+        <f>M46*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P46" s="17">
+        <f>N46-O46</f>
+        <v/>
+      </c>
+      <c r="Q46" s="54">
+        <f>N46-H46</f>
         <v/>
       </c>
     </row>
@@ -5285,37 +5453,41 @@
         <f>'08_Moteur'!AM44</f>
         <v/>
       </c>
-      <c r="I47" s="17">
-        <f>IF(N47="Ne pas ouvrir",0,E47)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J47" s="17">
-        <f>O47-I47</f>
-        <v/>
-      </c>
-      <c r="K47" s="69">
+      <c r="I47" s="68">
         <f>'08_Moteur'!AN44</f>
         <v/>
       </c>
-      <c r="L47" s="70">
-        <f>IF(H47&lt;0,"🔴 Ne pas ouvrir",IF(K47&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K47&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M47" s="71">
-        <f>IF(H47&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K47&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K47&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N47" s="21" t="inlineStr">
+      <c r="J47" s="69">
+        <f>IF(H47&lt;0,"🔴 Ne pas ouvrir",IF(I47&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I47&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K47" s="70">
+        <f>IF(H47&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I47&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I47&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L47" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M47" s="50">
+        <f>IF(L47="Ne pas ouvrir",0,IF(L47="Ouvrir +1 classe",E47+'08_Moteur'!O44,E47))</f>
+        <v/>
+      </c>
+      <c r="N47" s="17">
+        <f>IF(L47="Ne pas ouvrir",0,IF(L47="Ouvrir +1 classe",H47+'08_Moteur'!O44*('08_Moteur'!AE44*'08_Moteur'!AF44-('08_Moteur'!R44+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S44)-'08_Moteur'!U44,IF(L47="Économiser 1 classe",H47+('08_Moteur'!AI44-MAX(1,'08_Moteur'!AI44-1))*'08_Moteur'!U44,H47)))</f>
+        <v/>
+      </c>
       <c r="O47" s="17">
-        <f>IF(N47="Ne pas ouvrir",0,IF(N47="Ouvrir +1 classe",H47-'08_Moteur'!U44,IF(N47="Économiser 1 classe",H47+('08_Moteur'!AI44-MAX(1,'08_Moteur'!AI44-1))*'08_Moteur'!U44,H47)))</f>
-        <v/>
-      </c>
-      <c r="P47" s="54">
-        <f>O47-H47</f>
+        <f>M47*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P47" s="17">
+        <f>N47-O47</f>
+        <v/>
+      </c>
+      <c r="Q47" s="54">
+        <f>N47-H47</f>
         <v/>
       </c>
     </row>
@@ -5352,37 +5524,41 @@
         <f>'08_Moteur'!AM45</f>
         <v/>
       </c>
-      <c r="I48" s="17">
-        <f>IF(N48="Ne pas ouvrir",0,E48)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J48" s="17">
-        <f>O48-I48</f>
-        <v/>
-      </c>
-      <c r="K48" s="69">
+      <c r="I48" s="68">
         <f>'08_Moteur'!AN45</f>
         <v/>
       </c>
-      <c r="L48" s="70">
-        <f>IF(H48&lt;0,"🔴 Ne pas ouvrir",IF(K48&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K48&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M48" s="71">
-        <f>IF(H48&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K48&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K48&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N48" s="21" t="inlineStr">
+      <c r="J48" s="69">
+        <f>IF(H48&lt;0,"🔴 Ne pas ouvrir",IF(I48&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I48&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K48" s="70">
+        <f>IF(H48&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I48&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I48&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L48" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M48" s="50">
+        <f>IF(L48="Ne pas ouvrir",0,IF(L48="Ouvrir +1 classe",E48+'08_Moteur'!O45,E48))</f>
+        <v/>
+      </c>
+      <c r="N48" s="17">
+        <f>IF(L48="Ne pas ouvrir",0,IF(L48="Ouvrir +1 classe",H48+'08_Moteur'!O45*('08_Moteur'!AE45*'08_Moteur'!AF45-('08_Moteur'!R45+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S45)-'08_Moteur'!U45,IF(L48="Économiser 1 classe",H48+('08_Moteur'!AI45-MAX(1,'08_Moteur'!AI45-1))*'08_Moteur'!U45,H48)))</f>
+        <v/>
+      </c>
       <c r="O48" s="17">
-        <f>IF(N48="Ne pas ouvrir",0,IF(N48="Ouvrir +1 classe",H48-'08_Moteur'!U45,IF(N48="Économiser 1 classe",H48+('08_Moteur'!AI45-MAX(1,'08_Moteur'!AI45-1))*'08_Moteur'!U45,H48)))</f>
-        <v/>
-      </c>
-      <c r="P48" s="54">
-        <f>O48-H48</f>
+        <f>M48*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P48" s="17">
+        <f>N48-O48</f>
+        <v/>
+      </c>
+      <c r="Q48" s="54">
+        <f>N48-H48</f>
         <v/>
       </c>
     </row>
@@ -5419,37 +5595,41 @@
         <f>'08_Moteur'!AM46</f>
         <v/>
       </c>
-      <c r="I49" s="17">
-        <f>IF(N49="Ne pas ouvrir",0,E49)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J49" s="17">
-        <f>O49-I49</f>
-        <v/>
-      </c>
-      <c r="K49" s="69">
+      <c r="I49" s="68">
         <f>'08_Moteur'!AN46</f>
         <v/>
       </c>
-      <c r="L49" s="70">
-        <f>IF(H49&lt;0,"🔴 Ne pas ouvrir",IF(K49&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K49&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M49" s="71">
-        <f>IF(H49&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K49&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K49&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N49" s="21" t="inlineStr">
+      <c r="J49" s="69">
+        <f>IF(H49&lt;0,"🔴 Ne pas ouvrir",IF(I49&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I49&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K49" s="70">
+        <f>IF(H49&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I49&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I49&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L49" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M49" s="50">
+        <f>IF(L49="Ne pas ouvrir",0,IF(L49="Ouvrir +1 classe",E49+'08_Moteur'!O46,E49))</f>
+        <v/>
+      </c>
+      <c r="N49" s="17">
+        <f>IF(L49="Ne pas ouvrir",0,IF(L49="Ouvrir +1 classe",H49+'08_Moteur'!O46*('08_Moteur'!AE46*'08_Moteur'!AF46-('08_Moteur'!R46+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S46)-'08_Moteur'!U46,IF(L49="Économiser 1 classe",H49+('08_Moteur'!AI46-MAX(1,'08_Moteur'!AI46-1))*'08_Moteur'!U46,H49)))</f>
+        <v/>
+      </c>
       <c r="O49" s="17">
-        <f>IF(N49="Ne pas ouvrir",0,IF(N49="Ouvrir +1 classe",H49-'08_Moteur'!U46,IF(N49="Économiser 1 classe",H49+('08_Moteur'!AI46-MAX(1,'08_Moteur'!AI46-1))*'08_Moteur'!U46,H49)))</f>
-        <v/>
-      </c>
-      <c r="P49" s="54">
-        <f>O49-H49</f>
+        <f>M49*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P49" s="17">
+        <f>N49-O49</f>
+        <v/>
+      </c>
+      <c r="Q49" s="54">
+        <f>N49-H49</f>
         <v/>
       </c>
     </row>
@@ -5486,37 +5666,41 @@
         <f>'08_Moteur'!AM47</f>
         <v/>
       </c>
-      <c r="I50" s="17">
-        <f>IF(N50="Ne pas ouvrir",0,E50)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J50" s="17">
-        <f>O50-I50</f>
-        <v/>
-      </c>
-      <c r="K50" s="69">
+      <c r="I50" s="68">
         <f>'08_Moteur'!AN47</f>
         <v/>
       </c>
-      <c r="L50" s="70">
-        <f>IF(H50&lt;0,"🔴 Ne pas ouvrir",IF(K50&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K50&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M50" s="71">
-        <f>IF(H50&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K50&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K50&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N50" s="21" t="inlineStr">
+      <c r="J50" s="69">
+        <f>IF(H50&lt;0,"🔴 Ne pas ouvrir",IF(I50&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I50&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K50" s="70">
+        <f>IF(H50&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I50&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I50&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L50" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M50" s="50">
+        <f>IF(L50="Ne pas ouvrir",0,IF(L50="Ouvrir +1 classe",E50+'08_Moteur'!O47,E50))</f>
+        <v/>
+      </c>
+      <c r="N50" s="17">
+        <f>IF(L50="Ne pas ouvrir",0,IF(L50="Ouvrir +1 classe",H50+'08_Moteur'!O47*('08_Moteur'!AE47*'08_Moteur'!AF47-('08_Moteur'!R47+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S47)-'08_Moteur'!U47,IF(L50="Économiser 1 classe",H50+('08_Moteur'!AI47-MAX(1,'08_Moteur'!AI47-1))*'08_Moteur'!U47,H50)))</f>
+        <v/>
+      </c>
       <c r="O50" s="17">
-        <f>IF(N50="Ne pas ouvrir",0,IF(N50="Ouvrir +1 classe",H50-'08_Moteur'!U47,IF(N50="Économiser 1 classe",H50+('08_Moteur'!AI47-MAX(1,'08_Moteur'!AI47-1))*'08_Moteur'!U47,H50)))</f>
-        <v/>
-      </c>
-      <c r="P50" s="54">
-        <f>O50-H50</f>
+        <f>M50*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P50" s="17">
+        <f>N50-O50</f>
+        <v/>
+      </c>
+      <c r="Q50" s="54">
+        <f>N50-H50</f>
         <v/>
       </c>
     </row>
@@ -5553,37 +5737,41 @@
         <f>'08_Moteur'!AM48</f>
         <v/>
       </c>
-      <c r="I51" s="17">
-        <f>IF(N51="Ne pas ouvrir",0,E51)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J51" s="17">
-        <f>O51-I51</f>
-        <v/>
-      </c>
-      <c r="K51" s="69">
+      <c r="I51" s="68">
         <f>'08_Moteur'!AN48</f>
         <v/>
       </c>
-      <c r="L51" s="70">
-        <f>IF(H51&lt;0,"🔴 Ne pas ouvrir",IF(K51&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K51&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M51" s="71">
-        <f>IF(H51&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K51&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K51&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N51" s="21" t="inlineStr">
+      <c r="J51" s="69">
+        <f>IF(H51&lt;0,"🔴 Ne pas ouvrir",IF(I51&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I51&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K51" s="70">
+        <f>IF(H51&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I51&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I51&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L51" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M51" s="50">
+        <f>IF(L51="Ne pas ouvrir",0,IF(L51="Ouvrir +1 classe",E51+'08_Moteur'!O48,E51))</f>
+        <v/>
+      </c>
+      <c r="N51" s="17">
+        <f>IF(L51="Ne pas ouvrir",0,IF(L51="Ouvrir +1 classe",H51+'08_Moteur'!O48*('08_Moteur'!AE48*'08_Moteur'!AF48-('08_Moteur'!R48+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S48)-'08_Moteur'!U48,IF(L51="Économiser 1 classe",H51+('08_Moteur'!AI48-MAX(1,'08_Moteur'!AI48-1))*'08_Moteur'!U48,H51)))</f>
+        <v/>
+      </c>
       <c r="O51" s="17">
-        <f>IF(N51="Ne pas ouvrir",0,IF(N51="Ouvrir +1 classe",H51-'08_Moteur'!U48,IF(N51="Économiser 1 classe",H51+('08_Moteur'!AI48-MAX(1,'08_Moteur'!AI48-1))*'08_Moteur'!U48,H51)))</f>
-        <v/>
-      </c>
-      <c r="P51" s="54">
-        <f>O51-H51</f>
+        <f>M51*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P51" s="17">
+        <f>N51-O51</f>
+        <v/>
+      </c>
+      <c r="Q51" s="54">
+        <f>N51-H51</f>
         <v/>
       </c>
     </row>
@@ -5620,37 +5808,41 @@
         <f>'08_Moteur'!AM49</f>
         <v/>
       </c>
-      <c r="I52" s="17">
-        <f>IF(N52="Ne pas ouvrir",0,E52)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J52" s="17">
-        <f>O52-I52</f>
-        <v/>
-      </c>
-      <c r="K52" s="69">
+      <c r="I52" s="68">
         <f>'08_Moteur'!AN49</f>
         <v/>
       </c>
-      <c r="L52" s="70">
-        <f>IF(H52&lt;0,"🔴 Ne pas ouvrir",IF(K52&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K52&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M52" s="71">
-        <f>IF(H52&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K52&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K52&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N52" s="21" t="inlineStr">
+      <c r="J52" s="69">
+        <f>IF(H52&lt;0,"🔴 Ne pas ouvrir",IF(I52&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I52&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K52" s="70">
+        <f>IF(H52&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I52&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I52&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L52" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M52" s="50">
+        <f>IF(L52="Ne pas ouvrir",0,IF(L52="Ouvrir +1 classe",E52+'08_Moteur'!O49,E52))</f>
+        <v/>
+      </c>
+      <c r="N52" s="17">
+        <f>IF(L52="Ne pas ouvrir",0,IF(L52="Ouvrir +1 classe",H52+'08_Moteur'!O49*('08_Moteur'!AE49*'08_Moteur'!AF49-('08_Moteur'!R49+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S49)-'08_Moteur'!U49,IF(L52="Économiser 1 classe",H52+('08_Moteur'!AI49-MAX(1,'08_Moteur'!AI49-1))*'08_Moteur'!U49,H52)))</f>
+        <v/>
+      </c>
       <c r="O52" s="17">
-        <f>IF(N52="Ne pas ouvrir",0,IF(N52="Ouvrir +1 classe",H52-'08_Moteur'!U49,IF(N52="Économiser 1 classe",H52+('08_Moteur'!AI49-MAX(1,'08_Moteur'!AI49-1))*'08_Moteur'!U49,H52)))</f>
-        <v/>
-      </c>
-      <c r="P52" s="54">
-        <f>O52-H52</f>
+        <f>M52*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P52" s="17">
+        <f>N52-O52</f>
+        <v/>
+      </c>
+      <c r="Q52" s="54">
+        <f>N52-H52</f>
         <v/>
       </c>
     </row>
@@ -5687,37 +5879,41 @@
         <f>'08_Moteur'!AM50</f>
         <v/>
       </c>
-      <c r="I53" s="17">
-        <f>IF(N53="Ne pas ouvrir",0,E53)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J53" s="17">
-        <f>O53-I53</f>
-        <v/>
-      </c>
-      <c r="K53" s="69">
+      <c r="I53" s="68">
         <f>'08_Moteur'!AN50</f>
         <v/>
       </c>
-      <c r="L53" s="70">
-        <f>IF(H53&lt;0,"🔴 Ne pas ouvrir",IF(K53&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K53&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M53" s="71">
-        <f>IF(H53&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K53&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K53&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N53" s="21" t="inlineStr">
+      <c r="J53" s="69">
+        <f>IF(H53&lt;0,"🔴 Ne pas ouvrir",IF(I53&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I53&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K53" s="70">
+        <f>IF(H53&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I53&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I53&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L53" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M53" s="50">
+        <f>IF(L53="Ne pas ouvrir",0,IF(L53="Ouvrir +1 classe",E53+'08_Moteur'!O50,E53))</f>
+        <v/>
+      </c>
+      <c r="N53" s="17">
+        <f>IF(L53="Ne pas ouvrir",0,IF(L53="Ouvrir +1 classe",H53+'08_Moteur'!O50*('08_Moteur'!AE50*'08_Moteur'!AF50-('08_Moteur'!R50+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S50)-'08_Moteur'!U50,IF(L53="Économiser 1 classe",H53+('08_Moteur'!AI50-MAX(1,'08_Moteur'!AI50-1))*'08_Moteur'!U50,H53)))</f>
+        <v/>
+      </c>
       <c r="O53" s="17">
-        <f>IF(N53="Ne pas ouvrir",0,IF(N53="Ouvrir +1 classe",H53-'08_Moteur'!U50,IF(N53="Économiser 1 classe",H53+('08_Moteur'!AI50-MAX(1,'08_Moteur'!AI50-1))*'08_Moteur'!U50,H53)))</f>
-        <v/>
-      </c>
-      <c r="P53" s="54">
-        <f>O53-H53</f>
+        <f>M53*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P53" s="17">
+        <f>N53-O53</f>
+        <v/>
+      </c>
+      <c r="Q53" s="54">
+        <f>N53-H53</f>
         <v/>
       </c>
     </row>
@@ -5754,37 +5950,41 @@
         <f>'08_Moteur'!AM51</f>
         <v/>
       </c>
-      <c r="I54" s="17">
-        <f>IF(N54="Ne pas ouvrir",0,E54)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J54" s="17">
-        <f>O54-I54</f>
-        <v/>
-      </c>
-      <c r="K54" s="69">
+      <c r="I54" s="68">
         <f>'08_Moteur'!AN51</f>
         <v/>
       </c>
-      <c r="L54" s="70">
-        <f>IF(H54&lt;0,"🔴 Ne pas ouvrir",IF(K54&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K54&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M54" s="71">
-        <f>IF(H54&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K54&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K54&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N54" s="21" t="inlineStr">
+      <c r="J54" s="69">
+        <f>IF(H54&lt;0,"🔴 Ne pas ouvrir",IF(I54&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I54&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K54" s="70">
+        <f>IF(H54&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I54&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I54&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L54" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M54" s="50">
+        <f>IF(L54="Ne pas ouvrir",0,IF(L54="Ouvrir +1 classe",E54+'08_Moteur'!O51,E54))</f>
+        <v/>
+      </c>
+      <c r="N54" s="17">
+        <f>IF(L54="Ne pas ouvrir",0,IF(L54="Ouvrir +1 classe",H54+'08_Moteur'!O51*('08_Moteur'!AE51*'08_Moteur'!AF51-('08_Moteur'!R51+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S51)-'08_Moteur'!U51,IF(L54="Économiser 1 classe",H54+('08_Moteur'!AI51-MAX(1,'08_Moteur'!AI51-1))*'08_Moteur'!U51,H54)))</f>
+        <v/>
+      </c>
       <c r="O54" s="17">
-        <f>IF(N54="Ne pas ouvrir",0,IF(N54="Ouvrir +1 classe",H54-'08_Moteur'!U51,IF(N54="Économiser 1 classe",H54+('08_Moteur'!AI51-MAX(1,'08_Moteur'!AI51-1))*'08_Moteur'!U51,H54)))</f>
-        <v/>
-      </c>
-      <c r="P54" s="54">
-        <f>O54-H54</f>
+        <f>M54*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P54" s="17">
+        <f>N54-O54</f>
+        <v/>
+      </c>
+      <c r="Q54" s="54">
+        <f>N54-H54</f>
         <v/>
       </c>
     </row>
@@ -5821,37 +6021,41 @@
         <f>'08_Moteur'!AM52</f>
         <v/>
       </c>
-      <c r="I55" s="17">
-        <f>IF(N55="Ne pas ouvrir",0,E55)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J55" s="17">
-        <f>O55-I55</f>
-        <v/>
-      </c>
-      <c r="K55" s="69">
+      <c r="I55" s="68">
         <f>'08_Moteur'!AN52</f>
         <v/>
       </c>
-      <c r="L55" s="70">
-        <f>IF(H55&lt;0,"🔴 Ne pas ouvrir",IF(K55&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K55&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M55" s="71">
-        <f>IF(H55&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K55&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K55&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N55" s="21" t="inlineStr">
+      <c r="J55" s="69">
+        <f>IF(H55&lt;0,"🔴 Ne pas ouvrir",IF(I55&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I55&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K55" s="70">
+        <f>IF(H55&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I55&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I55&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L55" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M55" s="50">
+        <f>IF(L55="Ne pas ouvrir",0,IF(L55="Ouvrir +1 classe",E55+'08_Moteur'!O52,E55))</f>
+        <v/>
+      </c>
+      <c r="N55" s="17">
+        <f>IF(L55="Ne pas ouvrir",0,IF(L55="Ouvrir +1 classe",H55+'08_Moteur'!O52*('08_Moteur'!AE52*'08_Moteur'!AF52-('08_Moteur'!R52+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S52)-'08_Moteur'!U52,IF(L55="Économiser 1 classe",H55+('08_Moteur'!AI52-MAX(1,'08_Moteur'!AI52-1))*'08_Moteur'!U52,H55)))</f>
+        <v/>
+      </c>
       <c r="O55" s="17">
-        <f>IF(N55="Ne pas ouvrir",0,IF(N55="Ouvrir +1 classe",H55-'08_Moteur'!U52,IF(N55="Économiser 1 classe",H55+('08_Moteur'!AI52-MAX(1,'08_Moteur'!AI52-1))*'08_Moteur'!U52,H55)))</f>
-        <v/>
-      </c>
-      <c r="P55" s="54">
-        <f>O55-H55</f>
+        <f>M55*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P55" s="17">
+        <f>N55-O55</f>
+        <v/>
+      </c>
+      <c r="Q55" s="54">
+        <f>N55-H55</f>
         <v/>
       </c>
     </row>
@@ -5888,37 +6092,41 @@
         <f>'08_Moteur'!AM53</f>
         <v/>
       </c>
-      <c r="I56" s="17">
-        <f>IF(N56="Ne pas ouvrir",0,E56)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J56" s="17">
-        <f>O56-I56</f>
-        <v/>
-      </c>
-      <c r="K56" s="69">
+      <c r="I56" s="68">
         <f>'08_Moteur'!AN53</f>
         <v/>
       </c>
-      <c r="L56" s="70">
-        <f>IF(H56&lt;0,"🔴 Ne pas ouvrir",IF(K56&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K56&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M56" s="71">
-        <f>IF(H56&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K56&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K56&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N56" s="21" t="inlineStr">
+      <c r="J56" s="69">
+        <f>IF(H56&lt;0,"🔴 Ne pas ouvrir",IF(I56&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I56&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K56" s="70">
+        <f>IF(H56&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I56&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I56&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L56" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M56" s="50">
+        <f>IF(L56="Ne pas ouvrir",0,IF(L56="Ouvrir +1 classe",E56+'08_Moteur'!O53,E56))</f>
+        <v/>
+      </c>
+      <c r="N56" s="17">
+        <f>IF(L56="Ne pas ouvrir",0,IF(L56="Ouvrir +1 classe",H56+'08_Moteur'!O53*('08_Moteur'!AE53*'08_Moteur'!AF53-('08_Moteur'!R53+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S53)-'08_Moteur'!U53,IF(L56="Économiser 1 classe",H56+('08_Moteur'!AI53-MAX(1,'08_Moteur'!AI53-1))*'08_Moteur'!U53,H56)))</f>
+        <v/>
+      </c>
       <c r="O56" s="17">
-        <f>IF(N56="Ne pas ouvrir",0,IF(N56="Ouvrir +1 classe",H56-'08_Moteur'!U53,IF(N56="Économiser 1 classe",H56+('08_Moteur'!AI53-MAX(1,'08_Moteur'!AI53-1))*'08_Moteur'!U53,H56)))</f>
-        <v/>
-      </c>
-      <c r="P56" s="54">
-        <f>O56-H56</f>
+        <f>M56*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P56" s="17">
+        <f>N56-O56</f>
+        <v/>
+      </c>
+      <c r="Q56" s="54">
+        <f>N56-H56</f>
         <v/>
       </c>
     </row>
@@ -5955,37 +6163,41 @@
         <f>'08_Moteur'!AM54</f>
         <v/>
       </c>
-      <c r="I57" s="17">
-        <f>IF(N57="Ne pas ouvrir",0,E57)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J57" s="17">
-        <f>O57-I57</f>
-        <v/>
-      </c>
-      <c r="K57" s="69">
+      <c r="I57" s="68">
         <f>'08_Moteur'!AN54</f>
         <v/>
       </c>
-      <c r="L57" s="70">
-        <f>IF(H57&lt;0,"🔴 Ne pas ouvrir",IF(K57&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K57&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M57" s="71">
-        <f>IF(H57&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K57&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K57&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N57" s="21" t="inlineStr">
+      <c r="J57" s="69">
+        <f>IF(H57&lt;0,"🔴 Ne pas ouvrir",IF(I57&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I57&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K57" s="70">
+        <f>IF(H57&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I57&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I57&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L57" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M57" s="50">
+        <f>IF(L57="Ne pas ouvrir",0,IF(L57="Ouvrir +1 classe",E57+'08_Moteur'!O54,E57))</f>
+        <v/>
+      </c>
+      <c r="N57" s="17">
+        <f>IF(L57="Ne pas ouvrir",0,IF(L57="Ouvrir +1 classe",H57+'08_Moteur'!O54*('08_Moteur'!AE54*'08_Moteur'!AF54-('08_Moteur'!R54+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S54)-'08_Moteur'!U54,IF(L57="Économiser 1 classe",H57+('08_Moteur'!AI54-MAX(1,'08_Moteur'!AI54-1))*'08_Moteur'!U54,H57)))</f>
+        <v/>
+      </c>
       <c r="O57" s="17">
-        <f>IF(N57="Ne pas ouvrir",0,IF(N57="Ouvrir +1 classe",H57-'08_Moteur'!U54,IF(N57="Économiser 1 classe",H57+('08_Moteur'!AI54-MAX(1,'08_Moteur'!AI54-1))*'08_Moteur'!U54,H57)))</f>
-        <v/>
-      </c>
-      <c r="P57" s="54">
-        <f>O57-H57</f>
+        <f>M57*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P57" s="17">
+        <f>N57-O57</f>
+        <v/>
+      </c>
+      <c r="Q57" s="54">
+        <f>N57-H57</f>
         <v/>
       </c>
     </row>
@@ -6022,37 +6234,41 @@
         <f>'08_Moteur'!AM55</f>
         <v/>
       </c>
-      <c r="I58" s="17">
-        <f>IF(N58="Ne pas ouvrir",0,E58)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J58" s="17">
-        <f>O58-I58</f>
-        <v/>
-      </c>
-      <c r="K58" s="69">
+      <c r="I58" s="68">
         <f>'08_Moteur'!AN55</f>
         <v/>
       </c>
-      <c r="L58" s="70">
-        <f>IF(H58&lt;0,"🔴 Ne pas ouvrir",IF(K58&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K58&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M58" s="71">
-        <f>IF(H58&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K58&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K58&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N58" s="21" t="inlineStr">
+      <c r="J58" s="69">
+        <f>IF(H58&lt;0,"🔴 Ne pas ouvrir",IF(I58&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I58&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K58" s="70">
+        <f>IF(H58&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I58&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I58&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L58" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M58" s="50">
+        <f>IF(L58="Ne pas ouvrir",0,IF(L58="Ouvrir +1 classe",E58+'08_Moteur'!O55,E58))</f>
+        <v/>
+      </c>
+      <c r="N58" s="17">
+        <f>IF(L58="Ne pas ouvrir",0,IF(L58="Ouvrir +1 classe",H58+'08_Moteur'!O55*('08_Moteur'!AE55*'08_Moteur'!AF55-('08_Moteur'!R55+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S55)-'08_Moteur'!U55,IF(L58="Économiser 1 classe",H58+('08_Moteur'!AI55-MAX(1,'08_Moteur'!AI55-1))*'08_Moteur'!U55,H58)))</f>
+        <v/>
+      </c>
       <c r="O58" s="17">
-        <f>IF(N58="Ne pas ouvrir",0,IF(N58="Ouvrir +1 classe",H58-'08_Moteur'!U55,IF(N58="Économiser 1 classe",H58+('08_Moteur'!AI55-MAX(1,'08_Moteur'!AI55-1))*'08_Moteur'!U55,H58)))</f>
-        <v/>
-      </c>
-      <c r="P58" s="54">
-        <f>O58-H58</f>
+        <f>M58*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P58" s="17">
+        <f>N58-O58</f>
+        <v/>
+      </c>
+      <c r="Q58" s="54">
+        <f>N58-H58</f>
         <v/>
       </c>
     </row>
@@ -6089,37 +6305,41 @@
         <f>'08_Moteur'!AM56</f>
         <v/>
       </c>
-      <c r="I59" s="17">
-        <f>IF(N59="Ne pas ouvrir",0,E59)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J59" s="17">
-        <f>O59-I59</f>
-        <v/>
-      </c>
-      <c r="K59" s="69">
+      <c r="I59" s="68">
         <f>'08_Moteur'!AN56</f>
         <v/>
       </c>
-      <c r="L59" s="70">
-        <f>IF(H59&lt;0,"🔴 Ne pas ouvrir",IF(K59&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K59&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M59" s="71">
-        <f>IF(H59&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K59&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K59&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N59" s="21" t="inlineStr">
+      <c r="J59" s="69">
+        <f>IF(H59&lt;0,"🔴 Ne pas ouvrir",IF(I59&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I59&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K59" s="70">
+        <f>IF(H59&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I59&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I59&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L59" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M59" s="50">
+        <f>IF(L59="Ne pas ouvrir",0,IF(L59="Ouvrir +1 classe",E59+'08_Moteur'!O56,E59))</f>
+        <v/>
+      </c>
+      <c r="N59" s="17">
+        <f>IF(L59="Ne pas ouvrir",0,IF(L59="Ouvrir +1 classe",H59+'08_Moteur'!O56*('08_Moteur'!AE56*'08_Moteur'!AF56-('08_Moteur'!R56+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S56)-'08_Moteur'!U56,IF(L59="Économiser 1 classe",H59+('08_Moteur'!AI56-MAX(1,'08_Moteur'!AI56-1))*'08_Moteur'!U56,H59)))</f>
+        <v/>
+      </c>
       <c r="O59" s="17">
-        <f>IF(N59="Ne pas ouvrir",0,IF(N59="Ouvrir +1 classe",H59-'08_Moteur'!U56,IF(N59="Économiser 1 classe",H59+('08_Moteur'!AI56-MAX(1,'08_Moteur'!AI56-1))*'08_Moteur'!U56,H59)))</f>
-        <v/>
-      </c>
-      <c r="P59" s="54">
-        <f>O59-H59</f>
+        <f>M59*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P59" s="17">
+        <f>N59-O59</f>
+        <v/>
+      </c>
+      <c r="Q59" s="54">
+        <f>N59-H59</f>
         <v/>
       </c>
     </row>
@@ -6156,37 +6376,41 @@
         <f>'08_Moteur'!AM57</f>
         <v/>
       </c>
-      <c r="I60" s="17">
-        <f>IF(N60="Ne pas ouvrir",0,E60)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J60" s="17">
-        <f>O60-I60</f>
-        <v/>
-      </c>
-      <c r="K60" s="69">
+      <c r="I60" s="68">
         <f>'08_Moteur'!AN57</f>
         <v/>
       </c>
-      <c r="L60" s="70">
-        <f>IF(H60&lt;0,"🔴 Ne pas ouvrir",IF(K60&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K60&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M60" s="71">
-        <f>IF(H60&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K60&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K60&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N60" s="21" t="inlineStr">
+      <c r="J60" s="69">
+        <f>IF(H60&lt;0,"🔴 Ne pas ouvrir",IF(I60&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I60&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K60" s="70">
+        <f>IF(H60&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I60&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I60&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L60" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M60" s="50">
+        <f>IF(L60="Ne pas ouvrir",0,IF(L60="Ouvrir +1 classe",E60+'08_Moteur'!O57,E60))</f>
+        <v/>
+      </c>
+      <c r="N60" s="17">
+        <f>IF(L60="Ne pas ouvrir",0,IF(L60="Ouvrir +1 classe",H60+'08_Moteur'!O57*('08_Moteur'!AE57*'08_Moteur'!AF57-('08_Moteur'!R57+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S57)-'08_Moteur'!U57,IF(L60="Économiser 1 classe",H60+('08_Moteur'!AI57-MAX(1,'08_Moteur'!AI57-1))*'08_Moteur'!U57,H60)))</f>
+        <v/>
+      </c>
       <c r="O60" s="17">
-        <f>IF(N60="Ne pas ouvrir",0,IF(N60="Ouvrir +1 classe",H60-'08_Moteur'!U57,IF(N60="Économiser 1 classe",H60+('08_Moteur'!AI57-MAX(1,'08_Moteur'!AI57-1))*'08_Moteur'!U57,H60)))</f>
-        <v/>
-      </c>
-      <c r="P60" s="54">
-        <f>O60-H60</f>
+        <f>M60*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P60" s="17">
+        <f>N60-O60</f>
+        <v/>
+      </c>
+      <c r="Q60" s="54">
+        <f>N60-H60</f>
         <v/>
       </c>
     </row>
@@ -6223,37 +6447,41 @@
         <f>'08_Moteur'!AM58</f>
         <v/>
       </c>
-      <c r="I61" s="17">
-        <f>IF(N61="Ne pas ouvrir",0,E61)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J61" s="17">
-        <f>O61-I61</f>
-        <v/>
-      </c>
-      <c r="K61" s="69">
+      <c r="I61" s="68">
         <f>'08_Moteur'!AN58</f>
         <v/>
       </c>
-      <c r="L61" s="70">
-        <f>IF(H61&lt;0,"🔴 Ne pas ouvrir",IF(K61&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K61&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M61" s="71">
-        <f>IF(H61&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K61&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K61&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N61" s="21" t="inlineStr">
+      <c r="J61" s="69">
+        <f>IF(H61&lt;0,"🔴 Ne pas ouvrir",IF(I61&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I61&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K61" s="70">
+        <f>IF(H61&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I61&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I61&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L61" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M61" s="50">
+        <f>IF(L61="Ne pas ouvrir",0,IF(L61="Ouvrir +1 classe",E61+'08_Moteur'!O58,E61))</f>
+        <v/>
+      </c>
+      <c r="N61" s="17">
+        <f>IF(L61="Ne pas ouvrir",0,IF(L61="Ouvrir +1 classe",H61+'08_Moteur'!O58*('08_Moteur'!AE58*'08_Moteur'!AF58-('08_Moteur'!R58+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S58)-'08_Moteur'!U58,IF(L61="Économiser 1 classe",H61+('08_Moteur'!AI58-MAX(1,'08_Moteur'!AI58-1))*'08_Moteur'!U58,H61)))</f>
+        <v/>
+      </c>
       <c r="O61" s="17">
-        <f>IF(N61="Ne pas ouvrir",0,IF(N61="Ouvrir +1 classe",H61-'08_Moteur'!U58,IF(N61="Économiser 1 classe",H61+('08_Moteur'!AI58-MAX(1,'08_Moteur'!AI58-1))*'08_Moteur'!U58,H61)))</f>
-        <v/>
-      </c>
-      <c r="P61" s="54">
-        <f>O61-H61</f>
+        <f>M61*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P61" s="17">
+        <f>N61-O61</f>
+        <v/>
+      </c>
+      <c r="Q61" s="54">
+        <f>N61-H61</f>
         <v/>
       </c>
     </row>
@@ -6290,37 +6518,41 @@
         <f>'08_Moteur'!AM59</f>
         <v/>
       </c>
-      <c r="I62" s="17">
-        <f>IF(N62="Ne pas ouvrir",0,E62)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J62" s="17">
-        <f>O62-I62</f>
-        <v/>
-      </c>
-      <c r="K62" s="69">
+      <c r="I62" s="68">
         <f>'08_Moteur'!AN59</f>
         <v/>
       </c>
-      <c r="L62" s="70">
-        <f>IF(H62&lt;0,"🔴 Ne pas ouvrir",IF(K62&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K62&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M62" s="71">
-        <f>IF(H62&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K62&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K62&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N62" s="21" t="inlineStr">
+      <c r="J62" s="69">
+        <f>IF(H62&lt;0,"🔴 Ne pas ouvrir",IF(I62&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I62&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K62" s="70">
+        <f>IF(H62&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I62&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I62&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L62" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M62" s="50">
+        <f>IF(L62="Ne pas ouvrir",0,IF(L62="Ouvrir +1 classe",E62+'08_Moteur'!O59,E62))</f>
+        <v/>
+      </c>
+      <c r="N62" s="17">
+        <f>IF(L62="Ne pas ouvrir",0,IF(L62="Ouvrir +1 classe",H62+'08_Moteur'!O59*('08_Moteur'!AE59*'08_Moteur'!AF59-('08_Moteur'!R59+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S59)-'08_Moteur'!U59,IF(L62="Économiser 1 classe",H62+('08_Moteur'!AI59-MAX(1,'08_Moteur'!AI59-1))*'08_Moteur'!U59,H62)))</f>
+        <v/>
+      </c>
       <c r="O62" s="17">
-        <f>IF(N62="Ne pas ouvrir",0,IF(N62="Ouvrir +1 classe",H62-'08_Moteur'!U59,IF(N62="Économiser 1 classe",H62+('08_Moteur'!AI59-MAX(1,'08_Moteur'!AI59-1))*'08_Moteur'!U59,H62)))</f>
-        <v/>
-      </c>
-      <c r="P62" s="54">
-        <f>O62-H62</f>
+        <f>M62*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P62" s="17">
+        <f>N62-O62</f>
+        <v/>
+      </c>
+      <c r="Q62" s="54">
+        <f>N62-H62</f>
         <v/>
       </c>
     </row>
@@ -6357,56 +6589,60 @@
         <f>'08_Moteur'!AM60</f>
         <v/>
       </c>
-      <c r="I63" s="17">
-        <f>IF(N63="Ne pas ouvrir",0,E63)*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUMPRODUCT((N6:N63&lt;&gt;"Ne pas ouvrir")*E6:E63),0)</f>
-        <v/>
-      </c>
-      <c r="J63" s="17">
-        <f>O63-I63</f>
-        <v/>
-      </c>
-      <c r="K63" s="69">
+      <c r="I63" s="68">
         <f>'08_Moteur'!AN60</f>
         <v/>
       </c>
-      <c r="L63" s="70">
-        <f>IF(H63&lt;0,"🔴 Ne pas ouvrir",IF(K63&gt;=0.95,"🟢 Ouvrir +1 classe",IF(K63&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
-        <v/>
-      </c>
-      <c r="M63" s="71">
-        <f>IF(H63&lt;0,"Contribution négative : la fermer améliore l'EBITDA",IF(K63&gt;=0.95,"Quasi saturé : +1 classe capte la demande",IF(K63&lt;0.55,"Sous-rempli MAIS contribution positive → GARDER (fermer perdrait la marge, la structure resterait)","Sain")))</f>
-        <v/>
-      </c>
-      <c r="N63" s="21" t="inlineStr">
+      <c r="J63" s="69">
+        <f>IF(H63&lt;0,"🔴 Ne pas ouvrir",IF(I63&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I63&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <v/>
+      </c>
+      <c r="K63" s="70">
+        <f>IF(H63&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I63&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I63&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <v/>
+      </c>
+      <c r="L63" s="21" t="inlineStr">
         <is>
           <t>Maintenir</t>
         </is>
       </c>
+      <c r="M63" s="50">
+        <f>IF(L63="Ne pas ouvrir",0,IF(L63="Ouvrir +1 classe",E63+'08_Moteur'!O60,E63))</f>
+        <v/>
+      </c>
+      <c r="N63" s="17">
+        <f>IF(L63="Ne pas ouvrir",0,IF(L63="Ouvrir +1 classe",H63+'08_Moteur'!O60*('08_Moteur'!AE60*'08_Moteur'!AF60-('08_Moteur'!R60+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S60)-'08_Moteur'!U60,IF(L63="Économiser 1 classe",H63+('08_Moteur'!AI60-MAX(1,'08_Moteur'!AI60-1))*'08_Moteur'!U60,H63)))</f>
+        <v/>
+      </c>
       <c r="O63" s="17">
-        <f>IF(N63="Ne pas ouvrir",0,IF(N63="Ouvrir +1 classe",H63-'08_Moteur'!U60,IF(N63="Économiser 1 classe",H63+('08_Moteur'!AI60-MAX(1,'08_Moteur'!AI60-1))*'08_Moteur'!U60,H63)))</f>
-        <v/>
-      </c>
-      <c r="P63" s="54">
-        <f>O63-H63</f>
+        <f>M63*IFERROR(('09_Allocation'!E20+'09_Allocation'!F20+'09_Allocation'!I20)/SUM(M6:M63),0)</f>
+        <v/>
+      </c>
+      <c r="P63" s="17">
+        <f>N63-O63</f>
+        <v/>
+      </c>
+      <c r="Q63" s="54">
+        <f>N63-H63</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="M3:P3"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="K2:L2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M3:Q3"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="I3:J3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L45 L46 L47 L48 L49 L50 L51 L52 L53 L54 L55 L56 L57 L58 L59 L60 L61 L62 L63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Maintenir,Ne pas ouvrir,Ouvrir +1 classe,Économiser 1 classe"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6470,7 +6706,7 @@
         <f>0.01*SUMPRODUCT('08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60*'08_Moteur'!$AF$3:$AF$60)</f>
         <v/>
       </c>
-      <c r="D6" s="71" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>Tombe quasi intégralement en EBITDA.</t>
         </is>
@@ -6486,7 +6722,7 @@
         <f>0.01*SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$D$18)</f>
         <v/>
       </c>
-      <c r="D7" s="71" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>Nul si recouvrement=100 % ; sinon réduit la perte.</t>
         </is>
@@ -6502,7 +6738,7 @@
         <f>0.01*'02_Leviers'!$D$21*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$AM$3:$AM$60)-0.01*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$H$3:$H$60*'08_Moteur'!$S$3:$S$60*(1+'08_Moteur'!$Y$3:$Y$60))</f>
         <v/>
       </c>
-      <c r="D8" s="71" t="inlineStr">
+      <c r="D8" s="70" t="inlineStr">
         <is>
           <t>Plus de leads → plus d'inscrits, net du coût.</t>
         </is>
@@ -6518,7 +6754,7 @@
         <f>0.01*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=0)*'08_Moteur'!$K$3:$K$60)*IFERROR(SUM('08_Moteur'!$AM$3:$AM$60)/SUM('08_Moteur'!$AD$3:$AD$60),0)</f>
         <v/>
       </c>
-      <c r="D9" s="71" t="inlineStr">
+      <c r="D9" s="70" t="inlineStr">
         <is>
           <t>Rétention : + d'étudiants qui poursuivent.</t>
         </is>
@@ -6530,7 +6766,7 @@
           <t>Exposition financement alternance (€ à sécuriser) :</t>
         </is>
       </c>
-      <c r="D11" s="72">
+      <c r="D11" s="71">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$G$9)</f>
         <v/>
       </c>
@@ -6773,20 +7009,20 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="73" t="inlineStr">
+      <c r="B15" s="72" t="inlineStr">
         <is>
           <t>€ à sécuriser (exposition)</t>
         </is>
       </c>
-      <c r="C15" s="74">
+      <c r="C15" s="73">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$G$9)</f>
         <v/>
       </c>
-      <c r="D15" s="74">
+      <c r="D15" s="73">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$G$3:$G$60*'08_Moteur'!$L$3:$L$60)*(1-'02_Leviers'!$D$20)</f>
         <v/>
       </c>
-      <c r="E15" s="75">
+      <c r="E15" s="74">
         <f>IFERROR(C15/D15-1,0)</f>
         <v/>
       </c>
@@ -6848,7 +7084,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="76" t="inlineStr">
+      <c r="B6" s="75" t="inlineStr">
         <is>
           <t>Marque / Campus</t>
         </is>
@@ -6865,7 +7101,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="76" t="inlineStr">
+      <c r="B7" s="75" t="inlineStr">
         <is>
           <t>Programme × Année × Modalité</t>
         </is>
@@ -6882,7 +7118,7 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="76" t="inlineStr">
+      <c r="B8" s="75" t="inlineStr">
         <is>
           <t>Params (capacité, heures…)</t>
         </is>
@@ -6899,7 +7135,7 @@
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="76" t="inlineStr">
+      <c r="B9" s="75" t="inlineStr">
         <is>
           <t>Historique N-2/N-1</t>
         </is>
@@ -6916,7 +7152,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="76" t="inlineStr">
+      <c r="B10" s="75" t="inlineStr">
         <is>
           <t>Cohortes / taux de passage</t>
         </is>
@@ -6933,7 +7169,7 @@
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="76" t="inlineStr">
+      <c r="B11" s="75" t="inlineStr">
         <is>
           <t>Sécurisation &amp; recouvrement</t>
         </is>
@@ -6950,7 +7186,7 @@
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="76" t="inlineStr">
+      <c r="B12" s="75" t="inlineStr">
         <is>
           <t>Objectifs (cadrage)</t>
         </is>
@@ -6967,7 +7203,7 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="76" t="inlineStr">
+      <c r="B13" s="75" t="inlineStr">
         <is>
           <t>Décisions ouvrir/fermer</t>
         </is>
@@ -6984,7 +7220,7 @@
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="76" t="inlineStr">
+      <c r="B14" s="75" t="inlineStr">
         <is>
           <t>Allocation structure</t>
         </is>

</xml_diff>

<commit_message>
Simulateur : décisions dépendantes de l'année (entrée vs poursuite)
- Années d'ENTRÉE (B1/M1/BTS1) : recrutement décidable -> Maintenir / Ne pas
  lancer / Ouvrir +1 (capter) / Regrouper.
- Années de POURSUITE (B2/B3/M2/BTS2) : cohorte déjà inscrite (issue de la
  progression) -> on ne peut ni annuler ni capter ; seul levier = organisation
  des classes (Maintenir / Regrouper). Menu déroulant et reco restreints en
  conséquence ; reco 'Restructurer (mutualiser)' si contribution négative.

Vérifié : 0 erreur ; B1/M1 peuvent recevoir 'Ouvrir +1', B2/B3/M2 non.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -2547,11 +2547,11 @@
         <v/>
       </c>
       <c r="J6" s="69">
-        <f>IF(H6&lt;0,"🔴 Ne pas ouvrir",IF(I6&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I6&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H6&lt;0,"🔴 Ne pas lancer",IF(I6&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I6&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K6" s="70">
-        <f>IF(H6&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I6&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I6&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H6&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I6&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I6&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L6" s="21" t="inlineStr">
@@ -2560,11 +2560,11 @@
         </is>
       </c>
       <c r="M6" s="50">
-        <f>IF(L6="Ne pas ouvrir",0,IF(L6="Ouvrir +1 classe",E6+'08_Moteur'!O3,E6))</f>
+        <f>IF(L6="Ne pas lancer",0,IF(L6="Ouvrir +1 classe",E6+'08_Moteur'!O3,E6))</f>
         <v/>
       </c>
       <c r="N6" s="17">
-        <f>IF(L6="Ne pas ouvrir",0,IF(L6="Ouvrir +1 classe",H6+'08_Moteur'!O3*('08_Moteur'!AE3*'08_Moteur'!AF3-('08_Moteur'!R3+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S3)-'08_Moteur'!U3,IF(L6="Économiser 1 classe",H6+('08_Moteur'!AI3-MAX(1,'08_Moteur'!AI3-1))*'08_Moteur'!U3,H6)))</f>
+        <f>IF(L6="Ne pas lancer",0,IF(L6="Ouvrir +1 classe",H6+'08_Moteur'!O3*('08_Moteur'!AE3*'08_Moteur'!AF3-('08_Moteur'!R3+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S3)-'08_Moteur'!U3,IF(L6="Regrouper (-1 classe)",H6+('08_Moteur'!AI3-MAX(1,'08_Moteur'!AI3-1))*'08_Moteur'!U3,H6)))</f>
         <v/>
       </c>
       <c r="O6" s="17">
@@ -2618,11 +2618,11 @@
         <v/>
       </c>
       <c r="J7" s="69">
-        <f>IF(H7&lt;0,"🔴 Ne pas ouvrir",IF(I7&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I7&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H7&lt;0,"🔴 Restructurer (mutualiser)",IF(I7&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K7" s="70">
-        <f>IF(H7&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I7&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I7&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L7" s="21" t="inlineStr">
@@ -2631,11 +2631,11 @@
         </is>
       </c>
       <c r="M7" s="50">
-        <f>IF(L7="Ne pas ouvrir",0,IF(L7="Ouvrir +1 classe",E7+'08_Moteur'!O4,E7))</f>
+        <f>IF(L7="Ne pas lancer",0,IF(L7="Ouvrir +1 classe",E7+'08_Moteur'!O4,E7))</f>
         <v/>
       </c>
       <c r="N7" s="17">
-        <f>IF(L7="Ne pas ouvrir",0,IF(L7="Ouvrir +1 classe",H7+'08_Moteur'!O4*('08_Moteur'!AE4*'08_Moteur'!AF4-('08_Moteur'!R4+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S4)-'08_Moteur'!U4,IF(L7="Économiser 1 classe",H7+('08_Moteur'!AI4-MAX(1,'08_Moteur'!AI4-1))*'08_Moteur'!U4,H7)))</f>
+        <f>IF(L7="Ne pas lancer",0,IF(L7="Ouvrir +1 classe",H7+'08_Moteur'!O4*('08_Moteur'!AE4*'08_Moteur'!AF4-('08_Moteur'!R4+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S4)-'08_Moteur'!U4,IF(L7="Regrouper (-1 classe)",H7+('08_Moteur'!AI4-MAX(1,'08_Moteur'!AI4-1))*'08_Moteur'!U4,H7)))</f>
         <v/>
       </c>
       <c r="O7" s="17">
@@ -2689,11 +2689,11 @@
         <v/>
       </c>
       <c r="J8" s="69">
-        <f>IF(H8&lt;0,"🔴 Ne pas ouvrir",IF(I8&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I8&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H8&lt;0,"🔴 Restructurer (mutualiser)",IF(I8&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K8" s="70">
-        <f>IF(H8&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I8&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I8&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L8" s="21" t="inlineStr">
@@ -2702,11 +2702,11 @@
         </is>
       </c>
       <c r="M8" s="50">
-        <f>IF(L8="Ne pas ouvrir",0,IF(L8="Ouvrir +1 classe",E8+'08_Moteur'!O5,E8))</f>
+        <f>IF(L8="Ne pas lancer",0,IF(L8="Ouvrir +1 classe",E8+'08_Moteur'!O5,E8))</f>
         <v/>
       </c>
       <c r="N8" s="17">
-        <f>IF(L8="Ne pas ouvrir",0,IF(L8="Ouvrir +1 classe",H8+'08_Moteur'!O5*('08_Moteur'!AE5*'08_Moteur'!AF5-('08_Moteur'!R5+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S5)-'08_Moteur'!U5,IF(L8="Économiser 1 classe",H8+('08_Moteur'!AI5-MAX(1,'08_Moteur'!AI5-1))*'08_Moteur'!U5,H8)))</f>
+        <f>IF(L8="Ne pas lancer",0,IF(L8="Ouvrir +1 classe",H8+'08_Moteur'!O5*('08_Moteur'!AE5*'08_Moteur'!AF5-('08_Moteur'!R5+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S5)-'08_Moteur'!U5,IF(L8="Regrouper (-1 classe)",H8+('08_Moteur'!AI5-MAX(1,'08_Moteur'!AI5-1))*'08_Moteur'!U5,H8)))</f>
         <v/>
       </c>
       <c r="O8" s="17">
@@ -2760,11 +2760,11 @@
         <v/>
       </c>
       <c r="J9" s="69">
-        <f>IF(H9&lt;0,"🔴 Ne pas ouvrir",IF(I9&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I9&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H9&lt;0,"🔴 Ne pas lancer",IF(I9&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I9&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K9" s="70">
-        <f>IF(H9&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I9&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I9&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H9&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I9&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I9&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L9" s="21" t="inlineStr">
@@ -2773,11 +2773,11 @@
         </is>
       </c>
       <c r="M9" s="50">
-        <f>IF(L9="Ne pas ouvrir",0,IF(L9="Ouvrir +1 classe",E9+'08_Moteur'!O6,E9))</f>
+        <f>IF(L9="Ne pas lancer",0,IF(L9="Ouvrir +1 classe",E9+'08_Moteur'!O6,E9))</f>
         <v/>
       </c>
       <c r="N9" s="17">
-        <f>IF(L9="Ne pas ouvrir",0,IF(L9="Ouvrir +1 classe",H9+'08_Moteur'!O6*('08_Moteur'!AE6*'08_Moteur'!AF6-('08_Moteur'!R6+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S6)-'08_Moteur'!U6,IF(L9="Économiser 1 classe",H9+('08_Moteur'!AI6-MAX(1,'08_Moteur'!AI6-1))*'08_Moteur'!U6,H9)))</f>
+        <f>IF(L9="Ne pas lancer",0,IF(L9="Ouvrir +1 classe",H9+'08_Moteur'!O6*('08_Moteur'!AE6*'08_Moteur'!AF6-('08_Moteur'!R6+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S6)-'08_Moteur'!U6,IF(L9="Regrouper (-1 classe)",H9+('08_Moteur'!AI6-MAX(1,'08_Moteur'!AI6-1))*'08_Moteur'!U6,H9)))</f>
         <v/>
       </c>
       <c r="O9" s="17">
@@ -2831,11 +2831,11 @@
         <v/>
       </c>
       <c r="J10" s="69">
-        <f>IF(H10&lt;0,"🔴 Ne pas ouvrir",IF(I10&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I10&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H10&lt;0,"🔴 Restructurer (mutualiser)",IF(I10&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K10" s="70">
-        <f>IF(H10&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I10&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I10&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L10" s="21" t="inlineStr">
@@ -2844,11 +2844,11 @@
         </is>
       </c>
       <c r="M10" s="50">
-        <f>IF(L10="Ne pas ouvrir",0,IF(L10="Ouvrir +1 classe",E10+'08_Moteur'!O7,E10))</f>
+        <f>IF(L10="Ne pas lancer",0,IF(L10="Ouvrir +1 classe",E10+'08_Moteur'!O7,E10))</f>
         <v/>
       </c>
       <c r="N10" s="17">
-        <f>IF(L10="Ne pas ouvrir",0,IF(L10="Ouvrir +1 classe",H10+'08_Moteur'!O7*('08_Moteur'!AE7*'08_Moteur'!AF7-('08_Moteur'!R7+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S7)-'08_Moteur'!U7,IF(L10="Économiser 1 classe",H10+('08_Moteur'!AI7-MAX(1,'08_Moteur'!AI7-1))*'08_Moteur'!U7,H10)))</f>
+        <f>IF(L10="Ne pas lancer",0,IF(L10="Ouvrir +1 classe",H10+'08_Moteur'!O7*('08_Moteur'!AE7*'08_Moteur'!AF7-('08_Moteur'!R7+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S7)-'08_Moteur'!U7,IF(L10="Regrouper (-1 classe)",H10+('08_Moteur'!AI7-MAX(1,'08_Moteur'!AI7-1))*'08_Moteur'!U7,H10)))</f>
         <v/>
       </c>
       <c r="O10" s="17">
@@ -2902,11 +2902,11 @@
         <v/>
       </c>
       <c r="J11" s="69">
-        <f>IF(H11&lt;0,"🔴 Ne pas ouvrir",IF(I11&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I11&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H11&lt;0,"🔴 Ne pas lancer",IF(I11&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I11&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K11" s="70">
-        <f>IF(H11&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I11&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I11&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H11&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I11&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I11&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L11" s="21" t="inlineStr">
@@ -2915,11 +2915,11 @@
         </is>
       </c>
       <c r="M11" s="50">
-        <f>IF(L11="Ne pas ouvrir",0,IF(L11="Ouvrir +1 classe",E11+'08_Moteur'!O8,E11))</f>
+        <f>IF(L11="Ne pas lancer",0,IF(L11="Ouvrir +1 classe",E11+'08_Moteur'!O8,E11))</f>
         <v/>
       </c>
       <c r="N11" s="17">
-        <f>IF(L11="Ne pas ouvrir",0,IF(L11="Ouvrir +1 classe",H11+'08_Moteur'!O8*('08_Moteur'!AE8*'08_Moteur'!AF8-('08_Moteur'!R8+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S8)-'08_Moteur'!U8,IF(L11="Économiser 1 classe",H11+('08_Moteur'!AI8-MAX(1,'08_Moteur'!AI8-1))*'08_Moteur'!U8,H11)))</f>
+        <f>IF(L11="Ne pas lancer",0,IF(L11="Ouvrir +1 classe",H11+'08_Moteur'!O8*('08_Moteur'!AE8*'08_Moteur'!AF8-('08_Moteur'!R8+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S8)-'08_Moteur'!U8,IF(L11="Regrouper (-1 classe)",H11+('08_Moteur'!AI8-MAX(1,'08_Moteur'!AI8-1))*'08_Moteur'!U8,H11)))</f>
         <v/>
       </c>
       <c r="O11" s="17">
@@ -2973,11 +2973,11 @@
         <v/>
       </c>
       <c r="J12" s="69">
-        <f>IF(H12&lt;0,"🔴 Ne pas ouvrir",IF(I12&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I12&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H12&lt;0,"🔴 Restructurer (mutualiser)",IF(I12&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K12" s="70">
-        <f>IF(H12&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I12&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I12&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L12" s="21" t="inlineStr">
@@ -2986,11 +2986,11 @@
         </is>
       </c>
       <c r="M12" s="50">
-        <f>IF(L12="Ne pas ouvrir",0,IF(L12="Ouvrir +1 classe",E12+'08_Moteur'!O9,E12))</f>
+        <f>IF(L12="Ne pas lancer",0,IF(L12="Ouvrir +1 classe",E12+'08_Moteur'!O9,E12))</f>
         <v/>
       </c>
       <c r="N12" s="17">
-        <f>IF(L12="Ne pas ouvrir",0,IF(L12="Ouvrir +1 classe",H12+'08_Moteur'!O9*('08_Moteur'!AE9*'08_Moteur'!AF9-('08_Moteur'!R9+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S9)-'08_Moteur'!U9,IF(L12="Économiser 1 classe",H12+('08_Moteur'!AI9-MAX(1,'08_Moteur'!AI9-1))*'08_Moteur'!U9,H12)))</f>
+        <f>IF(L12="Ne pas lancer",0,IF(L12="Ouvrir +1 classe",H12+'08_Moteur'!O9*('08_Moteur'!AE9*'08_Moteur'!AF9-('08_Moteur'!R9+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S9)-'08_Moteur'!U9,IF(L12="Regrouper (-1 classe)",H12+('08_Moteur'!AI9-MAX(1,'08_Moteur'!AI9-1))*'08_Moteur'!U9,H12)))</f>
         <v/>
       </c>
       <c r="O12" s="17">
@@ -3044,11 +3044,11 @@
         <v/>
       </c>
       <c r="J13" s="69">
-        <f>IF(H13&lt;0,"🔴 Ne pas ouvrir",IF(I13&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I13&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H13&lt;0,"🔴 Restructurer (mutualiser)",IF(I13&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K13" s="70">
-        <f>IF(H13&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I13&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I13&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L13" s="21" t="inlineStr">
@@ -3057,11 +3057,11 @@
         </is>
       </c>
       <c r="M13" s="50">
-        <f>IF(L13="Ne pas ouvrir",0,IF(L13="Ouvrir +1 classe",E13+'08_Moteur'!O10,E13))</f>
+        <f>IF(L13="Ne pas lancer",0,IF(L13="Ouvrir +1 classe",E13+'08_Moteur'!O10,E13))</f>
         <v/>
       </c>
       <c r="N13" s="17">
-        <f>IF(L13="Ne pas ouvrir",0,IF(L13="Ouvrir +1 classe",H13+'08_Moteur'!O10*('08_Moteur'!AE10*'08_Moteur'!AF10-('08_Moteur'!R10+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S10)-'08_Moteur'!U10,IF(L13="Économiser 1 classe",H13+('08_Moteur'!AI10-MAX(1,'08_Moteur'!AI10-1))*'08_Moteur'!U10,H13)))</f>
+        <f>IF(L13="Ne pas lancer",0,IF(L13="Ouvrir +1 classe",H13+'08_Moteur'!O10*('08_Moteur'!AE10*'08_Moteur'!AF10-('08_Moteur'!R10+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S10)-'08_Moteur'!U10,IF(L13="Regrouper (-1 classe)",H13+('08_Moteur'!AI10-MAX(1,'08_Moteur'!AI10-1))*'08_Moteur'!U10,H13)))</f>
         <v/>
       </c>
       <c r="O13" s="17">
@@ -3115,11 +3115,11 @@
         <v/>
       </c>
       <c r="J14" s="69">
-        <f>IF(H14&lt;0,"🔴 Ne pas ouvrir",IF(I14&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I14&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H14&lt;0,"🔴 Ne pas lancer",IF(I14&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I14&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K14" s="70">
-        <f>IF(H14&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I14&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I14&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H14&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I14&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I14&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L14" s="21" t="inlineStr">
@@ -3128,11 +3128,11 @@
         </is>
       </c>
       <c r="M14" s="50">
-        <f>IF(L14="Ne pas ouvrir",0,IF(L14="Ouvrir +1 classe",E14+'08_Moteur'!O11,E14))</f>
+        <f>IF(L14="Ne pas lancer",0,IF(L14="Ouvrir +1 classe",E14+'08_Moteur'!O11,E14))</f>
         <v/>
       </c>
       <c r="N14" s="17">
-        <f>IF(L14="Ne pas ouvrir",0,IF(L14="Ouvrir +1 classe",H14+'08_Moteur'!O11*('08_Moteur'!AE11*'08_Moteur'!AF11-('08_Moteur'!R11+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S11)-'08_Moteur'!U11,IF(L14="Économiser 1 classe",H14+('08_Moteur'!AI11-MAX(1,'08_Moteur'!AI11-1))*'08_Moteur'!U11,H14)))</f>
+        <f>IF(L14="Ne pas lancer",0,IF(L14="Ouvrir +1 classe",H14+'08_Moteur'!O11*('08_Moteur'!AE11*'08_Moteur'!AF11-('08_Moteur'!R11+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S11)-'08_Moteur'!U11,IF(L14="Regrouper (-1 classe)",H14+('08_Moteur'!AI11-MAX(1,'08_Moteur'!AI11-1))*'08_Moteur'!U11,H14)))</f>
         <v/>
       </c>
       <c r="O14" s="17">
@@ -3186,11 +3186,11 @@
         <v/>
       </c>
       <c r="J15" s="69">
-        <f>IF(H15&lt;0,"🔴 Ne pas ouvrir",IF(I15&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I15&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H15&lt;0,"🔴 Restructurer (mutualiser)",IF(I15&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K15" s="70">
-        <f>IF(H15&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I15&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I15&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L15" s="21" t="inlineStr">
@@ -3199,11 +3199,11 @@
         </is>
       </c>
       <c r="M15" s="50">
-        <f>IF(L15="Ne pas ouvrir",0,IF(L15="Ouvrir +1 classe",E15+'08_Moteur'!O12,E15))</f>
+        <f>IF(L15="Ne pas lancer",0,IF(L15="Ouvrir +1 classe",E15+'08_Moteur'!O12,E15))</f>
         <v/>
       </c>
       <c r="N15" s="17">
-        <f>IF(L15="Ne pas ouvrir",0,IF(L15="Ouvrir +1 classe",H15+'08_Moteur'!O12*('08_Moteur'!AE12*'08_Moteur'!AF12-('08_Moteur'!R12+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S12)-'08_Moteur'!U12,IF(L15="Économiser 1 classe",H15+('08_Moteur'!AI12-MAX(1,'08_Moteur'!AI12-1))*'08_Moteur'!U12,H15)))</f>
+        <f>IF(L15="Ne pas lancer",0,IF(L15="Ouvrir +1 classe",H15+'08_Moteur'!O12*('08_Moteur'!AE12*'08_Moteur'!AF12-('08_Moteur'!R12+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S12)-'08_Moteur'!U12,IF(L15="Regrouper (-1 classe)",H15+('08_Moteur'!AI12-MAX(1,'08_Moteur'!AI12-1))*'08_Moteur'!U12,H15)))</f>
         <v/>
       </c>
       <c r="O15" s="17">
@@ -3257,11 +3257,11 @@
         <v/>
       </c>
       <c r="J16" s="69">
-        <f>IF(H16&lt;0,"🔴 Ne pas ouvrir",IF(I16&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I16&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H16&lt;0,"🔴 Ne pas lancer",IF(I16&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I16&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K16" s="70">
-        <f>IF(H16&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I16&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I16&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H16&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I16&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I16&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L16" s="21" t="inlineStr">
@@ -3270,11 +3270,11 @@
         </is>
       </c>
       <c r="M16" s="50">
-        <f>IF(L16="Ne pas ouvrir",0,IF(L16="Ouvrir +1 classe",E16+'08_Moteur'!O13,E16))</f>
+        <f>IF(L16="Ne pas lancer",0,IF(L16="Ouvrir +1 classe",E16+'08_Moteur'!O13,E16))</f>
         <v/>
       </c>
       <c r="N16" s="17">
-        <f>IF(L16="Ne pas ouvrir",0,IF(L16="Ouvrir +1 classe",H16+'08_Moteur'!O13*('08_Moteur'!AE13*'08_Moteur'!AF13-('08_Moteur'!R13+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S13)-'08_Moteur'!U13,IF(L16="Économiser 1 classe",H16+('08_Moteur'!AI13-MAX(1,'08_Moteur'!AI13-1))*'08_Moteur'!U13,H16)))</f>
+        <f>IF(L16="Ne pas lancer",0,IF(L16="Ouvrir +1 classe",H16+'08_Moteur'!O13*('08_Moteur'!AE13*'08_Moteur'!AF13-('08_Moteur'!R13+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S13)-'08_Moteur'!U13,IF(L16="Regrouper (-1 classe)",H16+('08_Moteur'!AI13-MAX(1,'08_Moteur'!AI13-1))*'08_Moteur'!U13,H16)))</f>
         <v/>
       </c>
       <c r="O16" s="17">
@@ -3328,11 +3328,11 @@
         <v/>
       </c>
       <c r="J17" s="69">
-        <f>IF(H17&lt;0,"🔴 Ne pas ouvrir",IF(I17&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I17&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H17&lt;0,"🔴 Restructurer (mutualiser)",IF(I17&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K17" s="70">
-        <f>IF(H17&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I17&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I17&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L17" s="21" t="inlineStr">
@@ -3341,11 +3341,11 @@
         </is>
       </c>
       <c r="M17" s="50">
-        <f>IF(L17="Ne pas ouvrir",0,IF(L17="Ouvrir +1 classe",E17+'08_Moteur'!O14,E17))</f>
+        <f>IF(L17="Ne pas lancer",0,IF(L17="Ouvrir +1 classe",E17+'08_Moteur'!O14,E17))</f>
         <v/>
       </c>
       <c r="N17" s="17">
-        <f>IF(L17="Ne pas ouvrir",0,IF(L17="Ouvrir +1 classe",H17+'08_Moteur'!O14*('08_Moteur'!AE14*'08_Moteur'!AF14-('08_Moteur'!R14+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S14)-'08_Moteur'!U14,IF(L17="Économiser 1 classe",H17+('08_Moteur'!AI14-MAX(1,'08_Moteur'!AI14-1))*'08_Moteur'!U14,H17)))</f>
+        <f>IF(L17="Ne pas lancer",0,IF(L17="Ouvrir +1 classe",H17+'08_Moteur'!O14*('08_Moteur'!AE14*'08_Moteur'!AF14-('08_Moteur'!R14+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S14)-'08_Moteur'!U14,IF(L17="Regrouper (-1 classe)",H17+('08_Moteur'!AI14-MAX(1,'08_Moteur'!AI14-1))*'08_Moteur'!U14,H17)))</f>
         <v/>
       </c>
       <c r="O17" s="17">
@@ -3399,11 +3399,11 @@
         <v/>
       </c>
       <c r="J18" s="69">
-        <f>IF(H18&lt;0,"🔴 Ne pas ouvrir",IF(I18&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I18&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H18&lt;0,"🔴 Restructurer (mutualiser)",IF(I18&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K18" s="70">
-        <f>IF(H18&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I18&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I18&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L18" s="21" t="inlineStr">
@@ -3412,11 +3412,11 @@
         </is>
       </c>
       <c r="M18" s="50">
-        <f>IF(L18="Ne pas ouvrir",0,IF(L18="Ouvrir +1 classe",E18+'08_Moteur'!O15,E18))</f>
+        <f>IF(L18="Ne pas lancer",0,IF(L18="Ouvrir +1 classe",E18+'08_Moteur'!O15,E18))</f>
         <v/>
       </c>
       <c r="N18" s="17">
-        <f>IF(L18="Ne pas ouvrir",0,IF(L18="Ouvrir +1 classe",H18+'08_Moteur'!O15*('08_Moteur'!AE15*'08_Moteur'!AF15-('08_Moteur'!R15+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S15)-'08_Moteur'!U15,IF(L18="Économiser 1 classe",H18+('08_Moteur'!AI15-MAX(1,'08_Moteur'!AI15-1))*'08_Moteur'!U15,H18)))</f>
+        <f>IF(L18="Ne pas lancer",0,IF(L18="Ouvrir +1 classe",H18+'08_Moteur'!O15*('08_Moteur'!AE15*'08_Moteur'!AF15-('08_Moteur'!R15+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S15)-'08_Moteur'!U15,IF(L18="Regrouper (-1 classe)",H18+('08_Moteur'!AI15-MAX(1,'08_Moteur'!AI15-1))*'08_Moteur'!U15,H18)))</f>
         <v/>
       </c>
       <c r="O18" s="17">
@@ -3470,11 +3470,11 @@
         <v/>
       </c>
       <c r="J19" s="69">
-        <f>IF(H19&lt;0,"🔴 Ne pas ouvrir",IF(I19&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I19&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H19&lt;0,"🔴 Ne pas lancer",IF(I19&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I19&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K19" s="70">
-        <f>IF(H19&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I19&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I19&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H19&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I19&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I19&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L19" s="21" t="inlineStr">
@@ -3483,11 +3483,11 @@
         </is>
       </c>
       <c r="M19" s="50">
-        <f>IF(L19="Ne pas ouvrir",0,IF(L19="Ouvrir +1 classe",E19+'08_Moteur'!O16,E19))</f>
+        <f>IF(L19="Ne pas lancer",0,IF(L19="Ouvrir +1 classe",E19+'08_Moteur'!O16,E19))</f>
         <v/>
       </c>
       <c r="N19" s="17">
-        <f>IF(L19="Ne pas ouvrir",0,IF(L19="Ouvrir +1 classe",H19+'08_Moteur'!O16*('08_Moteur'!AE16*'08_Moteur'!AF16-('08_Moteur'!R16+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S16)-'08_Moteur'!U16,IF(L19="Économiser 1 classe",H19+('08_Moteur'!AI16-MAX(1,'08_Moteur'!AI16-1))*'08_Moteur'!U16,H19)))</f>
+        <f>IF(L19="Ne pas lancer",0,IF(L19="Ouvrir +1 classe",H19+'08_Moteur'!O16*('08_Moteur'!AE16*'08_Moteur'!AF16-('08_Moteur'!R16+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S16)-'08_Moteur'!U16,IF(L19="Regrouper (-1 classe)",H19+('08_Moteur'!AI16-MAX(1,'08_Moteur'!AI16-1))*'08_Moteur'!U16,H19)))</f>
         <v/>
       </c>
       <c r="O19" s="17">
@@ -3541,11 +3541,11 @@
         <v/>
       </c>
       <c r="J20" s="69">
-        <f>IF(H20&lt;0,"🔴 Ne pas ouvrir",IF(I20&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I20&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H20&lt;0,"🔴 Restructurer (mutualiser)",IF(I20&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K20" s="70">
-        <f>IF(H20&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I20&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I20&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L20" s="21" t="inlineStr">
@@ -3554,11 +3554,11 @@
         </is>
       </c>
       <c r="M20" s="50">
-        <f>IF(L20="Ne pas ouvrir",0,IF(L20="Ouvrir +1 classe",E20+'08_Moteur'!O17,E20))</f>
+        <f>IF(L20="Ne pas lancer",0,IF(L20="Ouvrir +1 classe",E20+'08_Moteur'!O17,E20))</f>
         <v/>
       </c>
       <c r="N20" s="17">
-        <f>IF(L20="Ne pas ouvrir",0,IF(L20="Ouvrir +1 classe",H20+'08_Moteur'!O17*('08_Moteur'!AE17*'08_Moteur'!AF17-('08_Moteur'!R17+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S17)-'08_Moteur'!U17,IF(L20="Économiser 1 classe",H20+('08_Moteur'!AI17-MAX(1,'08_Moteur'!AI17-1))*'08_Moteur'!U17,H20)))</f>
+        <f>IF(L20="Ne pas lancer",0,IF(L20="Ouvrir +1 classe",H20+'08_Moteur'!O17*('08_Moteur'!AE17*'08_Moteur'!AF17-('08_Moteur'!R17+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S17)-'08_Moteur'!U17,IF(L20="Regrouper (-1 classe)",H20+('08_Moteur'!AI17-MAX(1,'08_Moteur'!AI17-1))*'08_Moteur'!U17,H20)))</f>
         <v/>
       </c>
       <c r="O20" s="17">
@@ -3612,11 +3612,11 @@
         <v/>
       </c>
       <c r="J21" s="69">
-        <f>IF(H21&lt;0,"🔴 Ne pas ouvrir",IF(I21&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I21&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H21&lt;0,"🔴 Ne pas lancer",IF(I21&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I21&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K21" s="70">
-        <f>IF(H21&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I21&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I21&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H21&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I21&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I21&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L21" s="21" t="inlineStr">
@@ -3625,11 +3625,11 @@
         </is>
       </c>
       <c r="M21" s="50">
-        <f>IF(L21="Ne pas ouvrir",0,IF(L21="Ouvrir +1 classe",E21+'08_Moteur'!O18,E21))</f>
+        <f>IF(L21="Ne pas lancer",0,IF(L21="Ouvrir +1 classe",E21+'08_Moteur'!O18,E21))</f>
         <v/>
       </c>
       <c r="N21" s="17">
-        <f>IF(L21="Ne pas ouvrir",0,IF(L21="Ouvrir +1 classe",H21+'08_Moteur'!O18*('08_Moteur'!AE18*'08_Moteur'!AF18-('08_Moteur'!R18+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S18)-'08_Moteur'!U18,IF(L21="Économiser 1 classe",H21+('08_Moteur'!AI18-MAX(1,'08_Moteur'!AI18-1))*'08_Moteur'!U18,H21)))</f>
+        <f>IF(L21="Ne pas lancer",0,IF(L21="Ouvrir +1 classe",H21+'08_Moteur'!O18*('08_Moteur'!AE18*'08_Moteur'!AF18-('08_Moteur'!R18+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S18)-'08_Moteur'!U18,IF(L21="Regrouper (-1 classe)",H21+('08_Moteur'!AI18-MAX(1,'08_Moteur'!AI18-1))*'08_Moteur'!U18,H21)))</f>
         <v/>
       </c>
       <c r="O21" s="17">
@@ -3683,11 +3683,11 @@
         <v/>
       </c>
       <c r="J22" s="69">
-        <f>IF(H22&lt;0,"🔴 Ne pas ouvrir",IF(I22&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I22&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H22&lt;0,"🔴 Restructurer (mutualiser)",IF(I22&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K22" s="70">
-        <f>IF(H22&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I22&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I22&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L22" s="21" t="inlineStr">
@@ -3696,11 +3696,11 @@
         </is>
       </c>
       <c r="M22" s="50">
-        <f>IF(L22="Ne pas ouvrir",0,IF(L22="Ouvrir +1 classe",E22+'08_Moteur'!O19,E22))</f>
+        <f>IF(L22="Ne pas lancer",0,IF(L22="Ouvrir +1 classe",E22+'08_Moteur'!O19,E22))</f>
         <v/>
       </c>
       <c r="N22" s="17">
-        <f>IF(L22="Ne pas ouvrir",0,IF(L22="Ouvrir +1 classe",H22+'08_Moteur'!O19*('08_Moteur'!AE19*'08_Moteur'!AF19-('08_Moteur'!R19+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S19)-'08_Moteur'!U19,IF(L22="Économiser 1 classe",H22+('08_Moteur'!AI19-MAX(1,'08_Moteur'!AI19-1))*'08_Moteur'!U19,H22)))</f>
+        <f>IF(L22="Ne pas lancer",0,IF(L22="Ouvrir +1 classe",H22+'08_Moteur'!O19*('08_Moteur'!AE19*'08_Moteur'!AF19-('08_Moteur'!R19+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S19)-'08_Moteur'!U19,IF(L22="Regrouper (-1 classe)",H22+('08_Moteur'!AI19-MAX(1,'08_Moteur'!AI19-1))*'08_Moteur'!U19,H22)))</f>
         <v/>
       </c>
       <c r="O22" s="17">
@@ -3754,11 +3754,11 @@
         <v/>
       </c>
       <c r="J23" s="69">
-        <f>IF(H23&lt;0,"🔴 Ne pas ouvrir",IF(I23&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I23&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H23&lt;0,"🔴 Restructurer (mutualiser)",IF(I23&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K23" s="70">
-        <f>IF(H23&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I23&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I23&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L23" s="21" t="inlineStr">
@@ -3767,11 +3767,11 @@
         </is>
       </c>
       <c r="M23" s="50">
-        <f>IF(L23="Ne pas ouvrir",0,IF(L23="Ouvrir +1 classe",E23+'08_Moteur'!O20,E23))</f>
+        <f>IF(L23="Ne pas lancer",0,IF(L23="Ouvrir +1 classe",E23+'08_Moteur'!O20,E23))</f>
         <v/>
       </c>
       <c r="N23" s="17">
-        <f>IF(L23="Ne pas ouvrir",0,IF(L23="Ouvrir +1 classe",H23+'08_Moteur'!O20*('08_Moteur'!AE20*'08_Moteur'!AF20-('08_Moteur'!R20+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S20)-'08_Moteur'!U20,IF(L23="Économiser 1 classe",H23+('08_Moteur'!AI20-MAX(1,'08_Moteur'!AI20-1))*'08_Moteur'!U20,H23)))</f>
+        <f>IF(L23="Ne pas lancer",0,IF(L23="Ouvrir +1 classe",H23+'08_Moteur'!O20*('08_Moteur'!AE20*'08_Moteur'!AF20-('08_Moteur'!R20+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S20)-'08_Moteur'!U20,IF(L23="Regrouper (-1 classe)",H23+('08_Moteur'!AI20-MAX(1,'08_Moteur'!AI20-1))*'08_Moteur'!U20,H23)))</f>
         <v/>
       </c>
       <c r="O23" s="17">
@@ -3825,11 +3825,11 @@
         <v/>
       </c>
       <c r="J24" s="69">
-        <f>IF(H24&lt;0,"🔴 Ne pas ouvrir",IF(I24&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I24&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H24&lt;0,"🔴 Ne pas lancer",IF(I24&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I24&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K24" s="70">
-        <f>IF(H24&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I24&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I24&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H24&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I24&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I24&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L24" s="21" t="inlineStr">
@@ -3838,11 +3838,11 @@
         </is>
       </c>
       <c r="M24" s="50">
-        <f>IF(L24="Ne pas ouvrir",0,IF(L24="Ouvrir +1 classe",E24+'08_Moteur'!O21,E24))</f>
+        <f>IF(L24="Ne pas lancer",0,IF(L24="Ouvrir +1 classe",E24+'08_Moteur'!O21,E24))</f>
         <v/>
       </c>
       <c r="N24" s="17">
-        <f>IF(L24="Ne pas ouvrir",0,IF(L24="Ouvrir +1 classe",H24+'08_Moteur'!O21*('08_Moteur'!AE21*'08_Moteur'!AF21-('08_Moteur'!R21+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S21)-'08_Moteur'!U21,IF(L24="Économiser 1 classe",H24+('08_Moteur'!AI21-MAX(1,'08_Moteur'!AI21-1))*'08_Moteur'!U21,H24)))</f>
+        <f>IF(L24="Ne pas lancer",0,IF(L24="Ouvrir +1 classe",H24+'08_Moteur'!O21*('08_Moteur'!AE21*'08_Moteur'!AF21-('08_Moteur'!R21+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S21)-'08_Moteur'!U21,IF(L24="Regrouper (-1 classe)",H24+('08_Moteur'!AI21-MAX(1,'08_Moteur'!AI21-1))*'08_Moteur'!U21,H24)))</f>
         <v/>
       </c>
       <c r="O24" s="17">
@@ -3896,11 +3896,11 @@
         <v/>
       </c>
       <c r="J25" s="69">
-        <f>IF(H25&lt;0,"🔴 Ne pas ouvrir",IF(I25&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I25&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H25&lt;0,"🔴 Restructurer (mutualiser)",IF(I25&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K25" s="70">
-        <f>IF(H25&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I25&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I25&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L25" s="21" t="inlineStr">
@@ -3909,11 +3909,11 @@
         </is>
       </c>
       <c r="M25" s="50">
-        <f>IF(L25="Ne pas ouvrir",0,IF(L25="Ouvrir +1 classe",E25+'08_Moteur'!O22,E25))</f>
+        <f>IF(L25="Ne pas lancer",0,IF(L25="Ouvrir +1 classe",E25+'08_Moteur'!O22,E25))</f>
         <v/>
       </c>
       <c r="N25" s="17">
-        <f>IF(L25="Ne pas ouvrir",0,IF(L25="Ouvrir +1 classe",H25+'08_Moteur'!O22*('08_Moteur'!AE22*'08_Moteur'!AF22-('08_Moteur'!R22+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S22)-'08_Moteur'!U22,IF(L25="Économiser 1 classe",H25+('08_Moteur'!AI22-MAX(1,'08_Moteur'!AI22-1))*'08_Moteur'!U22,H25)))</f>
+        <f>IF(L25="Ne pas lancer",0,IF(L25="Ouvrir +1 classe",H25+'08_Moteur'!O22*('08_Moteur'!AE22*'08_Moteur'!AF22-('08_Moteur'!R22+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S22)-'08_Moteur'!U22,IF(L25="Regrouper (-1 classe)",H25+('08_Moteur'!AI22-MAX(1,'08_Moteur'!AI22-1))*'08_Moteur'!U22,H25)))</f>
         <v/>
       </c>
       <c r="O25" s="17">
@@ -3967,11 +3967,11 @@
         <v/>
       </c>
       <c r="J26" s="69">
-        <f>IF(H26&lt;0,"🔴 Ne pas ouvrir",IF(I26&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I26&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H26&lt;0,"🔴 Ne pas lancer",IF(I26&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I26&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K26" s="70">
-        <f>IF(H26&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I26&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I26&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H26&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I26&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I26&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L26" s="21" t="inlineStr">
@@ -3980,11 +3980,11 @@
         </is>
       </c>
       <c r="M26" s="50">
-        <f>IF(L26="Ne pas ouvrir",0,IF(L26="Ouvrir +1 classe",E26+'08_Moteur'!O23,E26))</f>
+        <f>IF(L26="Ne pas lancer",0,IF(L26="Ouvrir +1 classe",E26+'08_Moteur'!O23,E26))</f>
         <v/>
       </c>
       <c r="N26" s="17">
-        <f>IF(L26="Ne pas ouvrir",0,IF(L26="Ouvrir +1 classe",H26+'08_Moteur'!O23*('08_Moteur'!AE23*'08_Moteur'!AF23-('08_Moteur'!R23+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S23)-'08_Moteur'!U23,IF(L26="Économiser 1 classe",H26+('08_Moteur'!AI23-MAX(1,'08_Moteur'!AI23-1))*'08_Moteur'!U23,H26)))</f>
+        <f>IF(L26="Ne pas lancer",0,IF(L26="Ouvrir +1 classe",H26+'08_Moteur'!O23*('08_Moteur'!AE23*'08_Moteur'!AF23-('08_Moteur'!R23+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S23)-'08_Moteur'!U23,IF(L26="Regrouper (-1 classe)",H26+('08_Moteur'!AI23-MAX(1,'08_Moteur'!AI23-1))*'08_Moteur'!U23,H26)))</f>
         <v/>
       </c>
       <c r="O26" s="17">
@@ -4038,11 +4038,11 @@
         <v/>
       </c>
       <c r="J27" s="69">
-        <f>IF(H27&lt;0,"🔴 Ne pas ouvrir",IF(I27&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I27&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H27&lt;0,"🔴 Restructurer (mutualiser)",IF(I27&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K27" s="70">
-        <f>IF(H27&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I27&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I27&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L27" s="21" t="inlineStr">
@@ -4051,11 +4051,11 @@
         </is>
       </c>
       <c r="M27" s="50">
-        <f>IF(L27="Ne pas ouvrir",0,IF(L27="Ouvrir +1 classe",E27+'08_Moteur'!O24,E27))</f>
+        <f>IF(L27="Ne pas lancer",0,IF(L27="Ouvrir +1 classe",E27+'08_Moteur'!O24,E27))</f>
         <v/>
       </c>
       <c r="N27" s="17">
-        <f>IF(L27="Ne pas ouvrir",0,IF(L27="Ouvrir +1 classe",H27+'08_Moteur'!O24*('08_Moteur'!AE24*'08_Moteur'!AF24-('08_Moteur'!R24+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S24)-'08_Moteur'!U24,IF(L27="Économiser 1 classe",H27+('08_Moteur'!AI24-MAX(1,'08_Moteur'!AI24-1))*'08_Moteur'!U24,H27)))</f>
+        <f>IF(L27="Ne pas lancer",0,IF(L27="Ouvrir +1 classe",H27+'08_Moteur'!O24*('08_Moteur'!AE24*'08_Moteur'!AF24-('08_Moteur'!R24+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S24)-'08_Moteur'!U24,IF(L27="Regrouper (-1 classe)",H27+('08_Moteur'!AI24-MAX(1,'08_Moteur'!AI24-1))*'08_Moteur'!U24,H27)))</f>
         <v/>
       </c>
       <c r="O27" s="17">
@@ -4109,11 +4109,11 @@
         <v/>
       </c>
       <c r="J28" s="69">
-        <f>IF(H28&lt;0,"🔴 Ne pas ouvrir",IF(I28&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I28&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H28&lt;0,"🔴 Restructurer (mutualiser)",IF(I28&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K28" s="70">
-        <f>IF(H28&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I28&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I28&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L28" s="21" t="inlineStr">
@@ -4122,11 +4122,11 @@
         </is>
       </c>
       <c r="M28" s="50">
-        <f>IF(L28="Ne pas ouvrir",0,IF(L28="Ouvrir +1 classe",E28+'08_Moteur'!O25,E28))</f>
+        <f>IF(L28="Ne pas lancer",0,IF(L28="Ouvrir +1 classe",E28+'08_Moteur'!O25,E28))</f>
         <v/>
       </c>
       <c r="N28" s="17">
-        <f>IF(L28="Ne pas ouvrir",0,IF(L28="Ouvrir +1 classe",H28+'08_Moteur'!O25*('08_Moteur'!AE25*'08_Moteur'!AF25-('08_Moteur'!R25+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S25)-'08_Moteur'!U25,IF(L28="Économiser 1 classe",H28+('08_Moteur'!AI25-MAX(1,'08_Moteur'!AI25-1))*'08_Moteur'!U25,H28)))</f>
+        <f>IF(L28="Ne pas lancer",0,IF(L28="Ouvrir +1 classe",H28+'08_Moteur'!O25*('08_Moteur'!AE25*'08_Moteur'!AF25-('08_Moteur'!R25+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S25)-'08_Moteur'!U25,IF(L28="Regrouper (-1 classe)",H28+('08_Moteur'!AI25-MAX(1,'08_Moteur'!AI25-1))*'08_Moteur'!U25,H28)))</f>
         <v/>
       </c>
       <c r="O28" s="17">
@@ -4180,11 +4180,11 @@
         <v/>
       </c>
       <c r="J29" s="69">
-        <f>IF(H29&lt;0,"🔴 Ne pas ouvrir",IF(I29&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I29&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H29&lt;0,"🔴 Ne pas lancer",IF(I29&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I29&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K29" s="70">
-        <f>IF(H29&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I29&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I29&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H29&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I29&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I29&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L29" s="21" t="inlineStr">
@@ -4193,11 +4193,11 @@
         </is>
       </c>
       <c r="M29" s="50">
-        <f>IF(L29="Ne pas ouvrir",0,IF(L29="Ouvrir +1 classe",E29+'08_Moteur'!O26,E29))</f>
+        <f>IF(L29="Ne pas lancer",0,IF(L29="Ouvrir +1 classe",E29+'08_Moteur'!O26,E29))</f>
         <v/>
       </c>
       <c r="N29" s="17">
-        <f>IF(L29="Ne pas ouvrir",0,IF(L29="Ouvrir +1 classe",H29+'08_Moteur'!O26*('08_Moteur'!AE26*'08_Moteur'!AF26-('08_Moteur'!R26+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S26)-'08_Moteur'!U26,IF(L29="Économiser 1 classe",H29+('08_Moteur'!AI26-MAX(1,'08_Moteur'!AI26-1))*'08_Moteur'!U26,H29)))</f>
+        <f>IF(L29="Ne pas lancer",0,IF(L29="Ouvrir +1 classe",H29+'08_Moteur'!O26*('08_Moteur'!AE26*'08_Moteur'!AF26-('08_Moteur'!R26+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S26)-'08_Moteur'!U26,IF(L29="Regrouper (-1 classe)",H29+('08_Moteur'!AI26-MAX(1,'08_Moteur'!AI26-1))*'08_Moteur'!U26,H29)))</f>
         <v/>
       </c>
       <c r="O29" s="17">
@@ -4251,11 +4251,11 @@
         <v/>
       </c>
       <c r="J30" s="69">
-        <f>IF(H30&lt;0,"🔴 Ne pas ouvrir",IF(I30&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I30&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H30&lt;0,"🔴 Restructurer (mutualiser)",IF(I30&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K30" s="70">
-        <f>IF(H30&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I30&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I30&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L30" s="21" t="inlineStr">
@@ -4264,11 +4264,11 @@
         </is>
       </c>
       <c r="M30" s="50">
-        <f>IF(L30="Ne pas ouvrir",0,IF(L30="Ouvrir +1 classe",E30+'08_Moteur'!O27,E30))</f>
+        <f>IF(L30="Ne pas lancer",0,IF(L30="Ouvrir +1 classe",E30+'08_Moteur'!O27,E30))</f>
         <v/>
       </c>
       <c r="N30" s="17">
-        <f>IF(L30="Ne pas ouvrir",0,IF(L30="Ouvrir +1 classe",H30+'08_Moteur'!O27*('08_Moteur'!AE27*'08_Moteur'!AF27-('08_Moteur'!R27+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S27)-'08_Moteur'!U27,IF(L30="Économiser 1 classe",H30+('08_Moteur'!AI27-MAX(1,'08_Moteur'!AI27-1))*'08_Moteur'!U27,H30)))</f>
+        <f>IF(L30="Ne pas lancer",0,IF(L30="Ouvrir +1 classe",H30+'08_Moteur'!O27*('08_Moteur'!AE27*'08_Moteur'!AF27-('08_Moteur'!R27+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S27)-'08_Moteur'!U27,IF(L30="Regrouper (-1 classe)",H30+('08_Moteur'!AI27-MAX(1,'08_Moteur'!AI27-1))*'08_Moteur'!U27,H30)))</f>
         <v/>
       </c>
       <c r="O30" s="17">
@@ -4322,11 +4322,11 @@
         <v/>
       </c>
       <c r="J31" s="69">
-        <f>IF(H31&lt;0,"🔴 Ne pas ouvrir",IF(I31&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I31&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H31&lt;0,"🔴 Ne pas lancer",IF(I31&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I31&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K31" s="70">
-        <f>IF(H31&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I31&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I31&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H31&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I31&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I31&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L31" s="21" t="inlineStr">
@@ -4335,11 +4335,11 @@
         </is>
       </c>
       <c r="M31" s="50">
-        <f>IF(L31="Ne pas ouvrir",0,IF(L31="Ouvrir +1 classe",E31+'08_Moteur'!O28,E31))</f>
+        <f>IF(L31="Ne pas lancer",0,IF(L31="Ouvrir +1 classe",E31+'08_Moteur'!O28,E31))</f>
         <v/>
       </c>
       <c r="N31" s="17">
-        <f>IF(L31="Ne pas ouvrir",0,IF(L31="Ouvrir +1 classe",H31+'08_Moteur'!O28*('08_Moteur'!AE28*'08_Moteur'!AF28-('08_Moteur'!R28+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S28)-'08_Moteur'!U28,IF(L31="Économiser 1 classe",H31+('08_Moteur'!AI28-MAX(1,'08_Moteur'!AI28-1))*'08_Moteur'!U28,H31)))</f>
+        <f>IF(L31="Ne pas lancer",0,IF(L31="Ouvrir +1 classe",H31+'08_Moteur'!O28*('08_Moteur'!AE28*'08_Moteur'!AF28-('08_Moteur'!R28+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S28)-'08_Moteur'!U28,IF(L31="Regrouper (-1 classe)",H31+('08_Moteur'!AI28-MAX(1,'08_Moteur'!AI28-1))*'08_Moteur'!U28,H31)))</f>
         <v/>
       </c>
       <c r="O31" s="17">
@@ -4393,11 +4393,11 @@
         <v/>
       </c>
       <c r="J32" s="69">
-        <f>IF(H32&lt;0,"🔴 Ne pas ouvrir",IF(I32&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I32&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H32&lt;0,"🔴 Restructurer (mutualiser)",IF(I32&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K32" s="70">
-        <f>IF(H32&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I32&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I32&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L32" s="21" t="inlineStr">
@@ -4406,11 +4406,11 @@
         </is>
       </c>
       <c r="M32" s="50">
-        <f>IF(L32="Ne pas ouvrir",0,IF(L32="Ouvrir +1 classe",E32+'08_Moteur'!O29,E32))</f>
+        <f>IF(L32="Ne pas lancer",0,IF(L32="Ouvrir +1 classe",E32+'08_Moteur'!O29,E32))</f>
         <v/>
       </c>
       <c r="N32" s="17">
-        <f>IF(L32="Ne pas ouvrir",0,IF(L32="Ouvrir +1 classe",H32+'08_Moteur'!O29*('08_Moteur'!AE29*'08_Moteur'!AF29-('08_Moteur'!R29+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S29)-'08_Moteur'!U29,IF(L32="Économiser 1 classe",H32+('08_Moteur'!AI29-MAX(1,'08_Moteur'!AI29-1))*'08_Moteur'!U29,H32)))</f>
+        <f>IF(L32="Ne pas lancer",0,IF(L32="Ouvrir +1 classe",H32+'08_Moteur'!O29*('08_Moteur'!AE29*'08_Moteur'!AF29-('08_Moteur'!R29+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S29)-'08_Moteur'!U29,IF(L32="Regrouper (-1 classe)",H32+('08_Moteur'!AI29-MAX(1,'08_Moteur'!AI29-1))*'08_Moteur'!U29,H32)))</f>
         <v/>
       </c>
       <c r="O32" s="17">
@@ -4464,11 +4464,11 @@
         <v/>
       </c>
       <c r="J33" s="69">
-        <f>IF(H33&lt;0,"🔴 Ne pas ouvrir",IF(I33&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I33&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H33&lt;0,"🔴 Restructurer (mutualiser)",IF(I33&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K33" s="70">
-        <f>IF(H33&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I33&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I33&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L33" s="21" t="inlineStr">
@@ -4477,11 +4477,11 @@
         </is>
       </c>
       <c r="M33" s="50">
-        <f>IF(L33="Ne pas ouvrir",0,IF(L33="Ouvrir +1 classe",E33+'08_Moteur'!O30,E33))</f>
+        <f>IF(L33="Ne pas lancer",0,IF(L33="Ouvrir +1 classe",E33+'08_Moteur'!O30,E33))</f>
         <v/>
       </c>
       <c r="N33" s="17">
-        <f>IF(L33="Ne pas ouvrir",0,IF(L33="Ouvrir +1 classe",H33+'08_Moteur'!O30*('08_Moteur'!AE30*'08_Moteur'!AF30-('08_Moteur'!R30+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S30)-'08_Moteur'!U30,IF(L33="Économiser 1 classe",H33+('08_Moteur'!AI30-MAX(1,'08_Moteur'!AI30-1))*'08_Moteur'!U30,H33)))</f>
+        <f>IF(L33="Ne pas lancer",0,IF(L33="Ouvrir +1 classe",H33+'08_Moteur'!O30*('08_Moteur'!AE30*'08_Moteur'!AF30-('08_Moteur'!R30+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S30)-'08_Moteur'!U30,IF(L33="Regrouper (-1 classe)",H33+('08_Moteur'!AI30-MAX(1,'08_Moteur'!AI30-1))*'08_Moteur'!U30,H33)))</f>
         <v/>
       </c>
       <c r="O33" s="17">
@@ -4535,11 +4535,11 @@
         <v/>
       </c>
       <c r="J34" s="69">
-        <f>IF(H34&lt;0,"🔴 Ne pas ouvrir",IF(I34&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I34&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H34&lt;0,"🔴 Ne pas lancer",IF(I34&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I34&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K34" s="70">
-        <f>IF(H34&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I34&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I34&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H34&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I34&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I34&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L34" s="21" t="inlineStr">
@@ -4548,11 +4548,11 @@
         </is>
       </c>
       <c r="M34" s="50">
-        <f>IF(L34="Ne pas ouvrir",0,IF(L34="Ouvrir +1 classe",E34+'08_Moteur'!O31,E34))</f>
+        <f>IF(L34="Ne pas lancer",0,IF(L34="Ouvrir +1 classe",E34+'08_Moteur'!O31,E34))</f>
         <v/>
       </c>
       <c r="N34" s="17">
-        <f>IF(L34="Ne pas ouvrir",0,IF(L34="Ouvrir +1 classe",H34+'08_Moteur'!O31*('08_Moteur'!AE31*'08_Moteur'!AF31-('08_Moteur'!R31+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S31)-'08_Moteur'!U31,IF(L34="Économiser 1 classe",H34+('08_Moteur'!AI31-MAX(1,'08_Moteur'!AI31-1))*'08_Moteur'!U31,H34)))</f>
+        <f>IF(L34="Ne pas lancer",0,IF(L34="Ouvrir +1 classe",H34+'08_Moteur'!O31*('08_Moteur'!AE31*'08_Moteur'!AF31-('08_Moteur'!R31+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S31)-'08_Moteur'!U31,IF(L34="Regrouper (-1 classe)",H34+('08_Moteur'!AI31-MAX(1,'08_Moteur'!AI31-1))*'08_Moteur'!U31,H34)))</f>
         <v/>
       </c>
       <c r="O34" s="17">
@@ -4606,11 +4606,11 @@
         <v/>
       </c>
       <c r="J35" s="69">
-        <f>IF(H35&lt;0,"🔴 Ne pas ouvrir",IF(I35&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I35&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H35&lt;0,"🔴 Restructurer (mutualiser)",IF(I35&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K35" s="70">
-        <f>IF(H35&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I35&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I35&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L35" s="21" t="inlineStr">
@@ -4619,11 +4619,11 @@
         </is>
       </c>
       <c r="M35" s="50">
-        <f>IF(L35="Ne pas ouvrir",0,IF(L35="Ouvrir +1 classe",E35+'08_Moteur'!O32,E35))</f>
+        <f>IF(L35="Ne pas lancer",0,IF(L35="Ouvrir +1 classe",E35+'08_Moteur'!O32,E35))</f>
         <v/>
       </c>
       <c r="N35" s="17">
-        <f>IF(L35="Ne pas ouvrir",0,IF(L35="Ouvrir +1 classe",H35+'08_Moteur'!O32*('08_Moteur'!AE32*'08_Moteur'!AF32-('08_Moteur'!R32+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S32)-'08_Moteur'!U32,IF(L35="Économiser 1 classe",H35+('08_Moteur'!AI32-MAX(1,'08_Moteur'!AI32-1))*'08_Moteur'!U32,H35)))</f>
+        <f>IF(L35="Ne pas lancer",0,IF(L35="Ouvrir +1 classe",H35+'08_Moteur'!O32*('08_Moteur'!AE32*'08_Moteur'!AF32-('08_Moteur'!R32+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S32)-'08_Moteur'!U32,IF(L35="Regrouper (-1 classe)",H35+('08_Moteur'!AI32-MAX(1,'08_Moteur'!AI32-1))*'08_Moteur'!U32,H35)))</f>
         <v/>
       </c>
       <c r="O35" s="17">
@@ -4677,11 +4677,11 @@
         <v/>
       </c>
       <c r="J36" s="69">
-        <f>IF(H36&lt;0,"🔴 Ne pas ouvrir",IF(I36&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I36&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H36&lt;0,"🔴 Ne pas lancer",IF(I36&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I36&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K36" s="70">
-        <f>IF(H36&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I36&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I36&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H36&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I36&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I36&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L36" s="21" t="inlineStr">
@@ -4690,11 +4690,11 @@
         </is>
       </c>
       <c r="M36" s="50">
-        <f>IF(L36="Ne pas ouvrir",0,IF(L36="Ouvrir +1 classe",E36+'08_Moteur'!O33,E36))</f>
+        <f>IF(L36="Ne pas lancer",0,IF(L36="Ouvrir +1 classe",E36+'08_Moteur'!O33,E36))</f>
         <v/>
       </c>
       <c r="N36" s="17">
-        <f>IF(L36="Ne pas ouvrir",0,IF(L36="Ouvrir +1 classe",H36+'08_Moteur'!O33*('08_Moteur'!AE33*'08_Moteur'!AF33-('08_Moteur'!R33+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S33)-'08_Moteur'!U33,IF(L36="Économiser 1 classe",H36+('08_Moteur'!AI33-MAX(1,'08_Moteur'!AI33-1))*'08_Moteur'!U33,H36)))</f>
+        <f>IF(L36="Ne pas lancer",0,IF(L36="Ouvrir +1 classe",H36+'08_Moteur'!O33*('08_Moteur'!AE33*'08_Moteur'!AF33-('08_Moteur'!R33+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S33)-'08_Moteur'!U33,IF(L36="Regrouper (-1 classe)",H36+('08_Moteur'!AI33-MAX(1,'08_Moteur'!AI33-1))*'08_Moteur'!U33,H36)))</f>
         <v/>
       </c>
       <c r="O36" s="17">
@@ -4748,11 +4748,11 @@
         <v/>
       </c>
       <c r="J37" s="69">
-        <f>IF(H37&lt;0,"🔴 Ne pas ouvrir",IF(I37&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I37&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H37&lt;0,"🔴 Restructurer (mutualiser)",IF(I37&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K37" s="70">
-        <f>IF(H37&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I37&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I37&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L37" s="21" t="inlineStr">
@@ -4761,11 +4761,11 @@
         </is>
       </c>
       <c r="M37" s="50">
-        <f>IF(L37="Ne pas ouvrir",0,IF(L37="Ouvrir +1 classe",E37+'08_Moteur'!O34,E37))</f>
+        <f>IF(L37="Ne pas lancer",0,IF(L37="Ouvrir +1 classe",E37+'08_Moteur'!O34,E37))</f>
         <v/>
       </c>
       <c r="N37" s="17">
-        <f>IF(L37="Ne pas ouvrir",0,IF(L37="Ouvrir +1 classe",H37+'08_Moteur'!O34*('08_Moteur'!AE34*'08_Moteur'!AF34-('08_Moteur'!R34+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S34)-'08_Moteur'!U34,IF(L37="Économiser 1 classe",H37+('08_Moteur'!AI34-MAX(1,'08_Moteur'!AI34-1))*'08_Moteur'!U34,H37)))</f>
+        <f>IF(L37="Ne pas lancer",0,IF(L37="Ouvrir +1 classe",H37+'08_Moteur'!O34*('08_Moteur'!AE34*'08_Moteur'!AF34-('08_Moteur'!R34+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S34)-'08_Moteur'!U34,IF(L37="Regrouper (-1 classe)",H37+('08_Moteur'!AI34-MAX(1,'08_Moteur'!AI34-1))*'08_Moteur'!U34,H37)))</f>
         <v/>
       </c>
       <c r="O37" s="17">
@@ -4819,11 +4819,11 @@
         <v/>
       </c>
       <c r="J38" s="69">
-        <f>IF(H38&lt;0,"🔴 Ne pas ouvrir",IF(I38&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I38&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H38&lt;0,"🔴 Restructurer (mutualiser)",IF(I38&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K38" s="70">
-        <f>IF(H38&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I38&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I38&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L38" s="21" t="inlineStr">
@@ -4832,11 +4832,11 @@
         </is>
       </c>
       <c r="M38" s="50">
-        <f>IF(L38="Ne pas ouvrir",0,IF(L38="Ouvrir +1 classe",E38+'08_Moteur'!O35,E38))</f>
+        <f>IF(L38="Ne pas lancer",0,IF(L38="Ouvrir +1 classe",E38+'08_Moteur'!O35,E38))</f>
         <v/>
       </c>
       <c r="N38" s="17">
-        <f>IF(L38="Ne pas ouvrir",0,IF(L38="Ouvrir +1 classe",H38+'08_Moteur'!O35*('08_Moteur'!AE35*'08_Moteur'!AF35-('08_Moteur'!R35+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S35)-'08_Moteur'!U35,IF(L38="Économiser 1 classe",H38+('08_Moteur'!AI35-MAX(1,'08_Moteur'!AI35-1))*'08_Moteur'!U35,H38)))</f>
+        <f>IF(L38="Ne pas lancer",0,IF(L38="Ouvrir +1 classe",H38+'08_Moteur'!O35*('08_Moteur'!AE35*'08_Moteur'!AF35-('08_Moteur'!R35+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S35)-'08_Moteur'!U35,IF(L38="Regrouper (-1 classe)",H38+('08_Moteur'!AI35-MAX(1,'08_Moteur'!AI35-1))*'08_Moteur'!U35,H38)))</f>
         <v/>
       </c>
       <c r="O38" s="17">
@@ -4890,11 +4890,11 @@
         <v/>
       </c>
       <c r="J39" s="69">
-        <f>IF(H39&lt;0,"🔴 Ne pas ouvrir",IF(I39&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I39&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H39&lt;0,"🔴 Ne pas lancer",IF(I39&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I39&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K39" s="70">
-        <f>IF(H39&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I39&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I39&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H39&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I39&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I39&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L39" s="21" t="inlineStr">
@@ -4903,11 +4903,11 @@
         </is>
       </c>
       <c r="M39" s="50">
-        <f>IF(L39="Ne pas ouvrir",0,IF(L39="Ouvrir +1 classe",E39+'08_Moteur'!O36,E39))</f>
+        <f>IF(L39="Ne pas lancer",0,IF(L39="Ouvrir +1 classe",E39+'08_Moteur'!O36,E39))</f>
         <v/>
       </c>
       <c r="N39" s="17">
-        <f>IF(L39="Ne pas ouvrir",0,IF(L39="Ouvrir +1 classe",H39+'08_Moteur'!O36*('08_Moteur'!AE36*'08_Moteur'!AF36-('08_Moteur'!R36+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S36)-'08_Moteur'!U36,IF(L39="Économiser 1 classe",H39+('08_Moteur'!AI36-MAX(1,'08_Moteur'!AI36-1))*'08_Moteur'!U36,H39)))</f>
+        <f>IF(L39="Ne pas lancer",0,IF(L39="Ouvrir +1 classe",H39+'08_Moteur'!O36*('08_Moteur'!AE36*'08_Moteur'!AF36-('08_Moteur'!R36+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S36)-'08_Moteur'!U36,IF(L39="Regrouper (-1 classe)",H39+('08_Moteur'!AI36-MAX(1,'08_Moteur'!AI36-1))*'08_Moteur'!U36,H39)))</f>
         <v/>
       </c>
       <c r="O39" s="17">
@@ -4961,11 +4961,11 @@
         <v/>
       </c>
       <c r="J40" s="69">
-        <f>IF(H40&lt;0,"🔴 Ne pas ouvrir",IF(I40&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I40&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H40&lt;0,"🔴 Restructurer (mutualiser)",IF(I40&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K40" s="70">
-        <f>IF(H40&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I40&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I40&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L40" s="21" t="inlineStr">
@@ -4974,11 +4974,11 @@
         </is>
       </c>
       <c r="M40" s="50">
-        <f>IF(L40="Ne pas ouvrir",0,IF(L40="Ouvrir +1 classe",E40+'08_Moteur'!O37,E40))</f>
+        <f>IF(L40="Ne pas lancer",0,IF(L40="Ouvrir +1 classe",E40+'08_Moteur'!O37,E40))</f>
         <v/>
       </c>
       <c r="N40" s="17">
-        <f>IF(L40="Ne pas ouvrir",0,IF(L40="Ouvrir +1 classe",H40+'08_Moteur'!O37*('08_Moteur'!AE37*'08_Moteur'!AF37-('08_Moteur'!R37+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S37)-'08_Moteur'!U37,IF(L40="Économiser 1 classe",H40+('08_Moteur'!AI37-MAX(1,'08_Moteur'!AI37-1))*'08_Moteur'!U37,H40)))</f>
+        <f>IF(L40="Ne pas lancer",0,IF(L40="Ouvrir +1 classe",H40+'08_Moteur'!O37*('08_Moteur'!AE37*'08_Moteur'!AF37-('08_Moteur'!R37+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S37)-'08_Moteur'!U37,IF(L40="Regrouper (-1 classe)",H40+('08_Moteur'!AI37-MAX(1,'08_Moteur'!AI37-1))*'08_Moteur'!U37,H40)))</f>
         <v/>
       </c>
       <c r="O40" s="17">
@@ -5032,11 +5032,11 @@
         <v/>
       </c>
       <c r="J41" s="69">
-        <f>IF(H41&lt;0,"🔴 Ne pas ouvrir",IF(I41&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I41&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H41&lt;0,"🔴 Ne pas lancer",IF(I41&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I41&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K41" s="70">
-        <f>IF(H41&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I41&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I41&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H41&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I41&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I41&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L41" s="21" t="inlineStr">
@@ -5045,11 +5045,11 @@
         </is>
       </c>
       <c r="M41" s="50">
-        <f>IF(L41="Ne pas ouvrir",0,IF(L41="Ouvrir +1 classe",E41+'08_Moteur'!O38,E41))</f>
+        <f>IF(L41="Ne pas lancer",0,IF(L41="Ouvrir +1 classe",E41+'08_Moteur'!O38,E41))</f>
         <v/>
       </c>
       <c r="N41" s="17">
-        <f>IF(L41="Ne pas ouvrir",0,IF(L41="Ouvrir +1 classe",H41+'08_Moteur'!O38*('08_Moteur'!AE38*'08_Moteur'!AF38-('08_Moteur'!R38+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S38)-'08_Moteur'!U38,IF(L41="Économiser 1 classe",H41+('08_Moteur'!AI38-MAX(1,'08_Moteur'!AI38-1))*'08_Moteur'!U38,H41)))</f>
+        <f>IF(L41="Ne pas lancer",0,IF(L41="Ouvrir +1 classe",H41+'08_Moteur'!O38*('08_Moteur'!AE38*'08_Moteur'!AF38-('08_Moteur'!R38+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S38)-'08_Moteur'!U38,IF(L41="Regrouper (-1 classe)",H41+('08_Moteur'!AI38-MAX(1,'08_Moteur'!AI38-1))*'08_Moteur'!U38,H41)))</f>
         <v/>
       </c>
       <c r="O41" s="17">
@@ -5103,11 +5103,11 @@
         <v/>
       </c>
       <c r="J42" s="69">
-        <f>IF(H42&lt;0,"🔴 Ne pas ouvrir",IF(I42&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I42&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H42&lt;0,"🔴 Restructurer (mutualiser)",IF(I42&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K42" s="70">
-        <f>IF(H42&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I42&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I42&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L42" s="21" t="inlineStr">
@@ -5116,11 +5116,11 @@
         </is>
       </c>
       <c r="M42" s="50">
-        <f>IF(L42="Ne pas ouvrir",0,IF(L42="Ouvrir +1 classe",E42+'08_Moteur'!O39,E42))</f>
+        <f>IF(L42="Ne pas lancer",0,IF(L42="Ouvrir +1 classe",E42+'08_Moteur'!O39,E42))</f>
         <v/>
       </c>
       <c r="N42" s="17">
-        <f>IF(L42="Ne pas ouvrir",0,IF(L42="Ouvrir +1 classe",H42+'08_Moteur'!O39*('08_Moteur'!AE39*'08_Moteur'!AF39-('08_Moteur'!R39+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S39)-'08_Moteur'!U39,IF(L42="Économiser 1 classe",H42+('08_Moteur'!AI39-MAX(1,'08_Moteur'!AI39-1))*'08_Moteur'!U39,H42)))</f>
+        <f>IF(L42="Ne pas lancer",0,IF(L42="Ouvrir +1 classe",H42+'08_Moteur'!O39*('08_Moteur'!AE39*'08_Moteur'!AF39-('08_Moteur'!R39+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S39)-'08_Moteur'!U39,IF(L42="Regrouper (-1 classe)",H42+('08_Moteur'!AI39-MAX(1,'08_Moteur'!AI39-1))*'08_Moteur'!U39,H42)))</f>
         <v/>
       </c>
       <c r="O42" s="17">
@@ -5174,11 +5174,11 @@
         <v/>
       </c>
       <c r="J43" s="69">
-        <f>IF(H43&lt;0,"🔴 Ne pas ouvrir",IF(I43&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I43&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H43&lt;0,"🔴 Restructurer (mutualiser)",IF(I43&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K43" s="70">
-        <f>IF(H43&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I43&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I43&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L43" s="21" t="inlineStr">
@@ -5187,11 +5187,11 @@
         </is>
       </c>
       <c r="M43" s="50">
-        <f>IF(L43="Ne pas ouvrir",0,IF(L43="Ouvrir +1 classe",E43+'08_Moteur'!O40,E43))</f>
+        <f>IF(L43="Ne pas lancer",0,IF(L43="Ouvrir +1 classe",E43+'08_Moteur'!O40,E43))</f>
         <v/>
       </c>
       <c r="N43" s="17">
-        <f>IF(L43="Ne pas ouvrir",0,IF(L43="Ouvrir +1 classe",H43+'08_Moteur'!O40*('08_Moteur'!AE40*'08_Moteur'!AF40-('08_Moteur'!R40+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S40)-'08_Moteur'!U40,IF(L43="Économiser 1 classe",H43+('08_Moteur'!AI40-MAX(1,'08_Moteur'!AI40-1))*'08_Moteur'!U40,H43)))</f>
+        <f>IF(L43="Ne pas lancer",0,IF(L43="Ouvrir +1 classe",H43+'08_Moteur'!O40*('08_Moteur'!AE40*'08_Moteur'!AF40-('08_Moteur'!R40+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S40)-'08_Moteur'!U40,IF(L43="Regrouper (-1 classe)",H43+('08_Moteur'!AI40-MAX(1,'08_Moteur'!AI40-1))*'08_Moteur'!U40,H43)))</f>
         <v/>
       </c>
       <c r="O43" s="17">
@@ -5245,11 +5245,11 @@
         <v/>
       </c>
       <c r="J44" s="69">
-        <f>IF(H44&lt;0,"🔴 Ne pas ouvrir",IF(I44&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I44&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H44&lt;0,"🔴 Ne pas lancer",IF(I44&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I44&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K44" s="70">
-        <f>IF(H44&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I44&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I44&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H44&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I44&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I44&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L44" s="21" t="inlineStr">
@@ -5258,11 +5258,11 @@
         </is>
       </c>
       <c r="M44" s="50">
-        <f>IF(L44="Ne pas ouvrir",0,IF(L44="Ouvrir +1 classe",E44+'08_Moteur'!O41,E44))</f>
+        <f>IF(L44="Ne pas lancer",0,IF(L44="Ouvrir +1 classe",E44+'08_Moteur'!O41,E44))</f>
         <v/>
       </c>
       <c r="N44" s="17">
-        <f>IF(L44="Ne pas ouvrir",0,IF(L44="Ouvrir +1 classe",H44+'08_Moteur'!O41*('08_Moteur'!AE41*'08_Moteur'!AF41-('08_Moteur'!R41+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S41)-'08_Moteur'!U41,IF(L44="Économiser 1 classe",H44+('08_Moteur'!AI41-MAX(1,'08_Moteur'!AI41-1))*'08_Moteur'!U41,H44)))</f>
+        <f>IF(L44="Ne pas lancer",0,IF(L44="Ouvrir +1 classe",H44+'08_Moteur'!O41*('08_Moteur'!AE41*'08_Moteur'!AF41-('08_Moteur'!R41+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S41)-'08_Moteur'!U41,IF(L44="Regrouper (-1 classe)",H44+('08_Moteur'!AI41-MAX(1,'08_Moteur'!AI41-1))*'08_Moteur'!U41,H44)))</f>
         <v/>
       </c>
       <c r="O44" s="17">
@@ -5316,11 +5316,11 @@
         <v/>
       </c>
       <c r="J45" s="69">
-        <f>IF(H45&lt;0,"🔴 Ne pas ouvrir",IF(I45&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I45&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H45&lt;0,"🔴 Restructurer (mutualiser)",IF(I45&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K45" s="70">
-        <f>IF(H45&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I45&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I45&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L45" s="21" t="inlineStr">
@@ -5329,11 +5329,11 @@
         </is>
       </c>
       <c r="M45" s="50">
-        <f>IF(L45="Ne pas ouvrir",0,IF(L45="Ouvrir +1 classe",E45+'08_Moteur'!O42,E45))</f>
+        <f>IF(L45="Ne pas lancer",0,IF(L45="Ouvrir +1 classe",E45+'08_Moteur'!O42,E45))</f>
         <v/>
       </c>
       <c r="N45" s="17">
-        <f>IF(L45="Ne pas ouvrir",0,IF(L45="Ouvrir +1 classe",H45+'08_Moteur'!O42*('08_Moteur'!AE42*'08_Moteur'!AF42-('08_Moteur'!R42+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S42)-'08_Moteur'!U42,IF(L45="Économiser 1 classe",H45+('08_Moteur'!AI42-MAX(1,'08_Moteur'!AI42-1))*'08_Moteur'!U42,H45)))</f>
+        <f>IF(L45="Ne pas lancer",0,IF(L45="Ouvrir +1 classe",H45+'08_Moteur'!O42*('08_Moteur'!AE42*'08_Moteur'!AF42-('08_Moteur'!R42+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S42)-'08_Moteur'!U42,IF(L45="Regrouper (-1 classe)",H45+('08_Moteur'!AI42-MAX(1,'08_Moteur'!AI42-1))*'08_Moteur'!U42,H45)))</f>
         <v/>
       </c>
       <c r="O45" s="17">
@@ -5387,11 +5387,11 @@
         <v/>
       </c>
       <c r="J46" s="69">
-        <f>IF(H46&lt;0,"🔴 Ne pas ouvrir",IF(I46&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I46&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H46&lt;0,"🔴 Restructurer (mutualiser)",IF(I46&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K46" s="70">
-        <f>IF(H46&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I46&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I46&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L46" s="21" t="inlineStr">
@@ -5400,11 +5400,11 @@
         </is>
       </c>
       <c r="M46" s="50">
-        <f>IF(L46="Ne pas ouvrir",0,IF(L46="Ouvrir +1 classe",E46+'08_Moteur'!O43,E46))</f>
+        <f>IF(L46="Ne pas lancer",0,IF(L46="Ouvrir +1 classe",E46+'08_Moteur'!O43,E46))</f>
         <v/>
       </c>
       <c r="N46" s="17">
-        <f>IF(L46="Ne pas ouvrir",0,IF(L46="Ouvrir +1 classe",H46+'08_Moteur'!O43*('08_Moteur'!AE43*'08_Moteur'!AF43-('08_Moteur'!R43+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S43)-'08_Moteur'!U43,IF(L46="Économiser 1 classe",H46+('08_Moteur'!AI43-MAX(1,'08_Moteur'!AI43-1))*'08_Moteur'!U43,H46)))</f>
+        <f>IF(L46="Ne pas lancer",0,IF(L46="Ouvrir +1 classe",H46+'08_Moteur'!O43*('08_Moteur'!AE43*'08_Moteur'!AF43-('08_Moteur'!R43+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S43)-'08_Moteur'!U43,IF(L46="Regrouper (-1 classe)",H46+('08_Moteur'!AI43-MAX(1,'08_Moteur'!AI43-1))*'08_Moteur'!U43,H46)))</f>
         <v/>
       </c>
       <c r="O46" s="17">
@@ -5458,11 +5458,11 @@
         <v/>
       </c>
       <c r="J47" s="69">
-        <f>IF(H47&lt;0,"🔴 Ne pas ouvrir",IF(I47&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I47&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H47&lt;0,"🔴 Ne pas lancer",IF(I47&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I47&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K47" s="70">
-        <f>IF(H47&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I47&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I47&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H47&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I47&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I47&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L47" s="21" t="inlineStr">
@@ -5471,11 +5471,11 @@
         </is>
       </c>
       <c r="M47" s="50">
-        <f>IF(L47="Ne pas ouvrir",0,IF(L47="Ouvrir +1 classe",E47+'08_Moteur'!O44,E47))</f>
+        <f>IF(L47="Ne pas lancer",0,IF(L47="Ouvrir +1 classe",E47+'08_Moteur'!O44,E47))</f>
         <v/>
       </c>
       <c r="N47" s="17">
-        <f>IF(L47="Ne pas ouvrir",0,IF(L47="Ouvrir +1 classe",H47+'08_Moteur'!O44*('08_Moteur'!AE44*'08_Moteur'!AF44-('08_Moteur'!R44+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S44)-'08_Moteur'!U44,IF(L47="Économiser 1 classe",H47+('08_Moteur'!AI44-MAX(1,'08_Moteur'!AI44-1))*'08_Moteur'!U44,H47)))</f>
+        <f>IF(L47="Ne pas lancer",0,IF(L47="Ouvrir +1 classe",H47+'08_Moteur'!O44*('08_Moteur'!AE44*'08_Moteur'!AF44-('08_Moteur'!R44+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S44)-'08_Moteur'!U44,IF(L47="Regrouper (-1 classe)",H47+('08_Moteur'!AI44-MAX(1,'08_Moteur'!AI44-1))*'08_Moteur'!U44,H47)))</f>
         <v/>
       </c>
       <c r="O47" s="17">
@@ -5529,11 +5529,11 @@
         <v/>
       </c>
       <c r="J48" s="69">
-        <f>IF(H48&lt;0,"🔴 Ne pas ouvrir",IF(I48&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I48&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H48&lt;0,"🔴 Restructurer (mutualiser)",IF(I48&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K48" s="70">
-        <f>IF(H48&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I48&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I48&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L48" s="21" t="inlineStr">
@@ -5542,11 +5542,11 @@
         </is>
       </c>
       <c r="M48" s="50">
-        <f>IF(L48="Ne pas ouvrir",0,IF(L48="Ouvrir +1 classe",E48+'08_Moteur'!O45,E48))</f>
+        <f>IF(L48="Ne pas lancer",0,IF(L48="Ouvrir +1 classe",E48+'08_Moteur'!O45,E48))</f>
         <v/>
       </c>
       <c r="N48" s="17">
-        <f>IF(L48="Ne pas ouvrir",0,IF(L48="Ouvrir +1 classe",H48+'08_Moteur'!O45*('08_Moteur'!AE45*'08_Moteur'!AF45-('08_Moteur'!R45+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S45)-'08_Moteur'!U45,IF(L48="Économiser 1 classe",H48+('08_Moteur'!AI45-MAX(1,'08_Moteur'!AI45-1))*'08_Moteur'!U45,H48)))</f>
+        <f>IF(L48="Ne pas lancer",0,IF(L48="Ouvrir +1 classe",H48+'08_Moteur'!O45*('08_Moteur'!AE45*'08_Moteur'!AF45-('08_Moteur'!R45+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S45)-'08_Moteur'!U45,IF(L48="Regrouper (-1 classe)",H48+('08_Moteur'!AI45-MAX(1,'08_Moteur'!AI45-1))*'08_Moteur'!U45,H48)))</f>
         <v/>
       </c>
       <c r="O48" s="17">
@@ -5600,11 +5600,11 @@
         <v/>
       </c>
       <c r="J49" s="69">
-        <f>IF(H49&lt;0,"🔴 Ne pas ouvrir",IF(I49&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I49&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H49&lt;0,"🔴 Restructurer (mutualiser)",IF(I49&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K49" s="70">
-        <f>IF(H49&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I49&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I49&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L49" s="21" t="inlineStr">
@@ -5613,11 +5613,11 @@
         </is>
       </c>
       <c r="M49" s="50">
-        <f>IF(L49="Ne pas ouvrir",0,IF(L49="Ouvrir +1 classe",E49+'08_Moteur'!O46,E49))</f>
+        <f>IF(L49="Ne pas lancer",0,IF(L49="Ouvrir +1 classe",E49+'08_Moteur'!O46,E49))</f>
         <v/>
       </c>
       <c r="N49" s="17">
-        <f>IF(L49="Ne pas ouvrir",0,IF(L49="Ouvrir +1 classe",H49+'08_Moteur'!O46*('08_Moteur'!AE46*'08_Moteur'!AF46-('08_Moteur'!R46+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S46)-'08_Moteur'!U46,IF(L49="Économiser 1 classe",H49+('08_Moteur'!AI46-MAX(1,'08_Moteur'!AI46-1))*'08_Moteur'!U46,H49)))</f>
+        <f>IF(L49="Ne pas lancer",0,IF(L49="Ouvrir +1 classe",H49+'08_Moteur'!O46*('08_Moteur'!AE46*'08_Moteur'!AF46-('08_Moteur'!R46+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S46)-'08_Moteur'!U46,IF(L49="Regrouper (-1 classe)",H49+('08_Moteur'!AI46-MAX(1,'08_Moteur'!AI46-1))*'08_Moteur'!U46,H49)))</f>
         <v/>
       </c>
       <c r="O49" s="17">
@@ -5671,11 +5671,11 @@
         <v/>
       </c>
       <c r="J50" s="69">
-        <f>IF(H50&lt;0,"🔴 Ne pas ouvrir",IF(I50&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I50&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H50&lt;0,"🔴 Ne pas lancer",IF(I50&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I50&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K50" s="70">
-        <f>IF(H50&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I50&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I50&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H50&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I50&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I50&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L50" s="21" t="inlineStr">
@@ -5684,11 +5684,11 @@
         </is>
       </c>
       <c r="M50" s="50">
-        <f>IF(L50="Ne pas ouvrir",0,IF(L50="Ouvrir +1 classe",E50+'08_Moteur'!O47,E50))</f>
+        <f>IF(L50="Ne pas lancer",0,IF(L50="Ouvrir +1 classe",E50+'08_Moteur'!O47,E50))</f>
         <v/>
       </c>
       <c r="N50" s="17">
-        <f>IF(L50="Ne pas ouvrir",0,IF(L50="Ouvrir +1 classe",H50+'08_Moteur'!O47*('08_Moteur'!AE47*'08_Moteur'!AF47-('08_Moteur'!R47+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S47)-'08_Moteur'!U47,IF(L50="Économiser 1 classe",H50+('08_Moteur'!AI47-MAX(1,'08_Moteur'!AI47-1))*'08_Moteur'!U47,H50)))</f>
+        <f>IF(L50="Ne pas lancer",0,IF(L50="Ouvrir +1 classe",H50+'08_Moteur'!O47*('08_Moteur'!AE47*'08_Moteur'!AF47-('08_Moteur'!R47+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S47)-'08_Moteur'!U47,IF(L50="Regrouper (-1 classe)",H50+('08_Moteur'!AI47-MAX(1,'08_Moteur'!AI47-1))*'08_Moteur'!U47,H50)))</f>
         <v/>
       </c>
       <c r="O50" s="17">
@@ -5742,11 +5742,11 @@
         <v/>
       </c>
       <c r="J51" s="69">
-        <f>IF(H51&lt;0,"🔴 Ne pas ouvrir",IF(I51&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I51&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H51&lt;0,"🔴 Restructurer (mutualiser)",IF(I51&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K51" s="70">
-        <f>IF(H51&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I51&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I51&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L51" s="21" t="inlineStr">
@@ -5755,11 +5755,11 @@
         </is>
       </c>
       <c r="M51" s="50">
-        <f>IF(L51="Ne pas ouvrir",0,IF(L51="Ouvrir +1 classe",E51+'08_Moteur'!O48,E51))</f>
+        <f>IF(L51="Ne pas lancer",0,IF(L51="Ouvrir +1 classe",E51+'08_Moteur'!O48,E51))</f>
         <v/>
       </c>
       <c r="N51" s="17">
-        <f>IF(L51="Ne pas ouvrir",0,IF(L51="Ouvrir +1 classe",H51+'08_Moteur'!O48*('08_Moteur'!AE48*'08_Moteur'!AF48-('08_Moteur'!R48+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S48)-'08_Moteur'!U48,IF(L51="Économiser 1 classe",H51+('08_Moteur'!AI48-MAX(1,'08_Moteur'!AI48-1))*'08_Moteur'!U48,H51)))</f>
+        <f>IF(L51="Ne pas lancer",0,IF(L51="Ouvrir +1 classe",H51+'08_Moteur'!O48*('08_Moteur'!AE48*'08_Moteur'!AF48-('08_Moteur'!R48+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S48)-'08_Moteur'!U48,IF(L51="Regrouper (-1 classe)",H51+('08_Moteur'!AI48-MAX(1,'08_Moteur'!AI48-1))*'08_Moteur'!U48,H51)))</f>
         <v/>
       </c>
       <c r="O51" s="17">
@@ -5813,11 +5813,11 @@
         <v/>
       </c>
       <c r="J52" s="69">
-        <f>IF(H52&lt;0,"🔴 Ne pas ouvrir",IF(I52&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I52&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H52&lt;0,"🔴 Ne pas lancer",IF(I52&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I52&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K52" s="70">
-        <f>IF(H52&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I52&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I52&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H52&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I52&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I52&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L52" s="21" t="inlineStr">
@@ -5826,11 +5826,11 @@
         </is>
       </c>
       <c r="M52" s="50">
-        <f>IF(L52="Ne pas ouvrir",0,IF(L52="Ouvrir +1 classe",E52+'08_Moteur'!O49,E52))</f>
+        <f>IF(L52="Ne pas lancer",0,IF(L52="Ouvrir +1 classe",E52+'08_Moteur'!O49,E52))</f>
         <v/>
       </c>
       <c r="N52" s="17">
-        <f>IF(L52="Ne pas ouvrir",0,IF(L52="Ouvrir +1 classe",H52+'08_Moteur'!O49*('08_Moteur'!AE49*'08_Moteur'!AF49-('08_Moteur'!R49+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S49)-'08_Moteur'!U49,IF(L52="Économiser 1 classe",H52+('08_Moteur'!AI49-MAX(1,'08_Moteur'!AI49-1))*'08_Moteur'!U49,H52)))</f>
+        <f>IF(L52="Ne pas lancer",0,IF(L52="Ouvrir +1 classe",H52+'08_Moteur'!O49*('08_Moteur'!AE49*'08_Moteur'!AF49-('08_Moteur'!R49+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S49)-'08_Moteur'!U49,IF(L52="Regrouper (-1 classe)",H52+('08_Moteur'!AI49-MAX(1,'08_Moteur'!AI49-1))*'08_Moteur'!U49,H52)))</f>
         <v/>
       </c>
       <c r="O52" s="17">
@@ -5884,11 +5884,11 @@
         <v/>
       </c>
       <c r="J53" s="69">
-        <f>IF(H53&lt;0,"🔴 Ne pas ouvrir",IF(I53&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I53&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H53&lt;0,"🔴 Restructurer (mutualiser)",IF(I53&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K53" s="70">
-        <f>IF(H53&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I53&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I53&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L53" s="21" t="inlineStr">
@@ -5897,11 +5897,11 @@
         </is>
       </c>
       <c r="M53" s="50">
-        <f>IF(L53="Ne pas ouvrir",0,IF(L53="Ouvrir +1 classe",E53+'08_Moteur'!O50,E53))</f>
+        <f>IF(L53="Ne pas lancer",0,IF(L53="Ouvrir +1 classe",E53+'08_Moteur'!O50,E53))</f>
         <v/>
       </c>
       <c r="N53" s="17">
-        <f>IF(L53="Ne pas ouvrir",0,IF(L53="Ouvrir +1 classe",H53+'08_Moteur'!O50*('08_Moteur'!AE50*'08_Moteur'!AF50-('08_Moteur'!R50+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S50)-'08_Moteur'!U50,IF(L53="Économiser 1 classe",H53+('08_Moteur'!AI50-MAX(1,'08_Moteur'!AI50-1))*'08_Moteur'!U50,H53)))</f>
+        <f>IF(L53="Ne pas lancer",0,IF(L53="Ouvrir +1 classe",H53+'08_Moteur'!O50*('08_Moteur'!AE50*'08_Moteur'!AF50-('08_Moteur'!R50+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S50)-'08_Moteur'!U50,IF(L53="Regrouper (-1 classe)",H53+('08_Moteur'!AI50-MAX(1,'08_Moteur'!AI50-1))*'08_Moteur'!U50,H53)))</f>
         <v/>
       </c>
       <c r="O53" s="17">
@@ -5955,11 +5955,11 @@
         <v/>
       </c>
       <c r="J54" s="69">
-        <f>IF(H54&lt;0,"🔴 Ne pas ouvrir",IF(I54&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I54&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H54&lt;0,"🔴 Ne pas lancer",IF(I54&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I54&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K54" s="70">
-        <f>IF(H54&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I54&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I54&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H54&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I54&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I54&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L54" s="21" t="inlineStr">
@@ -5968,11 +5968,11 @@
         </is>
       </c>
       <c r="M54" s="50">
-        <f>IF(L54="Ne pas ouvrir",0,IF(L54="Ouvrir +1 classe",E54+'08_Moteur'!O51,E54))</f>
+        <f>IF(L54="Ne pas lancer",0,IF(L54="Ouvrir +1 classe",E54+'08_Moteur'!O51,E54))</f>
         <v/>
       </c>
       <c r="N54" s="17">
-        <f>IF(L54="Ne pas ouvrir",0,IF(L54="Ouvrir +1 classe",H54+'08_Moteur'!O51*('08_Moteur'!AE51*'08_Moteur'!AF51-('08_Moteur'!R51+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S51)-'08_Moteur'!U51,IF(L54="Économiser 1 classe",H54+('08_Moteur'!AI51-MAX(1,'08_Moteur'!AI51-1))*'08_Moteur'!U51,H54)))</f>
+        <f>IF(L54="Ne pas lancer",0,IF(L54="Ouvrir +1 classe",H54+'08_Moteur'!O51*('08_Moteur'!AE51*'08_Moteur'!AF51-('08_Moteur'!R51+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S51)-'08_Moteur'!U51,IF(L54="Regrouper (-1 classe)",H54+('08_Moteur'!AI51-MAX(1,'08_Moteur'!AI51-1))*'08_Moteur'!U51,H54)))</f>
         <v/>
       </c>
       <c r="O54" s="17">
@@ -6026,11 +6026,11 @@
         <v/>
       </c>
       <c r="J55" s="69">
-        <f>IF(H55&lt;0,"🔴 Ne pas ouvrir",IF(I55&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I55&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H55&lt;0,"🔴 Restructurer (mutualiser)",IF(I55&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K55" s="70">
-        <f>IF(H55&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I55&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I55&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L55" s="21" t="inlineStr">
@@ -6039,11 +6039,11 @@
         </is>
       </c>
       <c r="M55" s="50">
-        <f>IF(L55="Ne pas ouvrir",0,IF(L55="Ouvrir +1 classe",E55+'08_Moteur'!O52,E55))</f>
+        <f>IF(L55="Ne pas lancer",0,IF(L55="Ouvrir +1 classe",E55+'08_Moteur'!O52,E55))</f>
         <v/>
       </c>
       <c r="N55" s="17">
-        <f>IF(L55="Ne pas ouvrir",0,IF(L55="Ouvrir +1 classe",H55+'08_Moteur'!O52*('08_Moteur'!AE52*'08_Moteur'!AF52-('08_Moteur'!R52+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S52)-'08_Moteur'!U52,IF(L55="Économiser 1 classe",H55+('08_Moteur'!AI52-MAX(1,'08_Moteur'!AI52-1))*'08_Moteur'!U52,H55)))</f>
+        <f>IF(L55="Ne pas lancer",0,IF(L55="Ouvrir +1 classe",H55+'08_Moteur'!O52*('08_Moteur'!AE52*'08_Moteur'!AF52-('08_Moteur'!R52+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S52)-'08_Moteur'!U52,IF(L55="Regrouper (-1 classe)",H55+('08_Moteur'!AI52-MAX(1,'08_Moteur'!AI52-1))*'08_Moteur'!U52,H55)))</f>
         <v/>
       </c>
       <c r="O55" s="17">
@@ -6097,11 +6097,11 @@
         <v/>
       </c>
       <c r="J56" s="69">
-        <f>IF(H56&lt;0,"🔴 Ne pas ouvrir",IF(I56&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I56&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H56&lt;0,"🔴 Ne pas lancer",IF(I56&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I56&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K56" s="70">
-        <f>IF(H56&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I56&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I56&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H56&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I56&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I56&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L56" s="21" t="inlineStr">
@@ -6110,11 +6110,11 @@
         </is>
       </c>
       <c r="M56" s="50">
-        <f>IF(L56="Ne pas ouvrir",0,IF(L56="Ouvrir +1 classe",E56+'08_Moteur'!O53,E56))</f>
+        <f>IF(L56="Ne pas lancer",0,IF(L56="Ouvrir +1 classe",E56+'08_Moteur'!O53,E56))</f>
         <v/>
       </c>
       <c r="N56" s="17">
-        <f>IF(L56="Ne pas ouvrir",0,IF(L56="Ouvrir +1 classe",H56+'08_Moteur'!O53*('08_Moteur'!AE53*'08_Moteur'!AF53-('08_Moteur'!R53+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S53)-'08_Moteur'!U53,IF(L56="Économiser 1 classe",H56+('08_Moteur'!AI53-MAX(1,'08_Moteur'!AI53-1))*'08_Moteur'!U53,H56)))</f>
+        <f>IF(L56="Ne pas lancer",0,IF(L56="Ouvrir +1 classe",H56+'08_Moteur'!O53*('08_Moteur'!AE53*'08_Moteur'!AF53-('08_Moteur'!R53+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S53)-'08_Moteur'!U53,IF(L56="Regrouper (-1 classe)",H56+('08_Moteur'!AI53-MAX(1,'08_Moteur'!AI53-1))*'08_Moteur'!U53,H56)))</f>
         <v/>
       </c>
       <c r="O56" s="17">
@@ -6168,11 +6168,11 @@
         <v/>
       </c>
       <c r="J57" s="69">
-        <f>IF(H57&lt;0,"🔴 Ne pas ouvrir",IF(I57&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I57&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H57&lt;0,"🔴 Restructurer (mutualiser)",IF(I57&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K57" s="70">
-        <f>IF(H57&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I57&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I57&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L57" s="21" t="inlineStr">
@@ -6181,11 +6181,11 @@
         </is>
       </c>
       <c r="M57" s="50">
-        <f>IF(L57="Ne pas ouvrir",0,IF(L57="Ouvrir +1 classe",E57+'08_Moteur'!O54,E57))</f>
+        <f>IF(L57="Ne pas lancer",0,IF(L57="Ouvrir +1 classe",E57+'08_Moteur'!O54,E57))</f>
         <v/>
       </c>
       <c r="N57" s="17">
-        <f>IF(L57="Ne pas ouvrir",0,IF(L57="Ouvrir +1 classe",H57+'08_Moteur'!O54*('08_Moteur'!AE54*'08_Moteur'!AF54-('08_Moteur'!R54+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S54)-'08_Moteur'!U54,IF(L57="Économiser 1 classe",H57+('08_Moteur'!AI54-MAX(1,'08_Moteur'!AI54-1))*'08_Moteur'!U54,H57)))</f>
+        <f>IF(L57="Ne pas lancer",0,IF(L57="Ouvrir +1 classe",H57+'08_Moteur'!O54*('08_Moteur'!AE54*'08_Moteur'!AF54-('08_Moteur'!R54+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S54)-'08_Moteur'!U54,IF(L57="Regrouper (-1 classe)",H57+('08_Moteur'!AI54-MAX(1,'08_Moteur'!AI54-1))*'08_Moteur'!U54,H57)))</f>
         <v/>
       </c>
       <c r="O57" s="17">
@@ -6239,11 +6239,11 @@
         <v/>
       </c>
       <c r="J58" s="69">
-        <f>IF(H58&lt;0,"🔴 Ne pas ouvrir",IF(I58&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I58&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H58&lt;0,"🔴 Ne pas lancer",IF(I58&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I58&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K58" s="70">
-        <f>IF(H58&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I58&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I58&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H58&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I58&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I58&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L58" s="21" t="inlineStr">
@@ -6252,11 +6252,11 @@
         </is>
       </c>
       <c r="M58" s="50">
-        <f>IF(L58="Ne pas ouvrir",0,IF(L58="Ouvrir +1 classe",E58+'08_Moteur'!O55,E58))</f>
+        <f>IF(L58="Ne pas lancer",0,IF(L58="Ouvrir +1 classe",E58+'08_Moteur'!O55,E58))</f>
         <v/>
       </c>
       <c r="N58" s="17">
-        <f>IF(L58="Ne pas ouvrir",0,IF(L58="Ouvrir +1 classe",H58+'08_Moteur'!O55*('08_Moteur'!AE55*'08_Moteur'!AF55-('08_Moteur'!R55+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S55)-'08_Moteur'!U55,IF(L58="Économiser 1 classe",H58+('08_Moteur'!AI55-MAX(1,'08_Moteur'!AI55-1))*'08_Moteur'!U55,H58)))</f>
+        <f>IF(L58="Ne pas lancer",0,IF(L58="Ouvrir +1 classe",H58+'08_Moteur'!O55*('08_Moteur'!AE55*'08_Moteur'!AF55-('08_Moteur'!R55+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S55)-'08_Moteur'!U55,IF(L58="Regrouper (-1 classe)",H58+('08_Moteur'!AI55-MAX(1,'08_Moteur'!AI55-1))*'08_Moteur'!U55,H58)))</f>
         <v/>
       </c>
       <c r="O58" s="17">
@@ -6310,11 +6310,11 @@
         <v/>
       </c>
       <c r="J59" s="69">
-        <f>IF(H59&lt;0,"🔴 Ne pas ouvrir",IF(I59&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I59&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H59&lt;0,"🔴 Restructurer (mutualiser)",IF(I59&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K59" s="70">
-        <f>IF(H59&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I59&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I59&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L59" s="21" t="inlineStr">
@@ -6323,11 +6323,11 @@
         </is>
       </c>
       <c r="M59" s="50">
-        <f>IF(L59="Ne pas ouvrir",0,IF(L59="Ouvrir +1 classe",E59+'08_Moteur'!O56,E59))</f>
+        <f>IF(L59="Ne pas lancer",0,IF(L59="Ouvrir +1 classe",E59+'08_Moteur'!O56,E59))</f>
         <v/>
       </c>
       <c r="N59" s="17">
-        <f>IF(L59="Ne pas ouvrir",0,IF(L59="Ouvrir +1 classe",H59+'08_Moteur'!O56*('08_Moteur'!AE56*'08_Moteur'!AF56-('08_Moteur'!R56+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S56)-'08_Moteur'!U56,IF(L59="Économiser 1 classe",H59+('08_Moteur'!AI56-MAX(1,'08_Moteur'!AI56-1))*'08_Moteur'!U56,H59)))</f>
+        <f>IF(L59="Ne pas lancer",0,IF(L59="Ouvrir +1 classe",H59+'08_Moteur'!O56*('08_Moteur'!AE56*'08_Moteur'!AF56-('08_Moteur'!R56+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S56)-'08_Moteur'!U56,IF(L59="Regrouper (-1 classe)",H59+('08_Moteur'!AI56-MAX(1,'08_Moteur'!AI56-1))*'08_Moteur'!U56,H59)))</f>
         <v/>
       </c>
       <c r="O59" s="17">
@@ -6381,11 +6381,11 @@
         <v/>
       </c>
       <c r="J60" s="69">
-        <f>IF(H60&lt;0,"🔴 Ne pas ouvrir",IF(I60&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I60&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H60&lt;0,"🔴 Restructurer (mutualiser)",IF(I60&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K60" s="70">
-        <f>IF(H60&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I60&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I60&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L60" s="21" t="inlineStr">
@@ -6394,11 +6394,11 @@
         </is>
       </c>
       <c r="M60" s="50">
-        <f>IF(L60="Ne pas ouvrir",0,IF(L60="Ouvrir +1 classe",E60+'08_Moteur'!O57,E60))</f>
+        <f>IF(L60="Ne pas lancer",0,IF(L60="Ouvrir +1 classe",E60+'08_Moteur'!O57,E60))</f>
         <v/>
       </c>
       <c r="N60" s="17">
-        <f>IF(L60="Ne pas ouvrir",0,IF(L60="Ouvrir +1 classe",H60+'08_Moteur'!O57*('08_Moteur'!AE57*'08_Moteur'!AF57-('08_Moteur'!R57+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S57)-'08_Moteur'!U57,IF(L60="Économiser 1 classe",H60+('08_Moteur'!AI57-MAX(1,'08_Moteur'!AI57-1))*'08_Moteur'!U57,H60)))</f>
+        <f>IF(L60="Ne pas lancer",0,IF(L60="Ouvrir +1 classe",H60+'08_Moteur'!O57*('08_Moteur'!AE57*'08_Moteur'!AF57-('08_Moteur'!R57+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S57)-'08_Moteur'!U57,IF(L60="Regrouper (-1 classe)",H60+('08_Moteur'!AI57-MAX(1,'08_Moteur'!AI57-1))*'08_Moteur'!U57,H60)))</f>
         <v/>
       </c>
       <c r="O60" s="17">
@@ -6452,11 +6452,11 @@
         <v/>
       </c>
       <c r="J61" s="69">
-        <f>IF(H61&lt;0,"🔴 Ne pas ouvrir",IF(I61&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I61&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H61&lt;0,"🔴 Ne pas lancer",IF(I61&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I61&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K61" s="70">
-        <f>IF(H61&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I61&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I61&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>IF(H61&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I61&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I61&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
       <c r="L61" s="21" t="inlineStr">
@@ -6465,11 +6465,11 @@
         </is>
       </c>
       <c r="M61" s="50">
-        <f>IF(L61="Ne pas ouvrir",0,IF(L61="Ouvrir +1 classe",E61+'08_Moteur'!O58,E61))</f>
+        <f>IF(L61="Ne pas lancer",0,IF(L61="Ouvrir +1 classe",E61+'08_Moteur'!O58,E61))</f>
         <v/>
       </c>
       <c r="N61" s="17">
-        <f>IF(L61="Ne pas ouvrir",0,IF(L61="Ouvrir +1 classe",H61+'08_Moteur'!O58*('08_Moteur'!AE58*'08_Moteur'!AF58-('08_Moteur'!R58+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S58)-'08_Moteur'!U58,IF(L61="Économiser 1 classe",H61+('08_Moteur'!AI58-MAX(1,'08_Moteur'!AI58-1))*'08_Moteur'!U58,H61)))</f>
+        <f>IF(L61="Ne pas lancer",0,IF(L61="Ouvrir +1 classe",H61+'08_Moteur'!O58*('08_Moteur'!AE58*'08_Moteur'!AF58-('08_Moteur'!R58+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S58)-'08_Moteur'!U58,IF(L61="Regrouper (-1 classe)",H61+('08_Moteur'!AI58-MAX(1,'08_Moteur'!AI58-1))*'08_Moteur'!U58,H61)))</f>
         <v/>
       </c>
       <c r="O61" s="17">
@@ -6523,11 +6523,11 @@
         <v/>
       </c>
       <c r="J62" s="69">
-        <f>IF(H62&lt;0,"🔴 Ne pas ouvrir",IF(I62&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I62&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H62&lt;0,"🔴 Restructurer (mutualiser)",IF(I62&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K62" s="70">
-        <f>IF(H62&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I62&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I62&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L62" s="21" t="inlineStr">
@@ -6536,11 +6536,11 @@
         </is>
       </c>
       <c r="M62" s="50">
-        <f>IF(L62="Ne pas ouvrir",0,IF(L62="Ouvrir +1 classe",E62+'08_Moteur'!O59,E62))</f>
+        <f>IF(L62="Ne pas lancer",0,IF(L62="Ouvrir +1 classe",E62+'08_Moteur'!O59,E62))</f>
         <v/>
       </c>
       <c r="N62" s="17">
-        <f>IF(L62="Ne pas ouvrir",0,IF(L62="Ouvrir +1 classe",H62+'08_Moteur'!O59*('08_Moteur'!AE59*'08_Moteur'!AF59-('08_Moteur'!R59+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S59)-'08_Moteur'!U59,IF(L62="Économiser 1 classe",H62+('08_Moteur'!AI59-MAX(1,'08_Moteur'!AI59-1))*'08_Moteur'!U59,H62)))</f>
+        <f>IF(L62="Ne pas lancer",0,IF(L62="Ouvrir +1 classe",H62+'08_Moteur'!O59*('08_Moteur'!AE59*'08_Moteur'!AF59-('08_Moteur'!R59+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S59)-'08_Moteur'!U59,IF(L62="Regrouper (-1 classe)",H62+('08_Moteur'!AI59-MAX(1,'08_Moteur'!AI59-1))*'08_Moteur'!U59,H62)))</f>
         <v/>
       </c>
       <c r="O62" s="17">
@@ -6594,11 +6594,11 @@
         <v/>
       </c>
       <c r="J63" s="69">
-        <f>IF(H63&lt;0,"🔴 Ne pas ouvrir",IF(I63&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I63&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
+        <f>IF(H63&lt;0,"🔴 Restructurer (mutualiser)",IF(I63&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
       <c r="K63" s="70">
-        <f>IF(H63&lt;0,"Contribution négative → fermer améliore l'EBITDA",IF(I63&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I63&lt;0.55,"Sous-rempli mais contribution positive → GARDER","Sain")))</f>
+        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
       <c r="L63" s="21" t="inlineStr">
@@ -6607,11 +6607,11 @@
         </is>
       </c>
       <c r="M63" s="50">
-        <f>IF(L63="Ne pas ouvrir",0,IF(L63="Ouvrir +1 classe",E63+'08_Moteur'!O60,E63))</f>
+        <f>IF(L63="Ne pas lancer",0,IF(L63="Ouvrir +1 classe",E63+'08_Moteur'!O60,E63))</f>
         <v/>
       </c>
       <c r="N63" s="17">
-        <f>IF(L63="Ne pas ouvrir",0,IF(L63="Ouvrir +1 classe",H63+'08_Moteur'!O60*('08_Moteur'!AE60*'08_Moteur'!AF60-('08_Moteur'!R60+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S60)-'08_Moteur'!U60,IF(L63="Économiser 1 classe",H63+('08_Moteur'!AI60-MAX(1,'08_Moteur'!AI60-1))*'08_Moteur'!U60,H63)))</f>
+        <f>IF(L63="Ne pas lancer",0,IF(L63="Ouvrir +1 classe",H63+'08_Moteur'!O60*('08_Moteur'!AE60*'08_Moteur'!AF60-('08_Moteur'!R60+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S60)-'08_Moteur'!U60,IF(L63="Regrouper (-1 classe)",H63+('08_Moteur'!AI60-MAX(1,'08_Moteur'!AI60-1))*'08_Moteur'!U60,H63)))</f>
         <v/>
       </c>
       <c r="O63" s="17">
@@ -6641,9 +6641,12 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="I3:J3"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L45 L46 L47 L48 L49 L50 L51 L52 L53 L54 L55 L56 L57 L58 L59 L60 L61 L62 L63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Maintenir,Ne pas ouvrir,Ouvrir +1 classe,Économiser 1 classe"</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="L6 L9 L11 L14 L16 L19 L21 L24 L26 L29 L31 L34 L36 L39 L41 L44 L47 L50 L52 L54 L56 L58 L61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Maintenir,Ne pas lancer,Ouvrir +1 classe,Regrouper (-1 classe)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L7 L8 L10 L12 L13 L15 L17 L18 L20 L22 L23 L25 L27 L28 L30 L32 L33 L35 L37 L38 L40 L42 L43 L45 L46 L48 L49 L51 L53 L55 L57 L59 L60 L62 L63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Maintenir,Regrouper (-1 classe)"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Simulateur : mention explicite 'bac à sable' (n'affecte pas le P&L officiel)
Décision : garder le simulateur isolé (what-if). Ajout d'un avertissement clair
sur la feuille 11 : les décisions montrent un impact SIMULÉ (encadré) mais
n'affectent pas 09_Allocation / 10_PnL / 13_Simulation, pilotés par les leviers (02).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -35,7 +35,7 @@
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;;(#,##0)&quot; €&quot;;&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,6 +88,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00000000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="8">
@@ -187,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -378,6 +384,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2416,6 +2425,13 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="68" t="inlineStr">
+        <is>
+          <t>🧪 BAC À SABLE : ces décisions montrent un impact SIMULÉ (encadré ci-dessus) — elles n'affectent PAS le budget officiel (feuilles 09_Allocation / 10_PnL / 13_Simulation), qui se pilote via les LEVIERS (feuille 02_Leviers).</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
@@ -2542,15 +2558,15 @@
         <f>'08_Moteur'!AM3</f>
         <v/>
       </c>
-      <c r="I6" s="68">
+      <c r="I6" s="69">
         <f>'08_Moteur'!AN3</f>
         <v/>
       </c>
-      <c r="J6" s="69">
+      <c r="J6" s="70">
         <f>IF(H6&lt;0,"🔴 Ne pas lancer",IF(I6&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I6&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K6" s="70">
+      <c r="K6" s="71">
         <f>IF(H6&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I6&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I6&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -2613,15 +2629,15 @@
         <f>'08_Moteur'!AM4</f>
         <v/>
       </c>
-      <c r="I7" s="68">
+      <c r="I7" s="69">
         <f>'08_Moteur'!AN4</f>
         <v/>
       </c>
-      <c r="J7" s="69">
+      <c r="J7" s="70">
         <f>IF(H7&lt;0,"🔴 Restructurer (mutualiser)",IF(I7&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K7" s="70">
+      <c r="K7" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -2684,15 +2700,15 @@
         <f>'08_Moteur'!AM5</f>
         <v/>
       </c>
-      <c r="I8" s="68">
+      <c r="I8" s="69">
         <f>'08_Moteur'!AN5</f>
         <v/>
       </c>
-      <c r="J8" s="69">
+      <c r="J8" s="70">
         <f>IF(H8&lt;0,"🔴 Restructurer (mutualiser)",IF(I8&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K8" s="70">
+      <c r="K8" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -2755,15 +2771,15 @@
         <f>'08_Moteur'!AM6</f>
         <v/>
       </c>
-      <c r="I9" s="68">
+      <c r="I9" s="69">
         <f>'08_Moteur'!AN6</f>
         <v/>
       </c>
-      <c r="J9" s="69">
+      <c r="J9" s="70">
         <f>IF(H9&lt;0,"🔴 Ne pas lancer",IF(I9&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I9&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K9" s="70">
+      <c r="K9" s="71">
         <f>IF(H9&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I9&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I9&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -2826,15 +2842,15 @@
         <f>'08_Moteur'!AM7</f>
         <v/>
       </c>
-      <c r="I10" s="68">
+      <c r="I10" s="69">
         <f>'08_Moteur'!AN7</f>
         <v/>
       </c>
-      <c r="J10" s="69">
+      <c r="J10" s="70">
         <f>IF(H10&lt;0,"🔴 Restructurer (mutualiser)",IF(I10&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K10" s="70">
+      <c r="K10" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -2897,15 +2913,15 @@
         <f>'08_Moteur'!AM8</f>
         <v/>
       </c>
-      <c r="I11" s="68">
+      <c r="I11" s="69">
         <f>'08_Moteur'!AN8</f>
         <v/>
       </c>
-      <c r="J11" s="69">
+      <c r="J11" s="70">
         <f>IF(H11&lt;0,"🔴 Ne pas lancer",IF(I11&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I11&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K11" s="70">
+      <c r="K11" s="71">
         <f>IF(H11&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I11&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I11&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -2968,15 +2984,15 @@
         <f>'08_Moteur'!AM9</f>
         <v/>
       </c>
-      <c r="I12" s="68">
+      <c r="I12" s="69">
         <f>'08_Moteur'!AN9</f>
         <v/>
       </c>
-      <c r="J12" s="69">
+      <c r="J12" s="70">
         <f>IF(H12&lt;0,"🔴 Restructurer (mutualiser)",IF(I12&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K12" s="70">
+      <c r="K12" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3039,15 +3055,15 @@
         <f>'08_Moteur'!AM10</f>
         <v/>
       </c>
-      <c r="I13" s="68">
+      <c r="I13" s="69">
         <f>'08_Moteur'!AN10</f>
         <v/>
       </c>
-      <c r="J13" s="69">
+      <c r="J13" s="70">
         <f>IF(H13&lt;0,"🔴 Restructurer (mutualiser)",IF(I13&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K13" s="70">
+      <c r="K13" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3110,15 +3126,15 @@
         <f>'08_Moteur'!AM11</f>
         <v/>
       </c>
-      <c r="I14" s="68">
+      <c r="I14" s="69">
         <f>'08_Moteur'!AN11</f>
         <v/>
       </c>
-      <c r="J14" s="69">
+      <c r="J14" s="70">
         <f>IF(H14&lt;0,"🔴 Ne pas lancer",IF(I14&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I14&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K14" s="70">
+      <c r="K14" s="71">
         <f>IF(H14&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I14&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I14&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -3181,15 +3197,15 @@
         <f>'08_Moteur'!AM12</f>
         <v/>
       </c>
-      <c r="I15" s="68">
+      <c r="I15" s="69">
         <f>'08_Moteur'!AN12</f>
         <v/>
       </c>
-      <c r="J15" s="69">
+      <c r="J15" s="70">
         <f>IF(H15&lt;0,"🔴 Restructurer (mutualiser)",IF(I15&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K15" s="70">
+      <c r="K15" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3252,15 +3268,15 @@
         <f>'08_Moteur'!AM13</f>
         <v/>
       </c>
-      <c r="I16" s="68">
+      <c r="I16" s="69">
         <f>'08_Moteur'!AN13</f>
         <v/>
       </c>
-      <c r="J16" s="69">
+      <c r="J16" s="70">
         <f>IF(H16&lt;0,"🔴 Ne pas lancer",IF(I16&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I16&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K16" s="70">
+      <c r="K16" s="71">
         <f>IF(H16&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I16&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I16&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -3323,15 +3339,15 @@
         <f>'08_Moteur'!AM14</f>
         <v/>
       </c>
-      <c r="I17" s="68">
+      <c r="I17" s="69">
         <f>'08_Moteur'!AN14</f>
         <v/>
       </c>
-      <c r="J17" s="69">
+      <c r="J17" s="70">
         <f>IF(H17&lt;0,"🔴 Restructurer (mutualiser)",IF(I17&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K17" s="70">
+      <c r="K17" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3394,15 +3410,15 @@
         <f>'08_Moteur'!AM15</f>
         <v/>
       </c>
-      <c r="I18" s="68">
+      <c r="I18" s="69">
         <f>'08_Moteur'!AN15</f>
         <v/>
       </c>
-      <c r="J18" s="69">
+      <c r="J18" s="70">
         <f>IF(H18&lt;0,"🔴 Restructurer (mutualiser)",IF(I18&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K18" s="70">
+      <c r="K18" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3465,15 +3481,15 @@
         <f>'08_Moteur'!AM16</f>
         <v/>
       </c>
-      <c r="I19" s="68">
+      <c r="I19" s="69">
         <f>'08_Moteur'!AN16</f>
         <v/>
       </c>
-      <c r="J19" s="69">
+      <c r="J19" s="70">
         <f>IF(H19&lt;0,"🔴 Ne pas lancer",IF(I19&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I19&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K19" s="70">
+      <c r="K19" s="71">
         <f>IF(H19&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I19&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I19&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -3536,15 +3552,15 @@
         <f>'08_Moteur'!AM17</f>
         <v/>
       </c>
-      <c r="I20" s="68">
+      <c r="I20" s="69">
         <f>'08_Moteur'!AN17</f>
         <v/>
       </c>
-      <c r="J20" s="69">
+      <c r="J20" s="70">
         <f>IF(H20&lt;0,"🔴 Restructurer (mutualiser)",IF(I20&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K20" s="70">
+      <c r="K20" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3607,15 +3623,15 @@
         <f>'08_Moteur'!AM18</f>
         <v/>
       </c>
-      <c r="I21" s="68">
+      <c r="I21" s="69">
         <f>'08_Moteur'!AN18</f>
         <v/>
       </c>
-      <c r="J21" s="69">
+      <c r="J21" s="70">
         <f>IF(H21&lt;0,"🔴 Ne pas lancer",IF(I21&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I21&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K21" s="70">
+      <c r="K21" s="71">
         <f>IF(H21&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I21&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I21&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -3678,15 +3694,15 @@
         <f>'08_Moteur'!AM19</f>
         <v/>
       </c>
-      <c r="I22" s="68">
+      <c r="I22" s="69">
         <f>'08_Moteur'!AN19</f>
         <v/>
       </c>
-      <c r="J22" s="69">
+      <c r="J22" s="70">
         <f>IF(H22&lt;0,"🔴 Restructurer (mutualiser)",IF(I22&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K22" s="70">
+      <c r="K22" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3749,15 +3765,15 @@
         <f>'08_Moteur'!AM20</f>
         <v/>
       </c>
-      <c r="I23" s="68">
+      <c r="I23" s="69">
         <f>'08_Moteur'!AN20</f>
         <v/>
       </c>
-      <c r="J23" s="69">
+      <c r="J23" s="70">
         <f>IF(H23&lt;0,"🔴 Restructurer (mutualiser)",IF(I23&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K23" s="70">
+      <c r="K23" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3820,15 +3836,15 @@
         <f>'08_Moteur'!AM21</f>
         <v/>
       </c>
-      <c r="I24" s="68">
+      <c r="I24" s="69">
         <f>'08_Moteur'!AN21</f>
         <v/>
       </c>
-      <c r="J24" s="69">
+      <c r="J24" s="70">
         <f>IF(H24&lt;0,"🔴 Ne pas lancer",IF(I24&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I24&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K24" s="70">
+      <c r="K24" s="71">
         <f>IF(H24&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I24&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I24&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -3891,15 +3907,15 @@
         <f>'08_Moteur'!AM22</f>
         <v/>
       </c>
-      <c r="I25" s="68">
+      <c r="I25" s="69">
         <f>'08_Moteur'!AN22</f>
         <v/>
       </c>
-      <c r="J25" s="69">
+      <c r="J25" s="70">
         <f>IF(H25&lt;0,"🔴 Restructurer (mutualiser)",IF(I25&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K25" s="70">
+      <c r="K25" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -3962,15 +3978,15 @@
         <f>'08_Moteur'!AM23</f>
         <v/>
       </c>
-      <c r="I26" s="68">
+      <c r="I26" s="69">
         <f>'08_Moteur'!AN23</f>
         <v/>
       </c>
-      <c r="J26" s="69">
+      <c r="J26" s="70">
         <f>IF(H26&lt;0,"🔴 Ne pas lancer",IF(I26&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I26&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K26" s="70">
+      <c r="K26" s="71">
         <f>IF(H26&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I26&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I26&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -4033,15 +4049,15 @@
         <f>'08_Moteur'!AM24</f>
         <v/>
       </c>
-      <c r="I27" s="68">
+      <c r="I27" s="69">
         <f>'08_Moteur'!AN24</f>
         <v/>
       </c>
-      <c r="J27" s="69">
+      <c r="J27" s="70">
         <f>IF(H27&lt;0,"🔴 Restructurer (mutualiser)",IF(I27&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K27" s="70">
+      <c r="K27" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4104,15 +4120,15 @@
         <f>'08_Moteur'!AM25</f>
         <v/>
       </c>
-      <c r="I28" s="68">
+      <c r="I28" s="69">
         <f>'08_Moteur'!AN25</f>
         <v/>
       </c>
-      <c r="J28" s="69">
+      <c r="J28" s="70">
         <f>IF(H28&lt;0,"🔴 Restructurer (mutualiser)",IF(I28&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K28" s="70">
+      <c r="K28" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4175,15 +4191,15 @@
         <f>'08_Moteur'!AM26</f>
         <v/>
       </c>
-      <c r="I29" s="68">
+      <c r="I29" s="69">
         <f>'08_Moteur'!AN26</f>
         <v/>
       </c>
-      <c r="J29" s="69">
+      <c r="J29" s="70">
         <f>IF(H29&lt;0,"🔴 Ne pas lancer",IF(I29&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I29&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K29" s="70">
+      <c r="K29" s="71">
         <f>IF(H29&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I29&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I29&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -4246,15 +4262,15 @@
         <f>'08_Moteur'!AM27</f>
         <v/>
       </c>
-      <c r="I30" s="68">
+      <c r="I30" s="69">
         <f>'08_Moteur'!AN27</f>
         <v/>
       </c>
-      <c r="J30" s="69">
+      <c r="J30" s="70">
         <f>IF(H30&lt;0,"🔴 Restructurer (mutualiser)",IF(I30&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K30" s="70">
+      <c r="K30" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4317,15 +4333,15 @@
         <f>'08_Moteur'!AM28</f>
         <v/>
       </c>
-      <c r="I31" s="68">
+      <c r="I31" s="69">
         <f>'08_Moteur'!AN28</f>
         <v/>
       </c>
-      <c r="J31" s="69">
+      <c r="J31" s="70">
         <f>IF(H31&lt;0,"🔴 Ne pas lancer",IF(I31&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I31&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K31" s="70">
+      <c r="K31" s="71">
         <f>IF(H31&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I31&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I31&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -4388,15 +4404,15 @@
         <f>'08_Moteur'!AM29</f>
         <v/>
       </c>
-      <c r="I32" s="68">
+      <c r="I32" s="69">
         <f>'08_Moteur'!AN29</f>
         <v/>
       </c>
-      <c r="J32" s="69">
+      <c r="J32" s="70">
         <f>IF(H32&lt;0,"🔴 Restructurer (mutualiser)",IF(I32&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K32" s="70">
+      <c r="K32" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4459,15 +4475,15 @@
         <f>'08_Moteur'!AM30</f>
         <v/>
       </c>
-      <c r="I33" s="68">
+      <c r="I33" s="69">
         <f>'08_Moteur'!AN30</f>
         <v/>
       </c>
-      <c r="J33" s="69">
+      <c r="J33" s="70">
         <f>IF(H33&lt;0,"🔴 Restructurer (mutualiser)",IF(I33&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K33" s="70">
+      <c r="K33" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4530,15 +4546,15 @@
         <f>'08_Moteur'!AM31</f>
         <v/>
       </c>
-      <c r="I34" s="68">
+      <c r="I34" s="69">
         <f>'08_Moteur'!AN31</f>
         <v/>
       </c>
-      <c r="J34" s="69">
+      <c r="J34" s="70">
         <f>IF(H34&lt;0,"🔴 Ne pas lancer",IF(I34&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I34&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K34" s="70">
+      <c r="K34" s="71">
         <f>IF(H34&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I34&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I34&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -4601,15 +4617,15 @@
         <f>'08_Moteur'!AM32</f>
         <v/>
       </c>
-      <c r="I35" s="68">
+      <c r="I35" s="69">
         <f>'08_Moteur'!AN32</f>
         <v/>
       </c>
-      <c r="J35" s="69">
+      <c r="J35" s="70">
         <f>IF(H35&lt;0,"🔴 Restructurer (mutualiser)",IF(I35&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K35" s="70">
+      <c r="K35" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4672,15 +4688,15 @@
         <f>'08_Moteur'!AM33</f>
         <v/>
       </c>
-      <c r="I36" s="68">
+      <c r="I36" s="69">
         <f>'08_Moteur'!AN33</f>
         <v/>
       </c>
-      <c r="J36" s="69">
+      <c r="J36" s="70">
         <f>IF(H36&lt;0,"🔴 Ne pas lancer",IF(I36&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I36&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K36" s="70">
+      <c r="K36" s="71">
         <f>IF(H36&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I36&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I36&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -4743,15 +4759,15 @@
         <f>'08_Moteur'!AM34</f>
         <v/>
       </c>
-      <c r="I37" s="68">
+      <c r="I37" s="69">
         <f>'08_Moteur'!AN34</f>
         <v/>
       </c>
-      <c r="J37" s="69">
+      <c r="J37" s="70">
         <f>IF(H37&lt;0,"🔴 Restructurer (mutualiser)",IF(I37&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K37" s="70">
+      <c r="K37" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4814,15 +4830,15 @@
         <f>'08_Moteur'!AM35</f>
         <v/>
       </c>
-      <c r="I38" s="68">
+      <c r="I38" s="69">
         <f>'08_Moteur'!AN35</f>
         <v/>
       </c>
-      <c r="J38" s="69">
+      <c r="J38" s="70">
         <f>IF(H38&lt;0,"🔴 Restructurer (mutualiser)",IF(I38&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K38" s="70">
+      <c r="K38" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -4885,15 +4901,15 @@
         <f>'08_Moteur'!AM36</f>
         <v/>
       </c>
-      <c r="I39" s="68">
+      <c r="I39" s="69">
         <f>'08_Moteur'!AN36</f>
         <v/>
       </c>
-      <c r="J39" s="69">
+      <c r="J39" s="70">
         <f>IF(H39&lt;0,"🔴 Ne pas lancer",IF(I39&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I39&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K39" s="70">
+      <c r="K39" s="71">
         <f>IF(H39&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I39&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I39&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -4956,15 +4972,15 @@
         <f>'08_Moteur'!AM37</f>
         <v/>
       </c>
-      <c r="I40" s="68">
+      <c r="I40" s="69">
         <f>'08_Moteur'!AN37</f>
         <v/>
       </c>
-      <c r="J40" s="69">
+      <c r="J40" s="70">
         <f>IF(H40&lt;0,"🔴 Restructurer (mutualiser)",IF(I40&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K40" s="70">
+      <c r="K40" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5027,15 +5043,15 @@
         <f>'08_Moteur'!AM38</f>
         <v/>
       </c>
-      <c r="I41" s="68">
+      <c r="I41" s="69">
         <f>'08_Moteur'!AN38</f>
         <v/>
       </c>
-      <c r="J41" s="69">
+      <c r="J41" s="70">
         <f>IF(H41&lt;0,"🔴 Ne pas lancer",IF(I41&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I41&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K41" s="70">
+      <c r="K41" s="71">
         <f>IF(H41&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I41&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I41&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -5098,15 +5114,15 @@
         <f>'08_Moteur'!AM39</f>
         <v/>
       </c>
-      <c r="I42" s="68">
+      <c r="I42" s="69">
         <f>'08_Moteur'!AN39</f>
         <v/>
       </c>
-      <c r="J42" s="69">
+      <c r="J42" s="70">
         <f>IF(H42&lt;0,"🔴 Restructurer (mutualiser)",IF(I42&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K42" s="70">
+      <c r="K42" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5169,15 +5185,15 @@
         <f>'08_Moteur'!AM40</f>
         <v/>
       </c>
-      <c r="I43" s="68">
+      <c r="I43" s="69">
         <f>'08_Moteur'!AN40</f>
         <v/>
       </c>
-      <c r="J43" s="69">
+      <c r="J43" s="70">
         <f>IF(H43&lt;0,"🔴 Restructurer (mutualiser)",IF(I43&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K43" s="70">
+      <c r="K43" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5240,15 +5256,15 @@
         <f>'08_Moteur'!AM41</f>
         <v/>
       </c>
-      <c r="I44" s="68">
+      <c r="I44" s="69">
         <f>'08_Moteur'!AN41</f>
         <v/>
       </c>
-      <c r="J44" s="69">
+      <c r="J44" s="70">
         <f>IF(H44&lt;0,"🔴 Ne pas lancer",IF(I44&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I44&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K44" s="70">
+      <c r="K44" s="71">
         <f>IF(H44&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I44&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I44&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -5311,15 +5327,15 @@
         <f>'08_Moteur'!AM42</f>
         <v/>
       </c>
-      <c r="I45" s="68">
+      <c r="I45" s="69">
         <f>'08_Moteur'!AN42</f>
         <v/>
       </c>
-      <c r="J45" s="69">
+      <c r="J45" s="70">
         <f>IF(H45&lt;0,"🔴 Restructurer (mutualiser)",IF(I45&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K45" s="70">
+      <c r="K45" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5382,15 +5398,15 @@
         <f>'08_Moteur'!AM43</f>
         <v/>
       </c>
-      <c r="I46" s="68">
+      <c r="I46" s="69">
         <f>'08_Moteur'!AN43</f>
         <v/>
       </c>
-      <c r="J46" s="69">
+      <c r="J46" s="70">
         <f>IF(H46&lt;0,"🔴 Restructurer (mutualiser)",IF(I46&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K46" s="70">
+      <c r="K46" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5453,15 +5469,15 @@
         <f>'08_Moteur'!AM44</f>
         <v/>
       </c>
-      <c r="I47" s="68">
+      <c r="I47" s="69">
         <f>'08_Moteur'!AN44</f>
         <v/>
       </c>
-      <c r="J47" s="69">
+      <c r="J47" s="70">
         <f>IF(H47&lt;0,"🔴 Ne pas lancer",IF(I47&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I47&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K47" s="70">
+      <c r="K47" s="71">
         <f>IF(H47&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I47&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I47&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -5524,15 +5540,15 @@
         <f>'08_Moteur'!AM45</f>
         <v/>
       </c>
-      <c r="I48" s="68">
+      <c r="I48" s="69">
         <f>'08_Moteur'!AN45</f>
         <v/>
       </c>
-      <c r="J48" s="69">
+      <c r="J48" s="70">
         <f>IF(H48&lt;0,"🔴 Restructurer (mutualiser)",IF(I48&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K48" s="70">
+      <c r="K48" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5595,15 +5611,15 @@
         <f>'08_Moteur'!AM46</f>
         <v/>
       </c>
-      <c r="I49" s="68">
+      <c r="I49" s="69">
         <f>'08_Moteur'!AN46</f>
         <v/>
       </c>
-      <c r="J49" s="69">
+      <c r="J49" s="70">
         <f>IF(H49&lt;0,"🔴 Restructurer (mutualiser)",IF(I49&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K49" s="70">
+      <c r="K49" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5666,15 +5682,15 @@
         <f>'08_Moteur'!AM47</f>
         <v/>
       </c>
-      <c r="I50" s="68">
+      <c r="I50" s="69">
         <f>'08_Moteur'!AN47</f>
         <v/>
       </c>
-      <c r="J50" s="69">
+      <c r="J50" s="70">
         <f>IF(H50&lt;0,"🔴 Ne pas lancer",IF(I50&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I50&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K50" s="70">
+      <c r="K50" s="71">
         <f>IF(H50&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I50&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I50&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -5737,15 +5753,15 @@
         <f>'08_Moteur'!AM48</f>
         <v/>
       </c>
-      <c r="I51" s="68">
+      <c r="I51" s="69">
         <f>'08_Moteur'!AN48</f>
         <v/>
       </c>
-      <c r="J51" s="69">
+      <c r="J51" s="70">
         <f>IF(H51&lt;0,"🔴 Restructurer (mutualiser)",IF(I51&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K51" s="70">
+      <c r="K51" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5808,15 +5824,15 @@
         <f>'08_Moteur'!AM49</f>
         <v/>
       </c>
-      <c r="I52" s="68">
+      <c r="I52" s="69">
         <f>'08_Moteur'!AN49</f>
         <v/>
       </c>
-      <c r="J52" s="69">
+      <c r="J52" s="70">
         <f>IF(H52&lt;0,"🔴 Ne pas lancer",IF(I52&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I52&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K52" s="70">
+      <c r="K52" s="71">
         <f>IF(H52&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I52&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I52&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -5879,15 +5895,15 @@
         <f>'08_Moteur'!AM50</f>
         <v/>
       </c>
-      <c r="I53" s="68">
+      <c r="I53" s="69">
         <f>'08_Moteur'!AN50</f>
         <v/>
       </c>
-      <c r="J53" s="69">
+      <c r="J53" s="70">
         <f>IF(H53&lt;0,"🔴 Restructurer (mutualiser)",IF(I53&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K53" s="70">
+      <c r="K53" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -5950,15 +5966,15 @@
         <f>'08_Moteur'!AM51</f>
         <v/>
       </c>
-      <c r="I54" s="68">
+      <c r="I54" s="69">
         <f>'08_Moteur'!AN51</f>
         <v/>
       </c>
-      <c r="J54" s="69">
+      <c r="J54" s="70">
         <f>IF(H54&lt;0,"🔴 Ne pas lancer",IF(I54&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I54&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K54" s="70">
+      <c r="K54" s="71">
         <f>IF(H54&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I54&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I54&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -6021,15 +6037,15 @@
         <f>'08_Moteur'!AM52</f>
         <v/>
       </c>
-      <c r="I55" s="68">
+      <c r="I55" s="69">
         <f>'08_Moteur'!AN52</f>
         <v/>
       </c>
-      <c r="J55" s="69">
+      <c r="J55" s="70">
         <f>IF(H55&lt;0,"🔴 Restructurer (mutualiser)",IF(I55&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K55" s="70">
+      <c r="K55" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -6092,15 +6108,15 @@
         <f>'08_Moteur'!AM53</f>
         <v/>
       </c>
-      <c r="I56" s="68">
+      <c r="I56" s="69">
         <f>'08_Moteur'!AN53</f>
         <v/>
       </c>
-      <c r="J56" s="69">
+      <c r="J56" s="70">
         <f>IF(H56&lt;0,"🔴 Ne pas lancer",IF(I56&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I56&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K56" s="70">
+      <c r="K56" s="71">
         <f>IF(H56&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I56&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I56&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -6163,15 +6179,15 @@
         <f>'08_Moteur'!AM54</f>
         <v/>
       </c>
-      <c r="I57" s="68">
+      <c r="I57" s="69">
         <f>'08_Moteur'!AN54</f>
         <v/>
       </c>
-      <c r="J57" s="69">
+      <c r="J57" s="70">
         <f>IF(H57&lt;0,"🔴 Restructurer (mutualiser)",IF(I57&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K57" s="70">
+      <c r="K57" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -6234,15 +6250,15 @@
         <f>'08_Moteur'!AM55</f>
         <v/>
       </c>
-      <c r="I58" s="68">
+      <c r="I58" s="69">
         <f>'08_Moteur'!AN55</f>
         <v/>
       </c>
-      <c r="J58" s="69">
+      <c r="J58" s="70">
         <f>IF(H58&lt;0,"🔴 Ne pas lancer",IF(I58&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I58&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K58" s="70">
+      <c r="K58" s="71">
         <f>IF(H58&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I58&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I58&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -6305,15 +6321,15 @@
         <f>'08_Moteur'!AM56</f>
         <v/>
       </c>
-      <c r="I59" s="68">
+      <c r="I59" s="69">
         <f>'08_Moteur'!AN56</f>
         <v/>
       </c>
-      <c r="J59" s="69">
+      <c r="J59" s="70">
         <f>IF(H59&lt;0,"🔴 Restructurer (mutualiser)",IF(I59&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K59" s="70">
+      <c r="K59" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -6376,15 +6392,15 @@
         <f>'08_Moteur'!AM57</f>
         <v/>
       </c>
-      <c r="I60" s="68">
+      <c r="I60" s="69">
         <f>'08_Moteur'!AN57</f>
         <v/>
       </c>
-      <c r="J60" s="69">
+      <c r="J60" s="70">
         <f>IF(H60&lt;0,"🔴 Restructurer (mutualiser)",IF(I60&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K60" s="70">
+      <c r="K60" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -6447,15 +6463,15 @@
         <f>'08_Moteur'!AM58</f>
         <v/>
       </c>
-      <c r="I61" s="68">
+      <c r="I61" s="69">
         <f>'08_Moteur'!AN58</f>
         <v/>
       </c>
-      <c r="J61" s="69">
+      <c r="J61" s="70">
         <f>IF(H61&lt;0,"🔴 Ne pas lancer",IF(I61&gt;=0.95,"🟢 Ouvrir +1 (capter+diluer)",IF(I61&lt;0.55,"🟡 Surveiller","🟢 Maintenir")))</f>
         <v/>
       </c>
-      <c r="K61" s="70">
+      <c r="K61" s="71">
         <f>IF(H61&lt;0,"Entrée à contribution négative → ne pas lancer cette cohorte",IF(I61&gt;=0.95,"Saturé → ouvrir capte des étudiants ET dilue la structure pour tous",IF(I61&lt;0.55,"Sous-rempli mais contribution positive → garder","Sain")))</f>
         <v/>
       </c>
@@ -6518,15 +6534,15 @@
         <f>'08_Moteur'!AM59</f>
         <v/>
       </c>
-      <c r="I62" s="68">
+      <c r="I62" s="69">
         <f>'08_Moteur'!AN59</f>
         <v/>
       </c>
-      <c r="J62" s="69">
+      <c r="J62" s="70">
         <f>IF(H62&lt;0,"🔴 Restructurer (mutualiser)",IF(I62&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K62" s="70">
+      <c r="K62" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -6589,15 +6605,15 @@
         <f>'08_Moteur'!AM60</f>
         <v/>
       </c>
-      <c r="I63" s="68">
+      <c r="I63" s="69">
         <f>'08_Moteur'!AN60</f>
         <v/>
       </c>
-      <c r="J63" s="69">
+      <c r="J63" s="70">
         <f>IF(H63&lt;0,"🔴 Restructurer (mutualiser)",IF(I63&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
         <v/>
       </c>
-      <c r="K63" s="70">
+      <c r="K63" s="71">
         <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
         <v/>
       </c>
@@ -6628,12 +6644,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="A4:Q4"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="G3:H3"/>
@@ -6709,7 +6726,7 @@
         <f>0.01*SUMPRODUCT('08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60*'08_Moteur'!$AF$3:$AF$60)</f>
         <v/>
       </c>
-      <c r="D6" s="70" t="inlineStr">
+      <c r="D6" s="71" t="inlineStr">
         <is>
           <t>Tombe quasi intégralement en EBITDA.</t>
         </is>
@@ -6725,7 +6742,7 @@
         <f>0.01*SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$D$18)</f>
         <v/>
       </c>
-      <c r="D7" s="70" t="inlineStr">
+      <c r="D7" s="71" t="inlineStr">
         <is>
           <t>Nul si recouvrement=100 % ; sinon réduit la perte.</t>
         </is>
@@ -6741,7 +6758,7 @@
         <f>0.01*'02_Leviers'!$D$21*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$AM$3:$AM$60)-0.01*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=1)*'08_Moteur'!$H$3:$H$60*'08_Moteur'!$S$3:$S$60*(1+'08_Moteur'!$Y$3:$Y$60))</f>
         <v/>
       </c>
-      <c r="D8" s="70" t="inlineStr">
+      <c r="D8" s="71" t="inlineStr">
         <is>
           <t>Plus de leads → plus d'inscrits, net du coût.</t>
         </is>
@@ -6757,7 +6774,7 @@
         <f>0.01*SUMPRODUCT(('08_Moteur'!$F$3:$F$60=0)*'08_Moteur'!$K$3:$K$60)*IFERROR(SUM('08_Moteur'!$AM$3:$AM$60)/SUM('08_Moteur'!$AD$3:$AD$60),0)</f>
         <v/>
       </c>
-      <c r="D9" s="70" t="inlineStr">
+      <c r="D9" s="71" t="inlineStr">
         <is>
           <t>Rétention : + d'étudiants qui poursuivent.</t>
         </is>
@@ -6769,7 +6786,7 @@
           <t>Exposition financement alternance (€ à sécuriser) :</t>
         </is>
       </c>
-      <c r="D11" s="71">
+      <c r="D11" s="72">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$G$9)</f>
         <v/>
       </c>
@@ -7012,20 +7029,20 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="72" t="inlineStr">
+      <c r="B15" s="73" t="inlineStr">
         <is>
           <t>€ à sécuriser (exposition)</t>
         </is>
       </c>
-      <c r="C15" s="73">
+      <c r="C15" s="74">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$G$9)</f>
         <v/>
       </c>
-      <c r="D15" s="73">
+      <c r="D15" s="74">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$G$3:$G$60*'08_Moteur'!$L$3:$L$60)*(1-'02_Leviers'!$D$20)</f>
         <v/>
       </c>
-      <c r="E15" s="74">
+      <c r="E15" s="75">
         <f>IFERROR(C15/D15-1,0)</f>
         <v/>
       </c>
@@ -7087,7 +7104,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="75" t="inlineStr">
+      <c r="B6" s="76" t="inlineStr">
         <is>
           <t>Marque / Campus</t>
         </is>
@@ -7104,7 +7121,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="75" t="inlineStr">
+      <c r="B7" s="76" t="inlineStr">
         <is>
           <t>Programme × Année × Modalité</t>
         </is>
@@ -7121,7 +7138,7 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="75" t="inlineStr">
+      <c r="B8" s="76" t="inlineStr">
         <is>
           <t>Params (capacité, heures…)</t>
         </is>
@@ -7138,7 +7155,7 @@
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="75" t="inlineStr">
+      <c r="B9" s="76" t="inlineStr">
         <is>
           <t>Historique N-2/N-1</t>
         </is>
@@ -7155,7 +7172,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="75" t="inlineStr">
+      <c r="B10" s="76" t="inlineStr">
         <is>
           <t>Cohortes / taux de passage</t>
         </is>
@@ -7172,7 +7189,7 @@
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="75" t="inlineStr">
+      <c r="B11" s="76" t="inlineStr">
         <is>
           <t>Sécurisation &amp; recouvrement</t>
         </is>
@@ -7189,7 +7206,7 @@
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="75" t="inlineStr">
+      <c r="B12" s="76" t="inlineStr">
         <is>
           <t>Objectifs (cadrage)</t>
         </is>
@@ -7206,7 +7223,7 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="75" t="inlineStr">
+      <c r="B13" s="76" t="inlineStr">
         <is>
           <t>Décisions ouvrir/fermer</t>
         </is>
@@ -7223,7 +7240,7 @@
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="75" t="inlineStr">
+      <c r="B14" s="76" t="inlineStr">
         <is>
           <t>Allocation structure</t>
         </is>

</xml_diff>

<commit_message>
Documentation : note explicative (info-bulle) sur chaque entête de chaque feuille
140 notes ajoutées (glossaire) sur les 13 feuilles à grille, dont les 42 colonnes
du moteur, les colonnes CFO du simulateur, les paramètres, l'historique, etc.
Survol d'un entête -> explication de ce qu'il contient / comment il est calculé.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -487,6 +487,836 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Indicateur de pilotage.</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Objectif fixé par la direction (saisie).</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Résultat du budget construit par les drivers (moteur).</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Budget construit − cible.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Ligne du compte de résultat.</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeur réelle de l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeur budgétée.</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Budget − Réalisé (en €).</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Variation en % vs l'an dernier.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Campus (ville). Une entité = Marque + Ville.</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Programme de formation (ex. Bachelor Management).</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Année d'études : B1/B2/B3 (Bachelor), M1/M2 (Mastère), 1/2 (BTS).</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif budget de la promo.</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Chiffre d'affaires budget de la promo.</t>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0">
+      <text>
+        <t>Coûts qui DISPARAISSENT si on ferme la promo (enseignement, pédago, marketing, autres variables).</t>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0">
+      <text>
+        <t>CA − coûts directs évitables. C'est LA métrique de décision : on ne ferme que si elle est négative.</t>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0">
+      <text>
+        <t>Taux de remplissage = effectif / (classes × capacité).</t>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0">
+      <text>
+        <t>Recommandation automatique (contribution + remplissage). Dépend de l'année : entrée (lancer/capter) vs poursuite (regrouper).</t>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="0" shapeId="0">
+      <text>
+        <t>Explication de la recommandation.</t>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0">
+      <text>
+        <t>Ton choix. Menu restreint selon l'année : entrée = lancer/capter ; poursuite = seulement regrouper.</t>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif après ta décision (0 si 'ne pas lancer' ; +1 classe captée si 'ouvrir').</t>
+      </text>
+    </comment>
+    <comment ref="N5" authorId="0" shapeId="0">
+      <text>
+        <t>Contribution recalculée selon ta décision.</t>
+      </text>
+    </comment>
+    <comment ref="O5" authorId="0" shapeId="0">
+      <text>
+        <t>Quote-part de structure fixe (loyer, permanents, siège) portée par la promo, RECALCULÉE après décisions : moins d'étudiants au total → chacun en porte plus (dilution).</t>
+      </text>
+    </comment>
+    <comment ref="P5" authorId="0" shapeId="0">
+      <text>
+        <t>Contribution après − structure allouée. Vue INFORMATIVE — surtout PAS un critère de fermeture.</t>
+      </text>
+    </comment>
+    <comment ref="Q5" authorId="0" shapeId="0">
+      <text>
+        <t>Impact sur l'EBITDA groupe = contribution après − contribution avant.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Levier testé et son incrément.</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Effet € sur l'EBITDA d'un pas du levier (approximation vivante).</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Interprétation.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment13.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Indicateur de pilotage.</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeur budgétée.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeur réelle de l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Variation Budget vs N-1.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="C3" authorId="0" shapeId="0">
+      <text>
+        <t>Scénario actif : change cette cellule et TOUT le budget se recalcule.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeurs du scénario Cadrage (central).</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeurs du scénario Optimiste.</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeurs du scénario Prudent.</t>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeur ACTIVE = celle du scénario sélectionné en C3.</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Croissance du budget d'acquisition → pilote le volume via l'élasticité mesurée.</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>Hausse tarifaire moyenne, modulée par marque (coeff prix).</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>Points de conversion candidature→inscrit gagnés (pilotage admissions).</t>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>Part des contrats d'alternance sécurisés dans les 3 mois → financement OPCO à 100 %.</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>Amélioration du taux de passage (réinscription) vs l'historique.</t>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>Inflation appliquée aux charges (pédago, loyers, autres).</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Revalorisation des rémunérations chargées (permanents + enseignement).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Coefficient appliqué à l'effort marketing du cadrage pour cette marque (&gt;1 = on pousse).</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Coefficient appliqué à la hausse tarifaire du cadrage pour cette marque.</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Lecture du positionnement (pousser / défendre / maintenir).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Campus (ville). Une entité = Marque + Ville.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Domaine d'activité de la marque.</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Année d'études (B1, B2, B3, M1, M2…).</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Devise de reporting.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="A3" authorId="0" shapeId="0">
+      <text>
+        <t>Clé technique 'programme|année' pour relier les paramètres au moteur.</t>
+      </text>
+    </comment>
+    <comment ref="B3" authorId="0" shapeId="0">
+      <text>
+        <t>Programme de formation (ex. Bachelor Management).</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="0" shapeId="0">
+      <text>
+        <t>Année d'études : B1/B2/B3 (Bachelor), M1/M2 (Mastère), 1/2 (BTS).</t>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="0" shapeId="0">
+      <text>
+        <t>Modalité : INIT = initial · ALT = alternance (financée OPCO/NPEC).</t>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="0" shapeId="0">
+      <text>
+        <t>Capacité cible d'une classe (nb d'étudiants).</t>
+      </text>
+    </comment>
+    <comment ref="G3" authorId="0" shapeId="0">
+      <text>
+        <t>Coût horaire chargé de l'enseignement (vacation), en €.</t>
+      </text>
+    </comment>
+    <comment ref="I3" authorId="0" shapeId="0">
+      <text>
+        <t>Coût d'acquisition variable (achat de leads) par nouvel inscrit. N'existe qu'en année d'entrée.</t>
+      </text>
+    </comment>
+    <comment ref="J3" authorId="0" shapeId="0">
+      <text>
+        <t>Taux de progression de l'année inférieure vers celle-ci (réinscription). Vide en année d'entrée.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="A3" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="B3" authorId="0" shapeId="0">
+      <text>
+        <t>Campus (ville). Une entité = Marque + Ville.</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="0" shapeId="0">
+      <text>
+        <t>Programme de formation (ex. Bachelor Management).</t>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="0" shapeId="0">
+      <text>
+        <t>Type de diplôme : BAC (Bachelor), MAST (Mastère), BTS.</t>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="0" shapeId="0">
+      <text>
+        <t>Année d'études : B1/B2/B3 (Bachelor), M1/M2 (Mastère), 1/2 (BTS).</t>
+      </text>
+    </comment>
+    <comment ref="F3" authorId="0" shapeId="0">
+      <text>
+        <t>Modalité : INIT = initial · ALT = alternance (financée OPCO/NPEC).</t>
+      </text>
+    </comment>
+    <comment ref="G3" authorId="0" shapeId="0">
+      <text>
+        <t>1 = année d'entrée (on recrute) · 0 = année de poursuite (cohorte progressée).</t>
+      </text>
+    </comment>
+    <comment ref="H3" authorId="0" shapeId="0">
+      <text>
+        <t>Candidatures l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="I3" authorId="0" shapeId="0">
+      <text>
+        <t>Nouveaux inscrits l'an dernier (entrants).</t>
+      </text>
+    </comment>
+    <comment ref="J3" authorId="0" shapeId="0">
+      <text>
+        <t>Réinscrits l'an dernier (étudiants qui poursuivent).</t>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif réel l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="L3" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif de l'année juste inférieure l'an dernier — base de la cohorte pour calculer la progression.</t>
+      </text>
+    </comment>
+    <comment ref="M3" authorId="0" shapeId="0">
+      <text>
+        <t>Tarif moyen l'an dernier (€/étudiant/an).</t>
+      </text>
+    </comment>
+    <comment ref="N3" authorId="0" shapeId="0">
+      <text>
+        <t>Nombre de classes l'an dernier.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="A3" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="B3" authorId="0" shapeId="0">
+      <text>
+        <t>Campus (ville). Une entité = Marque + Ville.</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif réel l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="0" shapeId="0">
+      <text>
+        <t>Chiffre d'affaires réel l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="E3" authorId="0" shapeId="0">
+      <text>
+        <t>Marge de contribution réelle l'an dernier (CA − coûts directs).</t>
+      </text>
+    </comment>
+    <comment ref="F3" authorId="0" shapeId="0">
+      <text>
+        <t>Loyer du campus l'an dernier (coût de structure, fixe).</t>
+      </text>
+    </comment>
+    <comment ref="G3" authorId="0" shapeId="0">
+      <text>
+        <t>Effectifs permanents (équivalent temps plein) du campus.</t>
+      </text>
+    </comment>
+    <comment ref="H3" authorId="0" shapeId="0">
+      <text>
+        <t>Masse salariale permanente = ETP × coût chargé par ETP.</t>
+      </text>
+    </comment>
+    <comment ref="I3" authorId="0" shapeId="0">
+      <text>
+        <t>Dotations aux amortissements l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="J3" authorId="0" shapeId="0">
+      <text>
+        <t>Surface du campus (utilisée comme driver d'allocation possible).</t>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="0" shapeId="0">
+      <text>
+        <t>EBITDA du campus = contribution − loyer − masse salariale permanente.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>Campus (ville). Une entité = Marque + Ville.</t>
+      </text>
+    </comment>
+    <comment ref="C2" authorId="0" shapeId="0">
+      <text>
+        <t>Programme de formation (ex. Bachelor Management).</t>
+      </text>
+    </comment>
+    <comment ref="D2" authorId="0" shapeId="0">
+      <text>
+        <t>Année d'études : B1/B2/B3 (Bachelor), M1/M2 (Mastère), 1/2 (BTS).</t>
+      </text>
+    </comment>
+    <comment ref="E2" authorId="0" shapeId="0">
+      <text>
+        <t>Modalité : INIT = initial (payé par la famille) · ALT = alternance (financé OPCO/NPEC).</t>
+      </text>
+    </comment>
+    <comment ref="F2" authorId="0" shapeId="0">
+      <text>
+        <t>1 = année d'entrée (on recrute) · 0 = année de poursuite (cohorte progressée).</t>
+      </text>
+    </comment>
+    <comment ref="G2" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif réel l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="0" shapeId="0">
+      <text>
+        <t>Nouveaux inscrits l'an dernier (entrants).</t>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="0" shapeId="0">
+      <text>
+        <t>Réinscrits l'an dernier (étudiants qui poursuivent).</t>
+      </text>
+    </comment>
+    <comment ref="J2" authorId="0" shapeId="0">
+      <text>
+        <t>Candidatures l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="K2" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif de l'année inférieure l'an dernier (base de progression de la cohorte).</t>
+      </text>
+    </comment>
+    <comment ref="L2" authorId="0" shapeId="0">
+      <text>
+        <t>Tarif moyen l'an dernier (€/étudiant/an).</t>
+      </text>
+    </comment>
+    <comment ref="M2" authorId="0" shapeId="0">
+      <text>
+        <t>Nombre de classes l'an dernier.</t>
+      </text>
+    </comment>
+    <comment ref="N2" authorId="0" shapeId="0">
+      <text>
+        <t>Clé programme|année pour retrouver les paramètres (feuille 05).</t>
+      </text>
+    </comment>
+    <comment ref="O2" authorId="0" shapeId="0">
+      <text>
+        <t>Capacité cible par classe (lue dans 05).</t>
+      </text>
+    </comment>
+    <comment ref="P2" authorId="0" shapeId="0">
+      <text>
+        <t>Heures d'enseignement par classe/an (05).</t>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="0" shapeId="0">
+      <text>
+        <t>Taux horaire chargé de l'enseignement (05).</t>
+      </text>
+    </comment>
+    <comment ref="R2" authorId="0" shapeId="0">
+      <text>
+        <t>Coût pédagogique par étudiant (05).</t>
+      </text>
+    </comment>
+    <comment ref="S2" authorId="0" shapeId="0">
+      <text>
+        <t>Coût d'acquisition variable par nouvel inscrit (05).</t>
+      </text>
+    </comment>
+    <comment ref="T2" authorId="0" shapeId="0">
+      <text>
+        <t>Taux de passage de l'année inférieure (05). 0 en année d'entrée.</t>
+      </text>
+    </comment>
+    <comment ref="U2" authorId="0" shapeId="0">
+      <text>
+        <t>Coût d'une classe = heures × taux horaire × (1 + politique salariale).</t>
+      </text>
+    </comment>
+    <comment ref="V2" authorId="0" shapeId="0">
+      <text>
+        <t>Coefficient stratégique MARKETING de la marque (feuille 03) — module l'effort par marque.</t>
+      </text>
+    </comment>
+    <comment ref="W2" authorId="0" shapeId="0">
+      <text>
+        <t>Coefficient stratégique PRIX de la marque (feuille 03) — module la hausse tarifaire par marque.</t>
+      </text>
+    </comment>
+    <comment ref="X2" authorId="0" shapeId="0">
+      <text>
+        <t>Élasticité marketing mesurée (06). Repli si historique manquant.</t>
+      </text>
+    </comment>
+    <comment ref="Y2" authorId="0" shapeId="0">
+      <text>
+        <t>Effort marketing appliqué = levier 'variation budget marketing' × coefficient marque.</t>
+      </text>
+    </comment>
+    <comment ref="Z2" authorId="0" shapeId="0">
+      <text>
+        <t>Candidatures budget = candidatures N-1 × (1 + élasticité × effort marketing).</t>
+      </text>
+    </comment>
+    <comment ref="AA2" authorId="0" shapeId="0">
+      <text>
+        <t>Taux de conversion candidature→inscrit (mesuré par cellule) + gain du levier conversion.</t>
+      </text>
+    </comment>
+    <comment ref="AB2" authorId="0" shapeId="0">
+      <text>
+        <t>Nouveaux inscrits budget = candidatures budget × taux de conversion.</t>
+      </text>
+    </comment>
+    <comment ref="AC2" authorId="0" shapeId="0">
+      <text>
+        <t>Réinscrits budget = effectif de l'année inférieure (N-1) × (taux de passage + amélioration).</t>
+      </text>
+    </comment>
+    <comment ref="AD2" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif budget = nouveaux + réinscrits.</t>
+      </text>
+    </comment>
+    <comment ref="AE2" authorId="0" shapeId="0">
+      <text>
+        <t>Tarif budget = tarif N-1 × (1 + hausse prix × coefficient marque).</t>
+      </text>
+    </comment>
+    <comment ref="AF2" authorId="0" shapeId="0">
+      <text>
+        <t>Facteur de financement alternance BUDGET (sécurisation + reste à charge recouvré). = 1 en initial.</t>
+      </text>
+    </comment>
+    <comment ref="AG2" authorId="0" shapeId="0">
+      <text>
+        <t>Facteur de financement alternance N-1 (référence pour le pont).</t>
+      </text>
+    </comment>
+    <comment ref="AH2" authorId="0" shapeId="0">
+      <text>
+        <t>CA budget = effectif × tarif × facteur financement + frais de dossier.</t>
+      </text>
+    </comment>
+    <comment ref="AI2" authorId="0" shapeId="0">
+      <text>
+        <t>Classes nécessaires = arrondi supérieur (effectif / capacité).</t>
+      </text>
+    </comment>
+    <comment ref="AJ2" authorId="0" shapeId="0">
+      <text>
+        <t>Coût d'enseignement = classes × coût par classe.</t>
+      </text>
+    </comment>
+    <comment ref="AK2" authorId="0" shapeId="0">
+      <text>
+        <t>Coût pédagogique = effectif × coût pédago/étudiant × (1 + inflation).</t>
+      </text>
+    </comment>
+    <comment ref="AL2" authorId="0" shapeId="0">
+      <text>
+        <t>Marketing = nouveaux × CAC variable × (1 + effort). = 0 en année de poursuite.</t>
+      </text>
+    </comment>
+    <comment ref="AM2" authorId="0" shapeId="0">
+      <text>
+        <t>MARGE DE CONTRIBUTION = CA − enseignement − pédago − marketing − autres charges.</t>
+      </text>
+    </comment>
+    <comment ref="AN2" authorId="0" shapeId="0">
+      <text>
+        <t>Taux de remplissage = effectif / (classes × capacité).</t>
+      </text>
+    </comment>
+    <comment ref="AO2" authorId="0" shapeId="0">
+      <text>
+        <t>Contribution par étudiant.</t>
+      </text>
+    </comment>
+    <comment ref="AP2" authorId="0" shapeId="0">
+      <text>
+        <t>Point mort = nb d'étudiants pour couvrir le coût des classes.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Campus (ville). Une entité = Marque + Ville.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Marge de contribution (CA − coûts directs évitables).</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Loyer du campus (structure fixe).</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Masse salariale permanente (structure fixe).</t>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeur du driver d'allocation (effectif, CA ou m² selon 02_Leviers).</t>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0">
+      <text>
+        <t>Part du campus dans le driver total.</t>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0">
+      <text>
+        <t>Frais de structure groupe alloués à ce campus.</t>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0">
+      <text>
+        <t>EBITDA du campus = contribution − loyer − permanents − structure allouée.</t>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="0" shapeId="0">
+      <text>
+        <t>Dotations aux amortissements.</t>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0">
+      <text>
+        <t>Résultat d'exploitation = EBITDA − D&amp;A.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1077,7 +1907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L20"/>
+  <dimension ref="A2:AS20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1907,6 +2737,7 @@
     <mergeCell ref="H3:I3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1916,7 +2747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F25"/>
+  <dimension ref="A2:AS25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2321,6 +3152,7 @@
     <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2330,7 +3162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q63"/>
+  <dimension ref="A1:AS63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6667,6 +7499,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -6676,7 +7509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D11"/>
+  <dimension ref="A2:AS11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6798,6 +7631,7 @@
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -6807,7 +7641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E15"/>
+  <dimension ref="A2:AS15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7052,6 +7886,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -7061,7 +7896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D14"/>
+  <dimension ref="A2:AS14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7271,7 +8106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E14"/>
+  <dimension ref="A2:AS14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7400,6 +8235,7 @@
     <mergeCell ref="B12:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -7919,6 +8755,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -7928,7 +8765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E10"/>
+  <dimension ref="A2:AS10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8065,6 +8902,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -8074,7 +8912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F32"/>
+  <dimension ref="A2:AS32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8823,6 +9661,7 @@
     <mergeCell ref="B22:F22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -8832,7 +9671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:AS23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9703,6 +10542,7 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -9712,7 +10552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:AS73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -13316,6 +14156,7 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -13325,7 +14166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:AS18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -14032,6 +14873,7 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -14041,7 +14883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP61"/>
+  <dimension ref="A1:AS61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -24247,5 +25089,6 @@
     <mergeCell ref="A1:AP1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CACvar : affiché uniquement en année d'entrée (0 en poursuite)
Le CAC variable (achat de leads) ne concerne que le recrutement, donc les années
d'entrée (B1/M1/BTS1). Auparavant la valeur s'affichait aussi sur les années de
poursuite (où nouveaux=0 -> coût 0, mais affichage trompeur). Désormais 0/'-' en
poursuite. Valeurs (320 Bachelor...) illustratives = part variable du CAC total
(~0,8-2k), le reste étant en marketing central fixe.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -9824,7 +9824,7 @@
         <v>400</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J5" s="25" t="n">
         <v>0.85</v>
@@ -9864,7 +9864,7 @@
         <v>400</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J6" s="25" t="n">
         <v>0.9</v>
@@ -9942,7 +9942,7 @@
         <v>520</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="J8" s="25" t="n">
         <v>0.92</v>
@@ -10020,7 +10020,7 @@
         <v>550</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J10" s="25" t="n">
         <v>0.85</v>
@@ -10060,7 +10060,7 @@
         <v>550</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J11" s="25" t="n">
         <v>0.9</v>
@@ -10138,7 +10138,7 @@
         <v>670</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="J13" s="25" t="n">
         <v>0.92</v>
@@ -10216,7 +10216,7 @@
         <v>380</v>
       </c>
       <c r="I15" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J15" s="25" t="n">
         <v>0.85</v>
@@ -10256,7 +10256,7 @@
         <v>380</v>
       </c>
       <c r="I16" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J16" s="25" t="n">
         <v>0.9</v>
@@ -10334,7 +10334,7 @@
         <v>350</v>
       </c>
       <c r="I18" s="28" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J18" s="25" t="n">
         <v>0.9</v>
@@ -10412,7 +10412,7 @@
         <v>380</v>
       </c>
       <c r="I20" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J20" s="25" t="n">
         <v>0.9</v>
@@ -10490,7 +10490,7 @@
         <v>450</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J22" s="25" t="n">
         <v>0.85</v>
@@ -10530,7 +10530,7 @@
         <v>450</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="J23" s="25" t="n">
         <v>0.9</v>

</xml_diff>

<commit_message>
Calibre la structure de coûts sur les comptes consolidés (personnel 46%)
Réduit le ratio d'ETP permanents (eff/28+2 -> eff/30+1) et relève les
autres charges d'exploitation (380 -> 934 €/étudiant) pour aligner la
répartition du P&L sur le réel EDUSERVICES 4.0 : personnel 45,5% (vs 46%),
achats/autres+pédago 16,9%, loyers 11%, D&A 6%, EBITDA 14,6%,
CA/étudiant 8 276 €. 0 erreur de formule.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -8632,7 +8632,7 @@
         </is>
       </c>
       <c r="D19" s="28" t="n">
-        <v>380</v>
+        <v>934</v>
       </c>
       <c r="E19" s="29" t="inlineStr">
         <is>
@@ -14264,13 +14264,13 @@
         <v>2467250</v>
       </c>
       <c r="E4" s="41" t="n">
-        <v>1785470</v>
+        <v>1624256</v>
       </c>
       <c r="F4" s="41" t="n">
         <v>271000</v>
       </c>
       <c r="G4" s="39" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H4" s="17">
         <f>G4*'02_Leviers'!$D$15</f>
@@ -14305,13 +14305,13 @@
         <v>2102540</v>
       </c>
       <c r="E5" s="41" t="n">
-        <v>1531180</v>
+        <v>1393788</v>
       </c>
       <c r="F5" s="41" t="n">
         <v>231000</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H5" s="17">
         <f>G5*'02_Leviers'!$D$15</f>
@@ -14346,13 +14346,13 @@
         <v>1898640</v>
       </c>
       <c r="E6" s="41" t="n">
-        <v>1351280</v>
+        <v>1227184</v>
       </c>
       <c r="F6" s="41" t="n">
         <v>209000</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H6" s="17">
         <f>G6*'02_Leviers'!$D$15</f>
@@ -14387,13 +14387,13 @@
         <v>1619880</v>
       </c>
       <c r="E7" s="41" t="n">
-        <v>1105220</v>
+        <v>999406</v>
       </c>
       <c r="F7" s="41" t="n">
         <v>178000</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H7" s="17">
         <f>G7*'02_Leviers'!$D$15</f>
@@ -14428,13 +14428,13 @@
         <v>2280350</v>
       </c>
       <c r="E8" s="41" t="n">
-        <v>1589820</v>
+        <v>1440794</v>
       </c>
       <c r="F8" s="41" t="n">
         <v>251000</v>
       </c>
       <c r="G8" s="39" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H8" s="17">
         <f>G8*'02_Leviers'!$D$15</f>
@@ -14469,13 +14469,13 @@
         <v>1585200</v>
       </c>
       <c r="E9" s="41" t="n">
-        <v>1025970</v>
+        <v>922372</v>
       </c>
       <c r="F9" s="41" t="n">
         <v>174000</v>
       </c>
       <c r="G9" s="39" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H9" s="17">
         <f>G9*'02_Leviers'!$D$15</f>
@@ -14510,13 +14510,13 @@
         <v>1483250</v>
       </c>
       <c r="E10" s="41" t="n">
-        <v>937820</v>
+        <v>840870</v>
       </c>
       <c r="F10" s="41" t="n">
         <v>163000</v>
       </c>
       <c r="G10" s="39" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H10" s="17">
         <f>G10*'02_Leviers'!$D$15</f>
@@ -14551,13 +14551,13 @@
         <v>1044500</v>
       </c>
       <c r="E11" s="41" t="n">
-        <v>734820</v>
+        <v>662800</v>
       </c>
       <c r="F11" s="41" t="n">
         <v>115000</v>
       </c>
       <c r="G11" s="39" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H11" s="17">
         <f>G11*'02_Leviers'!$D$15</f>
@@ -14592,13 +14592,13 @@
         <v>835600</v>
       </c>
       <c r="E12" s="41" t="n">
-        <v>579040</v>
+        <v>521424</v>
       </c>
       <c r="F12" s="41" t="n">
         <v>92000</v>
       </c>
       <c r="G12" s="39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H12" s="17">
         <f>G12*'02_Leviers'!$D$15</f>
@@ -14633,13 +14633,13 @@
         <v>835600</v>
       </c>
       <c r="E13" s="41" t="n">
-        <v>579040</v>
+        <v>521424</v>
       </c>
       <c r="F13" s="41" t="n">
         <v>92000</v>
       </c>
       <c r="G13" s="39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H13" s="17">
         <f>G13*'02_Leviers'!$D$15</f>
@@ -14674,13 +14674,13 @@
         <v>1130470</v>
       </c>
       <c r="E14" s="41" t="n">
-        <v>711410</v>
+        <v>628864</v>
       </c>
       <c r="F14" s="41" t="n">
         <v>124000</v>
       </c>
       <c r="G14" s="39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H14" s="17">
         <f>G14*'02_Leviers'!$D$15</f>
@@ -14715,13 +14715,13 @@
         <v>887850</v>
       </c>
       <c r="E15" s="41" t="n">
-        <v>605020</v>
+        <v>540202</v>
       </c>
       <c r="F15" s="41" t="n">
         <v>98000</v>
       </c>
       <c r="G15" s="39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H15" s="17">
         <f>G15*'02_Leviers'!$D$15</f>
@@ -14756,13 +14756,13 @@
         <v>980230</v>
       </c>
       <c r="E16" s="41" t="n">
-        <v>675770</v>
+        <v>608182</v>
       </c>
       <c r="F16" s="41" t="n">
         <v>108000</v>
       </c>
       <c r="G16" s="39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H16" s="17">
         <f>G16*'02_Leviers'!$D$15</f>
@@ -14797,13 +14797,13 @@
         <v>835600</v>
       </c>
       <c r="E17" s="41" t="n">
-        <v>577440</v>
+        <v>519824</v>
       </c>
       <c r="F17" s="41" t="n">
         <v>92000</v>
       </c>
       <c r="G17" s="39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H17" s="17">
         <f>G17*'02_Leviers'!$D$15</f>

</xml_diff>

<commit_message>
Simulateur : le regroupement (-1 classe) vérifie la capacité des classes restantes
Avant, "Regrouper (-1 classe)" créditait toujours l'économie d'une classe dès
2 classes, sans vérifier que les étudiants tiennent dans les classes restantes
— or le moteur dimensionne déjà au minimum (arrondi sup. effectif/capacité),
donc l'économie était systématiquement optimiste.

Désormais l'économie n'est créditée que si effectif <= (classes-1) x capacité
x 1,10 (tolérance salle +10%). Sinon aucune économie et la reco affiche
"infaisable : capacité". Le remplissage après regroupement est montré dans le
motif. Résultat sur les données : 6 promos regroupables, 24 infaisables.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -625,7 +625,7 @@
     </comment>
     <comment ref="N5" authorId="0" shapeId="0">
       <text>
-        <t>Contribution recalculée selon ta décision.</t>
+        <t>Contribution recalculée selon ta décision. Regrouper (−1 classe) n'est crédité (économie d'une classe) QUE si l'effectif tient dans les classes restantes : effectif ≤ (classes−1) × capacité × 1,10 (tolérance salle +10%). Sinon aucune économie : le regroupement déborderait la capacité.</t>
       </text>
     </comment>
     <comment ref="O5" authorId="0" shapeId="0">
@@ -3412,7 +3412,7 @@
         <v/>
       </c>
       <c r="N6" s="17">
-        <f>IF(L6="Ne pas lancer",0,IF(L6="Ouvrir +1 classe",H6+'08_Moteur'!O3*('08_Moteur'!AE3*'08_Moteur'!AF3-('08_Moteur'!R3+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S3)-'08_Moteur'!U3,IF(L6="Regrouper (-1 classe)",H6+('08_Moteur'!AI3-MAX(1,'08_Moteur'!AI3-1))*'08_Moteur'!U3,H6)))</f>
+        <f>IF(L6="Ne pas lancer",0,IF(L6="Ouvrir +1 classe",H6+'08_Moteur'!O3*('08_Moteur'!AE3*'08_Moteur'!AF3-('08_Moteur'!R3+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S3)-'08_Moteur'!U3,IF(L6="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI3&gt;=2,E6&lt;=('08_Moteur'!AI3-1)*'08_Moteur'!O3*1.1),H6+'08_Moteur'!U3,H6),H6)))</f>
         <v/>
       </c>
       <c r="O6" s="17">
@@ -3466,11 +3466,11 @@
         <v/>
       </c>
       <c r="J7" s="70">
-        <f>IF(H7&lt;0,"🔴 Restructurer (mutualiser)",IF(I7&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H7&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI4&gt;=2,E7&lt;=('08_Moteur'!AI4-1)*'08_Moteur'!O4*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I7&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K7" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI4&gt;=2,TEXT(IFERROR(E7/(('08_Moteur'!AI4-1)*'08_Moteur'!O4),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L7" s="21" t="inlineStr">
@@ -3483,7 +3483,7 @@
         <v/>
       </c>
       <c r="N7" s="17">
-        <f>IF(L7="Ne pas lancer",0,IF(L7="Ouvrir +1 classe",H7+'08_Moteur'!O4*('08_Moteur'!AE4*'08_Moteur'!AF4-('08_Moteur'!R4+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S4)-'08_Moteur'!U4,IF(L7="Regrouper (-1 classe)",H7+('08_Moteur'!AI4-MAX(1,'08_Moteur'!AI4-1))*'08_Moteur'!U4,H7)))</f>
+        <f>IF(L7="Ne pas lancer",0,IF(L7="Ouvrir +1 classe",H7+'08_Moteur'!O4*('08_Moteur'!AE4*'08_Moteur'!AF4-('08_Moteur'!R4+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S4)-'08_Moteur'!U4,IF(L7="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI4&gt;=2,E7&lt;=('08_Moteur'!AI4-1)*'08_Moteur'!O4*1.1),H7+'08_Moteur'!U4,H7),H7)))</f>
         <v/>
       </c>
       <c r="O7" s="17">
@@ -3537,11 +3537,11 @@
         <v/>
       </c>
       <c r="J8" s="70">
-        <f>IF(H8&lt;0,"🔴 Restructurer (mutualiser)",IF(I8&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H8&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI5&gt;=2,E8&lt;=('08_Moteur'!AI5-1)*'08_Moteur'!O5*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I8&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K8" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI5&gt;=2,TEXT(IFERROR(E8/(('08_Moteur'!AI5-1)*'08_Moteur'!O5),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L8" s="21" t="inlineStr">
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="N8" s="17">
-        <f>IF(L8="Ne pas lancer",0,IF(L8="Ouvrir +1 classe",H8+'08_Moteur'!O5*('08_Moteur'!AE5*'08_Moteur'!AF5-('08_Moteur'!R5+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S5)-'08_Moteur'!U5,IF(L8="Regrouper (-1 classe)",H8+('08_Moteur'!AI5-MAX(1,'08_Moteur'!AI5-1))*'08_Moteur'!U5,H8)))</f>
+        <f>IF(L8="Ne pas lancer",0,IF(L8="Ouvrir +1 classe",H8+'08_Moteur'!O5*('08_Moteur'!AE5*'08_Moteur'!AF5-('08_Moteur'!R5+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S5)-'08_Moteur'!U5,IF(L8="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI5&gt;=2,E8&lt;=('08_Moteur'!AI5-1)*'08_Moteur'!O5*1.1),H8+'08_Moteur'!U5,H8),H8)))</f>
         <v/>
       </c>
       <c r="O8" s="17">
@@ -3625,7 +3625,7 @@
         <v/>
       </c>
       <c r="N9" s="17">
-        <f>IF(L9="Ne pas lancer",0,IF(L9="Ouvrir +1 classe",H9+'08_Moteur'!O6*('08_Moteur'!AE6*'08_Moteur'!AF6-('08_Moteur'!R6+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S6)-'08_Moteur'!U6,IF(L9="Regrouper (-1 classe)",H9+('08_Moteur'!AI6-MAX(1,'08_Moteur'!AI6-1))*'08_Moteur'!U6,H9)))</f>
+        <f>IF(L9="Ne pas lancer",0,IF(L9="Ouvrir +1 classe",H9+'08_Moteur'!O6*('08_Moteur'!AE6*'08_Moteur'!AF6-('08_Moteur'!R6+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S6)-'08_Moteur'!U6,IF(L9="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI6&gt;=2,E9&lt;=('08_Moteur'!AI6-1)*'08_Moteur'!O6*1.1),H9+'08_Moteur'!U6,H9),H9)))</f>
         <v/>
       </c>
       <c r="O9" s="17">
@@ -3679,11 +3679,11 @@
         <v/>
       </c>
       <c r="J10" s="70">
-        <f>IF(H10&lt;0,"🔴 Restructurer (mutualiser)",IF(I10&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H10&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI7&gt;=2,E10&lt;=('08_Moteur'!AI7-1)*'08_Moteur'!O7*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I10&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K10" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI7&gt;=2,TEXT(IFERROR(E10/(('08_Moteur'!AI7-1)*'08_Moteur'!O7),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L10" s="21" t="inlineStr">
@@ -3696,7 +3696,7 @@
         <v/>
       </c>
       <c r="N10" s="17">
-        <f>IF(L10="Ne pas lancer",0,IF(L10="Ouvrir +1 classe",H10+'08_Moteur'!O7*('08_Moteur'!AE7*'08_Moteur'!AF7-('08_Moteur'!R7+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S7)-'08_Moteur'!U7,IF(L10="Regrouper (-1 classe)",H10+('08_Moteur'!AI7-MAX(1,'08_Moteur'!AI7-1))*'08_Moteur'!U7,H10)))</f>
+        <f>IF(L10="Ne pas lancer",0,IF(L10="Ouvrir +1 classe",H10+'08_Moteur'!O7*('08_Moteur'!AE7*'08_Moteur'!AF7-('08_Moteur'!R7+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S7)-'08_Moteur'!U7,IF(L10="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI7&gt;=2,E10&lt;=('08_Moteur'!AI7-1)*'08_Moteur'!O7*1.1),H10+'08_Moteur'!U7,H10),H10)))</f>
         <v/>
       </c>
       <c r="O10" s="17">
@@ -3767,7 +3767,7 @@
         <v/>
       </c>
       <c r="N11" s="17">
-        <f>IF(L11="Ne pas lancer",0,IF(L11="Ouvrir +1 classe",H11+'08_Moteur'!O8*('08_Moteur'!AE8*'08_Moteur'!AF8-('08_Moteur'!R8+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S8)-'08_Moteur'!U8,IF(L11="Regrouper (-1 classe)",H11+('08_Moteur'!AI8-MAX(1,'08_Moteur'!AI8-1))*'08_Moteur'!U8,H11)))</f>
+        <f>IF(L11="Ne pas lancer",0,IF(L11="Ouvrir +1 classe",H11+'08_Moteur'!O8*('08_Moteur'!AE8*'08_Moteur'!AF8-('08_Moteur'!R8+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S8)-'08_Moteur'!U8,IF(L11="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI8&gt;=2,E11&lt;=('08_Moteur'!AI8-1)*'08_Moteur'!O8*1.1),H11+'08_Moteur'!U8,H11),H11)))</f>
         <v/>
       </c>
       <c r="O11" s="17">
@@ -3821,11 +3821,11 @@
         <v/>
       </c>
       <c r="J12" s="70">
-        <f>IF(H12&lt;0,"🔴 Restructurer (mutualiser)",IF(I12&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H12&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI9&gt;=2,E12&lt;=('08_Moteur'!AI9-1)*'08_Moteur'!O9*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I12&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K12" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI9&gt;=2,TEXT(IFERROR(E12/(('08_Moteur'!AI9-1)*'08_Moteur'!O9),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L12" s="21" t="inlineStr">
@@ -3838,7 +3838,7 @@
         <v/>
       </c>
       <c r="N12" s="17">
-        <f>IF(L12="Ne pas lancer",0,IF(L12="Ouvrir +1 classe",H12+'08_Moteur'!O9*('08_Moteur'!AE9*'08_Moteur'!AF9-('08_Moteur'!R9+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S9)-'08_Moteur'!U9,IF(L12="Regrouper (-1 classe)",H12+('08_Moteur'!AI9-MAX(1,'08_Moteur'!AI9-1))*'08_Moteur'!U9,H12)))</f>
+        <f>IF(L12="Ne pas lancer",0,IF(L12="Ouvrir +1 classe",H12+'08_Moteur'!O9*('08_Moteur'!AE9*'08_Moteur'!AF9-('08_Moteur'!R9+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S9)-'08_Moteur'!U9,IF(L12="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI9&gt;=2,E12&lt;=('08_Moteur'!AI9-1)*'08_Moteur'!O9*1.1),H12+'08_Moteur'!U9,H12),H12)))</f>
         <v/>
       </c>
       <c r="O12" s="17">
@@ -3892,11 +3892,11 @@
         <v/>
       </c>
       <c r="J13" s="70">
-        <f>IF(H13&lt;0,"🔴 Restructurer (mutualiser)",IF(I13&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H13&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI10&gt;=2,E13&lt;=('08_Moteur'!AI10-1)*'08_Moteur'!O10*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I13&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K13" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI10&gt;=2,TEXT(IFERROR(E13/(('08_Moteur'!AI10-1)*'08_Moteur'!O10),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L13" s="21" t="inlineStr">
@@ -3909,7 +3909,7 @@
         <v/>
       </c>
       <c r="N13" s="17">
-        <f>IF(L13="Ne pas lancer",0,IF(L13="Ouvrir +1 classe",H13+'08_Moteur'!O10*('08_Moteur'!AE10*'08_Moteur'!AF10-('08_Moteur'!R10+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S10)-'08_Moteur'!U10,IF(L13="Regrouper (-1 classe)",H13+('08_Moteur'!AI10-MAX(1,'08_Moteur'!AI10-1))*'08_Moteur'!U10,H13)))</f>
+        <f>IF(L13="Ne pas lancer",0,IF(L13="Ouvrir +1 classe",H13+'08_Moteur'!O10*('08_Moteur'!AE10*'08_Moteur'!AF10-('08_Moteur'!R10+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S10)-'08_Moteur'!U10,IF(L13="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI10&gt;=2,E13&lt;=('08_Moteur'!AI10-1)*'08_Moteur'!O10*1.1),H13+'08_Moteur'!U10,H13),H13)))</f>
         <v/>
       </c>
       <c r="O13" s="17">
@@ -3980,7 +3980,7 @@
         <v/>
       </c>
       <c r="N14" s="17">
-        <f>IF(L14="Ne pas lancer",0,IF(L14="Ouvrir +1 classe",H14+'08_Moteur'!O11*('08_Moteur'!AE11*'08_Moteur'!AF11-('08_Moteur'!R11+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S11)-'08_Moteur'!U11,IF(L14="Regrouper (-1 classe)",H14+('08_Moteur'!AI11-MAX(1,'08_Moteur'!AI11-1))*'08_Moteur'!U11,H14)))</f>
+        <f>IF(L14="Ne pas lancer",0,IF(L14="Ouvrir +1 classe",H14+'08_Moteur'!O11*('08_Moteur'!AE11*'08_Moteur'!AF11-('08_Moteur'!R11+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S11)-'08_Moteur'!U11,IF(L14="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI11&gt;=2,E14&lt;=('08_Moteur'!AI11-1)*'08_Moteur'!O11*1.1),H14+'08_Moteur'!U11,H14),H14)))</f>
         <v/>
       </c>
       <c r="O14" s="17">
@@ -4034,11 +4034,11 @@
         <v/>
       </c>
       <c r="J15" s="70">
-        <f>IF(H15&lt;0,"🔴 Restructurer (mutualiser)",IF(I15&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H15&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI12&gt;=2,E15&lt;=('08_Moteur'!AI12-1)*'08_Moteur'!O12*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I15&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K15" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI12&gt;=2,TEXT(IFERROR(E15/(('08_Moteur'!AI12-1)*'08_Moteur'!O12),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L15" s="21" t="inlineStr">
@@ -4051,7 +4051,7 @@
         <v/>
       </c>
       <c r="N15" s="17">
-        <f>IF(L15="Ne pas lancer",0,IF(L15="Ouvrir +1 classe",H15+'08_Moteur'!O12*('08_Moteur'!AE12*'08_Moteur'!AF12-('08_Moteur'!R12+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S12)-'08_Moteur'!U12,IF(L15="Regrouper (-1 classe)",H15+('08_Moteur'!AI12-MAX(1,'08_Moteur'!AI12-1))*'08_Moteur'!U12,H15)))</f>
+        <f>IF(L15="Ne pas lancer",0,IF(L15="Ouvrir +1 classe",H15+'08_Moteur'!O12*('08_Moteur'!AE12*'08_Moteur'!AF12-('08_Moteur'!R12+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S12)-'08_Moteur'!U12,IF(L15="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI12&gt;=2,E15&lt;=('08_Moteur'!AI12-1)*'08_Moteur'!O12*1.1),H15+'08_Moteur'!U12,H15),H15)))</f>
         <v/>
       </c>
       <c r="O15" s="17">
@@ -4122,7 +4122,7 @@
         <v/>
       </c>
       <c r="N16" s="17">
-        <f>IF(L16="Ne pas lancer",0,IF(L16="Ouvrir +1 classe",H16+'08_Moteur'!O13*('08_Moteur'!AE13*'08_Moteur'!AF13-('08_Moteur'!R13+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S13)-'08_Moteur'!U13,IF(L16="Regrouper (-1 classe)",H16+('08_Moteur'!AI13-MAX(1,'08_Moteur'!AI13-1))*'08_Moteur'!U13,H16)))</f>
+        <f>IF(L16="Ne pas lancer",0,IF(L16="Ouvrir +1 classe",H16+'08_Moteur'!O13*('08_Moteur'!AE13*'08_Moteur'!AF13-('08_Moteur'!R13+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S13)-'08_Moteur'!U13,IF(L16="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI13&gt;=2,E16&lt;=('08_Moteur'!AI13-1)*'08_Moteur'!O13*1.1),H16+'08_Moteur'!U13,H16),H16)))</f>
         <v/>
       </c>
       <c r="O16" s="17">
@@ -4176,11 +4176,11 @@
         <v/>
       </c>
       <c r="J17" s="70">
-        <f>IF(H17&lt;0,"🔴 Restructurer (mutualiser)",IF(I17&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H17&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI14&gt;=2,E17&lt;=('08_Moteur'!AI14-1)*'08_Moteur'!O14*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I17&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K17" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI14&gt;=2,TEXT(IFERROR(E17/(('08_Moteur'!AI14-1)*'08_Moteur'!O14),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L17" s="21" t="inlineStr">
@@ -4193,7 +4193,7 @@
         <v/>
       </c>
       <c r="N17" s="17">
-        <f>IF(L17="Ne pas lancer",0,IF(L17="Ouvrir +1 classe",H17+'08_Moteur'!O14*('08_Moteur'!AE14*'08_Moteur'!AF14-('08_Moteur'!R14+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S14)-'08_Moteur'!U14,IF(L17="Regrouper (-1 classe)",H17+('08_Moteur'!AI14-MAX(1,'08_Moteur'!AI14-1))*'08_Moteur'!U14,H17)))</f>
+        <f>IF(L17="Ne pas lancer",0,IF(L17="Ouvrir +1 classe",H17+'08_Moteur'!O14*('08_Moteur'!AE14*'08_Moteur'!AF14-('08_Moteur'!R14+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S14)-'08_Moteur'!U14,IF(L17="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI14&gt;=2,E17&lt;=('08_Moteur'!AI14-1)*'08_Moteur'!O14*1.1),H17+'08_Moteur'!U14,H17),H17)))</f>
         <v/>
       </c>
       <c r="O17" s="17">
@@ -4247,11 +4247,11 @@
         <v/>
       </c>
       <c r="J18" s="70">
-        <f>IF(H18&lt;0,"🔴 Restructurer (mutualiser)",IF(I18&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H18&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI15&gt;=2,E18&lt;=('08_Moteur'!AI15-1)*'08_Moteur'!O15*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I18&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K18" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI15&gt;=2,TEXT(IFERROR(E18/(('08_Moteur'!AI15-1)*'08_Moteur'!O15),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L18" s="21" t="inlineStr">
@@ -4264,7 +4264,7 @@
         <v/>
       </c>
       <c r="N18" s="17">
-        <f>IF(L18="Ne pas lancer",0,IF(L18="Ouvrir +1 classe",H18+'08_Moteur'!O15*('08_Moteur'!AE15*'08_Moteur'!AF15-('08_Moteur'!R15+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S15)-'08_Moteur'!U15,IF(L18="Regrouper (-1 classe)",H18+('08_Moteur'!AI15-MAX(1,'08_Moteur'!AI15-1))*'08_Moteur'!U15,H18)))</f>
+        <f>IF(L18="Ne pas lancer",0,IF(L18="Ouvrir +1 classe",H18+'08_Moteur'!O15*('08_Moteur'!AE15*'08_Moteur'!AF15-('08_Moteur'!R15+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S15)-'08_Moteur'!U15,IF(L18="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI15&gt;=2,E18&lt;=('08_Moteur'!AI15-1)*'08_Moteur'!O15*1.1),H18+'08_Moteur'!U15,H18),H18)))</f>
         <v/>
       </c>
       <c r="O18" s="17">
@@ -4335,7 +4335,7 @@
         <v/>
       </c>
       <c r="N19" s="17">
-        <f>IF(L19="Ne pas lancer",0,IF(L19="Ouvrir +1 classe",H19+'08_Moteur'!O16*('08_Moteur'!AE16*'08_Moteur'!AF16-('08_Moteur'!R16+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S16)-'08_Moteur'!U16,IF(L19="Regrouper (-1 classe)",H19+('08_Moteur'!AI16-MAX(1,'08_Moteur'!AI16-1))*'08_Moteur'!U16,H19)))</f>
+        <f>IF(L19="Ne pas lancer",0,IF(L19="Ouvrir +1 classe",H19+'08_Moteur'!O16*('08_Moteur'!AE16*'08_Moteur'!AF16-('08_Moteur'!R16+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S16)-'08_Moteur'!U16,IF(L19="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI16&gt;=2,E19&lt;=('08_Moteur'!AI16-1)*'08_Moteur'!O16*1.1),H19+'08_Moteur'!U16,H19),H19)))</f>
         <v/>
       </c>
       <c r="O19" s="17">
@@ -4389,11 +4389,11 @@
         <v/>
       </c>
       <c r="J20" s="70">
-        <f>IF(H20&lt;0,"🔴 Restructurer (mutualiser)",IF(I20&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H20&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI17&gt;=2,E20&lt;=('08_Moteur'!AI17-1)*'08_Moteur'!O17*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I20&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K20" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI17&gt;=2,TEXT(IFERROR(E20/(('08_Moteur'!AI17-1)*'08_Moteur'!O17),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L20" s="21" t="inlineStr">
@@ -4406,7 +4406,7 @@
         <v/>
       </c>
       <c r="N20" s="17">
-        <f>IF(L20="Ne pas lancer",0,IF(L20="Ouvrir +1 classe",H20+'08_Moteur'!O17*('08_Moteur'!AE17*'08_Moteur'!AF17-('08_Moteur'!R17+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S17)-'08_Moteur'!U17,IF(L20="Regrouper (-1 classe)",H20+('08_Moteur'!AI17-MAX(1,'08_Moteur'!AI17-1))*'08_Moteur'!U17,H20)))</f>
+        <f>IF(L20="Ne pas lancer",0,IF(L20="Ouvrir +1 classe",H20+'08_Moteur'!O17*('08_Moteur'!AE17*'08_Moteur'!AF17-('08_Moteur'!R17+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S17)-'08_Moteur'!U17,IF(L20="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI17&gt;=2,E20&lt;=('08_Moteur'!AI17-1)*'08_Moteur'!O17*1.1),H20+'08_Moteur'!U17,H20),H20)))</f>
         <v/>
       </c>
       <c r="O20" s="17">
@@ -4477,7 +4477,7 @@
         <v/>
       </c>
       <c r="N21" s="17">
-        <f>IF(L21="Ne pas lancer",0,IF(L21="Ouvrir +1 classe",H21+'08_Moteur'!O18*('08_Moteur'!AE18*'08_Moteur'!AF18-('08_Moteur'!R18+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S18)-'08_Moteur'!U18,IF(L21="Regrouper (-1 classe)",H21+('08_Moteur'!AI18-MAX(1,'08_Moteur'!AI18-1))*'08_Moteur'!U18,H21)))</f>
+        <f>IF(L21="Ne pas lancer",0,IF(L21="Ouvrir +1 classe",H21+'08_Moteur'!O18*('08_Moteur'!AE18*'08_Moteur'!AF18-('08_Moteur'!R18+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S18)-'08_Moteur'!U18,IF(L21="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI18&gt;=2,E21&lt;=('08_Moteur'!AI18-1)*'08_Moteur'!O18*1.1),H21+'08_Moteur'!U18,H21),H21)))</f>
         <v/>
       </c>
       <c r="O21" s="17">
@@ -4531,11 +4531,11 @@
         <v/>
       </c>
       <c r="J22" s="70">
-        <f>IF(H22&lt;0,"🔴 Restructurer (mutualiser)",IF(I22&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H22&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI19&gt;=2,E22&lt;=('08_Moteur'!AI19-1)*'08_Moteur'!O19*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I22&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K22" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI19&gt;=2,TEXT(IFERROR(E22/(('08_Moteur'!AI19-1)*'08_Moteur'!O19),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L22" s="21" t="inlineStr">
@@ -4548,7 +4548,7 @@
         <v/>
       </c>
       <c r="N22" s="17">
-        <f>IF(L22="Ne pas lancer",0,IF(L22="Ouvrir +1 classe",H22+'08_Moteur'!O19*('08_Moteur'!AE19*'08_Moteur'!AF19-('08_Moteur'!R19+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S19)-'08_Moteur'!U19,IF(L22="Regrouper (-1 classe)",H22+('08_Moteur'!AI19-MAX(1,'08_Moteur'!AI19-1))*'08_Moteur'!U19,H22)))</f>
+        <f>IF(L22="Ne pas lancer",0,IF(L22="Ouvrir +1 classe",H22+'08_Moteur'!O19*('08_Moteur'!AE19*'08_Moteur'!AF19-('08_Moteur'!R19+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S19)-'08_Moteur'!U19,IF(L22="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI19&gt;=2,E22&lt;=('08_Moteur'!AI19-1)*'08_Moteur'!O19*1.1),H22+'08_Moteur'!U19,H22),H22)))</f>
         <v/>
       </c>
       <c r="O22" s="17">
@@ -4602,11 +4602,11 @@
         <v/>
       </c>
       <c r="J23" s="70">
-        <f>IF(H23&lt;0,"🔴 Restructurer (mutualiser)",IF(I23&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H23&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI20&gt;=2,E23&lt;=('08_Moteur'!AI20-1)*'08_Moteur'!O20*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I23&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K23" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI20&gt;=2,TEXT(IFERROR(E23/(('08_Moteur'!AI20-1)*'08_Moteur'!O20),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L23" s="21" t="inlineStr">
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="N23" s="17">
-        <f>IF(L23="Ne pas lancer",0,IF(L23="Ouvrir +1 classe",H23+'08_Moteur'!O20*('08_Moteur'!AE20*'08_Moteur'!AF20-('08_Moteur'!R20+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S20)-'08_Moteur'!U20,IF(L23="Regrouper (-1 classe)",H23+('08_Moteur'!AI20-MAX(1,'08_Moteur'!AI20-1))*'08_Moteur'!U20,H23)))</f>
+        <f>IF(L23="Ne pas lancer",0,IF(L23="Ouvrir +1 classe",H23+'08_Moteur'!O20*('08_Moteur'!AE20*'08_Moteur'!AF20-('08_Moteur'!R20+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S20)-'08_Moteur'!U20,IF(L23="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI20&gt;=2,E23&lt;=('08_Moteur'!AI20-1)*'08_Moteur'!O20*1.1),H23+'08_Moteur'!U20,H23),H23)))</f>
         <v/>
       </c>
       <c r="O23" s="17">
@@ -4690,7 +4690,7 @@
         <v/>
       </c>
       <c r="N24" s="17">
-        <f>IF(L24="Ne pas lancer",0,IF(L24="Ouvrir +1 classe",H24+'08_Moteur'!O21*('08_Moteur'!AE21*'08_Moteur'!AF21-('08_Moteur'!R21+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S21)-'08_Moteur'!U21,IF(L24="Regrouper (-1 classe)",H24+('08_Moteur'!AI21-MAX(1,'08_Moteur'!AI21-1))*'08_Moteur'!U21,H24)))</f>
+        <f>IF(L24="Ne pas lancer",0,IF(L24="Ouvrir +1 classe",H24+'08_Moteur'!O21*('08_Moteur'!AE21*'08_Moteur'!AF21-('08_Moteur'!R21+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S21)-'08_Moteur'!U21,IF(L24="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI21&gt;=2,E24&lt;=('08_Moteur'!AI21-1)*'08_Moteur'!O21*1.1),H24+'08_Moteur'!U21,H24),H24)))</f>
         <v/>
       </c>
       <c r="O24" s="17">
@@ -4744,11 +4744,11 @@
         <v/>
       </c>
       <c r="J25" s="70">
-        <f>IF(H25&lt;0,"🔴 Restructurer (mutualiser)",IF(I25&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H25&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI22&gt;=2,E25&lt;=('08_Moteur'!AI22-1)*'08_Moteur'!O22*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I25&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K25" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI22&gt;=2,TEXT(IFERROR(E25/(('08_Moteur'!AI22-1)*'08_Moteur'!O22),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L25" s="21" t="inlineStr">
@@ -4761,7 +4761,7 @@
         <v/>
       </c>
       <c r="N25" s="17">
-        <f>IF(L25="Ne pas lancer",0,IF(L25="Ouvrir +1 classe",H25+'08_Moteur'!O22*('08_Moteur'!AE22*'08_Moteur'!AF22-('08_Moteur'!R22+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S22)-'08_Moteur'!U22,IF(L25="Regrouper (-1 classe)",H25+('08_Moteur'!AI22-MAX(1,'08_Moteur'!AI22-1))*'08_Moteur'!U22,H25)))</f>
+        <f>IF(L25="Ne pas lancer",0,IF(L25="Ouvrir +1 classe",H25+'08_Moteur'!O22*('08_Moteur'!AE22*'08_Moteur'!AF22-('08_Moteur'!R22+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S22)-'08_Moteur'!U22,IF(L25="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI22&gt;=2,E25&lt;=('08_Moteur'!AI22-1)*'08_Moteur'!O22*1.1),H25+'08_Moteur'!U22,H25),H25)))</f>
         <v/>
       </c>
       <c r="O25" s="17">
@@ -4832,7 +4832,7 @@
         <v/>
       </c>
       <c r="N26" s="17">
-        <f>IF(L26="Ne pas lancer",0,IF(L26="Ouvrir +1 classe",H26+'08_Moteur'!O23*('08_Moteur'!AE23*'08_Moteur'!AF23-('08_Moteur'!R23+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S23)-'08_Moteur'!U23,IF(L26="Regrouper (-1 classe)",H26+('08_Moteur'!AI23-MAX(1,'08_Moteur'!AI23-1))*'08_Moteur'!U23,H26)))</f>
+        <f>IF(L26="Ne pas lancer",0,IF(L26="Ouvrir +1 classe",H26+'08_Moteur'!O23*('08_Moteur'!AE23*'08_Moteur'!AF23-('08_Moteur'!R23+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S23)-'08_Moteur'!U23,IF(L26="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI23&gt;=2,E26&lt;=('08_Moteur'!AI23-1)*'08_Moteur'!O23*1.1),H26+'08_Moteur'!U23,H26),H26)))</f>
         <v/>
       </c>
       <c r="O26" s="17">
@@ -4886,11 +4886,11 @@
         <v/>
       </c>
       <c r="J27" s="70">
-        <f>IF(H27&lt;0,"🔴 Restructurer (mutualiser)",IF(I27&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H27&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI24&gt;=2,E27&lt;=('08_Moteur'!AI24-1)*'08_Moteur'!O24*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I27&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K27" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI24&gt;=2,TEXT(IFERROR(E27/(('08_Moteur'!AI24-1)*'08_Moteur'!O24),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L27" s="21" t="inlineStr">
@@ -4903,7 +4903,7 @@
         <v/>
       </c>
       <c r="N27" s="17">
-        <f>IF(L27="Ne pas lancer",0,IF(L27="Ouvrir +1 classe",H27+'08_Moteur'!O24*('08_Moteur'!AE24*'08_Moteur'!AF24-('08_Moteur'!R24+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S24)-'08_Moteur'!U24,IF(L27="Regrouper (-1 classe)",H27+('08_Moteur'!AI24-MAX(1,'08_Moteur'!AI24-1))*'08_Moteur'!U24,H27)))</f>
+        <f>IF(L27="Ne pas lancer",0,IF(L27="Ouvrir +1 classe",H27+'08_Moteur'!O24*('08_Moteur'!AE24*'08_Moteur'!AF24-('08_Moteur'!R24+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S24)-'08_Moteur'!U24,IF(L27="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI24&gt;=2,E27&lt;=('08_Moteur'!AI24-1)*'08_Moteur'!O24*1.1),H27+'08_Moteur'!U24,H27),H27)))</f>
         <v/>
       </c>
       <c r="O27" s="17">
@@ -4957,11 +4957,11 @@
         <v/>
       </c>
       <c r="J28" s="70">
-        <f>IF(H28&lt;0,"🔴 Restructurer (mutualiser)",IF(I28&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H28&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI25&gt;=2,E28&lt;=('08_Moteur'!AI25-1)*'08_Moteur'!O25*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I28&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K28" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI25&gt;=2,TEXT(IFERROR(E28/(('08_Moteur'!AI25-1)*'08_Moteur'!O25),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L28" s="21" t="inlineStr">
@@ -4974,7 +4974,7 @@
         <v/>
       </c>
       <c r="N28" s="17">
-        <f>IF(L28="Ne pas lancer",0,IF(L28="Ouvrir +1 classe",H28+'08_Moteur'!O25*('08_Moteur'!AE25*'08_Moteur'!AF25-('08_Moteur'!R25+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S25)-'08_Moteur'!U25,IF(L28="Regrouper (-1 classe)",H28+('08_Moteur'!AI25-MAX(1,'08_Moteur'!AI25-1))*'08_Moteur'!U25,H28)))</f>
+        <f>IF(L28="Ne pas lancer",0,IF(L28="Ouvrir +1 classe",H28+'08_Moteur'!O25*('08_Moteur'!AE25*'08_Moteur'!AF25-('08_Moteur'!R25+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S25)-'08_Moteur'!U25,IF(L28="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI25&gt;=2,E28&lt;=('08_Moteur'!AI25-1)*'08_Moteur'!O25*1.1),H28+'08_Moteur'!U25,H28),H28)))</f>
         <v/>
       </c>
       <c r="O28" s="17">
@@ -5045,7 +5045,7 @@
         <v/>
       </c>
       <c r="N29" s="17">
-        <f>IF(L29="Ne pas lancer",0,IF(L29="Ouvrir +1 classe",H29+'08_Moteur'!O26*('08_Moteur'!AE26*'08_Moteur'!AF26-('08_Moteur'!R26+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S26)-'08_Moteur'!U26,IF(L29="Regrouper (-1 classe)",H29+('08_Moteur'!AI26-MAX(1,'08_Moteur'!AI26-1))*'08_Moteur'!U26,H29)))</f>
+        <f>IF(L29="Ne pas lancer",0,IF(L29="Ouvrir +1 classe",H29+'08_Moteur'!O26*('08_Moteur'!AE26*'08_Moteur'!AF26-('08_Moteur'!R26+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S26)-'08_Moteur'!U26,IF(L29="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI26&gt;=2,E29&lt;=('08_Moteur'!AI26-1)*'08_Moteur'!O26*1.1),H29+'08_Moteur'!U26,H29),H29)))</f>
         <v/>
       </c>
       <c r="O29" s="17">
@@ -5099,11 +5099,11 @@
         <v/>
       </c>
       <c r="J30" s="70">
-        <f>IF(H30&lt;0,"🔴 Restructurer (mutualiser)",IF(I30&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H30&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI27&gt;=2,E30&lt;=('08_Moteur'!AI27-1)*'08_Moteur'!O27*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I30&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K30" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI27&gt;=2,TEXT(IFERROR(E30/(('08_Moteur'!AI27-1)*'08_Moteur'!O27),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L30" s="21" t="inlineStr">
@@ -5116,7 +5116,7 @@
         <v/>
       </c>
       <c r="N30" s="17">
-        <f>IF(L30="Ne pas lancer",0,IF(L30="Ouvrir +1 classe",H30+'08_Moteur'!O27*('08_Moteur'!AE27*'08_Moteur'!AF27-('08_Moteur'!R27+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S27)-'08_Moteur'!U27,IF(L30="Regrouper (-1 classe)",H30+('08_Moteur'!AI27-MAX(1,'08_Moteur'!AI27-1))*'08_Moteur'!U27,H30)))</f>
+        <f>IF(L30="Ne pas lancer",0,IF(L30="Ouvrir +1 classe",H30+'08_Moteur'!O27*('08_Moteur'!AE27*'08_Moteur'!AF27-('08_Moteur'!R27+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S27)-'08_Moteur'!U27,IF(L30="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI27&gt;=2,E30&lt;=('08_Moteur'!AI27-1)*'08_Moteur'!O27*1.1),H30+'08_Moteur'!U27,H30),H30)))</f>
         <v/>
       </c>
       <c r="O30" s="17">
@@ -5187,7 +5187,7 @@
         <v/>
       </c>
       <c r="N31" s="17">
-        <f>IF(L31="Ne pas lancer",0,IF(L31="Ouvrir +1 classe",H31+'08_Moteur'!O28*('08_Moteur'!AE28*'08_Moteur'!AF28-('08_Moteur'!R28+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S28)-'08_Moteur'!U28,IF(L31="Regrouper (-1 classe)",H31+('08_Moteur'!AI28-MAX(1,'08_Moteur'!AI28-1))*'08_Moteur'!U28,H31)))</f>
+        <f>IF(L31="Ne pas lancer",0,IF(L31="Ouvrir +1 classe",H31+'08_Moteur'!O28*('08_Moteur'!AE28*'08_Moteur'!AF28-('08_Moteur'!R28+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S28)-'08_Moteur'!U28,IF(L31="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI28&gt;=2,E31&lt;=('08_Moteur'!AI28-1)*'08_Moteur'!O28*1.1),H31+'08_Moteur'!U28,H31),H31)))</f>
         <v/>
       </c>
       <c r="O31" s="17">
@@ -5241,11 +5241,11 @@
         <v/>
       </c>
       <c r="J32" s="70">
-        <f>IF(H32&lt;0,"🔴 Restructurer (mutualiser)",IF(I32&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H32&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI29&gt;=2,E32&lt;=('08_Moteur'!AI29-1)*'08_Moteur'!O29*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I32&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K32" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI29&gt;=2,TEXT(IFERROR(E32/(('08_Moteur'!AI29-1)*'08_Moteur'!O29),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L32" s="21" t="inlineStr">
@@ -5258,7 +5258,7 @@
         <v/>
       </c>
       <c r="N32" s="17">
-        <f>IF(L32="Ne pas lancer",0,IF(L32="Ouvrir +1 classe",H32+'08_Moteur'!O29*('08_Moteur'!AE29*'08_Moteur'!AF29-('08_Moteur'!R29+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S29)-'08_Moteur'!U29,IF(L32="Regrouper (-1 classe)",H32+('08_Moteur'!AI29-MAX(1,'08_Moteur'!AI29-1))*'08_Moteur'!U29,H32)))</f>
+        <f>IF(L32="Ne pas lancer",0,IF(L32="Ouvrir +1 classe",H32+'08_Moteur'!O29*('08_Moteur'!AE29*'08_Moteur'!AF29-('08_Moteur'!R29+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S29)-'08_Moteur'!U29,IF(L32="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI29&gt;=2,E32&lt;=('08_Moteur'!AI29-1)*'08_Moteur'!O29*1.1),H32+'08_Moteur'!U29,H32),H32)))</f>
         <v/>
       </c>
       <c r="O32" s="17">
@@ -5312,11 +5312,11 @@
         <v/>
       </c>
       <c r="J33" s="70">
-        <f>IF(H33&lt;0,"🔴 Restructurer (mutualiser)",IF(I33&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H33&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI30&gt;=2,E33&lt;=('08_Moteur'!AI30-1)*'08_Moteur'!O30*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I33&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K33" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI30&gt;=2,TEXT(IFERROR(E33/(('08_Moteur'!AI30-1)*'08_Moteur'!O30),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L33" s="21" t="inlineStr">
@@ -5329,7 +5329,7 @@
         <v/>
       </c>
       <c r="N33" s="17">
-        <f>IF(L33="Ne pas lancer",0,IF(L33="Ouvrir +1 classe",H33+'08_Moteur'!O30*('08_Moteur'!AE30*'08_Moteur'!AF30-('08_Moteur'!R30+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S30)-'08_Moteur'!U30,IF(L33="Regrouper (-1 classe)",H33+('08_Moteur'!AI30-MAX(1,'08_Moteur'!AI30-1))*'08_Moteur'!U30,H33)))</f>
+        <f>IF(L33="Ne pas lancer",0,IF(L33="Ouvrir +1 classe",H33+'08_Moteur'!O30*('08_Moteur'!AE30*'08_Moteur'!AF30-('08_Moteur'!R30+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S30)-'08_Moteur'!U30,IF(L33="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI30&gt;=2,E33&lt;=('08_Moteur'!AI30-1)*'08_Moteur'!O30*1.1),H33+'08_Moteur'!U30,H33),H33)))</f>
         <v/>
       </c>
       <c r="O33" s="17">
@@ -5400,7 +5400,7 @@
         <v/>
       </c>
       <c r="N34" s="17">
-        <f>IF(L34="Ne pas lancer",0,IF(L34="Ouvrir +1 classe",H34+'08_Moteur'!O31*('08_Moteur'!AE31*'08_Moteur'!AF31-('08_Moteur'!R31+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S31)-'08_Moteur'!U31,IF(L34="Regrouper (-1 classe)",H34+('08_Moteur'!AI31-MAX(1,'08_Moteur'!AI31-1))*'08_Moteur'!U31,H34)))</f>
+        <f>IF(L34="Ne pas lancer",0,IF(L34="Ouvrir +1 classe",H34+'08_Moteur'!O31*('08_Moteur'!AE31*'08_Moteur'!AF31-('08_Moteur'!R31+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S31)-'08_Moteur'!U31,IF(L34="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI31&gt;=2,E34&lt;=('08_Moteur'!AI31-1)*'08_Moteur'!O31*1.1),H34+'08_Moteur'!U31,H34),H34)))</f>
         <v/>
       </c>
       <c r="O34" s="17">
@@ -5454,11 +5454,11 @@
         <v/>
       </c>
       <c r="J35" s="70">
-        <f>IF(H35&lt;0,"🔴 Restructurer (mutualiser)",IF(I35&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H35&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI32&gt;=2,E35&lt;=('08_Moteur'!AI32-1)*'08_Moteur'!O32*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I35&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K35" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI32&gt;=2,TEXT(IFERROR(E35/(('08_Moteur'!AI32-1)*'08_Moteur'!O32),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L35" s="21" t="inlineStr">
@@ -5471,7 +5471,7 @@
         <v/>
       </c>
       <c r="N35" s="17">
-        <f>IF(L35="Ne pas lancer",0,IF(L35="Ouvrir +1 classe",H35+'08_Moteur'!O32*('08_Moteur'!AE32*'08_Moteur'!AF32-('08_Moteur'!R32+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S32)-'08_Moteur'!U32,IF(L35="Regrouper (-1 classe)",H35+('08_Moteur'!AI32-MAX(1,'08_Moteur'!AI32-1))*'08_Moteur'!U32,H35)))</f>
+        <f>IF(L35="Ne pas lancer",0,IF(L35="Ouvrir +1 classe",H35+'08_Moteur'!O32*('08_Moteur'!AE32*'08_Moteur'!AF32-('08_Moteur'!R32+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S32)-'08_Moteur'!U32,IF(L35="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI32&gt;=2,E35&lt;=('08_Moteur'!AI32-1)*'08_Moteur'!O32*1.1),H35+'08_Moteur'!U32,H35),H35)))</f>
         <v/>
       </c>
       <c r="O35" s="17">
@@ -5542,7 +5542,7 @@
         <v/>
       </c>
       <c r="N36" s="17">
-        <f>IF(L36="Ne pas lancer",0,IF(L36="Ouvrir +1 classe",H36+'08_Moteur'!O33*('08_Moteur'!AE33*'08_Moteur'!AF33-('08_Moteur'!R33+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S33)-'08_Moteur'!U33,IF(L36="Regrouper (-1 classe)",H36+('08_Moteur'!AI33-MAX(1,'08_Moteur'!AI33-1))*'08_Moteur'!U33,H36)))</f>
+        <f>IF(L36="Ne pas lancer",0,IF(L36="Ouvrir +1 classe",H36+'08_Moteur'!O33*('08_Moteur'!AE33*'08_Moteur'!AF33-('08_Moteur'!R33+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S33)-'08_Moteur'!U33,IF(L36="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI33&gt;=2,E36&lt;=('08_Moteur'!AI33-1)*'08_Moteur'!O33*1.1),H36+'08_Moteur'!U33,H36),H36)))</f>
         <v/>
       </c>
       <c r="O36" s="17">
@@ -5596,11 +5596,11 @@
         <v/>
       </c>
       <c r="J37" s="70">
-        <f>IF(H37&lt;0,"🔴 Restructurer (mutualiser)",IF(I37&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H37&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI34&gt;=2,E37&lt;=('08_Moteur'!AI34-1)*'08_Moteur'!O34*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I37&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K37" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI34&gt;=2,TEXT(IFERROR(E37/(('08_Moteur'!AI34-1)*'08_Moteur'!O34),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L37" s="21" t="inlineStr">
@@ -5613,7 +5613,7 @@
         <v/>
       </c>
       <c r="N37" s="17">
-        <f>IF(L37="Ne pas lancer",0,IF(L37="Ouvrir +1 classe",H37+'08_Moteur'!O34*('08_Moteur'!AE34*'08_Moteur'!AF34-('08_Moteur'!R34+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S34)-'08_Moteur'!U34,IF(L37="Regrouper (-1 classe)",H37+('08_Moteur'!AI34-MAX(1,'08_Moteur'!AI34-1))*'08_Moteur'!U34,H37)))</f>
+        <f>IF(L37="Ne pas lancer",0,IF(L37="Ouvrir +1 classe",H37+'08_Moteur'!O34*('08_Moteur'!AE34*'08_Moteur'!AF34-('08_Moteur'!R34+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S34)-'08_Moteur'!U34,IF(L37="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI34&gt;=2,E37&lt;=('08_Moteur'!AI34-1)*'08_Moteur'!O34*1.1),H37+'08_Moteur'!U34,H37),H37)))</f>
         <v/>
       </c>
       <c r="O37" s="17">
@@ -5667,11 +5667,11 @@
         <v/>
       </c>
       <c r="J38" s="70">
-        <f>IF(H38&lt;0,"🔴 Restructurer (mutualiser)",IF(I38&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H38&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI35&gt;=2,E38&lt;=('08_Moteur'!AI35-1)*'08_Moteur'!O35*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I38&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K38" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI35&gt;=2,TEXT(IFERROR(E38/(('08_Moteur'!AI35-1)*'08_Moteur'!O35),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L38" s="21" t="inlineStr">
@@ -5684,7 +5684,7 @@
         <v/>
       </c>
       <c r="N38" s="17">
-        <f>IF(L38="Ne pas lancer",0,IF(L38="Ouvrir +1 classe",H38+'08_Moteur'!O35*('08_Moteur'!AE35*'08_Moteur'!AF35-('08_Moteur'!R35+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S35)-'08_Moteur'!U35,IF(L38="Regrouper (-1 classe)",H38+('08_Moteur'!AI35-MAX(1,'08_Moteur'!AI35-1))*'08_Moteur'!U35,H38)))</f>
+        <f>IF(L38="Ne pas lancer",0,IF(L38="Ouvrir +1 classe",H38+'08_Moteur'!O35*('08_Moteur'!AE35*'08_Moteur'!AF35-('08_Moteur'!R35+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S35)-'08_Moteur'!U35,IF(L38="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI35&gt;=2,E38&lt;=('08_Moteur'!AI35-1)*'08_Moteur'!O35*1.1),H38+'08_Moteur'!U35,H38),H38)))</f>
         <v/>
       </c>
       <c r="O38" s="17">
@@ -5755,7 +5755,7 @@
         <v/>
       </c>
       <c r="N39" s="17">
-        <f>IF(L39="Ne pas lancer",0,IF(L39="Ouvrir +1 classe",H39+'08_Moteur'!O36*('08_Moteur'!AE36*'08_Moteur'!AF36-('08_Moteur'!R36+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S36)-'08_Moteur'!U36,IF(L39="Regrouper (-1 classe)",H39+('08_Moteur'!AI36-MAX(1,'08_Moteur'!AI36-1))*'08_Moteur'!U36,H39)))</f>
+        <f>IF(L39="Ne pas lancer",0,IF(L39="Ouvrir +1 classe",H39+'08_Moteur'!O36*('08_Moteur'!AE36*'08_Moteur'!AF36-('08_Moteur'!R36+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S36)-'08_Moteur'!U36,IF(L39="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI36&gt;=2,E39&lt;=('08_Moteur'!AI36-1)*'08_Moteur'!O36*1.1),H39+'08_Moteur'!U36,H39),H39)))</f>
         <v/>
       </c>
       <c r="O39" s="17">
@@ -5809,11 +5809,11 @@
         <v/>
       </c>
       <c r="J40" s="70">
-        <f>IF(H40&lt;0,"🔴 Restructurer (mutualiser)",IF(I40&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H40&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI37&gt;=2,E40&lt;=('08_Moteur'!AI37-1)*'08_Moteur'!O37*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I40&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K40" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI37&gt;=2,TEXT(IFERROR(E40/(('08_Moteur'!AI37-1)*'08_Moteur'!O37),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L40" s="21" t="inlineStr">
@@ -5826,7 +5826,7 @@
         <v/>
       </c>
       <c r="N40" s="17">
-        <f>IF(L40="Ne pas lancer",0,IF(L40="Ouvrir +1 classe",H40+'08_Moteur'!O37*('08_Moteur'!AE37*'08_Moteur'!AF37-('08_Moteur'!R37+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S37)-'08_Moteur'!U37,IF(L40="Regrouper (-1 classe)",H40+('08_Moteur'!AI37-MAX(1,'08_Moteur'!AI37-1))*'08_Moteur'!U37,H40)))</f>
+        <f>IF(L40="Ne pas lancer",0,IF(L40="Ouvrir +1 classe",H40+'08_Moteur'!O37*('08_Moteur'!AE37*'08_Moteur'!AF37-('08_Moteur'!R37+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S37)-'08_Moteur'!U37,IF(L40="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI37&gt;=2,E40&lt;=('08_Moteur'!AI37-1)*'08_Moteur'!O37*1.1),H40+'08_Moteur'!U37,H40),H40)))</f>
         <v/>
       </c>
       <c r="O40" s="17">
@@ -5897,7 +5897,7 @@
         <v/>
       </c>
       <c r="N41" s="17">
-        <f>IF(L41="Ne pas lancer",0,IF(L41="Ouvrir +1 classe",H41+'08_Moteur'!O38*('08_Moteur'!AE38*'08_Moteur'!AF38-('08_Moteur'!R38+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S38)-'08_Moteur'!U38,IF(L41="Regrouper (-1 classe)",H41+('08_Moteur'!AI38-MAX(1,'08_Moteur'!AI38-1))*'08_Moteur'!U38,H41)))</f>
+        <f>IF(L41="Ne pas lancer",0,IF(L41="Ouvrir +1 classe",H41+'08_Moteur'!O38*('08_Moteur'!AE38*'08_Moteur'!AF38-('08_Moteur'!R38+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S38)-'08_Moteur'!U38,IF(L41="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI38&gt;=2,E41&lt;=('08_Moteur'!AI38-1)*'08_Moteur'!O38*1.1),H41+'08_Moteur'!U38,H41),H41)))</f>
         <v/>
       </c>
       <c r="O41" s="17">
@@ -5951,11 +5951,11 @@
         <v/>
       </c>
       <c r="J42" s="70">
-        <f>IF(H42&lt;0,"🔴 Restructurer (mutualiser)",IF(I42&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H42&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI39&gt;=2,E42&lt;=('08_Moteur'!AI39-1)*'08_Moteur'!O39*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I42&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K42" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI39&gt;=2,TEXT(IFERROR(E42/(('08_Moteur'!AI39-1)*'08_Moteur'!O39),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L42" s="21" t="inlineStr">
@@ -5968,7 +5968,7 @@
         <v/>
       </c>
       <c r="N42" s="17">
-        <f>IF(L42="Ne pas lancer",0,IF(L42="Ouvrir +1 classe",H42+'08_Moteur'!O39*('08_Moteur'!AE39*'08_Moteur'!AF39-('08_Moteur'!R39+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S39)-'08_Moteur'!U39,IF(L42="Regrouper (-1 classe)",H42+('08_Moteur'!AI39-MAX(1,'08_Moteur'!AI39-1))*'08_Moteur'!U39,H42)))</f>
+        <f>IF(L42="Ne pas lancer",0,IF(L42="Ouvrir +1 classe",H42+'08_Moteur'!O39*('08_Moteur'!AE39*'08_Moteur'!AF39-('08_Moteur'!R39+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S39)-'08_Moteur'!U39,IF(L42="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI39&gt;=2,E42&lt;=('08_Moteur'!AI39-1)*'08_Moteur'!O39*1.1),H42+'08_Moteur'!U39,H42),H42)))</f>
         <v/>
       </c>
       <c r="O42" s="17">
@@ -6022,11 +6022,11 @@
         <v/>
       </c>
       <c r="J43" s="70">
-        <f>IF(H43&lt;0,"🔴 Restructurer (mutualiser)",IF(I43&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H43&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI40&gt;=2,E43&lt;=('08_Moteur'!AI40-1)*'08_Moteur'!O40*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I43&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K43" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI40&gt;=2,TEXT(IFERROR(E43/(('08_Moteur'!AI40-1)*'08_Moteur'!O40),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L43" s="21" t="inlineStr">
@@ -6039,7 +6039,7 @@
         <v/>
       </c>
       <c r="N43" s="17">
-        <f>IF(L43="Ne pas lancer",0,IF(L43="Ouvrir +1 classe",H43+'08_Moteur'!O40*('08_Moteur'!AE40*'08_Moteur'!AF40-('08_Moteur'!R40+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S40)-'08_Moteur'!U40,IF(L43="Regrouper (-1 classe)",H43+('08_Moteur'!AI40-MAX(1,'08_Moteur'!AI40-1))*'08_Moteur'!U40,H43)))</f>
+        <f>IF(L43="Ne pas lancer",0,IF(L43="Ouvrir +1 classe",H43+'08_Moteur'!O40*('08_Moteur'!AE40*'08_Moteur'!AF40-('08_Moteur'!R40+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S40)-'08_Moteur'!U40,IF(L43="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI40&gt;=2,E43&lt;=('08_Moteur'!AI40-1)*'08_Moteur'!O40*1.1),H43+'08_Moteur'!U40,H43),H43)))</f>
         <v/>
       </c>
       <c r="O43" s="17">
@@ -6110,7 +6110,7 @@
         <v/>
       </c>
       <c r="N44" s="17">
-        <f>IF(L44="Ne pas lancer",0,IF(L44="Ouvrir +1 classe",H44+'08_Moteur'!O41*('08_Moteur'!AE41*'08_Moteur'!AF41-('08_Moteur'!R41+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S41)-'08_Moteur'!U41,IF(L44="Regrouper (-1 classe)",H44+('08_Moteur'!AI41-MAX(1,'08_Moteur'!AI41-1))*'08_Moteur'!U41,H44)))</f>
+        <f>IF(L44="Ne pas lancer",0,IF(L44="Ouvrir +1 classe",H44+'08_Moteur'!O41*('08_Moteur'!AE41*'08_Moteur'!AF41-('08_Moteur'!R41+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S41)-'08_Moteur'!U41,IF(L44="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI41&gt;=2,E44&lt;=('08_Moteur'!AI41-1)*'08_Moteur'!O41*1.1),H44+'08_Moteur'!U41,H44),H44)))</f>
         <v/>
       </c>
       <c r="O44" s="17">
@@ -6164,11 +6164,11 @@
         <v/>
       </c>
       <c r="J45" s="70">
-        <f>IF(H45&lt;0,"🔴 Restructurer (mutualiser)",IF(I45&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H45&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI42&gt;=2,E45&lt;=('08_Moteur'!AI42-1)*'08_Moteur'!O42*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I45&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K45" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI42&gt;=2,TEXT(IFERROR(E45/(('08_Moteur'!AI42-1)*'08_Moteur'!O42),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L45" s="21" t="inlineStr">
@@ -6181,7 +6181,7 @@
         <v/>
       </c>
       <c r="N45" s="17">
-        <f>IF(L45="Ne pas lancer",0,IF(L45="Ouvrir +1 classe",H45+'08_Moteur'!O42*('08_Moteur'!AE42*'08_Moteur'!AF42-('08_Moteur'!R42+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S42)-'08_Moteur'!U42,IF(L45="Regrouper (-1 classe)",H45+('08_Moteur'!AI42-MAX(1,'08_Moteur'!AI42-1))*'08_Moteur'!U42,H45)))</f>
+        <f>IF(L45="Ne pas lancer",0,IF(L45="Ouvrir +1 classe",H45+'08_Moteur'!O42*('08_Moteur'!AE42*'08_Moteur'!AF42-('08_Moteur'!R42+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S42)-'08_Moteur'!U42,IF(L45="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI42&gt;=2,E45&lt;=('08_Moteur'!AI42-1)*'08_Moteur'!O42*1.1),H45+'08_Moteur'!U42,H45),H45)))</f>
         <v/>
       </c>
       <c r="O45" s="17">
@@ -6235,11 +6235,11 @@
         <v/>
       </c>
       <c r="J46" s="70">
-        <f>IF(H46&lt;0,"🔴 Restructurer (mutualiser)",IF(I46&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H46&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI43&gt;=2,E46&lt;=('08_Moteur'!AI43-1)*'08_Moteur'!O43*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I46&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K46" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI43&gt;=2,TEXT(IFERROR(E46/(('08_Moteur'!AI43-1)*'08_Moteur'!O43),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L46" s="21" t="inlineStr">
@@ -6252,7 +6252,7 @@
         <v/>
       </c>
       <c r="N46" s="17">
-        <f>IF(L46="Ne pas lancer",0,IF(L46="Ouvrir +1 classe",H46+'08_Moteur'!O43*('08_Moteur'!AE43*'08_Moteur'!AF43-('08_Moteur'!R43+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S43)-'08_Moteur'!U43,IF(L46="Regrouper (-1 classe)",H46+('08_Moteur'!AI43-MAX(1,'08_Moteur'!AI43-1))*'08_Moteur'!U43,H46)))</f>
+        <f>IF(L46="Ne pas lancer",0,IF(L46="Ouvrir +1 classe",H46+'08_Moteur'!O43*('08_Moteur'!AE43*'08_Moteur'!AF43-('08_Moteur'!R43+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S43)-'08_Moteur'!U43,IF(L46="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI43&gt;=2,E46&lt;=('08_Moteur'!AI43-1)*'08_Moteur'!O43*1.1),H46+'08_Moteur'!U43,H46),H46)))</f>
         <v/>
       </c>
       <c r="O46" s="17">
@@ -6323,7 +6323,7 @@
         <v/>
       </c>
       <c r="N47" s="17">
-        <f>IF(L47="Ne pas lancer",0,IF(L47="Ouvrir +1 classe",H47+'08_Moteur'!O44*('08_Moteur'!AE44*'08_Moteur'!AF44-('08_Moteur'!R44+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S44)-'08_Moteur'!U44,IF(L47="Regrouper (-1 classe)",H47+('08_Moteur'!AI44-MAX(1,'08_Moteur'!AI44-1))*'08_Moteur'!U44,H47)))</f>
+        <f>IF(L47="Ne pas lancer",0,IF(L47="Ouvrir +1 classe",H47+'08_Moteur'!O44*('08_Moteur'!AE44*'08_Moteur'!AF44-('08_Moteur'!R44+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S44)-'08_Moteur'!U44,IF(L47="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI44&gt;=2,E47&lt;=('08_Moteur'!AI44-1)*'08_Moteur'!O44*1.1),H47+'08_Moteur'!U44,H47),H47)))</f>
         <v/>
       </c>
       <c r="O47" s="17">
@@ -6377,11 +6377,11 @@
         <v/>
       </c>
       <c r="J48" s="70">
-        <f>IF(H48&lt;0,"🔴 Restructurer (mutualiser)",IF(I48&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H48&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI45&gt;=2,E48&lt;=('08_Moteur'!AI45-1)*'08_Moteur'!O45*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I48&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K48" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI45&gt;=2,TEXT(IFERROR(E48/(('08_Moteur'!AI45-1)*'08_Moteur'!O45),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L48" s="21" t="inlineStr">
@@ -6394,7 +6394,7 @@
         <v/>
       </c>
       <c r="N48" s="17">
-        <f>IF(L48="Ne pas lancer",0,IF(L48="Ouvrir +1 classe",H48+'08_Moteur'!O45*('08_Moteur'!AE45*'08_Moteur'!AF45-('08_Moteur'!R45+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S45)-'08_Moteur'!U45,IF(L48="Regrouper (-1 classe)",H48+('08_Moteur'!AI45-MAX(1,'08_Moteur'!AI45-1))*'08_Moteur'!U45,H48)))</f>
+        <f>IF(L48="Ne pas lancer",0,IF(L48="Ouvrir +1 classe",H48+'08_Moteur'!O45*('08_Moteur'!AE45*'08_Moteur'!AF45-('08_Moteur'!R45+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S45)-'08_Moteur'!U45,IF(L48="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI45&gt;=2,E48&lt;=('08_Moteur'!AI45-1)*'08_Moteur'!O45*1.1),H48+'08_Moteur'!U45,H48),H48)))</f>
         <v/>
       </c>
       <c r="O48" s="17">
@@ -6448,11 +6448,11 @@
         <v/>
       </c>
       <c r="J49" s="70">
-        <f>IF(H49&lt;0,"🔴 Restructurer (mutualiser)",IF(I49&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H49&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI46&gt;=2,E49&lt;=('08_Moteur'!AI46-1)*'08_Moteur'!O46*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I49&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K49" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI46&gt;=2,TEXT(IFERROR(E49/(('08_Moteur'!AI46-1)*'08_Moteur'!O46),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L49" s="21" t="inlineStr">
@@ -6465,7 +6465,7 @@
         <v/>
       </c>
       <c r="N49" s="17">
-        <f>IF(L49="Ne pas lancer",0,IF(L49="Ouvrir +1 classe",H49+'08_Moteur'!O46*('08_Moteur'!AE46*'08_Moteur'!AF46-('08_Moteur'!R46+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S46)-'08_Moteur'!U46,IF(L49="Regrouper (-1 classe)",H49+('08_Moteur'!AI46-MAX(1,'08_Moteur'!AI46-1))*'08_Moteur'!U46,H49)))</f>
+        <f>IF(L49="Ne pas lancer",0,IF(L49="Ouvrir +1 classe",H49+'08_Moteur'!O46*('08_Moteur'!AE46*'08_Moteur'!AF46-('08_Moteur'!R46+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S46)-'08_Moteur'!U46,IF(L49="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI46&gt;=2,E49&lt;=('08_Moteur'!AI46-1)*'08_Moteur'!O46*1.1),H49+'08_Moteur'!U46,H49),H49)))</f>
         <v/>
       </c>
       <c r="O49" s="17">
@@ -6536,7 +6536,7 @@
         <v/>
       </c>
       <c r="N50" s="17">
-        <f>IF(L50="Ne pas lancer",0,IF(L50="Ouvrir +1 classe",H50+'08_Moteur'!O47*('08_Moteur'!AE47*'08_Moteur'!AF47-('08_Moteur'!R47+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S47)-'08_Moteur'!U47,IF(L50="Regrouper (-1 classe)",H50+('08_Moteur'!AI47-MAX(1,'08_Moteur'!AI47-1))*'08_Moteur'!U47,H50)))</f>
+        <f>IF(L50="Ne pas lancer",0,IF(L50="Ouvrir +1 classe",H50+'08_Moteur'!O47*('08_Moteur'!AE47*'08_Moteur'!AF47-('08_Moteur'!R47+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S47)-'08_Moteur'!U47,IF(L50="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI47&gt;=2,E50&lt;=('08_Moteur'!AI47-1)*'08_Moteur'!O47*1.1),H50+'08_Moteur'!U47,H50),H50)))</f>
         <v/>
       </c>
       <c r="O50" s="17">
@@ -6590,11 +6590,11 @@
         <v/>
       </c>
       <c r="J51" s="70">
-        <f>IF(H51&lt;0,"🔴 Restructurer (mutualiser)",IF(I51&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H51&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI48&gt;=2,E51&lt;=('08_Moteur'!AI48-1)*'08_Moteur'!O48*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I51&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K51" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI48&gt;=2,TEXT(IFERROR(E51/(('08_Moteur'!AI48-1)*'08_Moteur'!O48),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L51" s="21" t="inlineStr">
@@ -6607,7 +6607,7 @@
         <v/>
       </c>
       <c r="N51" s="17">
-        <f>IF(L51="Ne pas lancer",0,IF(L51="Ouvrir +1 classe",H51+'08_Moteur'!O48*('08_Moteur'!AE48*'08_Moteur'!AF48-('08_Moteur'!R48+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S48)-'08_Moteur'!U48,IF(L51="Regrouper (-1 classe)",H51+('08_Moteur'!AI48-MAX(1,'08_Moteur'!AI48-1))*'08_Moteur'!U48,H51)))</f>
+        <f>IF(L51="Ne pas lancer",0,IF(L51="Ouvrir +1 classe",H51+'08_Moteur'!O48*('08_Moteur'!AE48*'08_Moteur'!AF48-('08_Moteur'!R48+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S48)-'08_Moteur'!U48,IF(L51="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI48&gt;=2,E51&lt;=('08_Moteur'!AI48-1)*'08_Moteur'!O48*1.1),H51+'08_Moteur'!U48,H51),H51)))</f>
         <v/>
       </c>
       <c r="O51" s="17">
@@ -6678,7 +6678,7 @@
         <v/>
       </c>
       <c r="N52" s="17">
-        <f>IF(L52="Ne pas lancer",0,IF(L52="Ouvrir +1 classe",H52+'08_Moteur'!O49*('08_Moteur'!AE49*'08_Moteur'!AF49-('08_Moteur'!R49+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S49)-'08_Moteur'!U49,IF(L52="Regrouper (-1 classe)",H52+('08_Moteur'!AI49-MAX(1,'08_Moteur'!AI49-1))*'08_Moteur'!U49,H52)))</f>
+        <f>IF(L52="Ne pas lancer",0,IF(L52="Ouvrir +1 classe",H52+'08_Moteur'!O49*('08_Moteur'!AE49*'08_Moteur'!AF49-('08_Moteur'!R49+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S49)-'08_Moteur'!U49,IF(L52="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI49&gt;=2,E52&lt;=('08_Moteur'!AI49-1)*'08_Moteur'!O49*1.1),H52+'08_Moteur'!U49,H52),H52)))</f>
         <v/>
       </c>
       <c r="O52" s="17">
@@ -6732,11 +6732,11 @@
         <v/>
       </c>
       <c r="J53" s="70">
-        <f>IF(H53&lt;0,"🔴 Restructurer (mutualiser)",IF(I53&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H53&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI50&gt;=2,E53&lt;=('08_Moteur'!AI50-1)*'08_Moteur'!O50*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I53&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K53" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI50&gt;=2,TEXT(IFERROR(E53/(('08_Moteur'!AI50-1)*'08_Moteur'!O50),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L53" s="21" t="inlineStr">
@@ -6749,7 +6749,7 @@
         <v/>
       </c>
       <c r="N53" s="17">
-        <f>IF(L53="Ne pas lancer",0,IF(L53="Ouvrir +1 classe",H53+'08_Moteur'!O50*('08_Moteur'!AE50*'08_Moteur'!AF50-('08_Moteur'!R50+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S50)-'08_Moteur'!U50,IF(L53="Regrouper (-1 classe)",H53+('08_Moteur'!AI50-MAX(1,'08_Moteur'!AI50-1))*'08_Moteur'!U50,H53)))</f>
+        <f>IF(L53="Ne pas lancer",0,IF(L53="Ouvrir +1 classe",H53+'08_Moteur'!O50*('08_Moteur'!AE50*'08_Moteur'!AF50-('08_Moteur'!R50+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S50)-'08_Moteur'!U50,IF(L53="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI50&gt;=2,E53&lt;=('08_Moteur'!AI50-1)*'08_Moteur'!O50*1.1),H53+'08_Moteur'!U50,H53),H53)))</f>
         <v/>
       </c>
       <c r="O53" s="17">
@@ -6820,7 +6820,7 @@
         <v/>
       </c>
       <c r="N54" s="17">
-        <f>IF(L54="Ne pas lancer",0,IF(L54="Ouvrir +1 classe",H54+'08_Moteur'!O51*('08_Moteur'!AE51*'08_Moteur'!AF51-('08_Moteur'!R51+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S51)-'08_Moteur'!U51,IF(L54="Regrouper (-1 classe)",H54+('08_Moteur'!AI51-MAX(1,'08_Moteur'!AI51-1))*'08_Moteur'!U51,H54)))</f>
+        <f>IF(L54="Ne pas lancer",0,IF(L54="Ouvrir +1 classe",H54+'08_Moteur'!O51*('08_Moteur'!AE51*'08_Moteur'!AF51-('08_Moteur'!R51+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S51)-'08_Moteur'!U51,IF(L54="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI51&gt;=2,E54&lt;=('08_Moteur'!AI51-1)*'08_Moteur'!O51*1.1),H54+'08_Moteur'!U51,H54),H54)))</f>
         <v/>
       </c>
       <c r="O54" s="17">
@@ -6874,11 +6874,11 @@
         <v/>
       </c>
       <c r="J55" s="70">
-        <f>IF(H55&lt;0,"🔴 Restructurer (mutualiser)",IF(I55&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H55&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI52&gt;=2,E55&lt;=('08_Moteur'!AI52-1)*'08_Moteur'!O52*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I55&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K55" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI52&gt;=2,TEXT(IFERROR(E55/(('08_Moteur'!AI52-1)*'08_Moteur'!O52),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L55" s="21" t="inlineStr">
@@ -6891,7 +6891,7 @@
         <v/>
       </c>
       <c r="N55" s="17">
-        <f>IF(L55="Ne pas lancer",0,IF(L55="Ouvrir +1 classe",H55+'08_Moteur'!O52*('08_Moteur'!AE52*'08_Moteur'!AF52-('08_Moteur'!R52+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S52)-'08_Moteur'!U52,IF(L55="Regrouper (-1 classe)",H55+('08_Moteur'!AI52-MAX(1,'08_Moteur'!AI52-1))*'08_Moteur'!U52,H55)))</f>
+        <f>IF(L55="Ne pas lancer",0,IF(L55="Ouvrir +1 classe",H55+'08_Moteur'!O52*('08_Moteur'!AE52*'08_Moteur'!AF52-('08_Moteur'!R52+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S52)-'08_Moteur'!U52,IF(L55="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI52&gt;=2,E55&lt;=('08_Moteur'!AI52-1)*'08_Moteur'!O52*1.1),H55+'08_Moteur'!U52,H55),H55)))</f>
         <v/>
       </c>
       <c r="O55" s="17">
@@ -6962,7 +6962,7 @@
         <v/>
       </c>
       <c r="N56" s="17">
-        <f>IF(L56="Ne pas lancer",0,IF(L56="Ouvrir +1 classe",H56+'08_Moteur'!O53*('08_Moteur'!AE53*'08_Moteur'!AF53-('08_Moteur'!R53+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S53)-'08_Moteur'!U53,IF(L56="Regrouper (-1 classe)",H56+('08_Moteur'!AI53-MAX(1,'08_Moteur'!AI53-1))*'08_Moteur'!U53,H56)))</f>
+        <f>IF(L56="Ne pas lancer",0,IF(L56="Ouvrir +1 classe",H56+'08_Moteur'!O53*('08_Moteur'!AE53*'08_Moteur'!AF53-('08_Moteur'!R53+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S53)-'08_Moteur'!U53,IF(L56="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI53&gt;=2,E56&lt;=('08_Moteur'!AI53-1)*'08_Moteur'!O53*1.1),H56+'08_Moteur'!U53,H56),H56)))</f>
         <v/>
       </c>
       <c r="O56" s="17">
@@ -7016,11 +7016,11 @@
         <v/>
       </c>
       <c r="J57" s="70">
-        <f>IF(H57&lt;0,"🔴 Restructurer (mutualiser)",IF(I57&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H57&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI54&gt;=2,E57&lt;=('08_Moteur'!AI54-1)*'08_Moteur'!O54*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I57&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K57" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI54&gt;=2,TEXT(IFERROR(E57/(('08_Moteur'!AI54-1)*'08_Moteur'!O54),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L57" s="21" t="inlineStr">
@@ -7033,7 +7033,7 @@
         <v/>
       </c>
       <c r="N57" s="17">
-        <f>IF(L57="Ne pas lancer",0,IF(L57="Ouvrir +1 classe",H57+'08_Moteur'!O54*('08_Moteur'!AE54*'08_Moteur'!AF54-('08_Moteur'!R54+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S54)-'08_Moteur'!U54,IF(L57="Regrouper (-1 classe)",H57+('08_Moteur'!AI54-MAX(1,'08_Moteur'!AI54-1))*'08_Moteur'!U54,H57)))</f>
+        <f>IF(L57="Ne pas lancer",0,IF(L57="Ouvrir +1 classe",H57+'08_Moteur'!O54*('08_Moteur'!AE54*'08_Moteur'!AF54-('08_Moteur'!R54+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S54)-'08_Moteur'!U54,IF(L57="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI54&gt;=2,E57&lt;=('08_Moteur'!AI54-1)*'08_Moteur'!O54*1.1),H57+'08_Moteur'!U54,H57),H57)))</f>
         <v/>
       </c>
       <c r="O57" s="17">
@@ -7104,7 +7104,7 @@
         <v/>
       </c>
       <c r="N58" s="17">
-        <f>IF(L58="Ne pas lancer",0,IF(L58="Ouvrir +1 classe",H58+'08_Moteur'!O55*('08_Moteur'!AE55*'08_Moteur'!AF55-('08_Moteur'!R55+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S55)-'08_Moteur'!U55,IF(L58="Regrouper (-1 classe)",H58+('08_Moteur'!AI55-MAX(1,'08_Moteur'!AI55-1))*'08_Moteur'!U55,H58)))</f>
+        <f>IF(L58="Ne pas lancer",0,IF(L58="Ouvrir +1 classe",H58+'08_Moteur'!O55*('08_Moteur'!AE55*'08_Moteur'!AF55-('08_Moteur'!R55+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S55)-'08_Moteur'!U55,IF(L58="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI55&gt;=2,E58&lt;=('08_Moteur'!AI55-1)*'08_Moteur'!O55*1.1),H58+'08_Moteur'!U55,H58),H58)))</f>
         <v/>
       </c>
       <c r="O58" s="17">
@@ -7158,11 +7158,11 @@
         <v/>
       </c>
       <c r="J59" s="70">
-        <f>IF(H59&lt;0,"🔴 Restructurer (mutualiser)",IF(I59&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H59&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI56&gt;=2,E59&lt;=('08_Moteur'!AI56-1)*'08_Moteur'!O56*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I59&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K59" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI56&gt;=2,TEXT(IFERROR(E59/(('08_Moteur'!AI56-1)*'08_Moteur'!O56),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L59" s="21" t="inlineStr">
@@ -7175,7 +7175,7 @@
         <v/>
       </c>
       <c r="N59" s="17">
-        <f>IF(L59="Ne pas lancer",0,IF(L59="Ouvrir +1 classe",H59+'08_Moteur'!O56*('08_Moteur'!AE56*'08_Moteur'!AF56-('08_Moteur'!R56+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S56)-'08_Moteur'!U56,IF(L59="Regrouper (-1 classe)",H59+('08_Moteur'!AI56-MAX(1,'08_Moteur'!AI56-1))*'08_Moteur'!U56,H59)))</f>
+        <f>IF(L59="Ne pas lancer",0,IF(L59="Ouvrir +1 classe",H59+'08_Moteur'!O56*('08_Moteur'!AE56*'08_Moteur'!AF56-('08_Moteur'!R56+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S56)-'08_Moteur'!U56,IF(L59="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI56&gt;=2,E59&lt;=('08_Moteur'!AI56-1)*'08_Moteur'!O56*1.1),H59+'08_Moteur'!U56,H59),H59)))</f>
         <v/>
       </c>
       <c r="O59" s="17">
@@ -7229,11 +7229,11 @@
         <v/>
       </c>
       <c r="J60" s="70">
-        <f>IF(H60&lt;0,"🔴 Restructurer (mutualiser)",IF(I60&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H60&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI57&gt;=2,E60&lt;=('08_Moteur'!AI57-1)*'08_Moteur'!O57*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I60&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K60" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI57&gt;=2,TEXT(IFERROR(E60/(('08_Moteur'!AI57-1)*'08_Moteur'!O57),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L60" s="21" t="inlineStr">
@@ -7246,7 +7246,7 @@
         <v/>
       </c>
       <c r="N60" s="17">
-        <f>IF(L60="Ne pas lancer",0,IF(L60="Ouvrir +1 classe",H60+'08_Moteur'!O57*('08_Moteur'!AE57*'08_Moteur'!AF57-('08_Moteur'!R57+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S57)-'08_Moteur'!U57,IF(L60="Regrouper (-1 classe)",H60+('08_Moteur'!AI57-MAX(1,'08_Moteur'!AI57-1))*'08_Moteur'!U57,H60)))</f>
+        <f>IF(L60="Ne pas lancer",0,IF(L60="Ouvrir +1 classe",H60+'08_Moteur'!O57*('08_Moteur'!AE57*'08_Moteur'!AF57-('08_Moteur'!R57+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S57)-'08_Moteur'!U57,IF(L60="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI57&gt;=2,E60&lt;=('08_Moteur'!AI57-1)*'08_Moteur'!O57*1.1),H60+'08_Moteur'!U57,H60),H60)))</f>
         <v/>
       </c>
       <c r="O60" s="17">
@@ -7317,7 +7317,7 @@
         <v/>
       </c>
       <c r="N61" s="17">
-        <f>IF(L61="Ne pas lancer",0,IF(L61="Ouvrir +1 classe",H61+'08_Moteur'!O58*('08_Moteur'!AE58*'08_Moteur'!AF58-('08_Moteur'!R58+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S58)-'08_Moteur'!U58,IF(L61="Regrouper (-1 classe)",H61+('08_Moteur'!AI58-MAX(1,'08_Moteur'!AI58-1))*'08_Moteur'!U58,H61)))</f>
+        <f>IF(L61="Ne pas lancer",0,IF(L61="Ouvrir +1 classe",H61+'08_Moteur'!O58*('08_Moteur'!AE58*'08_Moteur'!AF58-('08_Moteur'!R58+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S58)-'08_Moteur'!U58,IF(L61="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI58&gt;=2,E61&lt;=('08_Moteur'!AI58-1)*'08_Moteur'!O58*1.1),H61+'08_Moteur'!U58,H61),H61)))</f>
         <v/>
       </c>
       <c r="O61" s="17">
@@ -7371,11 +7371,11 @@
         <v/>
       </c>
       <c r="J62" s="70">
-        <f>IF(H62&lt;0,"🔴 Restructurer (mutualiser)",IF(I62&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H62&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI59&gt;=2,E62&lt;=('08_Moteur'!AI59-1)*'08_Moteur'!O59*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I62&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K62" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI59&gt;=2,TEXT(IFERROR(E62/(('08_Moteur'!AI59-1)*'08_Moteur'!O59),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L62" s="21" t="inlineStr">
@@ -7388,7 +7388,7 @@
         <v/>
       </c>
       <c r="N62" s="17">
-        <f>IF(L62="Ne pas lancer",0,IF(L62="Ouvrir +1 classe",H62+'08_Moteur'!O59*('08_Moteur'!AE59*'08_Moteur'!AF59-('08_Moteur'!R59+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S59)-'08_Moteur'!U59,IF(L62="Regrouper (-1 classe)",H62+('08_Moteur'!AI59-MAX(1,'08_Moteur'!AI59-1))*'08_Moteur'!U59,H62)))</f>
+        <f>IF(L62="Ne pas lancer",0,IF(L62="Ouvrir +1 classe",H62+'08_Moteur'!O59*('08_Moteur'!AE59*'08_Moteur'!AF59-('08_Moteur'!R59+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S59)-'08_Moteur'!U59,IF(L62="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI59&gt;=2,E62&lt;=('08_Moteur'!AI59-1)*'08_Moteur'!O59*1.1),H62+'08_Moteur'!U59,H62),H62)))</f>
         <v/>
       </c>
       <c r="O62" s="17">
@@ -7442,11 +7442,11 @@
         <v/>
       </c>
       <c r="J63" s="70">
-        <f>IF(H63&lt;0,"🔴 Restructurer (mutualiser)",IF(I63&lt;0.55,"🟡 Regrouper les classes","🟢 Maintenir"))</f>
+        <f>IF(H63&lt;0,"🔴 Restructurer (mutualiser)",IF(AND('08_Moteur'!AI60&gt;=2,E63&lt;=('08_Moteur'!AI60-1)*'08_Moteur'!O60*1.1),"🟡 Regroupable (−1 classe tient en capacité)",IF(I63&lt;0.55,"🟠 Sous-rempli mais −1 classe déborderait","🟢 Maintenir")))</f>
         <v/>
       </c>
       <c r="K63" s="71">
-        <f>"Poursuite : cohorte déjà inscrite (issue de l'année inférieure) → ni lancement ni capture ; seul levier = regrouper / mutualiser les classes"</f>
+        <f>"Poursuite : cohorte déjà inscrite → seul levier = regrouper. −1 classe créditée uniquement si l'effectif tient dans les classes restantes (capacité +10% tolérée). Remplissage si −1 classe : "&amp;IF('08_Moteur'!AI60&gt;=2,TEXT(IFERROR(E63/(('08_Moteur'!AI60-1)*'08_Moteur'!O60),0),"0%"),"n/a (1 seule classe)")</f>
         <v/>
       </c>
       <c r="L63" s="21" t="inlineStr">
@@ -7459,7 +7459,7 @@
         <v/>
       </c>
       <c r="N63" s="17">
-        <f>IF(L63="Ne pas lancer",0,IF(L63="Ouvrir +1 classe",H63+'08_Moteur'!O60*('08_Moteur'!AE60*'08_Moteur'!AF60-('08_Moteur'!R60+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S60)-'08_Moteur'!U60,IF(L63="Regrouper (-1 classe)",H63+('08_Moteur'!AI60-MAX(1,'08_Moteur'!AI60-1))*'08_Moteur'!U60,H63)))</f>
+        <f>IF(L63="Ne pas lancer",0,IF(L63="Ouvrir +1 classe",H63+'08_Moteur'!O60*('08_Moteur'!AE60*'08_Moteur'!AF60-('08_Moteur'!R60+'02_Leviers'!$D$19)*(1+'02_Leviers'!$G$11)-'08_Moteur'!S60)-'08_Moteur'!U60,IF(L63="Regrouper (-1 classe)",IF(AND('08_Moteur'!AI60&gt;=2,E63&lt;=('08_Moteur'!AI60-1)*'08_Moteur'!O60*1.1),H63+'08_Moteur'!U60,H63),H63)))</f>
         <v/>
       </c>
       <c r="O63" s="17">

</xml_diff>

<commit_message>
Nouvelle feuille 11c_Cascade : allocation en cascade + effet d'une fermeture
Cas d'école (bac à sable) qui implémente l'allocation descendante de la
structure non-évitable : siège groupe → marque (au CA) → campus (au nb
d'étudiants) → promo (au NOMBRE DE CLASSES). Deux enseignements montrés
d'emblée :
- Fermer une promo à contribution NÉGATIVE (Mastère 2) fait MONTER l'EBITDA
  campus (Δ +15 000 €).
- La structure non-évitable se redivise sur les classes restantes → le
  résultat tout compris d'une promo marginale (Bachelor 3) bascule en rouge,
  bien que l'EBITDA groupe s'améliore (effet d'ALLOCATION, pas une vraie perte).
Décision Maintenir/Fermer par promo, mise en rouge auto des résultats négatifs,
EBITDA campus avant/après. N'affecte pas le P&L officiel.

0 erreur de formule ; EBITDA N-1 maintenu à 14,6 % ; 17 feuilles.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -20,9 +20,10 @@
     <sheet name="10_PnL" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="11_Simulateur" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="11b_Mutualisation" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="12_Sensibilite" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="13_Simulation" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="14_Mapping_Tagetik" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="11c_Cascade" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="12_Sensibilite" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="13_Simulation" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="14_Mapping_Tagetik" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -195,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -404,6 +405,9 @@
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -423,6 +427,20 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -721,6 +739,26 @@
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="C21" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif budget de la promo.</t>
+      </text>
+    </comment>
+    <comment ref="I21" authorId="0" shapeId="0">
+      <text>
+        <t>Ton choix. Menu restreint selon l'année : entrée = lancer/capter ; poursuite = seulement regrouper.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment14.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Levier testé et son incrément.</t>
@@ -740,7 +778,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment15.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
@@ -1679,7 +1717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D29"/>
+  <dimension ref="B2:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1858,109 +1896,122 @@
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>12_Sensibilite</t>
+          <t>11c_Cascade</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Impact € sur l'EBITDA par levier (sens unique)</t>
+          <t>Allocation EN CASCADE (marque→campus→classe) + effet d'une fermeture (bénéfique vs entraînement)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>13_Simulation</t>
+          <t>12_Sensibilite</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>KPIs, € à risque, taux d'alternance/sécurisation</t>
+          <t>Impact € sur l'EBITDA par levier (sens unique)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
+          <t>13_Simulation</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>KPIs, € à risque, taux d'alternance/sécurisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
           <t>14_Mapping_Tagetik</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Passerelle Tagetik</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Légende</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="7" t="inlineStr">
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve"> exemple </t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Saisie / donnée réelle</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="9" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve"> exemple </t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Formule</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="10" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve"> exemple </t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Lien inter-feuilles</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="11" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> exemple </t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Hypothèse à remplir</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="12" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Marques/campus réels EDUSERVICES ; montants ILLUSTRATIFS calibrés sur des ordres de grandeur sourcés (scolarité 8-11 k€, NPEC ~7-10 k€, marge EBITDA ~20 %, classe ~30). À remplacer par le réel.</t>
         </is>
       </c>
     </row>
-    <row r="29"/>
+    <row r="30"/>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="25">
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="C15:D15"/>
+    <mergeCell ref="B23:D23"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C20:D20"/>
@@ -1970,14 +2021,14 @@
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="B5:D5"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="B29:D30"/>
     <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C27:D27"/>
     <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C23:D23"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B28:D29"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="B22:D22"/>
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="C18:D18"/>
@@ -8822,6 +8873,683 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A2:AS33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Allocation de la structure EN CASCADE (marque → campus → classe) &amp; effet d'une fermeture</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Cas d'école (bac à sable, montants illustratifs). La structure NON-ÉVITABLE descend en cascade : au CA par marque, puis au nb d'étudiants par campus, puis au NB DE CLASSES par promo (3 classes → /3). Fermer une promo ne supprime pas la structure : elle se redivise sur les classes restantes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>1) Descente de la structure non-évitable  —  siège groupe → marque (au CA) → campus (au nb d'étudiants)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Siège / structure GROUPE à répartir (€) :</t>
+        </is>
+      </c>
+      <c r="E6" s="74" t="n">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Marque</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>CA (€)</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Part CA</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Siège alloué marque</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>MBway (focus)</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="D9" s="52">
+        <f>IFERROR(C9/SUM($C$9:$C$11),0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="17">
+        <f>D9*$E$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>ISCOM</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D10" s="52">
+        <f>IFERROR(C10/SUM($C$9:$C$11),0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="17">
+        <f>D10*$E$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Pigier</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D11" s="52">
+        <f>IFERROR(C11/SUM($C$9:$C$11),0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="17">
+        <f>D11*$E$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C12" s="46">
+        <f>SUM(C9:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="44" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="E12" s="46">
+        <f>SUM(E9:E11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Campus MBway</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Effectif</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Part effectif</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Siège campus</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Fixe campus (loyer+perm)</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>Envelope campus</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Lyon (focus)</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="n">
+        <v>260</v>
+      </c>
+      <c r="D15" s="52">
+        <f>IFERROR(C15/SUM($C$15:$C$17),0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="17">
+        <f>D15*$E$9</f>
+        <v/>
+      </c>
+      <c r="F15" s="41" t="n">
+        <v>205000</v>
+      </c>
+      <c r="G15" s="54">
+        <f>E15+F15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="n">
+        <v>310</v>
+      </c>
+      <c r="D16" s="52">
+        <f>IFERROR(C16/SUM($C$15:$C$17),0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="17">
+        <f>D16*$E$9</f>
+        <v/>
+      </c>
+      <c r="F16" s="41" t="n">
+        <v>300000</v>
+      </c>
+      <c r="G16" s="54">
+        <f>E16+F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="n">
+        <v>240</v>
+      </c>
+      <c r="D17" s="52">
+        <f>IFERROR(C17/SUM($C$15:$C$17),0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="17">
+        <f>D17*$E$9</f>
+        <v/>
+      </c>
+      <c r="F17" s="41" t="n">
+        <v>240000</v>
+      </c>
+      <c r="G17" s="54">
+        <f>E17+F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C18" s="45">
+        <f>SUM(C15:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="44" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="E18" s="46">
+        <f>SUM(E15:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="46">
+        <f>SUM(F15:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="46">
+        <f>SUM(G15:G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2) Répartition campus → promos AU NOMBRE DE CLASSES  —  Campus focus : MBway Lyon  (décide sur la CONTRIBUTION ; la structure se redivise)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Promo (MBway Lyon)</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Effectif</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Classes</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Contribution
+(évitable)</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Struct/classe
+(avant)</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>Struct allouée
+(avant)</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Résultat t.c.
+(avant)</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>Décision</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>Classes
+après</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>Struct allouée
+(après)</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>Résultat t.c.
+(après)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Bachelor 1</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="n">
+        <v>66</v>
+      </c>
+      <c r="D22" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="41" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F22" s="17">
+        <f>IFERROR($G$15/SUM($D$22:$D$25),0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="17">
+        <f>D22*F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="54">
+        <f>E22-G22</f>
+        <v/>
+      </c>
+      <c r="I22" s="21" t="inlineStr">
+        <is>
+          <t>Maintenir</t>
+        </is>
+      </c>
+      <c r="J22" s="50">
+        <f>IF(I22="Fermer",0,D22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="17">
+        <f>IF(I22="Fermer",0,J22*IFERROR($G$15/SUM($J$22:$J$25),0))</f>
+        <v/>
+      </c>
+      <c r="L22" s="54">
+        <f>IF(I22="Fermer",0,E22-K22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Bachelor 2</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="n">
+        <v>56</v>
+      </c>
+      <c r="D23" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="41" t="n">
+        <v>120000</v>
+      </c>
+      <c r="F23" s="17">
+        <f>IFERROR($G$15/SUM($D$22:$D$25),0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="17">
+        <f>D23*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="54">
+        <f>E23-G23</f>
+        <v/>
+      </c>
+      <c r="I23" s="21" t="inlineStr">
+        <is>
+          <t>Maintenir</t>
+        </is>
+      </c>
+      <c r="J23" s="50">
+        <f>IF(I23="Fermer",0,D23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="17">
+        <f>IF(I23="Fermer",0,J23*IFERROR($G$15/SUM($J$22:$J$25),0))</f>
+        <v/>
+      </c>
+      <c r="L23" s="54">
+        <f>IF(I23="Fermer",0,E23-K23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Bachelor 3</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="n">
+        <v>50</v>
+      </c>
+      <c r="D24" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="41" t="n">
+        <v>105000</v>
+      </c>
+      <c r="F24" s="17">
+        <f>IFERROR($G$15/SUM($D$22:$D$25),0)</f>
+        <v/>
+      </c>
+      <c r="G24" s="17">
+        <f>D24*F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="54">
+        <f>E24-G24</f>
+        <v/>
+      </c>
+      <c r="I24" s="21" t="inlineStr">
+        <is>
+          <t>Maintenir</t>
+        </is>
+      </c>
+      <c r="J24" s="50">
+        <f>IF(I24="Fermer",0,D24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="17">
+        <f>IF(I24="Fermer",0,J24*IFERROR($G$15/SUM($J$22:$J$25),0))</f>
+        <v/>
+      </c>
+      <c r="L24" s="54">
+        <f>IF(I24="Fermer",0,E24-K24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Mastère 2 (sous-rempli)</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="41" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="F25" s="17">
+        <f>IFERROR($G$15/SUM($D$22:$D$25),0)</f>
+        <v/>
+      </c>
+      <c r="G25" s="17">
+        <f>D25*F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="54">
+        <f>E25-G25</f>
+        <v/>
+      </c>
+      <c r="I25" s="21" t="inlineStr">
+        <is>
+          <t>Fermer</t>
+        </is>
+      </c>
+      <c r="J25" s="50">
+        <f>IF(I25="Fermer",0,D25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="17">
+        <f>IF(I25="Fermer",0,J25*IFERROR($G$15/SUM($J$22:$J$25),0))</f>
+        <v/>
+      </c>
+      <c r="L25" s="54">
+        <f>IF(I25="Fermer",0,E25-K25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="43" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C26" s="45">
+        <f>SUM(C22:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="45">
+        <f>SUM(D22:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="46">
+        <f>SUM(E22:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="44" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G26" s="46">
+        <f>SUM(G22:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="46">
+        <f>SUM(H22:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="44" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="J26" s="45">
+        <f>SUM(J22:J25)</f>
+        <v/>
+      </c>
+      <c r="K26" s="46">
+        <f>SUM(K22:K25)</f>
+        <v/>
+      </c>
+      <c r="L26" s="46">
+        <f>SUM(L22:L25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>EBITDA campus AVANT :</t>
+        </is>
+      </c>
+      <c r="E28" s="54">
+        <f>SUM(E22:E25)-$G$15</f>
+        <v/>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>EBITDA campus APRÈS :</t>
+        </is>
+      </c>
+      <c r="I28" s="46">
+        <f>SUMIFS(E22:E25,I22:I25,"&lt;&gt;Fermer")-$G$15</f>
+        <v/>
+      </c>
+      <c r="J28" s="30" t="n"/>
+      <c r="K28" s="19" t="inlineStr">
+        <is>
+          <t>Δ EBITDA :</t>
+        </is>
+      </c>
+      <c r="L28" s="20">
+        <f>I28-E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>🧪 LECTURE (deux enseignements). ① On DÉCIDE sur la CONTRIBUTION (évitable) : fermer la promo à contribution NÉGATIVE (Mastère 2) fait MONTER l'EBITDA campus (Δ = +15 000 € = la perte évitée). ② MAIS la structure est NON-ÉVITABLE : en fermant, ses classes quittent le dénominateur → la structure se redivise sur les classes restantes (÷ nb de classes) → le « résultat tout compris » d'une promo marginale (Bachelor 3) bascule EN ROUGE, alors même que l'EBITDA groupe s'est amélioré. Le drag est un effet d'ALLOCATION (comptable), pas une vraie perte : la structure était déjà là. À l'inverse, fermer une promo à contribution POSITIVE (essaie Bachelor 1) fait CHUTER l'EBITDA et enfonce toutes les voisines. N'affecte pas le P&amp;L officiel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="B20:L20"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B30:L33"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="B6:D6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H22:H25">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L22:L25">
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="I22 I23 I24 I25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Maintenir,Fermer"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A2:AS11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8932,7 +9660,7 @@
           <t>Exposition financement alternance (€ à sécuriser) :</t>
         </is>
       </c>
-      <c r="D11" s="74">
+      <c r="D11" s="75">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$G$9)</f>
         <v/>
       </c>
@@ -8948,7 +9676,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9176,20 +9904,20 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="75" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>€ à sécuriser (exposition)</t>
         </is>
       </c>
-      <c r="C15" s="76">
+      <c r="C15" s="77">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$AD$3:$AD$60*'08_Moteur'!$AE$3:$AE$60)*(1-'02_Leviers'!$G$9)</f>
         <v/>
       </c>
-      <c r="D15" s="76">
+      <c r="D15" s="77">
         <f>SUMPRODUCT(('08_Moteur'!$E$3:$E$60="ALT")*'08_Moteur'!$G$3:$G$60*'08_Moteur'!$L$3:$L$60)*(1-'02_Leviers'!$D$20)</f>
         <v/>
       </c>
-      <c r="E15" s="77">
+      <c r="E15" s="78">
         <f>IFERROR(C15/D15-1,0)</f>
         <v/>
       </c>
@@ -9203,7 +9931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9252,7 +9980,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="78" t="inlineStr">
+      <c r="B6" s="79" t="inlineStr">
         <is>
           <t>Marque / Campus</t>
         </is>
@@ -9269,7 +9997,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="78" t="inlineStr">
+      <c r="B7" s="79" t="inlineStr">
         <is>
           <t>Programme × Année × Modalité</t>
         </is>
@@ -9286,7 +10014,7 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="78" t="inlineStr">
+      <c r="B8" s="79" t="inlineStr">
         <is>
           <t>Params (capacité, heures…)</t>
         </is>
@@ -9303,7 +10031,7 @@
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="78" t="inlineStr">
+      <c r="B9" s="79" t="inlineStr">
         <is>
           <t>Historique N-2/N-1</t>
         </is>
@@ -9320,7 +10048,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="78" t="inlineStr">
+      <c r="B10" s="79" t="inlineStr">
         <is>
           <t>Cohortes / taux de passage</t>
         </is>
@@ -9337,7 +10065,7 @@
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="78" t="inlineStr">
+      <c r="B11" s="79" t="inlineStr">
         <is>
           <t>Sécurisation &amp; recouvrement</t>
         </is>
@@ -9354,7 +10082,7 @@
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="78" t="inlineStr">
+      <c r="B12" s="79" t="inlineStr">
         <is>
           <t>Objectifs (cadrage)</t>
         </is>
@@ -9371,7 +10099,7 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="78" t="inlineStr">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>Décisions ouvrir/fermer</t>
         </is>
@@ -9388,7 +10116,7 @@
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="78" t="inlineStr">
+      <c r="B14" s="79" t="inlineStr">
         <is>
           <t>Allocation structure</t>
         </is>

</xml_diff>

<commit_message>
11c_Cascade : campus focus = ISCOM Toulouse (petit campus, marges fines)
Bascule le cas cascade sur ISCOM Toulouse, où les trois enseignements se
voient d'un coup, sur données réelles et EBITDA campus positif (+66 k€) :
- Mastère 2 en extinction (contribution négative) → fermer bénéfique (Δ +2 976).
- Bachelor 3 (résultat tout compris +19 k€) bascule EN ROUGE (-1,4 k€) quand on
  ferme M2 : effet d'entraînement (redivision de la structure).
- Mastère 1 EN ROUGE en résultat tout compris (-24 k€) mais contribution
  POSITIVE (+140 k€) → le piège : ne pas le fermer.
Onglet parametré (marque/campus focus en variables) ; objet de l'onglet explicité.

0 erreur ; EBITDA N-1 14,6 %.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -8882,7 +8882,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
@@ -8905,21 +8905,21 @@
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Allocation EN CASCADE sur un VRAI campus (MBway Lyon) &amp; effet d'une fermeture</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1">
+          <t>Allocation EN CASCADE sur un VRAI campus (ISCOM Toulouse) &amp; effet d'une fermeture</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Chiffres RÉELS du moteur (structure, CA, effectifs, économie unitaire feuille 05). La structure NON-ÉVITABLE descend en cascade : groupe → marque au CA → campus au nb d'étudiants → promo au NOMBRE DE CLASSES. Change l'effectif SCÉNARIO (bleu) d'une promo : sa contribution se recalcule, et tu vois quand fermer devient bénéfique… ou pas.</t>
+          <t>OBJET DE L'ONGLET : montrer, sur un vrai campus, QUAND fermer une promo est bénéfique (ou pas). Chiffres RÉELS du moteur. La structure NON-ÉVITABLE descend en cascade : groupe → marque au CA → campus au nb d'étudiants → promo au NOMBRE DE CLASSES. On DÉCIDE sur la CONTRIBUTION (évitable) ; le « résultat tout compris » (après structure) n'est qu'informatif. Change l'effectif SCÉNARIO (bleu) : contribution et classes se recalculent.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>1) Structure non-évitable de MBway Lyon  —  siège groupe cascadé (CA marque → effectif campus) + loyer &amp; permanents directs (réels, feuille 09)</t>
+          <t>1) Structure non-évitable de ISCOM Toulouse  —  siège groupe cascadé (CA marque → effectif campus) + loyer &amp; permanents directs (réels, feuille 09)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -8949,16 +8949,16 @@
     <row r="7">
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>× Part MBway au CA :</t>
+          <t>× Part ISCOM au CA :</t>
         </is>
       </c>
       <c r="G7" s="69">
-        <f>IFERROR(SUMIFS('08_Moteur'!$AH$3:$AH$60,'08_Moteur'!$A$3:$A$60,"MBway")/SUM('08_Moteur'!$AH$3:$AH$60),0)</f>
+        <f>IFERROR(SUMIFS('08_Moteur'!$AH$3:$AH$60,'08_Moteur'!$A$3:$A$60,"ISCOM")/SUM('08_Moteur'!$AH$3:$AH$60),0)</f>
         <v/>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>→ Siège MBway :</t>
+          <t>→ Siège ISCOM :</t>
         </is>
       </c>
       <c r="I7" s="17">
@@ -8969,16 +8969,16 @@
     <row r="8">
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>× Part Lyon dans MBway (aux effectifs) :</t>
+          <t>× Part Toulouse dans ISCOM (aux effectifs) :</t>
         </is>
       </c>
       <c r="G8" s="69">
-        <f>IFERROR(SUMIFS('08_Moteur'!$AD$3:$AD$60,'08_Moteur'!$A$3:$A$60,"MBway",'08_Moteur'!$B$3:$B$60,"Lyon")/SUMIFS('08_Moteur'!$AD$3:$AD$60,'08_Moteur'!$A$3:$A$60,"MBway"),0)</f>
+        <f>IFERROR(SUMIFS('08_Moteur'!$AD$3:$AD$60,'08_Moteur'!$A$3:$A$60,"ISCOM",'08_Moteur'!$B$3:$B$60,"Toulouse")/SUMIFS('08_Moteur'!$AD$3:$AD$60,'08_Moteur'!$A$3:$A$60,"ISCOM"),0)</f>
         <v/>
       </c>
       <c r="H8" s="19" t="inlineStr">
         <is>
-          <t>→ Siège Lyon :</t>
+          <t>→ Siège Toulouse :</t>
         </is>
       </c>
       <c r="I8" s="17">
@@ -8989,29 +8989,29 @@
     <row r="9">
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Loyer Lyon (réel, feuille 09) :</t>
+          <t>Loyer Toulouse (réel, feuille 09) :</t>
         </is>
       </c>
       <c r="I9" s="16">
-        <f>'09_Allocation'!E7</f>
+        <f>'09_Allocation'!E12</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Permanents Lyon (réel, feuille 09) :</t>
+          <t>Permanents Toulouse (réel, feuille 09) :</t>
         </is>
       </c>
       <c r="I10" s="16">
-        <f>'09_Allocation'!F7</f>
+        <f>'09_Allocation'!F12</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>ENVELOPE Lyon = siège Lyon + loyer + permanents (NON-ÉVITABLE) :</t>
+          <t>ENVELOPE Toulouse = siège + loyer + permanents (NON-ÉVITABLE) :</t>
         </is>
       </c>
       <c r="I11" s="46">
@@ -9022,7 +9022,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2) Répartition Lyon → promos AU NOMBRE DE CLASSES + décision  (change l'effectif bleu ; le rouge = résultat tout compris &lt; 0)</t>
+          <t>2) Répartition campus → promos AU NOMBRE DE CLASSES + décision  (change l'effectif bleu ; le rouge = résultat tout compris &lt; 0)</t>
         </is>
       </c>
       <c r="C13" s="4" t="n"/>
@@ -9046,7 +9046,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Promo (MBway Lyon)</t>
+          <t>Promo (ISCOM Toulouse)</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -9148,11 +9148,11 @@
         </is>
       </c>
       <c r="C15" s="48">
-        <f>'08_Moteur'!AD8</f>
+        <f>'08_Moteur'!AD33</f>
         <v/>
       </c>
       <c r="D15" s="74" t="n">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="E15" s="50">
         <f>IF(D15&lt;=0,0,MAX(1,ROUNDUP(D15/P15,0)))</f>
@@ -9199,13 +9199,13 @@
         <v>32</v>
       </c>
       <c r="Q15" s="41" t="n">
-        <v>34800</v>
+        <v>37200</v>
       </c>
       <c r="R15" s="41" t="n">
         <v>8500</v>
       </c>
       <c r="S15" s="41" t="n">
-        <v>1334</v>
+        <v>1484</v>
       </c>
       <c r="T15" s="41" t="n">
         <v>320</v>
@@ -9218,11 +9218,11 @@
         </is>
       </c>
       <c r="C16" s="48">
-        <f>'08_Moteur'!AD9</f>
+        <f>'08_Moteur'!AD34</f>
         <v/>
       </c>
       <c r="D16" s="74" t="n">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="E16" s="50">
         <f>IF(D16&lt;=0,0,MAX(1,ROUNDUP(D16/P16,0)))</f>
@@ -9269,13 +9269,13 @@
         <v>32</v>
       </c>
       <c r="Q16" s="41" t="n">
-        <v>32480</v>
+        <v>34720</v>
       </c>
       <c r="R16" s="41" t="n">
         <v>8000</v>
       </c>
       <c r="S16" s="41" t="n">
-        <v>1334</v>
+        <v>1484</v>
       </c>
       <c r="T16" s="41" t="n">
         <v>0</v>
@@ -9288,11 +9288,11 @@
         </is>
       </c>
       <c r="C17" s="48">
-        <f>'08_Moteur'!AD10</f>
+        <f>'08_Moteur'!AD35</f>
         <v/>
       </c>
       <c r="D17" s="74" t="n">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E17" s="50">
         <f>IF(D17&lt;=0,0,MAX(1,ROUNDUP(D17/P17,0)))</f>
@@ -9339,13 +9339,13 @@
         <v>32</v>
       </c>
       <c r="Q17" s="41" t="n">
-        <v>30160</v>
+        <v>32240</v>
       </c>
       <c r="R17" s="41" t="n">
         <v>8000</v>
       </c>
       <c r="S17" s="41" t="n">
-        <v>1334</v>
+        <v>1484</v>
       </c>
       <c r="T17" s="41" t="n">
         <v>0</v>
@@ -9354,15 +9354,15 @@
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Mastère 1 (ALT)</t>
+          <t>Mastère 1 (ALT — piège)</t>
         </is>
       </c>
       <c r="C18" s="48">
-        <f>'08_Moteur'!AD11</f>
+        <f>'08_Moteur'!AD36</f>
         <v/>
       </c>
       <c r="D18" s="74" t="n">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="E18" s="50">
         <f>IF(D18&lt;=0,0,MAX(1,ROUNDUP(D18/P18,0)))</f>
@@ -9409,13 +9409,13 @@
         <v>26</v>
       </c>
       <c r="Q18" s="41" t="n">
-        <v>33600</v>
+        <v>35520</v>
       </c>
       <c r="R18" s="41" t="n">
         <v>9000</v>
       </c>
       <c r="S18" s="41" t="n">
-        <v>1454</v>
+        <v>1604</v>
       </c>
       <c r="T18" s="41" t="n">
         <v>600</v>
@@ -9428,11 +9428,11 @@
         </is>
       </c>
       <c r="C19" s="48">
-        <f>'08_Moteur'!AD12</f>
+        <f>'08_Moteur'!AD37</f>
         <v/>
       </c>
       <c r="D19" s="74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" s="50">
         <f>IF(D19&lt;=0,0,MAX(1,ROUNDUP(D19/P19,0)))</f>
@@ -9479,13 +9479,13 @@
         <v>26</v>
       </c>
       <c r="Q19" s="41" t="n">
-        <v>30800</v>
+        <v>32560</v>
       </c>
       <c r="R19" s="41" t="n">
         <v>9000</v>
       </c>
       <c r="S19" s="41" t="n">
-        <v>1454</v>
+        <v>1604</v>
       </c>
       <c r="T19" s="41" t="n">
         <v>0</v>
@@ -9580,7 +9580,7 @@
     <row r="24">
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>🧪 LECTURE (vrai campus, bac à sable). On DÉCIDE sur la CONTRIBUTION (évitable). ① Le Mastère 2 est ici en EXTINCTION (3 étudiants) : sa contribution est NÉGATIVE (une classe coûte plus qu'elle ne rapporte, seuil de rentabilité ≈ 4-5 étudiants) → le fermer fait MONTER l'EBITDA campus = fermeture BÉNÉFIQUE. ② À l'inverse, remets une promo bien remplie (Bachelor 1) sur « Fermer » : l'EBITDA CHUTE (on perd sa contribution) et la structure non-évitable se redivise sur les classes restantes (÷ nb de classes) → le résultat tout compris des voisines se dégrade. Remarque HONNÊTE : avec des promos normalement remplies l'économie unitaire est saine (rentables dès ~5 étudiants), donc fermer n'est JAMAIS bénéfique — ça ne le devient que pour une promo réellement sous-remplie / en extinction. Baisse les effectifs bleus pour rendre une promo marginale et voir l'effet d'entraînement basculer une voisine EN ROUGE. N'affecte pas le P&amp;L officiel.</t>
+          <t>🧪 LECTURE (vrai campus ISCOM Toulouse, bac à sable). On DÉCIDE sur la CONTRIBUTION (évitable), JAMAIS sur le résultat tout compris. Trois enseignements visibles ici : ① FERMER BÉNÉFIQUE — le Mastère 2 est en EXTINCTION (4 étudiants) : sa CONTRIBUTION est négative (une classe coûte plus qu'elle ne rapporte) → le fermer fait MONTER l'EBITDA campus (Δ = perte évitée). ② EFFET D'ENTRAÎNEMENT — en fermant, la structure non-évitable se redivise sur les classes restantes (÷ nb de classes) → le résultat tout compris du Bachelor 3 (déjà mince) bascule EN ROUGE, alors que l'EBITDA s'est amélioré : c'est un effet d'ALLOCATION comptable, pas une vraie perte. ③ LE PIÈGE — le Mastère 1 est EN ROUGE en résultat tout compris (il porte beaucoup de structure) MAIS sa CONTRIBUTION est POSITIVE (~+119 k€) → il NE FAUT PAS le fermer : le fermer FERAIT PERDRE cette contribution et alourdirait tout le monde. Essaie : mets le Mastère 1 sur « Fermer » → l'EBITDA CHUTE. N'affecte pas le P&amp;L officiel.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Documentation complète : objet de chaque onglet + toutes les entêtes annotées
- Note « OBJET DE L'ONGLET » explicite sur le titre des 17 feuilles (guide le
  consultant : à quoi sert la feuille, comment s'en servir).
- Toutes les entêtes de toutes les feuilles ont désormais une note explicative
  (glossaire complété : 11c_Cascade, coefficients marque|campus, params
  programme×année, passerelle Tagetik).

0 erreur de formule.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
+++ b/eduservices/EDUSERVICES_Modele_Pilotage_Budget.xlsx
@@ -519,24 +519,9 @@
     <author>Guide</author>
   </authors>
   <commentList>
-    <comment ref="B5" authorId="0" shapeId="0">
+    <comment ref="B2" authorId="0" shapeId="0">
       <text>
-        <t>Indicateur de pilotage.</t>
-      </text>
-    </comment>
-    <comment ref="C5" authorId="0" shapeId="0">
-      <text>
-        <t>Objectif fixé par la direction (saisie).</t>
-      </text>
-    </comment>
-    <comment ref="D5" authorId="0" shapeId="0">
-      <text>
-        <t>Résultat du budget construit par les drivers (moteur).</t>
-      </text>
-    </comment>
-    <comment ref="E5" authorId="0" shapeId="0">
-      <text>
-        <t>Budget construit − cible.</t>
+        <t>OBJET DE L'ONGLET — Sommaire et mode d'emploi du classeur : rôle de chaque feuille, légende des couleurs, périmètre. Commence ici.</t>
       </text>
     </comment>
   </commentList>
@@ -549,6 +534,81 @@
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Répartir les frais de structure FIXES sur les campus selon un driver (effectifs / CA / m²).</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Campus (ville). Une entité = Marque + Ville.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Marge de contribution (CA − coûts directs évitables).</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Loyer du campus (structure fixe).</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0">
+      <text>
+        <t>Masse salariale permanente (structure fixe).</t>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0">
+      <text>
+        <t>Valeur du driver d'allocation (effectif, CA ou m² selon 02_Leviers).</t>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0">
+      <text>
+        <t>Part du campus dans le driver total.</t>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0">
+      <text>
+        <t>Frais de structure groupe alloués à ce campus.</t>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0">
+      <text>
+        <t>EBITDA du campus = contribution − loyer − permanents − structure allouée.</t>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="0" shapeId="0">
+      <text>
+        <t>Dotations aux amortissements.</t>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0">
+      <text>
+        <t>Résultat d'exploitation = EBITDA − D&amp;A.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Compte de résultat consolidé N-1 vs Budget + PONT d'explication du CA (volume / tarif / sécurisation / frais).</t>
+      </text>
+    </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Ligne du compte de résultat.</t>
@@ -578,12 +638,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — BAC À SABLE de décisions à la maille PROMO (ouvrir / fermer / regrouper) → impact EBITDA AVANT/APRÈS. N'affecte PAS le budget officiel.</t>
+      </text>
+    </comment>
     <comment ref="A5" authorId="0" shapeId="0">
       <text>
         <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
@@ -673,12 +738,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment13.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — BAC À SABLE à la maille CAMPUS × CYCLE : combien de classes / € récupérables en mutualisant le tronc commun, sans dépasser la capacité.</t>
+      </text>
+    </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
@@ -733,15 +803,60 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment14.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — BAC À SABLE : allocation de la structure EN CASCADE (marque→campus→classe) et démonstration de QUAND fermer une promo est bénéfique ou non, sur un vrai campus.</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Promotion = programme × année du campus focus (ISCOM Toulouse).</t>
+      </text>
+    </comment>
+    <comment ref="C14" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif budget RÉEL calculé par le moteur (feuille 08) pour cette promo — sert de référence en regard du scénario.</t>
+      </text>
+    </comment>
+    <comment ref="D14" authorId="0" shapeId="0">
+      <text>
+        <t>Effectif que TU testes (bleu, éditable). Baisse-le pour simuler une promo sous-remplie / en extinction et voir l'effet.</t>
+      </text>
+    </comment>
+    <comment ref="E14" authorId="0" shapeId="0">
+      <text>
+        <t>Nombre de classes = arrondi supérieur (effectif scénario / capacité).</t>
+      </text>
+    </comment>
     <comment ref="F14" authorId="0" shapeId="0">
       <text>
         <t>Chiffre d'affaires budget de la promo.</t>
+      </text>
+    </comment>
+    <comment ref="G14" authorId="0" shapeId="0">
+      <text>
+        <t>CA − coûts directs évitables (enseignement + charge/étu + CAC). C'est LA métrique de décision : on ne ferme que si elle est négative.</t>
+      </text>
+    </comment>
+    <comment ref="H14" authorId="0" shapeId="0">
+      <text>
+        <t>Structure non-évitable du campus (envelope) ÷ nombre total de classes. C'est ce qui se REDIVISE quand on ferme une promo.</t>
+      </text>
+    </comment>
+    <comment ref="I14" authorId="0" shapeId="0">
+      <text>
+        <t>Structure portée par la promo = ses classes × structure/classe.</t>
+      </text>
+    </comment>
+    <comment ref="J14" authorId="0" shapeId="0">
+      <text>
+        <t>Résultat TOUT COMPRIS = contribution − structure allouée. INFORMATIF : peut être négatif alors que la contribution est positive (le piège). JAMAIS un critère de fermeture.</t>
       </text>
     </comment>
     <comment ref="K14" authorId="0" shapeId="0">
@@ -749,21 +864,61 @@
         <t>Ton choix. Menu restreint selon l'année : entrée = lancer/capter ; poursuite = seulement regrouper.</t>
       </text>
     </comment>
+    <comment ref="L14" authorId="0" shapeId="0">
+      <text>
+        <t>Nombre de classes après ta décision (0 si Fermer).</t>
+      </text>
+    </comment>
+    <comment ref="M14" authorId="0" shapeId="0">
+      <text>
+        <t>Structure allouée après décisions : l'envelope (inchangée, non-évitable) se redivise sur les classes RESTANTES → chacune en porte plus.</t>
+      </text>
+    </comment>
+    <comment ref="N14" authorId="0" shapeId="0">
+      <text>
+        <t>Résultat tout compris recalculé après décisions. En ROUGE si &lt; 0 : rend visible l'effet d'entraînement.</t>
+      </text>
+    </comment>
     <comment ref="P14" authorId="0" shapeId="0">
       <text>
         <t>Capacité cible d'une classe (nb d'étudiants).</t>
+      </text>
+    </comment>
+    <comment ref="Q14" authorId="0" shapeId="0">
+      <text>
+        <t>Coût d'enseignement d'une classe (heures × taux horaire), issu du modèle (feuille 05).</t>
+      </text>
+    </comment>
+    <comment ref="R14" authorId="0" shapeId="0">
+      <text>
+        <t>Tarif de scolarité par étudiant et par an (feuille 05).</t>
+      </text>
+    </comment>
+    <comment ref="S14" authorId="0" shapeId="0">
+      <text>
+        <t>Charges variables par étudiant = coût pédagogique + autres charges d'exploitation (feuille 05).</t>
+      </text>
+    </comment>
+    <comment ref="T14" authorId="0" shapeId="0">
+      <text>
+        <t>Coût d'acquisition (achat de leads) par étudiant — uniquement en année d'entrée.</t>
       </text>
     </comment>
   </commentList>
 </comments>
 </file>
 
-<file path=xl/comments/comment14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment15.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Classer les LEVIERS par impact € sur l'EBITDA, pour savoir lequel actionner afin de combler l'écart de cadrage.</t>
+      </text>
+    </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Levier testé et son incrément.</t>
@@ -783,12 +938,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment16.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — TABLEAU DE BORD : KPIs clés Budget vs N-1 (effectif, CA, EBITDA, taux d'alternance, sécurisation, € à sécuriser).</t>
+      </text>
+    </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Indicateur de pilotage.</t>
@@ -813,12 +973,82 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment17.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — PASSERELLE : correspondance entre les objets du modèle Excel et leur implémentation dans CCH Tagetik.</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Notion du modèle Excel à transposer dans Tagetik.</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Objet CCH Tagetik correspondant (dimension, hiérarchie, règle de calcul, workflow…).</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Précision sur la correspondance et le paramétrage Tagetik.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Cadrage TOP-DOWN : la direction saisit les cibles CA/EBITDA ; la feuille affiche l'écart avec le budget CONSTRUIT par les leviers.</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Indicateur de pilotage.</t>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0">
+      <text>
+        <t>Objectif fixé par la direction (saisie).</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Résultat du budget construit par les drivers (moteur).</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>Budget construit − cible.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Guide</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Poste de pilotage : régler les hypothèses (en %), choisir le scénario, et voir les constantes de référence (mesuré vs repli). Tout le budget se recalcule à partir d'ici.</t>
+      </text>
+    </comment>
     <comment ref="C3" authorId="0" shapeId="0">
       <text>
         <t>Scénario actif : change cette cellule et TOUT le budget se recalcule.</t>
@@ -883,12 +1113,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Moduler l'intensité MARKETING et PRIX par marque ET par campus : effort appliqué = levier (feuille 02) × coefficient.</t>
+      </text>
+    </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
@@ -914,16 +1149,26 @@
         <t>Lecture du positionnement (pousser / défendre / maintenir).</t>
       </text>
     </comment>
+    <comment ref="H5" authorId="0" shapeId="0">
+      <text>
+        <t>Clé technique marque|campus : le moteur s'en sert pour retrouver le bon coefficient stratégique du campus.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
-<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Dimensions et plan de comptes du modèle (entités Groupe→Marque→Campus, comptes fixe/variable) — le socle de structuration.</t>
+      </text>
+    </comment>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
         <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
@@ -953,12 +1198,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Données de référence UNITAIRES par programme × année (capacité, heures, taux, pédago, CAC, passage) qui alimentent le moteur. À charger avec le réel.</t>
+      </text>
+    </comment>
     <comment ref="A3" authorId="0" shapeId="0">
       <text>
         <t>Clé technique 'programme|année' pour relier les paramètres au moteur.</t>
@@ -984,9 +1234,19 @@
         <t>Capacité cible d'une classe (nb d'étudiants).</t>
       </text>
     </comment>
+    <comment ref="F3" authorId="0" shapeId="0">
+      <text>
+        <t>Heures d'enseignement délivrées par classe et par an.</t>
+      </text>
+    </comment>
     <comment ref="G3" authorId="0" shapeId="0">
       <text>
         <t>Coût horaire chargé de l'enseignement (vacation), en €.</t>
+      </text>
+    </comment>
+    <comment ref="H3" authorId="0" shapeId="0">
+      <text>
+        <t>Coût pédagogique par étudiant/an, HORS salaires des intervenants (supports, licences, LMS, jury/examens, certifications). 350-670 € selon le domaine.</t>
       </text>
     </comment>
     <comment ref="I3" authorId="0" shapeId="0">
@@ -1003,12 +1263,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Réalisé N-1 par cellule (funnel + cohorte) et historique marketing N-2/N-1 servant à MESURER la conversion, le passage et l'élasticité (pas d'invention).</t>
+      </text>
+    </comment>
     <comment ref="A3" authorId="0" shapeId="0">
       <text>
         <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
@@ -1083,12 +1348,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — Réalisé N-1 par CAMPUS (loyers, ETP permanents, D&amp;A, m²) : la base des coûts de structure.</t>
+      </text>
+    </comment>
     <comment ref="A3" authorId="0" shapeId="0">
       <text>
         <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
@@ -1148,12 +1418,17 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Guide</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>OBJET DE L'ONGLET — CŒUR DE CALCUL : construit le budget de CHAQUE cellule (cohortes, marketing→volume, tarif, financement alternance, point mort). Toutes les feuilles de résultat en découlent.</t>
+      </text>
+    </comment>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
         <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
@@ -1362,71 +1637,6 @@
     <comment ref="AP2" authorId="0" shapeId="0">
       <text>
         <t>Point mort = nb d'étudiants pour couvrir le coût des classes.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Guide</author>
-  </authors>
-  <commentList>
-    <comment ref="B5" authorId="0" shapeId="0">
-      <text>
-        <t>Marque / école du groupe (dimension Entity dans Tagetik).</t>
-      </text>
-    </comment>
-    <comment ref="C5" authorId="0" shapeId="0">
-      <text>
-        <t>Campus (ville). Une entité = Marque + Ville.</t>
-      </text>
-    </comment>
-    <comment ref="D5" authorId="0" shapeId="0">
-      <text>
-        <t>Marge de contribution (CA − coûts directs évitables).</t>
-      </text>
-    </comment>
-    <comment ref="E5" authorId="0" shapeId="0">
-      <text>
-        <t>Loyer du campus (structure fixe).</t>
-      </text>
-    </comment>
-    <comment ref="F5" authorId="0" shapeId="0">
-      <text>
-        <t>Masse salariale permanente (structure fixe).</t>
-      </text>
-    </comment>
-    <comment ref="G5" authorId="0" shapeId="0">
-      <text>
-        <t>Valeur du driver d'allocation (effectif, CA ou m² selon 02_Leviers).</t>
-      </text>
-    </comment>
-    <comment ref="H5" authorId="0" shapeId="0">
-      <text>
-        <t>Part du campus dans le driver total.</t>
-      </text>
-    </comment>
-    <comment ref="I5" authorId="0" shapeId="0">
-      <text>
-        <t>Frais de structure groupe alloués à ce campus.</t>
-      </text>
-    </comment>
-    <comment ref="J5" authorId="0" shapeId="0">
-      <text>
-        <t>EBITDA du campus = contribution − loyer − permanents − structure allouée.</t>
-      </text>
-    </comment>
-    <comment ref="K5" authorId="0" shapeId="0">
-      <text>
-        <t>Dotations aux amortissements.</t>
-      </text>
-    </comment>
-    <comment ref="L5" authorId="0" shapeId="0">
-      <text>
-        <t>Résultat d'exploitation = EBITDA − D&amp;A.</t>
       </text>
     </comment>
   </commentList>
@@ -1722,7 +1932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D30"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1731,6 +1941,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="30" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2040,6 +2251,7 @@
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2049,7 +2261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS20"/>
+  <dimension ref="A1:AS20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2066,6 +2278,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2889,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS25"/>
+  <dimension ref="A1:AS25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2900,6 +3113,7 @@
     <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -7651,7 +7865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS35"/>
+  <dimension ref="A1:AS35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7667,6 +7881,7 @@
     <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -8878,7 +9093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS28"/>
+  <dimension ref="A1:AS28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8902,6 +9117,7 @@
     <col width="11" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -9631,7 +9847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS11"/>
+  <dimension ref="A1:AS11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9640,6 +9856,7 @@
     <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -9763,7 +9980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS15"/>
+  <dimension ref="A1:AS15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9773,6 +9990,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -10018,7 +10236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS14"/>
+  <dimension ref="A1:AS14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -10027,6 +10245,7 @@
     <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -10219,6 +10438,7 @@
     <mergeCell ref="B4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -10228,7 +10448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS14"/>
+  <dimension ref="A1:AS14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -10238,6 +10458,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -10367,7 +10588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -10379,6 +10600,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -10887,7 +11109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS19"/>
+  <dimension ref="A1:AS19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -10900,6 +11122,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -11326,7 +11549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AS32"/>
+  <dimension ref="A1:AS32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11337,6 +11560,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>

</xml_diff>